<commit_message>
Upload SDGym Benchmark Results (SDGym_results_01_01_2026) - Modality: single_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="37">
   <si>
     <t>Dataset</t>
   </si>
@@ -73,13 +73,55 @@
     <t>fake_hotels</t>
   </si>
   <si>
+    <t>child</t>
+  </si>
+  <si>
+    <t>covtype</t>
+  </si>
+  <si>
+    <t>news</t>
+  </si>
+  <si>
+    <t>insurance</t>
+  </si>
+  <si>
+    <t>alarm</t>
+  </si>
+  <si>
+    <t>adult</t>
+  </si>
+  <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>intrusion</t>
+  </si>
+  <si>
+    <t>expedia_hotel_logs</t>
+  </si>
+  <si>
     <t>multi_table</t>
   </si>
   <si>
+    <t>single_table</t>
+  </si>
+  <si>
     <t>IndependentSynthesizer</t>
   </si>
   <si>
     <t>HSASynthesizer</t>
+  </si>
+  <si>
+    <t>GaussianCopulaSynthesizer</t>
+  </si>
+  <si>
+    <t>CTGANSynthesizer</t>
+  </si>
+  <si>
+    <t>RealTabFormerSynthesizer</t>
+  </si>
+  <si>
+    <t>TVAESynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -440,7 +482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -486,10 +528,10 @@
         <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D2">
         <v>33</v>
@@ -513,7 +555,7 @@
         <v>3</v>
       </c>
       <c r="K2" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="L2">
         <v>0.15</v>
@@ -524,10 +566,10 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D3">
         <v>16</v>
@@ -551,7 +593,7 @@
         <v>2</v>
       </c>
       <c r="K3" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="L3">
         <v>0.09</v>
@@ -562,10 +604,10 @@
         <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="D4">
         <v>12</v>
@@ -589,7 +631,7 @@
         <v>3</v>
       </c>
       <c r="K4" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="L4">
         <v>0.6899999999999999</v>
@@ -600,10 +642,10 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="D5">
         <v>16</v>
@@ -627,7 +669,7 @@
         <v>3</v>
       </c>
       <c r="K5" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="L5">
         <v>0.57</v>
@@ -638,10 +680,10 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D6">
         <v>55</v>
@@ -665,7 +707,7 @@
         <v>4</v>
       </c>
       <c r="K6" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="L6">
         <v>85.38</v>
@@ -676,10 +718,10 @@
         <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D7">
         <v>22</v>
@@ -703,7 +745,7 @@
         <v>2</v>
       </c>
       <c r="K7" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="L7">
         <v>293.14</v>
@@ -714,10 +756,10 @@
         <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="D8">
         <v>15</v>
@@ -741,10 +783,352 @@
         <v>2</v>
       </c>
       <c r="K8" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="L8">
         <v>0.05</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9">
+        <v>20</v>
+      </c>
+      <c r="E9">
+        <v>20000</v>
+      </c>
+      <c r="F9">
+        <v>20</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9" t="s">
+        <v>36</v>
+      </c>
+      <c r="L9">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10">
+        <v>55</v>
+      </c>
+      <c r="E10">
+        <v>581012</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>54</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10" t="s">
+        <v>36</v>
+      </c>
+      <c r="L10">
+        <v>255.65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11">
+        <v>59</v>
+      </c>
+      <c r="E11">
+        <v>39644</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>59</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11" t="s">
+        <v>36</v>
+      </c>
+      <c r="L11">
+        <v>18.71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12">
+        <v>27</v>
+      </c>
+      <c r="E12">
+        <v>20000</v>
+      </c>
+      <c r="F12">
+        <v>27</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>1</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
+      <c r="K12" t="s">
+        <v>36</v>
+      </c>
+      <c r="L12">
+        <v>3.34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13">
+        <v>37</v>
+      </c>
+      <c r="E13">
+        <v>20000</v>
+      </c>
+      <c r="F13">
+        <v>37</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>1</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
+      </c>
+      <c r="K13" t="s">
+        <v>36</v>
+      </c>
+      <c r="L13">
+        <v>4.52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14">
+        <v>15</v>
+      </c>
+      <c r="E14">
+        <v>32561</v>
+      </c>
+      <c r="F14">
+        <v>9</v>
+      </c>
+      <c r="G14">
+        <v>6</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>1</v>
+      </c>
+      <c r="K14" t="s">
+        <v>36</v>
+      </c>
+      <c r="L14">
+        <v>3.91</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15">
+        <v>41</v>
+      </c>
+      <c r="E15">
+        <v>299285</v>
+      </c>
+      <c r="F15">
+        <v>29</v>
+      </c>
+      <c r="G15">
+        <v>12</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+      <c r="K15" t="s">
+        <v>36</v>
+      </c>
+      <c r="L15">
+        <v>98.17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16">
+        <v>41</v>
+      </c>
+      <c r="E16">
+        <v>494021</v>
+      </c>
+      <c r="F16">
+        <v>4</v>
+      </c>
+      <c r="G16">
+        <v>37</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>1</v>
+      </c>
+      <c r="K16" t="s">
+        <v>36</v>
+      </c>
+      <c r="L16">
+        <v>162.04</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" t="s">
+        <v>32</v>
+      </c>
+      <c r="D17">
+        <v>25</v>
+      </c>
+      <c r="E17">
+        <v>1000</v>
+      </c>
+      <c r="F17">
+        <v>16</v>
+      </c>
+      <c r="G17">
+        <v>5</v>
+      </c>
+      <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+      <c r="K17" t="s">
+        <v>36</v>
+      </c>
+      <c r="L17">
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_12_23_2025) - Modality: multi_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -52,76 +52,76 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>expedia_hotel_logs</t>
+  </si>
+  <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>alarm</t>
+  </si>
+  <si>
+    <t>intrusion</t>
+  </si>
+  <si>
+    <t>news</t>
+  </si>
+  <si>
+    <t>adult</t>
+  </si>
+  <si>
+    <t>insurance</t>
+  </si>
+  <si>
+    <t>covtype</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
+    <t>fake_hotels</t>
+  </si>
+  <si>
+    <t>financial</t>
+  </si>
+  <si>
+    <t>airbnb-simplified</t>
+  </si>
+  <si>
     <t>NBA</t>
   </si>
   <si>
+    <t>Biodegradability</t>
+  </si>
+  <si>
     <t>Student_loan</t>
   </si>
   <si>
     <t>restbase</t>
   </si>
   <si>
-    <t>Biodegradability</t>
-  </si>
-  <si>
-    <t>financial</t>
-  </si>
-  <si>
-    <t>airbnb-simplified</t>
-  </si>
-  <si>
-    <t>fake_hotels</t>
-  </si>
-  <si>
-    <t>expedia_hotel_logs</t>
-  </si>
-  <si>
-    <t>intrusion</t>
-  </si>
-  <si>
-    <t>adult</t>
-  </si>
-  <si>
-    <t>news</t>
-  </si>
-  <si>
-    <t>child</t>
-  </si>
-  <si>
-    <t>alarm</t>
-  </si>
-  <si>
-    <t>census</t>
-  </si>
-  <si>
-    <t>covtype</t>
-  </si>
-  <si>
-    <t>insurance</t>
+    <t>single_table</t>
   </si>
   <si>
     <t>multi_table</t>
   </si>
   <si>
-    <t>single_table</t>
+    <t>GaussianCopulaSynthesizer</t>
+  </si>
+  <si>
+    <t>RealTabFormerSynthesizer</t>
+  </si>
+  <si>
+    <t>TVAESynthesizer</t>
+  </si>
+  <si>
+    <t>CTGANSynthesizer</t>
+  </si>
+  <si>
+    <t>HSASynthesizer</t>
   </si>
   <si>
     <t>IndependentSynthesizer</t>
-  </si>
-  <si>
-    <t>HSASynthesizer</t>
-  </si>
-  <si>
-    <t>GaussianCopulaSynthesizer</t>
-  </si>
-  <si>
-    <t>TVAESynthesizer</t>
-  </si>
-  <si>
-    <t>RealTabFormerSynthesizer</t>
-  </si>
-  <si>
-    <t>CTGANSynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -534,31 +534,31 @@
         <v>30</v>
       </c>
       <c r="D2">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E2">
-        <v>1219</v>
+        <v>1000</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="G2">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2" t="s">
         <v>36</v>
       </c>
       <c r="L2">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -569,34 +569,34 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D3">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="E3">
-        <v>5288</v>
+        <v>299285</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H3">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" t="s">
         <v>36</v>
       </c>
       <c r="L3">
-        <v>0.09</v>
+        <v>98.17</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -607,34 +607,34 @@
         <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D4">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="E4">
-        <v>19297</v>
+        <v>20000</v>
       </c>
       <c r="F4">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="G4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4" t="s">
         <v>36</v>
       </c>
       <c r="L4">
-        <v>0.6899999999999999</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -645,34 +645,34 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D5">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="E5">
-        <v>21895</v>
+        <v>494021</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K5" t="s">
         <v>36</v>
       </c>
       <c r="L5">
-        <v>0.57</v>
+        <v>162.04</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -683,34 +683,34 @@
         <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D6">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E6">
-        <v>1079680</v>
+        <v>39644</v>
       </c>
       <c r="F6">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>21</v>
+        <v>59</v>
       </c>
       <c r="H6">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I6">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K6" t="s">
         <v>36</v>
       </c>
       <c r="L6">
-        <v>85.38</v>
+        <v>18.71</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -721,34 +721,34 @@
         <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D7">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E7">
-        <v>5751408</v>
+        <v>32561</v>
       </c>
       <c r="F7">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" t="s">
         <v>36</v>
       </c>
       <c r="L7">
-        <v>293.14</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -759,34 +759,34 @@
         <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D8">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E8">
-        <v>668</v>
+        <v>20000</v>
       </c>
       <c r="F8">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="G8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8" t="s">
         <v>36</v>
       </c>
       <c r="L8">
-        <v>0.05</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -794,22 +794,22 @@
         <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D9">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="E9">
-        <v>1000</v>
+        <v>581012</v>
       </c>
       <c r="F9">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G9">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -824,7 +824,7 @@
         <v>36</v>
       </c>
       <c r="L9">
-        <v>0.2</v>
+        <v>255.65</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -832,22 +832,22 @@
         <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D10">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="E10">
-        <v>494021</v>
+        <v>20000</v>
       </c>
       <c r="F10">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="G10">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -862,7 +862,7 @@
         <v>36</v>
       </c>
       <c r="L10">
-        <v>162.04</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -879,28 +879,28 @@
         <v>15</v>
       </c>
       <c r="E11">
-        <v>32561</v>
+        <v>668</v>
       </c>
       <c r="F11">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G11">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K11" t="s">
         <v>36</v>
       </c>
       <c r="L11">
-        <v>3.91</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -914,31 +914,31 @@
         <v>35</v>
       </c>
       <c r="D12">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E12">
-        <v>39644</v>
+        <v>1079680</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G12">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I12">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K12" t="s">
         <v>36</v>
       </c>
       <c r="L12">
-        <v>18.71</v>
+        <v>85.38</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -949,34 +949,34 @@
         <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D13">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E13">
-        <v>20000</v>
+        <v>5751408</v>
       </c>
       <c r="F13">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" t="s">
         <v>36</v>
       </c>
       <c r="L13">
-        <v>3.2</v>
+        <v>293.14</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -987,34 +987,34 @@
         <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D14">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="E14">
-        <v>20000</v>
+        <v>1219</v>
       </c>
       <c r="F14">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I14">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K14" t="s">
         <v>36</v>
       </c>
       <c r="L14">
-        <v>4.52</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1028,31 +1028,31 @@
         <v>34</v>
       </c>
       <c r="D15">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="E15">
-        <v>299285</v>
+        <v>21895</v>
       </c>
       <c r="F15">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="G15">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I15">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K15" t="s">
         <v>36</v>
       </c>
       <c r="L15">
-        <v>98.17</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1066,31 +1066,31 @@
         <v>35</v>
       </c>
       <c r="D16">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="E16">
-        <v>581012</v>
+        <v>5288</v>
       </c>
       <c r="F16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G16">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I16">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K16" t="s">
         <v>36</v>
       </c>
       <c r="L16">
-        <v>255.65</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1101,34 +1101,34 @@
         <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D17">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="E17">
-        <v>20000</v>
+        <v>19297</v>
       </c>
       <c r="F17">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K17" t="s">
         <v>36</v>
       </c>
       <c r="L17">
-        <v>3.34</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_02_01_2026) - Modality: single_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="35">
   <si>
     <t>Dataset</t>
   </si>
@@ -73,27 +73,27 @@
     <t>NBA</t>
   </si>
   <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>news</t>
+  </si>
+  <si>
     <t>intrusion</t>
   </si>
   <si>
-    <t>news</t>
+    <t>alarm</t>
   </si>
   <si>
     <t>insurance</t>
   </si>
   <si>
-    <t>alarm</t>
+    <t>adult</t>
   </si>
   <si>
     <t>covtype</t>
   </si>
   <si>
-    <t>census</t>
-  </si>
-  <si>
-    <t>adult</t>
-  </si>
-  <si>
     <t>child</t>
   </si>
   <si>
@@ -112,16 +112,10 @@
     <t>HSASynthesizer</t>
   </si>
   <si>
-    <t>TVAESynthesizer</t>
-  </si>
-  <si>
-    <t>CTGANSynthesizer</t>
+    <t>RealTabFormerSynthesizer</t>
   </si>
   <si>
     <t>GaussianCopulaSynthesizer</t>
-  </si>
-  <si>
-    <t>RealTabFormerSynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -555,7 +549,7 @@
         <v>4</v>
       </c>
       <c r="K2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L2">
         <v>85.38</v>
@@ -593,7 +587,7 @@
         <v>2</v>
       </c>
       <c r="K3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L3">
         <v>0.05</v>
@@ -631,7 +625,7 @@
         <v>3</v>
       </c>
       <c r="K4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L4">
         <v>0.57</v>
@@ -669,7 +663,7 @@
         <v>3</v>
       </c>
       <c r="K5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L5">
         <v>0.6899999999999999</v>
@@ -707,7 +701,7 @@
         <v>2</v>
       </c>
       <c r="K6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L6">
         <v>0.09</v>
@@ -745,7 +739,7 @@
         <v>2</v>
       </c>
       <c r="K7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L7">
         <v>293.14</v>
@@ -783,7 +777,7 @@
         <v>3</v>
       </c>
       <c r="K8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L8">
         <v>0.15</v>
@@ -803,13 +797,13 @@
         <v>41</v>
       </c>
       <c r="E9">
-        <v>494021</v>
+        <v>299285</v>
       </c>
       <c r="F9">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="G9">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -821,10 +815,10 @@
         <v>1</v>
       </c>
       <c r="K9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L9">
-        <v>162.04</v>
+        <v>98.17</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -835,7 +829,7 @@
         <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D10">
         <v>59</v>
@@ -859,7 +853,7 @@
         <v>1</v>
       </c>
       <c r="K10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L10">
         <v>18.71</v>
@@ -873,19 +867,19 @@
         <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D11">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="E11">
-        <v>20000</v>
+        <v>494021</v>
       </c>
       <c r="F11">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -897,10 +891,10 @@
         <v>1</v>
       </c>
       <c r="K11" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L11">
-        <v>3.34</v>
+        <v>162.04</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -911,7 +905,7 @@
         <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D12">
         <v>37</v>
@@ -935,7 +929,7 @@
         <v>1</v>
       </c>
       <c r="K12" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L12">
         <v>4.52</v>
@@ -952,16 +946,16 @@
         <v>33</v>
       </c>
       <c r="D13">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="E13">
-        <v>581012</v>
+        <v>20000</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="G13">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="H13">
         <v>1</v>
@@ -973,10 +967,10 @@
         <v>1</v>
       </c>
       <c r="K13" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L13">
-        <v>255.65</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -987,19 +981,19 @@
         <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D14">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="E14">
-        <v>299285</v>
+        <v>32561</v>
       </c>
       <c r="F14">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="G14">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -1011,10 +1005,10 @@
         <v>1</v>
       </c>
       <c r="K14" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L14">
-        <v>98.17</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1025,19 +1019,19 @@
         <v>29</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D15">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="E15">
-        <v>32561</v>
+        <v>581012</v>
       </c>
       <c r="F15">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G15">
-        <v>6</v>
+        <v>54</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -1049,10 +1043,10 @@
         <v>1</v>
       </c>
       <c r="K15" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L15">
-        <v>3.91</v>
+        <v>255.65</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1063,7 +1057,7 @@
         <v>29</v>
       </c>
       <c r="C16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D16">
         <v>20</v>
@@ -1087,7 +1081,7 @@
         <v>1</v>
       </c>
       <c r="K16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L16">
         <v>3.2</v>
@@ -1101,7 +1095,7 @@
         <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D17">
         <v>25</v>
@@ -1125,7 +1119,7 @@
         <v>1</v>
       </c>
       <c r="K17" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L17">
         <v>0.2</v>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_02_01_2026) - Modality: multi_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="84">
   <si>
     <t>Dataset</t>
   </si>
@@ -52,70 +52,217 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>news</t>
+  </si>
+  <si>
+    <t>intrusion</t>
+  </si>
+  <si>
+    <t>alarm</t>
+  </si>
+  <si>
+    <t>insurance</t>
+  </si>
+  <si>
+    <t>adult</t>
+  </si>
+  <si>
+    <t>covtype</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
+    <t>expedia_hotel_logs</t>
+  </si>
+  <si>
+    <t>Elti</t>
+  </si>
+  <si>
     <t>financial</t>
   </si>
   <si>
+    <t>got_families</t>
+  </si>
+  <si>
+    <t>nations</t>
+  </si>
+  <si>
+    <t>restbase</t>
+  </si>
+  <si>
+    <t>SAT</t>
+  </si>
+  <si>
+    <t>AustralianFootball</t>
+  </si>
+  <si>
+    <t>Same_gen</t>
+  </si>
+  <si>
+    <t>Student_loan</t>
+  </si>
+  <si>
+    <t>university</t>
+  </si>
+  <si>
+    <t>Biodegradability</t>
+  </si>
+  <si>
+    <t>legalActs</t>
+  </si>
+  <si>
+    <t>imdb_ijs</t>
+  </si>
+  <si>
+    <t>Mesh</t>
+  </si>
+  <si>
+    <t>TubePricing</t>
+  </si>
+  <si>
+    <t>world</t>
+  </si>
+  <si>
+    <t>genes</t>
+  </si>
+  <si>
+    <t>Hepatitis_std</t>
+  </si>
+  <si>
+    <t>Countries</t>
+  </si>
+  <si>
     <t>fake_hotels</t>
   </si>
   <si>
-    <t>Biodegradability</t>
-  </si>
-  <si>
-    <t>restbase</t>
-  </si>
-  <si>
-    <t>Student_loan</t>
+    <t>Toxicology</t>
+  </si>
+  <si>
+    <t>DCG</t>
+  </si>
+  <si>
+    <t>UW_std</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>fake_hotels_extended</t>
+  </si>
+  <si>
+    <t>Dunur</t>
+  </si>
+  <si>
+    <t>imdb_MovieLens</t>
+  </si>
+  <si>
+    <t>imdb_small</t>
+  </si>
+  <si>
+    <t>NBA</t>
+  </si>
+  <si>
+    <t>Pyrimidine</t>
+  </si>
+  <si>
+    <t>CORA</t>
+  </si>
+  <si>
+    <t>Triazine</t>
+  </si>
+  <si>
+    <t>FNHK</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>MuskSmall</t>
+  </si>
+  <si>
+    <t>PremierLeague</t>
+  </si>
+  <si>
+    <t>ftp</t>
+  </si>
+  <si>
+    <t>WebKP</t>
+  </si>
+  <si>
+    <t>Accidents</t>
   </si>
   <si>
     <t>airbnb-simplified</t>
   </si>
   <si>
-    <t>NBA</t>
-  </si>
-  <si>
-    <t>census</t>
-  </si>
-  <si>
-    <t>news</t>
-  </si>
-  <si>
-    <t>intrusion</t>
-  </si>
-  <si>
-    <t>alarm</t>
-  </si>
-  <si>
-    <t>insurance</t>
-  </si>
-  <si>
-    <t>adult</t>
-  </si>
-  <si>
-    <t>covtype</t>
-  </si>
-  <si>
-    <t>child</t>
-  </si>
-  <si>
-    <t>expedia_hotel_logs</t>
+    <t>trains</t>
+  </si>
+  <si>
+    <t>Pima</t>
+  </si>
+  <si>
+    <t>UTube</t>
+  </si>
+  <si>
+    <t>PTE</t>
+  </si>
+  <si>
+    <t>mutagenesis</t>
+  </si>
+  <si>
+    <t>Carcinogenesis</t>
+  </si>
+  <si>
+    <t>Mooney_Family</t>
+  </si>
+  <si>
+    <t>OMOP_CDM_dayz</t>
+  </si>
+  <si>
+    <t>Bupa</t>
+  </si>
+  <si>
+    <t>SalesDB</t>
+  </si>
+  <si>
+    <t>Chess</t>
+  </si>
+  <si>
+    <t>multi_table_ID_demo_dataset</t>
+  </si>
+  <si>
+    <t>Atherosclerosis</t>
+  </si>
+  <si>
+    <t>NCAA</t>
+  </si>
+  <si>
+    <t>single_table</t>
   </si>
   <si>
     <t>multi_table</t>
   </si>
   <si>
-    <t>single_table</t>
+    <t>RealTabFormerSynthesizer</t>
+  </si>
+  <si>
+    <t>GaussianCopulaSynthesizer</t>
+  </si>
+  <si>
+    <t>HSASynthesizer</t>
   </si>
   <si>
     <t>IndependentSynthesizer</t>
   </si>
   <si>
-    <t>HSASynthesizer</t>
-  </si>
-  <si>
-    <t>RealTabFormerSynthesizer</t>
-  </si>
-  <si>
-    <t>GaussianCopulaSynthesizer</t>
+    <t>MultiTableUniformSynthesizer</t>
+  </si>
+  <si>
+    <t>HMASynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -476,7 +623,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -522,37 +669,37 @@
         <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="D2">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="E2">
-        <v>1079680</v>
+        <v>299285</v>
       </c>
       <c r="F2">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="G2">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="H2">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L2">
-        <v>85.38</v>
+        <v>98.17</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -560,37 +707,37 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>77</v>
       </c>
       <c r="D3">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="E3">
-        <v>668</v>
+        <v>39644</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L3">
-        <v>0.05</v>
+        <v>18.71</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -598,37 +745,37 @@
         <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
+        <v>77</v>
       </c>
       <c r="D4">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="E4">
-        <v>21895</v>
+        <v>494021</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="H4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L4">
-        <v>0.57</v>
+        <v>162.04</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -636,37 +783,37 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>78</v>
       </c>
       <c r="D5">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="E5">
-        <v>19297</v>
+        <v>20000</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K5" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L5">
-        <v>0.6899999999999999</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -674,37 +821,37 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="D6">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="E6">
-        <v>5288</v>
+        <v>20000</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="G6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I6">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L6">
-        <v>0.09</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -712,37 +859,37 @@
         <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="C7" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="D7">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E7">
-        <v>5751408</v>
+        <v>32561</v>
       </c>
       <c r="F7">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L7">
-        <v>293.14</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -750,37 +897,37 @@
         <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="D8">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="E8">
-        <v>1219</v>
+        <v>581012</v>
       </c>
       <c r="F8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G8">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="H8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K8" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L8">
-        <v>0.15</v>
+        <v>255.65</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -788,22 +935,22 @@
         <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="D9">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="E9">
-        <v>299285</v>
+        <v>20000</v>
       </c>
       <c r="F9">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="G9">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -815,10 +962,10 @@
         <v>1</v>
       </c>
       <c r="K9" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L9">
-        <v>98.17</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -826,22 +973,22 @@
         <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="D10">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="E10">
-        <v>39644</v>
+        <v>1000</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G10">
-        <v>59</v>
+        <v>5</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -853,10 +1000,10 @@
         <v>1</v>
       </c>
       <c r="K10" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L10">
-        <v>18.71</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -864,37 +1011,37 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="C11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11">
         <v>32</v>
       </c>
-      <c r="D11">
-        <v>41</v>
-      </c>
       <c r="E11">
-        <v>494021</v>
+        <v>1352</v>
       </c>
       <c r="F11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G11">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K11" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L11">
-        <v>162.04</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -902,37 +1049,37 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="C12" t="s">
-        <v>33</v>
+        <v>80</v>
       </c>
       <c r="D12">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="E12">
-        <v>20000</v>
+        <v>1079680</v>
       </c>
       <c r="F12">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I12">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K12" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L12">
-        <v>4.52</v>
+        <v>85.38</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -940,37 +1087,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>81</v>
       </c>
       <c r="D13">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E13">
-        <v>20000</v>
+        <v>23</v>
       </c>
       <c r="F13">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="G13">
+        <v>2</v>
+      </c>
+      <c r="H13">
+        <v>3</v>
+      </c>
+      <c r="I13">
+        <v>2</v>
+      </c>
+      <c r="J13">
+        <v>2</v>
+      </c>
+      <c r="K13" t="s">
+        <v>83</v>
+      </c>
+      <c r="L13">
         <v>0</v>
-      </c>
-      <c r="H13">
-        <v>1</v>
-      </c>
-      <c r="I13">
-        <v>0</v>
-      </c>
-      <c r="J13">
-        <v>1</v>
-      </c>
-      <c r="K13" t="s">
-        <v>34</v>
-      </c>
-      <c r="L13">
-        <v>3.34</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -978,37 +1125,37 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>82</v>
       </c>
       <c r="D14">
-        <v>15</v>
+        <v>119</v>
       </c>
       <c r="E14">
-        <v>32561</v>
+        <v>11004</v>
       </c>
       <c r="F14">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G14">
-        <v>6</v>
+        <v>112</v>
       </c>
       <c r="H14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L14">
-        <v>3.91</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1016,37 +1163,37 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="C15" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="D15">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="E15">
-        <v>581012</v>
+        <v>19297</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G15">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I15">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K15" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L15">
-        <v>255.65</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1054,37 +1201,37 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="C16" t="s">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="D16">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="E16">
-        <v>20000</v>
+        <v>19867</v>
       </c>
       <c r="F16">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="G16">
         <v>0</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="I16">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="J16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K16" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="L16">
-        <v>3.2</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1092,37 +1239,1823 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" t="s">
+        <v>79</v>
+      </c>
+      <c r="D17">
+        <v>78</v>
+      </c>
+      <c r="E17">
+        <v>139179</v>
+      </c>
+      <c r="F17">
+        <v>12</v>
+      </c>
+      <c r="G17">
+        <v>57</v>
+      </c>
+      <c r="H17">
+        <v>4</v>
+      </c>
+      <c r="I17">
+        <v>5</v>
+      </c>
+      <c r="J17">
+        <v>3</v>
+      </c>
+      <c r="K17" t="s">
+        <v>83</v>
+      </c>
+      <c r="L17">
+        <v>31.18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C18" t="s">
+        <v>79</v>
+      </c>
+      <c r="D18">
+        <v>11</v>
+      </c>
+      <c r="E18">
+        <v>1536</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>4</v>
+      </c>
+      <c r="I18">
+        <v>6</v>
+      </c>
+      <c r="J18">
+        <v>2</v>
+      </c>
+      <c r="K18" t="s">
+        <v>83</v>
+      </c>
+      <c r="L18">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" t="s">
         <v>29</v>
       </c>
-      <c r="C17" t="s">
+      <c r="B19" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" t="s">
+        <v>79</v>
+      </c>
+      <c r="D19">
+        <v>16</v>
+      </c>
+      <c r="E19">
+        <v>5288</v>
+      </c>
+      <c r="F19">
+        <v>2</v>
+      </c>
+      <c r="G19">
+        <v>2</v>
+      </c>
+      <c r="H19">
+        <v>10</v>
+      </c>
+      <c r="I19">
+        <v>9</v>
+      </c>
+      <c r="J19">
+        <v>2</v>
+      </c>
+      <c r="K19" t="s">
+        <v>83</v>
+      </c>
+      <c r="L19">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" t="s">
+        <v>79</v>
+      </c>
+      <c r="D20">
+        <v>19</v>
+      </c>
+      <c r="E20">
+        <v>171</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>9</v>
+      </c>
+      <c r="H20">
+        <v>5</v>
+      </c>
+      <c r="I20">
+        <v>4</v>
+      </c>
+      <c r="J20">
+        <v>2</v>
+      </c>
+      <c r="K20" t="s">
+        <v>83</v>
+      </c>
+      <c r="L20">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" t="s">
+        <v>79</v>
+      </c>
+      <c r="D21">
+        <v>16</v>
+      </c>
+      <c r="E21">
+        <v>21895</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+      <c r="G21">
+        <v>4</v>
+      </c>
+      <c r="H21">
+        <v>5</v>
+      </c>
+      <c r="I21">
+        <v>5</v>
+      </c>
+      <c r="J21">
+        <v>3</v>
+      </c>
+      <c r="K21" t="s">
+        <v>83</v>
+      </c>
+      <c r="L21">
+        <v>0.57</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" t="s">
+        <v>76</v>
+      </c>
+      <c r="C22" t="s">
+        <v>80</v>
+      </c>
+      <c r="D22">
+        <v>35</v>
+      </c>
+      <c r="E22">
+        <v>1754397</v>
+      </c>
+      <c r="F22">
+        <v>18</v>
+      </c>
+      <c r="G22">
+        <v>8</v>
+      </c>
+      <c r="H22">
+        <v>5</v>
+      </c>
+      <c r="I22">
+        <v>5</v>
+      </c>
+      <c r="J22">
+        <v>2</v>
+      </c>
+      <c r="K22" t="s">
+        <v>83</v>
+      </c>
+      <c r="L22">
+        <v>130.3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" t="s">
         <v>33</v>
       </c>
-      <c r="D17">
+      <c r="B23" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" t="s">
+        <v>80</v>
+      </c>
+      <c r="D23">
         <v>25</v>
       </c>
-      <c r="E17">
-        <v>1000</v>
-      </c>
-      <c r="F17">
+      <c r="E23">
+        <v>5647694</v>
+      </c>
+      <c r="F23">
+        <v>9</v>
+      </c>
+      <c r="G23">
+        <v>3</v>
+      </c>
+      <c r="H23">
+        <v>7</v>
+      </c>
+      <c r="I23">
+        <v>6</v>
+      </c>
+      <c r="J23">
+        <v>2</v>
+      </c>
+      <c r="K23" t="s">
+        <v>83</v>
+      </c>
+      <c r="L23">
+        <v>173.9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" t="s">
+        <v>76</v>
+      </c>
+      <c r="C24" t="s">
+        <v>79</v>
+      </c>
+      <c r="D24">
+        <v>41</v>
+      </c>
+      <c r="E24">
+        <v>2700</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>2</v>
+      </c>
+      <c r="H24">
+        <v>29</v>
+      </c>
+      <c r="I24">
+        <v>33</v>
+      </c>
+      <c r="J24">
+        <v>2</v>
+      </c>
+      <c r="K24" t="s">
+        <v>83</v>
+      </c>
+      <c r="L24">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" t="s">
+        <v>79</v>
+      </c>
+      <c r="D25">
+        <v>192</v>
+      </c>
+      <c r="E25">
+        <v>154899</v>
+      </c>
+      <c r="F25">
+        <v>54</v>
+      </c>
+      <c r="G25">
+        <v>92</v>
+      </c>
+      <c r="H25">
+        <v>20</v>
+      </c>
+      <c r="I25">
+        <v>39</v>
+      </c>
+      <c r="J25">
+        <v>3</v>
+      </c>
+      <c r="K25" t="s">
+        <v>83</v>
+      </c>
+      <c r="L25">
+        <v>9.67</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" t="s">
+        <v>76</v>
+      </c>
+      <c r="C26" t="s">
+        <v>79</v>
+      </c>
+      <c r="D26">
+        <v>25</v>
+      </c>
+      <c r="E26">
+        <v>5302</v>
+      </c>
+      <c r="F26">
+        <v>11</v>
+      </c>
+      <c r="G26">
+        <v>9</v>
+      </c>
+      <c r="H26">
+        <v>3</v>
+      </c>
+      <c r="I26">
+        <v>2</v>
+      </c>
+      <c r="J26">
+        <v>2</v>
+      </c>
+      <c r="K26" t="s">
+        <v>83</v>
+      </c>
+      <c r="L26">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" t="s">
+        <v>79</v>
+      </c>
+      <c r="D27">
         <v>16</v>
       </c>
-      <c r="G17">
+      <c r="E27">
+        <v>6118</v>
+      </c>
+      <c r="F27">
+        <v>9</v>
+      </c>
+      <c r="G27">
+        <v>2</v>
+      </c>
+      <c r="H27">
+        <v>3</v>
+      </c>
+      <c r="I27">
+        <v>3</v>
+      </c>
+      <c r="J27">
+        <v>2</v>
+      </c>
+      <c r="K27" t="s">
+        <v>83</v>
+      </c>
+      <c r="L27">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B28" t="s">
+        <v>76</v>
+      </c>
+      <c r="C28" t="s">
+        <v>80</v>
+      </c>
+      <c r="D28">
+        <v>29</v>
+      </c>
+      <c r="E28">
+        <v>12927</v>
+      </c>
+      <c r="F28">
+        <v>2</v>
+      </c>
+      <c r="G28">
+        <v>14</v>
+      </c>
+      <c r="H28">
+        <v>7</v>
+      </c>
+      <c r="I28">
+        <v>6</v>
+      </c>
+      <c r="J28">
+        <v>2</v>
+      </c>
+      <c r="K28" t="s">
+        <v>83</v>
+      </c>
+      <c r="L28">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29" t="s">
+        <v>39</v>
+      </c>
+      <c r="B29" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29" t="s">
+        <v>79</v>
+      </c>
+      <c r="D29">
+        <v>68</v>
+      </c>
+      <c r="E29">
+        <v>22318</v>
+      </c>
+      <c r="F29">
+        <v>9</v>
+      </c>
+      <c r="G29">
+        <v>53</v>
+      </c>
+      <c r="H29">
+        <v>4</v>
+      </c>
+      <c r="I29">
+        <v>3</v>
+      </c>
+      <c r="J29">
+        <v>2</v>
+      </c>
+      <c r="K29" t="s">
+        <v>83</v>
+      </c>
+      <c r="L29">
+        <v>9.93</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" t="s">
+        <v>40</v>
+      </c>
+      <c r="B30" t="s">
+        <v>76</v>
+      </c>
+      <c r="C30" t="s">
+        <v>79</v>
+      </c>
+      <c r="D30">
+        <v>15</v>
+      </c>
+      <c r="E30">
+        <v>668</v>
+      </c>
+      <c r="F30">
         <v>5</v>
       </c>
-      <c r="H17">
-        <v>1</v>
-      </c>
-      <c r="I17">
+      <c r="G30">
+        <v>3</v>
+      </c>
+      <c r="H30">
+        <v>2</v>
+      </c>
+      <c r="I30">
+        <v>1</v>
+      </c>
+      <c r="J30">
+        <v>2</v>
+      </c>
+      <c r="K30" t="s">
+        <v>83</v>
+      </c>
+      <c r="L30">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" t="s">
+        <v>41</v>
+      </c>
+      <c r="B31" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31" t="s">
+        <v>79</v>
+      </c>
+      <c r="D31">
+        <v>12</v>
+      </c>
+      <c r="E31">
+        <v>36922</v>
+      </c>
+      <c r="F31">
+        <v>3</v>
+      </c>
+      <c r="G31">
         <v>0</v>
       </c>
-      <c r="J17">
-        <v>1</v>
-      </c>
-      <c r="K17" t="s">
-        <v>34</v>
-      </c>
-      <c r="L17">
-        <v>0.2</v>
+      <c r="H31">
+        <v>4</v>
+      </c>
+      <c r="I31">
+        <v>5</v>
+      </c>
+      <c r="J31">
+        <v>3</v>
+      </c>
+      <c r="K31" t="s">
+        <v>83</v>
+      </c>
+      <c r="L31">
+        <v>1.03</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" t="s">
+        <v>76</v>
+      </c>
+      <c r="C32" t="s">
+        <v>79</v>
+      </c>
+      <c r="D32">
+        <v>6</v>
+      </c>
+      <c r="E32">
+        <v>8258</v>
+      </c>
+      <c r="F32">
+        <v>2</v>
+      </c>
+      <c r="G32">
+        <v>1</v>
+      </c>
+      <c r="H32">
+        <v>2</v>
+      </c>
+      <c r="I32">
+        <v>1</v>
+      </c>
+      <c r="J32">
+        <v>2</v>
+      </c>
+      <c r="K32" t="s">
+        <v>83</v>
+      </c>
+      <c r="L32">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12">
+      <c r="A33" t="s">
+        <v>43</v>
+      </c>
+      <c r="B33" t="s">
+        <v>76</v>
+      </c>
+      <c r="C33" t="s">
+        <v>79</v>
+      </c>
+      <c r="D33">
+        <v>14</v>
+      </c>
+      <c r="E33">
+        <v>712</v>
+      </c>
+      <c r="F33">
+        <v>4</v>
+      </c>
+      <c r="G33">
+        <v>2</v>
+      </c>
+      <c r="H33">
+        <v>4</v>
+      </c>
+      <c r="I33">
+        <v>4</v>
+      </c>
+      <c r="J33">
+        <v>2</v>
+      </c>
+      <c r="K33" t="s">
+        <v>83</v>
+      </c>
+      <c r="L33">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12">
+      <c r="A34" t="s">
+        <v>44</v>
+      </c>
+      <c r="B34" t="s">
+        <v>76</v>
+      </c>
+      <c r="C34" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34">
+        <v>42</v>
+      </c>
+      <c r="E34">
+        <v>3841029</v>
+      </c>
+      <c r="F34">
+        <v>9</v>
+      </c>
+      <c r="G34">
+        <v>27</v>
+      </c>
+      <c r="H34">
+        <v>4</v>
+      </c>
+      <c r="I34">
+        <v>3</v>
+      </c>
+      <c r="J34">
+        <v>3</v>
+      </c>
+      <c r="K34" t="s">
+        <v>83</v>
+      </c>
+      <c r="L34">
+        <v>148.44</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12">
+      <c r="A35" t="s">
+        <v>45</v>
+      </c>
+      <c r="B35" t="s">
+        <v>76</v>
+      </c>
+      <c r="C35" t="s">
+        <v>79</v>
+      </c>
+      <c r="D35">
+        <v>19</v>
+      </c>
+      <c r="E35">
+        <v>668</v>
+      </c>
+      <c r="F35">
+        <v>3</v>
+      </c>
+      <c r="G35">
+        <v>3</v>
+      </c>
+      <c r="H35">
+        <v>2</v>
+      </c>
+      <c r="I35">
+        <v>1</v>
+      </c>
+      <c r="J35">
+        <v>2</v>
+      </c>
+      <c r="K35" t="s">
+        <v>83</v>
+      </c>
+      <c r="L35">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12">
+      <c r="A36" t="s">
+        <v>46</v>
+      </c>
+      <c r="B36" t="s">
+        <v>76</v>
+      </c>
+      <c r="C36" t="s">
+        <v>79</v>
+      </c>
+      <c r="D36">
+        <v>50</v>
+      </c>
+      <c r="E36">
+        <v>440</v>
+      </c>
+      <c r="F36">
+        <v>1</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36">
+        <v>17</v>
+      </c>
+      <c r="I36">
+        <v>32</v>
+      </c>
+      <c r="J36">
+        <v>2</v>
+      </c>
+      <c r="K36" t="s">
+        <v>83</v>
+      </c>
+      <c r="L36">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12">
+      <c r="A37" t="s">
+        <v>47</v>
+      </c>
+      <c r="B37" t="s">
+        <v>76</v>
+      </c>
+      <c r="C37" t="s">
+        <v>79</v>
+      </c>
+      <c r="D37">
+        <v>27</v>
+      </c>
+      <c r="E37">
+        <v>1249411</v>
+      </c>
+      <c r="F37">
+        <v>5</v>
+      </c>
+      <c r="G37">
+        <v>9</v>
+      </c>
+      <c r="H37">
+        <v>7</v>
+      </c>
+      <c r="I37">
+        <v>6</v>
+      </c>
+      <c r="J37">
+        <v>2</v>
+      </c>
+      <c r="K37" t="s">
+        <v>83</v>
+      </c>
+      <c r="L37">
+        <v>39.2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12">
+      <c r="A38" t="s">
+        <v>48</v>
+      </c>
+      <c r="B38" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38" t="s">
+        <v>79</v>
+      </c>
+      <c r="D38">
+        <v>25</v>
+      </c>
+      <c r="E38">
+        <v>4395</v>
+      </c>
+      <c r="F38">
+        <v>9</v>
+      </c>
+      <c r="G38">
+        <v>4</v>
+      </c>
+      <c r="H38">
+        <v>7</v>
+      </c>
+      <c r="I38">
+        <v>6</v>
+      </c>
+      <c r="J38">
+        <v>2</v>
+      </c>
+      <c r="K38" t="s">
+        <v>83</v>
+      </c>
+      <c r="L38">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12">
+      <c r="A39" t="s">
+        <v>49</v>
+      </c>
+      <c r="B39" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" t="s">
+        <v>79</v>
+      </c>
+      <c r="D39">
+        <v>33</v>
+      </c>
+      <c r="E39">
+        <v>1219</v>
+      </c>
+      <c r="F39">
+        <v>4</v>
+      </c>
+      <c r="G39">
+        <v>20</v>
+      </c>
+      <c r="H39">
+        <v>4</v>
+      </c>
+      <c r="I39">
+        <v>5</v>
+      </c>
+      <c r="J39">
+        <v>3</v>
+      </c>
+      <c r="K39" t="s">
+        <v>83</v>
+      </c>
+      <c r="L39">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12">
+      <c r="A40" t="s">
+        <v>50</v>
+      </c>
+      <c r="B40" t="s">
+        <v>76</v>
+      </c>
+      <c r="C40" t="s">
+        <v>80</v>
+      </c>
+      <c r="D40">
+        <v>14</v>
+      </c>
+      <c r="E40">
+        <v>296</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40">
+        <v>11</v>
+      </c>
+      <c r="H40">
+        <v>2</v>
+      </c>
+      <c r="I40">
+        <v>1</v>
+      </c>
+      <c r="J40">
+        <v>2</v>
+      </c>
+      <c r="K40" t="s">
+        <v>83</v>
+      </c>
+      <c r="L40">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12">
+      <c r="A41" t="s">
+        <v>51</v>
+      </c>
+      <c r="B41" t="s">
+        <v>76</v>
+      </c>
+      <c r="C41" t="s">
+        <v>79</v>
+      </c>
+      <c r="D41">
+        <v>10</v>
+      </c>
+      <c r="E41">
+        <v>57353</v>
+      </c>
+      <c r="F41">
+        <v>2</v>
+      </c>
+      <c r="G41">
+        <v>2</v>
+      </c>
+      <c r="H41">
+        <v>3</v>
+      </c>
+      <c r="I41">
+        <v>3</v>
+      </c>
+      <c r="J41">
+        <v>2</v>
+      </c>
+      <c r="K41" t="s">
+        <v>83</v>
+      </c>
+      <c r="L41">
+        <v>1.79</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12">
+      <c r="A42" t="s">
+        <v>52</v>
+      </c>
+      <c r="B42" t="s">
+        <v>76</v>
+      </c>
+      <c r="C42" t="s">
+        <v>82</v>
+      </c>
+      <c r="D42">
+        <v>15</v>
+      </c>
+      <c r="E42">
+        <v>1302</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42">
+        <v>12</v>
+      </c>
+      <c r="H42">
+        <v>2</v>
+      </c>
+      <c r="I42">
+        <v>1</v>
+      </c>
+      <c r="J42">
+        <v>2</v>
+      </c>
+      <c r="K42" t="s">
+        <v>83</v>
+      </c>
+      <c r="L42">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12">
+      <c r="A43" t="s">
+        <v>53</v>
+      </c>
+      <c r="B43" t="s">
+        <v>76</v>
+      </c>
+      <c r="C43" t="s">
+        <v>79</v>
+      </c>
+      <c r="D43">
+        <v>26</v>
+      </c>
+      <c r="E43">
+        <v>2113275</v>
+      </c>
+      <c r="F43">
+        <v>7</v>
+      </c>
+      <c r="G43">
+        <v>10</v>
+      </c>
+      <c r="H43">
+        <v>3</v>
+      </c>
+      <c r="I43">
+        <v>2</v>
+      </c>
+      <c r="J43">
+        <v>2</v>
+      </c>
+      <c r="K43" t="s">
+        <v>83</v>
+      </c>
+      <c r="L43">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12">
+      <c r="A44" t="s">
+        <v>54</v>
+      </c>
+      <c r="B44" t="s">
+        <v>76</v>
+      </c>
+      <c r="C44" t="s">
+        <v>79</v>
+      </c>
+      <c r="D44">
+        <v>266</v>
+      </c>
+      <c r="E44">
+        <v>10173</v>
+      </c>
+      <c r="F44">
+        <v>262</v>
+      </c>
+      <c r="G44">
+        <v>0</v>
+      </c>
+      <c r="H44">
+        <v>2</v>
+      </c>
+      <c r="I44">
+        <v>2</v>
+      </c>
+      <c r="J44">
+        <v>2</v>
+      </c>
+      <c r="K44" t="s">
+        <v>83</v>
+      </c>
+      <c r="L44">
+        <v>1.38</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12">
+      <c r="A45" t="s">
+        <v>55</v>
+      </c>
+      <c r="B45" t="s">
+        <v>76</v>
+      </c>
+      <c r="C45" t="s">
+        <v>79</v>
+      </c>
+      <c r="D45">
+        <v>170</v>
+      </c>
+      <c r="E45">
+        <v>568</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <v>167</v>
+      </c>
+      <c r="H45">
+        <v>2</v>
+      </c>
+      <c r="I45">
+        <v>1</v>
+      </c>
+      <c r="J45">
+        <v>2</v>
+      </c>
+      <c r="K45" t="s">
+        <v>83</v>
+      </c>
+      <c r="L45">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12">
+      <c r="A46" t="s">
+        <v>56</v>
+      </c>
+      <c r="B46" t="s">
+        <v>76</v>
+      </c>
+      <c r="C46" t="s">
+        <v>79</v>
+      </c>
+      <c r="D46">
+        <v>218</v>
+      </c>
+      <c r="E46">
+        <v>11308</v>
+      </c>
+      <c r="F46">
+        <v>5</v>
+      </c>
+      <c r="G46">
+        <v>204</v>
+      </c>
+      <c r="H46">
+        <v>4</v>
+      </c>
+      <c r="I46">
+        <v>5</v>
+      </c>
+      <c r="J46">
+        <v>3</v>
+      </c>
+      <c r="K46" t="s">
+        <v>83</v>
+      </c>
+      <c r="L46">
+        <v>17.2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12">
+      <c r="A47" t="s">
+        <v>57</v>
+      </c>
+      <c r="B47" t="s">
+        <v>76</v>
+      </c>
+      <c r="C47" t="s">
+        <v>79</v>
+      </c>
+      <c r="D47">
+        <v>11</v>
+      </c>
+      <c r="E47">
+        <v>96491</v>
+      </c>
+      <c r="F47">
+        <v>5</v>
+      </c>
+      <c r="G47">
+        <v>1</v>
+      </c>
+      <c r="H47">
+        <v>2</v>
+      </c>
+      <c r="I47">
+        <v>1</v>
+      </c>
+      <c r="J47">
+        <v>2</v>
+      </c>
+      <c r="K47" t="s">
+        <v>83</v>
+      </c>
+      <c r="L47">
+        <v>4.68</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12">
+      <c r="A48" t="s">
+        <v>58</v>
+      </c>
+      <c r="B48" t="s">
+        <v>76</v>
+      </c>
+      <c r="C48" t="s">
+        <v>79</v>
+      </c>
+      <c r="D48">
+        <v>8</v>
+      </c>
+      <c r="E48">
+        <v>81850</v>
+      </c>
+      <c r="F48">
+        <v>2</v>
+      </c>
+      <c r="G48">
+        <v>0</v>
+      </c>
+      <c r="H48">
+        <v>3</v>
+      </c>
+      <c r="I48">
+        <v>3</v>
+      </c>
+      <c r="J48">
+        <v>2</v>
+      </c>
+      <c r="K48" t="s">
+        <v>83</v>
+      </c>
+      <c r="L48">
+        <v>1.96</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12">
+      <c r="A49" t="s">
+        <v>59</v>
+      </c>
+      <c r="B49" t="s">
+        <v>76</v>
+      </c>
+      <c r="C49" t="s">
+        <v>79</v>
+      </c>
+      <c r="D49">
+        <v>43</v>
+      </c>
+      <c r="E49">
+        <v>1463093</v>
+      </c>
+      <c r="F49">
+        <v>24</v>
+      </c>
+      <c r="G49">
+        <v>14</v>
+      </c>
+      <c r="H49">
+        <v>3</v>
+      </c>
+      <c r="I49">
+        <v>3</v>
+      </c>
+      <c r="J49">
+        <v>3</v>
+      </c>
+      <c r="K49" t="s">
+        <v>83</v>
+      </c>
+      <c r="L49">
+        <v>219.33</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12">
+      <c r="A50" t="s">
+        <v>60</v>
+      </c>
+      <c r="B50" t="s">
+        <v>76</v>
+      </c>
+      <c r="C50" t="s">
+        <v>80</v>
+      </c>
+      <c r="D50">
+        <v>22</v>
+      </c>
+      <c r="E50">
+        <v>5751408</v>
+      </c>
+      <c r="F50">
+        <v>15</v>
+      </c>
+      <c r="G50">
+        <v>2</v>
+      </c>
+      <c r="H50">
+        <v>2</v>
+      </c>
+      <c r="I50">
+        <v>1</v>
+      </c>
+      <c r="J50">
+        <v>2</v>
+      </c>
+      <c r="K50" t="s">
+        <v>83</v>
+      </c>
+      <c r="L50">
+        <v>293.14</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12">
+      <c r="A51" t="s">
+        <v>61</v>
+      </c>
+      <c r="B51" t="s">
+        <v>76</v>
+      </c>
+      <c r="C51" t="s">
+        <v>79</v>
+      </c>
+      <c r="D51">
+        <v>13</v>
+      </c>
+      <c r="E51">
+        <v>83</v>
+      </c>
+      <c r="F51">
+        <v>6</v>
+      </c>
+      <c r="G51">
+        <v>4</v>
+      </c>
+      <c r="H51">
+        <v>2</v>
+      </c>
+      <c r="I51">
+        <v>1</v>
+      </c>
+      <c r="J51">
+        <v>2</v>
+      </c>
+      <c r="K51" t="s">
+        <v>83</v>
+      </c>
+      <c r="L51">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12">
+      <c r="A52" t="s">
+        <v>62</v>
+      </c>
+      <c r="B52" t="s">
+        <v>76</v>
+      </c>
+      <c r="C52" t="s">
+        <v>80</v>
+      </c>
+      <c r="D52">
+        <v>18</v>
+      </c>
+      <c r="E52">
+        <v>6912</v>
+      </c>
+      <c r="F52">
+        <v>1</v>
+      </c>
+      <c r="G52">
+        <v>8</v>
+      </c>
+      <c r="H52">
+        <v>9</v>
+      </c>
+      <c r="I52">
+        <v>8</v>
+      </c>
+      <c r="J52">
+        <v>2</v>
+      </c>
+      <c r="K52" t="s">
+        <v>83</v>
+      </c>
+      <c r="L52">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12">
+      <c r="A53" t="s">
+        <v>63</v>
+      </c>
+      <c r="B53" t="s">
+        <v>76</v>
+      </c>
+      <c r="C53" t="s">
+        <v>80</v>
+      </c>
+      <c r="D53">
+        <v>8</v>
+      </c>
+      <c r="E53">
+        <v>2735</v>
+      </c>
+      <c r="F53">
+        <v>5</v>
+      </c>
+      <c r="G53">
+        <v>0</v>
+      </c>
+      <c r="H53">
+        <v>2</v>
+      </c>
+      <c r="I53">
+        <v>1</v>
+      </c>
+      <c r="J53">
+        <v>2</v>
+      </c>
+      <c r="K53" t="s">
+        <v>83</v>
+      </c>
+      <c r="L53">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12">
+      <c r="A54" t="s">
+        <v>64</v>
+      </c>
+      <c r="B54" t="s">
+        <v>76</v>
+      </c>
+      <c r="C54" t="s">
+        <v>79</v>
+      </c>
+      <c r="D54">
+        <v>97</v>
+      </c>
+      <c r="E54">
+        <v>29850</v>
+      </c>
+      <c r="F54">
+        <v>25</v>
+      </c>
+      <c r="G54">
+        <v>9</v>
+      </c>
+      <c r="H54">
+        <v>38</v>
+      </c>
+      <c r="I54">
+        <v>39</v>
+      </c>
+      <c r="J54">
+        <v>3</v>
+      </c>
+      <c r="K54" t="s">
+        <v>83</v>
+      </c>
+      <c r="L54">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12">
+      <c r="A55" t="s">
+        <v>65</v>
+      </c>
+      <c r="B55" t="s">
+        <v>76</v>
+      </c>
+      <c r="C55" t="s">
+        <v>80</v>
+      </c>
+      <c r="D55">
+        <v>15</v>
+      </c>
+      <c r="E55">
+        <v>10324</v>
+      </c>
+      <c r="F55">
+        <v>2</v>
+      </c>
+      <c r="G55">
+        <v>7</v>
+      </c>
+      <c r="H55">
+        <v>3</v>
+      </c>
+      <c r="I55">
+        <v>3</v>
+      </c>
+      <c r="J55">
+        <v>3</v>
+      </c>
+      <c r="K55" t="s">
+        <v>83</v>
+      </c>
+      <c r="L55">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12">
+      <c r="A56" t="s">
+        <v>66</v>
+      </c>
+      <c r="B56" t="s">
+        <v>76</v>
+      </c>
+      <c r="C56" t="s">
+        <v>79</v>
+      </c>
+      <c r="D56">
+        <v>23</v>
+      </c>
+      <c r="E56">
+        <v>27443</v>
+      </c>
+      <c r="F56">
+        <v>2</v>
+      </c>
+      <c r="G56">
+        <v>2</v>
+      </c>
+      <c r="H56">
+        <v>6</v>
+      </c>
+      <c r="I56">
+        <v>13</v>
+      </c>
+      <c r="J56">
+        <v>3</v>
+      </c>
+      <c r="K56" t="s">
+        <v>83</v>
+      </c>
+      <c r="L56">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12">
+      <c r="A57" t="s">
+        <v>67</v>
+      </c>
+      <c r="B57" t="s">
+        <v>76</v>
+      </c>
+      <c r="C57" t="s">
+        <v>79</v>
+      </c>
+      <c r="D57">
+        <v>202</v>
+      </c>
+      <c r="E57">
+        <v>4425</v>
+      </c>
+      <c r="F57">
+        <v>0</v>
+      </c>
+      <c r="G57">
+        <v>0</v>
+      </c>
+      <c r="H57">
+        <v>68</v>
+      </c>
+      <c r="I57">
+        <v>134</v>
+      </c>
+      <c r="J57">
+        <v>2</v>
+      </c>
+      <c r="K57" t="s">
+        <v>83</v>
+      </c>
+      <c r="L57">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12">
+      <c r="A58" t="s">
+        <v>68</v>
+      </c>
+      <c r="B58" t="s">
+        <v>76</v>
+      </c>
+      <c r="C58" t="s">
+        <v>79</v>
+      </c>
+      <c r="D58">
+        <v>432</v>
+      </c>
+      <c r="E58">
+        <v>39000</v>
+      </c>
+      <c r="F58">
+        <v>108</v>
+      </c>
+      <c r="G58">
+        <v>51</v>
+      </c>
+      <c r="H58">
+        <v>39</v>
+      </c>
+      <c r="I58">
+        <v>171</v>
+      </c>
+      <c r="J58">
+        <v>9</v>
+      </c>
+      <c r="K58" t="s">
+        <v>83</v>
+      </c>
+      <c r="L58">
+        <v>3.45</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12">
+      <c r="A59" t="s">
+        <v>69</v>
+      </c>
+      <c r="B59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C59" t="s">
+        <v>80</v>
+      </c>
+      <c r="D59">
+        <v>17</v>
+      </c>
+      <c r="E59">
+        <v>2762</v>
+      </c>
+      <c r="F59">
+        <v>0</v>
+      </c>
+      <c r="G59">
+        <v>7</v>
+      </c>
+      <c r="H59">
+        <v>9</v>
+      </c>
+      <c r="I59">
+        <v>8</v>
+      </c>
+      <c r="J59">
+        <v>2</v>
+      </c>
+      <c r="K59" t="s">
+        <v>83</v>
+      </c>
+      <c r="L59">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12">
+      <c r="A60" t="s">
+        <v>70</v>
+      </c>
+      <c r="B60" t="s">
+        <v>76</v>
+      </c>
+      <c r="C60" t="s">
+        <v>80</v>
+      </c>
+      <c r="D60">
+        <v>16</v>
+      </c>
+      <c r="E60">
+        <v>6735507</v>
+      </c>
+      <c r="F60">
+        <v>7</v>
+      </c>
+      <c r="G60">
+        <v>2</v>
+      </c>
+      <c r="H60">
+        <v>4</v>
+      </c>
+      <c r="I60">
+        <v>3</v>
+      </c>
+      <c r="J60">
+        <v>2</v>
+      </c>
+      <c r="K60" t="s">
+        <v>83</v>
+      </c>
+      <c r="L60">
+        <v>269.25</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12">
+      <c r="A61" t="s">
+        <v>71</v>
+      </c>
+      <c r="B61" t="s">
+        <v>76</v>
+      </c>
+      <c r="C61" t="s">
+        <v>79</v>
+      </c>
+      <c r="D61">
+        <v>46</v>
+      </c>
+      <c r="E61">
+        <v>2052</v>
+      </c>
+      <c r="F61">
+        <v>39</v>
+      </c>
+      <c r="G61">
+        <v>4</v>
+      </c>
+      <c r="H61">
+        <v>2</v>
+      </c>
+      <c r="I61">
+        <v>1</v>
+      </c>
+      <c r="J61">
+        <v>2</v>
+      </c>
+      <c r="K61" t="s">
+        <v>83</v>
+      </c>
+      <c r="L61">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12">
+      <c r="A62" t="s">
+        <v>72</v>
+      </c>
+      <c r="B62" t="s">
+        <v>76</v>
+      </c>
+      <c r="C62" t="s">
+        <v>80</v>
+      </c>
+      <c r="D62">
+        <v>22</v>
+      </c>
+      <c r="E62">
+        <v>11150</v>
+      </c>
+      <c r="F62">
+        <v>4</v>
+      </c>
+      <c r="G62">
+        <v>3</v>
+      </c>
+      <c r="H62">
+        <v>4</v>
+      </c>
+      <c r="I62">
+        <v>3</v>
+      </c>
+      <c r="J62">
+        <v>3</v>
+      </c>
+      <c r="K62" t="s">
+        <v>83</v>
+      </c>
+      <c r="L62">
+        <v>0.6928000000000001</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12">
+      <c r="A63" t="s">
+        <v>73</v>
+      </c>
+      <c r="B63" t="s">
+        <v>76</v>
+      </c>
+      <c r="C63" t="s">
+        <v>79</v>
+      </c>
+      <c r="D63">
+        <v>198</v>
+      </c>
+      <c r="E63">
+        <v>12781</v>
+      </c>
+      <c r="F63">
+        <v>0</v>
+      </c>
+      <c r="G63">
+        <v>193</v>
+      </c>
+      <c r="H63">
+        <v>4</v>
+      </c>
+      <c r="I63">
+        <v>3</v>
+      </c>
+      <c r="J63">
+        <v>2</v>
+      </c>
+      <c r="K63" t="s">
+        <v>83</v>
+      </c>
+      <c r="L63">
+        <v>6.62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12">
+      <c r="A64" t="s">
+        <v>74</v>
+      </c>
+      <c r="B64" t="s">
+        <v>76</v>
+      </c>
+      <c r="C64" t="s">
+        <v>80</v>
+      </c>
+      <c r="D64">
+        <v>112</v>
+      </c>
+      <c r="E64">
+        <v>202305</v>
+      </c>
+      <c r="F64">
+        <v>14</v>
+      </c>
+      <c r="G64">
+        <v>72</v>
+      </c>
+      <c r="H64">
+        <v>9</v>
+      </c>
+      <c r="I64">
+        <v>17</v>
+      </c>
+      <c r="J64">
+        <v>2</v>
+      </c>
+      <c r="K64" t="s">
+        <v>83</v>
+      </c>
+      <c r="L64">
+        <v>27.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_03_01_2026) - Modality: single_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="86">
   <si>
     <t>Dataset</t>
   </si>
@@ -52,199 +52,211 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>ftp</t>
+  </si>
+  <si>
+    <t>world</t>
+  </si>
+  <si>
+    <t>NCAA</t>
+  </si>
+  <si>
+    <t>Countries</t>
+  </si>
+  <si>
+    <t>PremierLeague</t>
+  </si>
+  <si>
+    <t>university</t>
+  </si>
+  <si>
+    <t>Bupa</t>
+  </si>
+  <si>
+    <t>nations</t>
+  </si>
+  <si>
+    <t>Student_loan</t>
+  </si>
+  <si>
+    <t>DCG</t>
+  </si>
+  <si>
+    <t>got_families</t>
+  </si>
+  <si>
+    <t>legalActs</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>imdb_small</t>
+  </si>
+  <si>
+    <t>Same_gen</t>
+  </si>
+  <si>
+    <t>trains</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>genes</t>
+  </si>
+  <si>
+    <t>Pyrimidine</t>
+  </si>
+  <si>
+    <t>imdb_ijs</t>
+  </si>
+  <si>
+    <t>Pima</t>
+  </si>
+  <si>
+    <t>AustralianFootball</t>
+  </si>
+  <si>
+    <t>OMOP_CDM_dayz</t>
+  </si>
+  <si>
+    <t>TubePricing</t>
+  </si>
+  <si>
+    <t>restbase</t>
+  </si>
+  <si>
+    <t>financial</t>
+  </si>
+  <si>
+    <t>Mooney_Family</t>
+  </si>
+  <si>
+    <t>Atherosclerosis</t>
+  </si>
+  <si>
+    <t>Triazine</t>
+  </si>
+  <si>
+    <t>UW_std</t>
+  </si>
+  <si>
+    <t>fake_hotels_extended</t>
+  </si>
+  <si>
+    <t>CORA</t>
+  </si>
+  <si>
+    <t>Mesh</t>
+  </si>
+  <si>
+    <t>Chess</t>
+  </si>
+  <si>
+    <t>Biodegradability</t>
+  </si>
+  <si>
+    <t>PTE</t>
+  </si>
+  <si>
+    <t>SalesDB</t>
+  </si>
+  <si>
+    <t>MuskSmall</t>
+  </si>
+  <si>
+    <t>Dunur</t>
+  </si>
+  <si>
+    <t>SAT</t>
+  </si>
+  <si>
+    <t>WebKP</t>
+  </si>
+  <si>
+    <t>FNHK</t>
+  </si>
+  <si>
+    <t>UTube</t>
+  </si>
+  <si>
+    <t>NBA</t>
+  </si>
+  <si>
+    <t>imdb_MovieLens</t>
+  </si>
+  <si>
+    <t>Elti</t>
+  </si>
+  <si>
+    <t>airbnb-simplified</t>
+  </si>
+  <si>
+    <t>multi_table_ID_demo_dataset</t>
+  </si>
+  <si>
+    <t>mutagenesis</t>
+  </si>
+  <si>
+    <t>Toxicology</t>
+  </si>
+  <si>
+    <t>Carcinogenesis</t>
+  </si>
+  <si>
+    <t>fake_hotels</t>
+  </si>
+  <si>
+    <t>Hepatitis_std</t>
+  </si>
+  <si>
+    <t>Accidents</t>
+  </si>
+  <si>
     <t>census</t>
   </si>
   <si>
+    <t>expedia_hotel_logs</t>
+  </si>
+  <si>
+    <t>insurance</t>
+  </si>
+  <si>
     <t>news</t>
   </si>
   <si>
+    <t>covtype</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
     <t>intrusion</t>
   </si>
   <si>
     <t>alarm</t>
   </si>
   <si>
-    <t>insurance</t>
-  </si>
-  <si>
     <t>adult</t>
   </si>
   <si>
-    <t>covtype</t>
-  </si>
-  <si>
-    <t>child</t>
-  </si>
-  <si>
-    <t>expedia_hotel_logs</t>
-  </si>
-  <si>
-    <t>ftp</t>
-  </si>
-  <si>
-    <t>world</t>
-  </si>
-  <si>
-    <t>NCAA</t>
-  </si>
-  <si>
-    <t>Countries</t>
-  </si>
-  <si>
-    <t>PremierLeague</t>
-  </si>
-  <si>
-    <t>university</t>
-  </si>
-  <si>
-    <t>Bupa</t>
-  </si>
-  <si>
-    <t>nations</t>
-  </si>
-  <si>
-    <t>Student_loan</t>
-  </si>
-  <si>
-    <t>DCG</t>
-  </si>
-  <si>
-    <t>got_families</t>
-  </si>
-  <si>
-    <t>legalActs</t>
-  </si>
-  <si>
-    <t>SAP</t>
-  </si>
-  <si>
-    <t>imdb_small</t>
-  </si>
-  <si>
-    <t>Same_gen</t>
-  </si>
-  <si>
-    <t>trains</t>
-  </si>
-  <si>
-    <t>Facebook</t>
-  </si>
-  <si>
-    <t>genes</t>
-  </si>
-  <si>
-    <t>Pyrimidine</t>
-  </si>
-  <si>
-    <t>imdb_ijs</t>
-  </si>
-  <si>
-    <t>Pima</t>
-  </si>
-  <si>
-    <t>AustralianFootball</t>
-  </si>
-  <si>
-    <t>OMOP_CDM_dayz</t>
-  </si>
-  <si>
-    <t>TubePricing</t>
-  </si>
-  <si>
-    <t>restbase</t>
-  </si>
-  <si>
-    <t>financial</t>
-  </si>
-  <si>
-    <t>Mooney_Family</t>
-  </si>
-  <si>
-    <t>Atherosclerosis</t>
-  </si>
-  <si>
-    <t>Triazine</t>
-  </si>
-  <si>
-    <t>UW_std</t>
-  </si>
-  <si>
-    <t>fake_hotels_extended</t>
-  </si>
-  <si>
-    <t>CORA</t>
-  </si>
-  <si>
-    <t>Mesh</t>
-  </si>
-  <si>
-    <t>Chess</t>
-  </si>
-  <si>
-    <t>Biodegradability</t>
-  </si>
-  <si>
-    <t>PTE</t>
-  </si>
-  <si>
-    <t>SalesDB</t>
-  </si>
-  <si>
-    <t>MuskSmall</t>
-  </si>
-  <si>
-    <t>Dunur</t>
-  </si>
-  <si>
-    <t>SAT</t>
-  </si>
-  <si>
-    <t>WebKP</t>
-  </si>
-  <si>
-    <t>FNHK</t>
-  </si>
-  <si>
-    <t>UTube</t>
-  </si>
-  <si>
-    <t>NBA</t>
-  </si>
-  <si>
-    <t>imdb_MovieLens</t>
-  </si>
-  <si>
-    <t>Elti</t>
-  </si>
-  <si>
-    <t>airbnb-simplified</t>
-  </si>
-  <si>
-    <t>multi_table_ID_demo_dataset</t>
-  </si>
-  <si>
-    <t>mutagenesis</t>
-  </si>
-  <si>
-    <t>Toxicology</t>
-  </si>
-  <si>
-    <t>Carcinogenesis</t>
-  </si>
-  <si>
-    <t>fake_hotels</t>
-  </si>
-  <si>
-    <t>Hepatitis_std</t>
-  </si>
-  <si>
-    <t>Accidents</t>
+    <t>multi_table</t>
   </si>
   <si>
     <t>single_table</t>
   </si>
   <si>
-    <t>multi_table</t>
+    <t>HSASynthesizer</t>
+  </si>
+  <si>
+    <t>HMASynthesizer</t>
+  </si>
+  <si>
+    <t>IndependentSynthesizer</t>
+  </si>
+  <si>
+    <t>MultiTableUniformSynthesizer</t>
   </si>
   <si>
     <t>RealTabFormerSynthesizer</t>
@@ -253,16 +265,10 @@
     <t>GaussianCopulaSynthesizer</t>
   </si>
   <si>
-    <t>HSASynthesizer</t>
-  </si>
-  <si>
-    <t>HMASynthesizer</t>
-  </si>
-  <si>
-    <t>IndependentSynthesizer</t>
-  </si>
-  <si>
-    <t>MultiTableUniformSynthesizer</t>
+    <t>SegmentSynthesizer</t>
+  </si>
+  <si>
+    <t>TVAESynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -675,31 +681,31 @@
         <v>77</v>
       </c>
       <c r="D2">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="E2">
-        <v>299285</v>
+        <v>96491</v>
       </c>
       <c r="F2">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="G2">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L2">
-        <v>98.17</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -710,34 +716,34 @@
         <v>75</v>
       </c>
       <c r="C3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D3">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="E3">
-        <v>39644</v>
+        <v>5302</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G3">
-        <v>59</v>
+        <v>9</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L3">
-        <v>18.71</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -748,34 +754,34 @@
         <v>75</v>
       </c>
       <c r="C4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D4">
-        <v>41</v>
+        <v>112</v>
       </c>
       <c r="E4">
-        <v>494021</v>
+        <v>202305</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="G4">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="J4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L4">
-        <v>162.04</v>
+        <v>27.15</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -786,34 +792,34 @@
         <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D5">
-        <v>37</v>
+        <v>68</v>
       </c>
       <c r="E5">
-        <v>20000</v>
+        <v>22318</v>
       </c>
       <c r="F5">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L5">
-        <v>4.52</v>
+        <v>9.93</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -824,34 +830,34 @@
         <v>75</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D6">
-        <v>27</v>
+        <v>218</v>
       </c>
       <c r="E6">
-        <v>20000</v>
+        <v>11308</v>
       </c>
       <c r="F6">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L6">
-        <v>3.34</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -862,34 +868,34 @@
         <v>75</v>
       </c>
       <c r="C7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D7">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E7">
-        <v>32561</v>
+        <v>171</v>
       </c>
       <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
         <v>9</v>
       </c>
-      <c r="G7">
-        <v>6</v>
-      </c>
       <c r="H7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L7">
-        <v>3.91</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -900,34 +906,34 @@
         <v>75</v>
       </c>
       <c r="C8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D8">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="E8">
-        <v>581012</v>
+        <v>2762</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>54</v>
+        <v>7</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L8">
-        <v>255.65</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -941,31 +947,31 @@
         <v>78</v>
       </c>
       <c r="D9">
-        <v>20</v>
+        <v>119</v>
       </c>
       <c r="E9">
-        <v>20000</v>
+        <v>11004</v>
       </c>
       <c r="F9">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L9">
-        <v>3.2</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -976,34 +982,34 @@
         <v>75</v>
       </c>
       <c r="C10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D10">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E10">
-        <v>1000</v>
+        <v>5288</v>
       </c>
       <c r="F10">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L10">
-        <v>0.2</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1011,19 +1017,19 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C11" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D11">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E11">
-        <v>96491</v>
+        <v>8258</v>
       </c>
       <c r="F11">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G11">
         <v>1</v>
@@ -1038,10 +1044,10 @@
         <v>2</v>
       </c>
       <c r="K11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L11">
-        <v>4.68</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1049,22 +1055,22 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C12" t="s">
         <v>80</v>
       </c>
       <c r="D12">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="E12">
-        <v>5302</v>
+        <v>23</v>
       </c>
       <c r="F12">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="G12">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H12">
         <v>3</v>
@@ -1076,10 +1082,10 @@
         <v>2</v>
       </c>
       <c r="K12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L12">
-        <v>0.23</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1087,37 +1093,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D13">
-        <v>112</v>
+        <v>35</v>
       </c>
       <c r="E13">
-        <v>202305</v>
+        <v>1754397</v>
       </c>
       <c r="F13">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G13">
-        <v>72</v>
+        <v>8</v>
       </c>
       <c r="H13">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I13">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="J13">
         <v>2</v>
       </c>
       <c r="K13" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L13">
-        <v>27.15</v>
+        <v>130.3</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1125,22 +1131,22 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C14" t="s">
         <v>79</v>
       </c>
       <c r="D14">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="E14">
-        <v>22318</v>
+        <v>3841029</v>
       </c>
       <c r="F14">
         <v>9</v>
       </c>
       <c r="G14">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="H14">
         <v>4</v>
@@ -1149,13 +1155,13 @@
         <v>3</v>
       </c>
       <c r="J14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L14">
-        <v>9.93</v>
+        <v>148.44</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1163,37 +1169,37 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C15" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D15">
-        <v>218</v>
+        <v>25</v>
       </c>
       <c r="E15">
-        <v>11308</v>
+        <v>4395</v>
       </c>
       <c r="F15">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G15">
-        <v>204</v>
+        <v>4</v>
       </c>
       <c r="H15">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L15">
-        <v>17.2</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1201,37 +1207,37 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C16" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D16">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E16">
-        <v>171</v>
+        <v>1536</v>
       </c>
       <c r="F16">
         <v>1</v>
       </c>
       <c r="G16">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I16">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J16">
         <v>2</v>
       </c>
       <c r="K16" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L16">
-        <v>0.01</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1239,37 +1245,37 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C17" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D17">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E17">
-        <v>2762</v>
+        <v>83</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G17">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H17">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I17">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J17">
         <v>2</v>
       </c>
       <c r="K17" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L17">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1277,37 +1283,37 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D18">
-        <v>119</v>
+        <v>266</v>
       </c>
       <c r="E18">
-        <v>11004</v>
+        <v>10173</v>
       </c>
       <c r="F18">
-        <v>2</v>
+        <v>262</v>
       </c>
       <c r="G18">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J18">
         <v>2</v>
       </c>
       <c r="K18" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L18">
-        <v>0.45</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1315,37 +1321,37 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D19">
         <v>16</v>
       </c>
       <c r="E19">
-        <v>5288</v>
+        <v>6118</v>
       </c>
       <c r="F19">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G19">
         <v>2</v>
       </c>
       <c r="H19">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I19">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J19">
         <v>2</v>
       </c>
       <c r="K19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L19">
-        <v>0.09</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1353,22 +1359,22 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C20" t="s">
         <v>79</v>
       </c>
       <c r="D20">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E20">
-        <v>8258</v>
+        <v>296</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="H20">
         <v>2</v>
@@ -1380,10 +1386,10 @@
         <v>2</v>
       </c>
       <c r="K20" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L20">
-        <v>0.25</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1391,37 +1397,37 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C21" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D21">
+        <v>25</v>
+      </c>
+      <c r="E21">
+        <v>5647694</v>
+      </c>
+      <c r="F21">
         <v>9</v>
       </c>
-      <c r="E21">
-        <v>23</v>
-      </c>
-      <c r="F21">
-        <v>3</v>
-      </c>
       <c r="G21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H21">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I21">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J21">
         <v>2</v>
       </c>
       <c r="K21" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L21">
-        <v>0</v>
+        <v>173.9</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1429,37 +1435,37 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C22" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D22">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E22">
-        <v>1754397</v>
+        <v>6912</v>
       </c>
       <c r="F22">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="G22">
         <v>8</v>
       </c>
       <c r="H22">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I22">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J22">
         <v>2</v>
       </c>
       <c r="K22" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L22">
-        <v>130.3</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1467,37 +1473,37 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C23" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D23">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="E23">
-        <v>3841029</v>
+        <v>139179</v>
       </c>
       <c r="F23">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G23">
-        <v>27</v>
+        <v>57</v>
       </c>
       <c r="H23">
         <v>4</v>
       </c>
       <c r="I23">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J23">
         <v>3</v>
       </c>
       <c r="K23" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L23">
-        <v>148.44</v>
+        <v>31.18</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1505,37 +1511,37 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C24" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D24">
-        <v>25</v>
+        <v>432</v>
       </c>
       <c r="E24">
-        <v>4395</v>
+        <v>39000</v>
       </c>
       <c r="F24">
+        <v>108</v>
+      </c>
+      <c r="G24">
+        <v>51</v>
+      </c>
+      <c r="H24">
+        <v>39</v>
+      </c>
+      <c r="I24">
+        <v>171</v>
+      </c>
+      <c r="J24">
         <v>9</v>
       </c>
-      <c r="G24">
-        <v>4</v>
-      </c>
-      <c r="H24">
-        <v>7</v>
-      </c>
-      <c r="I24">
-        <v>6</v>
-      </c>
-      <c r="J24">
-        <v>2</v>
-      </c>
       <c r="K24" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L24">
-        <v>0.15</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1543,37 +1549,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D25">
-        <v>11</v>
+        <v>192</v>
       </c>
       <c r="E25">
-        <v>1536</v>
+        <v>154899</v>
       </c>
       <c r="F25">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="H25">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="I25">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="J25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K25" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L25">
-        <v>0.04</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1581,37 +1587,37 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C26" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D26">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E26">
-        <v>83</v>
+        <v>19297</v>
       </c>
       <c r="F26">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G26">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K26" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L26">
-        <v>0.01</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1619,37 +1625,37 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C27" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D27">
-        <v>266</v>
+        <v>55</v>
       </c>
       <c r="E27">
-        <v>10173</v>
+        <v>1079680</v>
       </c>
       <c r="F27">
-        <v>262</v>
+        <v>14</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H27">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I27">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J27">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K27" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L27">
-        <v>1.38</v>
+        <v>85.38</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1657,37 +1663,37 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C28" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D28">
-        <v>16</v>
+        <v>202</v>
       </c>
       <c r="E28">
-        <v>6118</v>
+        <v>4425</v>
       </c>
       <c r="F28">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H28">
-        <v>3</v>
+        <v>68</v>
       </c>
       <c r="I28">
-        <v>3</v>
+        <v>134</v>
       </c>
       <c r="J28">
         <v>2</v>
       </c>
       <c r="K28" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L28">
-        <v>0.36</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1695,37 +1701,37 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C29" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D29">
-        <v>14</v>
+        <v>198</v>
       </c>
       <c r="E29">
-        <v>296</v>
+        <v>12781</v>
       </c>
       <c r="F29">
         <v>0</v>
       </c>
       <c r="G29">
-        <v>11</v>
+        <v>193</v>
       </c>
       <c r="H29">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I29">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J29">
         <v>2</v>
       </c>
       <c r="K29" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L29">
-        <v>0.02</v>
+        <v>6.62</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1733,37 +1739,37 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C30" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D30">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E30">
-        <v>5647694</v>
+        <v>1302</v>
       </c>
       <c r="F30">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G30">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H30">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I30">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J30">
         <v>2</v>
       </c>
       <c r="K30" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L30">
-        <v>173.9</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1771,37 +1777,37 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C31" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D31">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E31">
-        <v>6912</v>
+        <v>712</v>
       </c>
       <c r="F31">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G31">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H31">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I31">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J31">
         <v>2</v>
       </c>
       <c r="K31" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L31">
-        <v>0.11</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1809,37 +1815,37 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C32" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D32">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="E32">
-        <v>139179</v>
+        <v>668</v>
       </c>
       <c r="F32">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="G32">
-        <v>57</v>
+        <v>3</v>
       </c>
       <c r="H32">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I32">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J32">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K32" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L32">
-        <v>31.18</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1847,37 +1853,37 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C33" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D33">
-        <v>432</v>
+        <v>10</v>
       </c>
       <c r="E33">
-        <v>39000</v>
+        <v>57353</v>
       </c>
       <c r="F33">
-        <v>108</v>
+        <v>2</v>
       </c>
       <c r="G33">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="H33">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="I33">
-        <v>171</v>
+        <v>3</v>
       </c>
       <c r="J33">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L33">
-        <v>3.45</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1885,37 +1891,37 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C34" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D34">
-        <v>192</v>
+        <v>41</v>
       </c>
       <c r="E34">
-        <v>154899</v>
+        <v>2700</v>
       </c>
       <c r="F34">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="G34">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="H34">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="I34">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="J34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L34">
-        <v>9.67</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1923,37 +1929,37 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C35" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D35">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="E35">
-        <v>19297</v>
+        <v>2052</v>
       </c>
       <c r="F35">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="G35">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H35">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I35">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J35">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K35" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L35">
-        <v>0.6899999999999999</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -1961,37 +1967,37 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C36" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D36">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="E36">
-        <v>1079680</v>
+        <v>21895</v>
       </c>
       <c r="F36">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G36">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="H36">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I36">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K36" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L36">
-        <v>85.38</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -1999,37 +2005,37 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C37" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D37">
-        <v>202</v>
+        <v>97</v>
       </c>
       <c r="E37">
-        <v>4425</v>
+        <v>29850</v>
       </c>
       <c r="F37">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G37">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H37">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="I37">
-        <v>134</v>
+        <v>39</v>
       </c>
       <c r="J37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K37" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L37">
-        <v>0.1</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2037,22 +2043,22 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C38" t="s">
         <v>79</v>
       </c>
       <c r="D38">
-        <v>198</v>
+        <v>16</v>
       </c>
       <c r="E38">
-        <v>12781</v>
+        <v>6735507</v>
       </c>
       <c r="F38">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G38">
-        <v>193</v>
+        <v>2</v>
       </c>
       <c r="H38">
         <v>4</v>
@@ -2064,10 +2070,10 @@
         <v>2</v>
       </c>
       <c r="K38" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L38">
-        <v>6.62</v>
+        <v>269.25</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2075,22 +2081,22 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C39" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D39">
-        <v>15</v>
+        <v>170</v>
       </c>
       <c r="E39">
-        <v>1302</v>
+        <v>568</v>
       </c>
       <c r="F39">
         <v>0</v>
       </c>
       <c r="G39">
-        <v>12</v>
+        <v>167</v>
       </c>
       <c r="H39">
         <v>2</v>
@@ -2102,10 +2108,10 @@
         <v>2</v>
       </c>
       <c r="K39" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L39">
-        <v>0.12</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2113,37 +2119,37 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C40" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D40">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="E40">
-        <v>712</v>
+        <v>440</v>
       </c>
       <c r="F40">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G40">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H40">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I40">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="J40">
         <v>2</v>
       </c>
       <c r="K40" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L40">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2151,37 +2157,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C41" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D41">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="E41">
-        <v>668</v>
+        <v>19867</v>
       </c>
       <c r="F41">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G41">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H41">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="I41">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="J41">
         <v>2</v>
       </c>
       <c r="K41" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L41">
-        <v>0.07000000000000001</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2189,22 +2195,22 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C42" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D42">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E42">
-        <v>57353</v>
+        <v>81850</v>
       </c>
       <c r="F42">
         <v>2</v>
       </c>
       <c r="G42">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H42">
         <v>3</v>
@@ -2216,10 +2222,10 @@
         <v>2</v>
       </c>
       <c r="K42" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L42">
-        <v>1.79</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2227,37 +2233,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C43" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D43">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="E43">
-        <v>2700</v>
+        <v>2113275</v>
       </c>
       <c r="F43">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G43">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H43">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="I43">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="J43">
         <v>2</v>
       </c>
       <c r="K43" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L43">
-        <v>0.04</v>
+        <v>120</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2265,22 +2271,22 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C44" t="s">
         <v>79</v>
       </c>
       <c r="D44">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="E44">
-        <v>2052</v>
+        <v>2735</v>
       </c>
       <c r="F44">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="G44">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H44">
         <v>2</v>
@@ -2292,10 +2298,10 @@
         <v>2</v>
       </c>
       <c r="K44" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L44">
-        <v>0.25</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2303,25 +2309,25 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C45" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D45">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E45">
-        <v>21895</v>
+        <v>1219</v>
       </c>
       <c r="F45">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G45">
+        <v>20</v>
+      </c>
+      <c r="H45">
         <v>4</v>
-      </c>
-      <c r="H45">
-        <v>5</v>
       </c>
       <c r="I45">
         <v>5</v>
@@ -2330,10 +2336,10 @@
         <v>3</v>
       </c>
       <c r="K45" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L45">
-        <v>0.57</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2341,37 +2347,37 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C46" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D46">
-        <v>97</v>
+        <v>27</v>
       </c>
       <c r="E46">
-        <v>29850</v>
+        <v>1249411</v>
       </c>
       <c r="F46">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="G46">
         <v>9</v>
       </c>
       <c r="H46">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="I46">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="J46">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K46" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L46">
-        <v>0.95</v>
+        <v>39.2</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2379,37 +2385,37 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C47" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D47">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E47">
-        <v>6735507</v>
+        <v>1352</v>
       </c>
       <c r="F47">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G47">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H47">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I47">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="J47">
         <v>2</v>
       </c>
       <c r="K47" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L47">
-        <v>269.25</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2417,22 +2423,22 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C48" t="s">
         <v>79</v>
       </c>
       <c r="D48">
-        <v>170</v>
+        <v>22</v>
       </c>
       <c r="E48">
-        <v>568</v>
+        <v>5751408</v>
       </c>
       <c r="F48">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G48">
-        <v>167</v>
+        <v>2</v>
       </c>
       <c r="H48">
         <v>2</v>
@@ -2444,10 +2450,10 @@
         <v>2</v>
       </c>
       <c r="K48" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L48">
-        <v>0.64</v>
+        <v>293.14</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2455,37 +2461,37 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C49" t="s">
         <v>79</v>
       </c>
       <c r="D49">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="E49">
-        <v>440</v>
+        <v>11150</v>
       </c>
       <c r="F49">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G49">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H49">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I49">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="J49">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K49" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L49">
-        <v>0.01</v>
+        <v>0.6928000000000001</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2493,37 +2499,37 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C50" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D50">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="E50">
-        <v>19867</v>
+        <v>10324</v>
       </c>
       <c r="F50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G50">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H50">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="I50">
-        <v>65</v>
+        <v>3</v>
       </c>
       <c r="J50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K50" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L50">
-        <v>0.32</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2531,37 +2537,37 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C51" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D51">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E51">
-        <v>81850</v>
+        <v>36922</v>
       </c>
       <c r="F51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G51">
         <v>0</v>
       </c>
       <c r="H51">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I51">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K51" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L51">
-        <v>1.96</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2569,37 +2575,37 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C52" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D52">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E52">
-        <v>2113275</v>
+        <v>27443</v>
       </c>
       <c r="F52">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G52">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H52">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I52">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="J52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K52" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L52">
-        <v>120</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2607,22 +2613,22 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C53" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D53">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E53">
-        <v>2735</v>
+        <v>668</v>
       </c>
       <c r="F53">
         <v>5</v>
       </c>
       <c r="G53">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H53">
         <v>2</v>
@@ -2634,10 +2640,10 @@
         <v>2</v>
       </c>
       <c r="K53" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L53">
-        <v>0.11</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2645,37 +2651,37 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C54" t="s">
         <v>79</v>
       </c>
       <c r="D54">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E54">
-        <v>1219</v>
+        <v>12927</v>
       </c>
       <c r="F54">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G54">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H54">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I54">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K54" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L54">
-        <v>0.15</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2683,37 +2689,37 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C55" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D55">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="E55">
-        <v>1249411</v>
+        <v>1463093</v>
       </c>
       <c r="F55">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="G55">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="H55">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I55">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J55">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K55" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L55">
-        <v>39.2</v>
+        <v>219.33</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2724,34 +2730,34 @@
         <v>76</v>
       </c>
       <c r="C56" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D56">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="E56">
-        <v>1352</v>
+        <v>299285</v>
       </c>
       <c r="F56">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="G56">
+        <v>12</v>
+      </c>
+      <c r="H56">
+        <v>1</v>
+      </c>
+      <c r="I56">
         <v>0</v>
       </c>
-      <c r="H56">
-        <v>11</v>
-      </c>
-      <c r="I56">
-        <v>20</v>
-      </c>
       <c r="J56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K56" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L56">
-        <v>0.05</v>
+        <v>98.17</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2762,34 +2768,34 @@
         <v>76</v>
       </c>
       <c r="C57" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D57">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E57">
-        <v>5751408</v>
+        <v>1000</v>
       </c>
       <c r="F57">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G57">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I57">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K57" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L57">
-        <v>293.14</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2800,34 +2806,34 @@
         <v>76</v>
       </c>
       <c r="C58" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D58">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E58">
-        <v>11150</v>
+        <v>20000</v>
       </c>
       <c r="F58">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="G58">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H58">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I58">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J58">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K58" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L58">
-        <v>0.6928000000000001</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2838,34 +2844,34 @@
         <v>76</v>
       </c>
       <c r="C59" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D59">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="E59">
-        <v>10324</v>
+        <v>39644</v>
       </c>
       <c r="F59">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G59">
-        <v>7</v>
+        <v>59</v>
       </c>
       <c r="H59">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I59">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J59">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K59" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L59">
-        <v>0.37</v>
+        <v>18.71</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2876,34 +2882,34 @@
         <v>76</v>
       </c>
       <c r="C60" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D60">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="E60">
-        <v>36922</v>
+        <v>581012</v>
       </c>
       <c r="F60">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G60">
+        <v>54</v>
+      </c>
+      <c r="H60">
+        <v>1</v>
+      </c>
+      <c r="I60">
         <v>0</v>
       </c>
-      <c r="H60">
-        <v>4</v>
-      </c>
-      <c r="I60">
-        <v>5</v>
-      </c>
       <c r="J60">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K60" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L60">
-        <v>1.03</v>
+        <v>255.65</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2914,34 +2920,34 @@
         <v>76</v>
       </c>
       <c r="C61" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D61">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E61">
-        <v>27443</v>
+        <v>20000</v>
       </c>
       <c r="F61">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="G61">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H61">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I61">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J61">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K61" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L61">
-        <v>0.9399999999999999</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -2952,34 +2958,34 @@
         <v>76</v>
       </c>
       <c r="C62" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D62">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="E62">
-        <v>668</v>
+        <v>494021</v>
       </c>
       <c r="F62">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G62">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="H62">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I62">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J62">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K62" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L62">
-        <v>0.05</v>
+        <v>162.04</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -2990,34 +2996,34 @@
         <v>76</v>
       </c>
       <c r="C63" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D63">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="E63">
-        <v>12927</v>
+        <v>20000</v>
       </c>
       <c r="F63">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="G63">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="H63">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I63">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J63">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K63" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L63">
-        <v>0.68</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3028,34 +3034,34 @@
         <v>76</v>
       </c>
       <c r="C64" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D64">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="E64">
-        <v>1463093</v>
+        <v>32561</v>
       </c>
       <c r="F64">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="G64">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H64">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I64">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J64">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K64" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L64">
-        <v>219.33</v>
+        <v>3.91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_03_01_2026) - Modality: multi_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -52,223 +52,223 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>expedia_hotel_logs</t>
+  </si>
+  <si>
+    <t>insurance</t>
+  </si>
+  <si>
+    <t>news</t>
+  </si>
+  <si>
+    <t>covtype</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
+    <t>intrusion</t>
+  </si>
+  <si>
+    <t>alarm</t>
+  </si>
+  <si>
+    <t>adult</t>
+  </si>
+  <si>
+    <t>NBA</t>
+  </si>
+  <si>
+    <t>Accidents</t>
+  </si>
+  <si>
+    <t>OMOP_CDM_dayz</t>
+  </si>
+  <si>
+    <t>UW_std</t>
+  </si>
+  <si>
+    <t>multi_table_ID_demo_dataset</t>
+  </si>
+  <si>
+    <t>UTube</t>
+  </si>
+  <si>
+    <t>imdb_ijs</t>
+  </si>
+  <si>
+    <t>trains</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>CORA</t>
+  </si>
+  <si>
+    <t>legalActs</t>
+  </si>
+  <si>
+    <t>SalesDB</t>
+  </si>
+  <si>
+    <t>Bupa</t>
+  </si>
+  <si>
+    <t>Atherosclerosis</t>
+  </si>
+  <si>
+    <t>airbnb-simplified</t>
+  </si>
+  <si>
+    <t>SAT</t>
+  </si>
+  <si>
+    <t>Mooney_Family</t>
+  </si>
+  <si>
+    <t>Biodegradability</t>
+  </si>
+  <si>
     <t>ftp</t>
   </si>
   <si>
+    <t>Dunur</t>
+  </si>
+  <si>
+    <t>genes</t>
+  </si>
+  <si>
+    <t>university</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>Pima</t>
+  </si>
+  <si>
+    <t>Triazine</t>
+  </si>
+  <si>
     <t>world</t>
   </si>
   <si>
+    <t>Elti</t>
+  </si>
+  <si>
+    <t>mutagenesis</t>
+  </si>
+  <si>
+    <t>Pyrimidine</t>
+  </si>
+  <si>
+    <t>FNHK</t>
+  </si>
+  <si>
+    <t>Toxicology</t>
+  </si>
+  <si>
+    <t>Carcinogenesis</t>
+  </si>
+  <si>
+    <t>restbase</t>
+  </si>
+  <si>
+    <t>fake_hotels</t>
+  </si>
+  <si>
+    <t>fake_hotels_extended</t>
+  </si>
+  <si>
+    <t>financial</t>
+  </si>
+  <si>
+    <t>Student_loan</t>
+  </si>
+  <si>
+    <t>Hepatitis_std</t>
+  </si>
+  <si>
+    <t>AustralianFootball</t>
+  </si>
+  <si>
+    <t>PremierLeague</t>
+  </si>
+  <si>
+    <t>MuskSmall</t>
+  </si>
+  <si>
+    <t>got_families</t>
+  </si>
+  <si>
+    <t>Same_gen</t>
+  </si>
+  <si>
+    <t>PTE</t>
+  </si>
+  <si>
+    <t>Chess</t>
+  </si>
+  <si>
+    <t>Countries</t>
+  </si>
+  <si>
+    <t>nations</t>
+  </si>
+  <si>
+    <t>WebKP</t>
+  </si>
+  <si>
+    <t>DCG</t>
+  </si>
+  <si>
+    <t>Mesh</t>
+  </si>
+  <si>
+    <t>imdb_small</t>
+  </si>
+  <si>
+    <t>TubePricing</t>
+  </si>
+  <si>
+    <t>imdb_MovieLens</t>
+  </si>
+  <si>
     <t>NCAA</t>
   </si>
   <si>
-    <t>Countries</t>
-  </si>
-  <si>
-    <t>PremierLeague</t>
-  </si>
-  <si>
-    <t>university</t>
-  </si>
-  <si>
-    <t>Bupa</t>
-  </si>
-  <si>
-    <t>nations</t>
-  </si>
-  <si>
-    <t>Student_loan</t>
-  </si>
-  <si>
-    <t>DCG</t>
-  </si>
-  <si>
-    <t>got_families</t>
-  </si>
-  <si>
-    <t>legalActs</t>
-  </si>
-  <si>
-    <t>SAP</t>
-  </si>
-  <si>
-    <t>imdb_small</t>
-  </si>
-  <si>
-    <t>Same_gen</t>
-  </si>
-  <si>
-    <t>trains</t>
-  </si>
-  <si>
-    <t>Facebook</t>
-  </si>
-  <si>
-    <t>genes</t>
-  </si>
-  <si>
-    <t>Pyrimidine</t>
-  </si>
-  <si>
-    <t>imdb_ijs</t>
-  </si>
-  <si>
-    <t>Pima</t>
-  </si>
-  <si>
-    <t>AustralianFootball</t>
-  </si>
-  <si>
-    <t>OMOP_CDM_dayz</t>
-  </si>
-  <si>
-    <t>TubePricing</t>
-  </si>
-  <si>
-    <t>restbase</t>
-  </si>
-  <si>
-    <t>financial</t>
-  </si>
-  <si>
-    <t>Mooney_Family</t>
-  </si>
-  <si>
-    <t>Atherosclerosis</t>
-  </si>
-  <si>
-    <t>Triazine</t>
-  </si>
-  <si>
-    <t>UW_std</t>
-  </si>
-  <si>
-    <t>fake_hotels_extended</t>
-  </si>
-  <si>
-    <t>CORA</t>
-  </si>
-  <si>
-    <t>Mesh</t>
-  </si>
-  <si>
-    <t>Chess</t>
-  </si>
-  <si>
-    <t>Biodegradability</t>
-  </si>
-  <si>
-    <t>PTE</t>
-  </si>
-  <si>
-    <t>SalesDB</t>
-  </si>
-  <si>
-    <t>MuskSmall</t>
-  </si>
-  <si>
-    <t>Dunur</t>
-  </si>
-  <si>
-    <t>SAT</t>
-  </si>
-  <si>
-    <t>WebKP</t>
-  </si>
-  <si>
-    <t>FNHK</t>
-  </si>
-  <si>
-    <t>UTube</t>
-  </si>
-  <si>
-    <t>NBA</t>
-  </si>
-  <si>
-    <t>imdb_MovieLens</t>
-  </si>
-  <si>
-    <t>Elti</t>
-  </si>
-  <si>
-    <t>airbnb-simplified</t>
-  </si>
-  <si>
-    <t>multi_table_ID_demo_dataset</t>
-  </si>
-  <si>
-    <t>mutagenesis</t>
-  </si>
-  <si>
-    <t>Toxicology</t>
-  </si>
-  <si>
-    <t>Carcinogenesis</t>
-  </si>
-  <si>
-    <t>fake_hotels</t>
-  </si>
-  <si>
-    <t>Hepatitis_std</t>
-  </si>
-  <si>
-    <t>Accidents</t>
-  </si>
-  <si>
-    <t>census</t>
-  </si>
-  <si>
-    <t>expedia_hotel_logs</t>
-  </si>
-  <si>
-    <t>insurance</t>
-  </si>
-  <si>
-    <t>news</t>
-  </si>
-  <si>
-    <t>covtype</t>
-  </si>
-  <si>
-    <t>child</t>
-  </si>
-  <si>
-    <t>intrusion</t>
-  </si>
-  <si>
-    <t>alarm</t>
-  </si>
-  <si>
-    <t>adult</t>
+    <t>single_table</t>
   </si>
   <si>
     <t>multi_table</t>
   </si>
   <si>
-    <t>single_table</t>
+    <t>RealTabFormerSynthesizer</t>
+  </si>
+  <si>
+    <t>GaussianCopulaSynthesizer</t>
+  </si>
+  <si>
+    <t>SegmentSynthesizer</t>
+  </si>
+  <si>
+    <t>TVAESynthesizer</t>
   </si>
   <si>
     <t>HSASynthesizer</t>
   </si>
   <si>
+    <t>IndependentSynthesizer</t>
+  </si>
+  <si>
     <t>HMASynthesizer</t>
   </si>
   <si>
-    <t>IndependentSynthesizer</t>
-  </si>
-  <si>
     <t>MultiTableUniformSynthesizer</t>
-  </si>
-  <si>
-    <t>RealTabFormerSynthesizer</t>
-  </si>
-  <si>
-    <t>GaussianCopulaSynthesizer</t>
-  </si>
-  <si>
-    <t>SegmentSynthesizer</t>
-  </si>
-  <si>
-    <t>TVAESynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -681,31 +681,31 @@
         <v>77</v>
       </c>
       <c r="D2">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="E2">
-        <v>96491</v>
+        <v>299285</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2" t="s">
         <v>85</v>
       </c>
       <c r="L2">
-        <v>4.68</v>
+        <v>98.17</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -722,28 +722,28 @@
         <v>25</v>
       </c>
       <c r="E3">
-        <v>5302</v>
+        <v>1000</v>
       </c>
       <c r="F3">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="G3">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" t="s">
         <v>85</v>
       </c>
       <c r="L3">
-        <v>0.23</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -757,31 +757,31 @@
         <v>79</v>
       </c>
       <c r="D4">
-        <v>112</v>
+        <v>27</v>
       </c>
       <c r="E4">
-        <v>202305</v>
+        <v>20000</v>
       </c>
       <c r="F4">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="G4">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K4" t="s">
         <v>85</v>
       </c>
       <c r="L4">
-        <v>27.15</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -795,31 +795,31 @@
         <v>77</v>
       </c>
       <c r="D5">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E5">
-        <v>22318</v>
+        <v>39644</v>
       </c>
       <c r="F5">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="H5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5" t="s">
         <v>85</v>
       </c>
       <c r="L5">
-        <v>9.93</v>
+        <v>18.71</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -830,34 +830,34 @@
         <v>75</v>
       </c>
       <c r="C6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D6">
-        <v>218</v>
+        <v>55</v>
       </c>
       <c r="E6">
-        <v>11308</v>
+        <v>581012</v>
       </c>
       <c r="F6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G6">
-        <v>204</v>
+        <v>54</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I6">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K6" t="s">
         <v>85</v>
       </c>
       <c r="L6">
-        <v>17.2</v>
+        <v>255.65</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -868,34 +868,34 @@
         <v>75</v>
       </c>
       <c r="C7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D7">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E7">
-        <v>171</v>
+        <v>20000</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="G7">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" t="s">
         <v>85</v>
       </c>
       <c r="L7">
-        <v>0.01</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -906,34 +906,34 @@
         <v>75</v>
       </c>
       <c r="C8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D8">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="E8">
-        <v>2762</v>
+        <v>494021</v>
       </c>
       <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="G8">
+        <v>37</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
         <v>0</v>
       </c>
-      <c r="G8">
-        <v>7</v>
-      </c>
-      <c r="H8">
-        <v>9</v>
-      </c>
-      <c r="I8">
-        <v>8</v>
-      </c>
       <c r="J8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8" t="s">
         <v>85</v>
       </c>
       <c r="L8">
-        <v>0.04</v>
+        <v>162.04</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -944,34 +944,34 @@
         <v>75</v>
       </c>
       <c r="C9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D9">
-        <v>119</v>
+        <v>37</v>
       </c>
       <c r="E9">
-        <v>11004</v>
+        <v>20000</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="G9">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" t="s">
         <v>85</v>
       </c>
       <c r="L9">
-        <v>0.45</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -985,31 +985,31 @@
         <v>77</v>
       </c>
       <c r="D10">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E10">
-        <v>5288</v>
+        <v>32561</v>
       </c>
       <c r="F10">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G10">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H10">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I10">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" t="s">
         <v>85</v>
       </c>
       <c r="L10">
-        <v>0.09</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1017,37 +1017,37 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C11" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D11">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E11">
-        <v>8258</v>
+        <v>1219</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K11" t="s">
         <v>85</v>
       </c>
       <c r="L11">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1055,37 +1055,37 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D12">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E12">
-        <v>23</v>
+        <v>1463093</v>
       </c>
       <c r="F12">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="G12">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H12">
         <v>3</v>
       </c>
       <c r="I12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K12" t="s">
         <v>85</v>
       </c>
       <c r="L12">
-        <v>0</v>
+        <v>219.33</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1093,37 +1093,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D13">
-        <v>35</v>
+        <v>432</v>
       </c>
       <c r="E13">
-        <v>1754397</v>
+        <v>39000</v>
       </c>
       <c r="F13">
-        <v>18</v>
+        <v>108</v>
       </c>
       <c r="G13">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="H13">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="I13">
-        <v>5</v>
+        <v>171</v>
       </c>
       <c r="J13">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="K13" t="s">
         <v>85</v>
       </c>
       <c r="L13">
-        <v>130.3</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1131,37 +1131,37 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C14" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D14">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="E14">
-        <v>3841029</v>
+        <v>712</v>
       </c>
       <c r="F14">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G14">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="H14">
         <v>4</v>
       </c>
       <c r="I14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" t="s">
         <v>85</v>
       </c>
       <c r="L14">
-        <v>148.44</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1169,37 +1169,37 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C15" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D15">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E15">
-        <v>4395</v>
+        <v>11150</v>
       </c>
       <c r="F15">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G15">
+        <v>3</v>
+      </c>
+      <c r="H15">
         <v>4</v>
       </c>
-      <c r="H15">
-        <v>7</v>
-      </c>
       <c r="I15">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K15" t="s">
         <v>85</v>
       </c>
       <c r="L15">
-        <v>0.15</v>
+        <v>0.6928000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1207,28 +1207,28 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C16" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D16">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E16">
-        <v>1536</v>
+        <v>2735</v>
       </c>
       <c r="F16">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G16">
         <v>0</v>
       </c>
       <c r="H16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I16">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J16">
         <v>2</v>
@@ -1237,7 +1237,7 @@
         <v>85</v>
       </c>
       <c r="L16">
-        <v>0.04</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1245,29 +1245,29 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C17" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D17">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E17">
-        <v>83</v>
+        <v>5647694</v>
       </c>
       <c r="F17">
+        <v>9</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+      <c r="H17">
+        <v>7</v>
+      </c>
+      <c r="I17">
         <v>6</v>
       </c>
-      <c r="G17">
-        <v>4</v>
-      </c>
-      <c r="H17">
-        <v>2</v>
-      </c>
-      <c r="I17">
-        <v>1</v>
-      </c>
       <c r="J17">
         <v>2</v>
       </c>
@@ -1275,7 +1275,7 @@
         <v>85</v>
       </c>
       <c r="L17">
-        <v>0.01</v>
+        <v>173.9</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1283,28 +1283,28 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C18" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D18">
-        <v>266</v>
+        <v>13</v>
       </c>
       <c r="E18">
-        <v>10173</v>
+        <v>83</v>
       </c>
       <c r="F18">
-        <v>262</v>
+        <v>6</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H18">
         <v>2</v>
       </c>
       <c r="I18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J18">
         <v>2</v>
@@ -1313,7 +1313,7 @@
         <v>85</v>
       </c>
       <c r="L18">
-        <v>1.38</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1321,28 +1321,28 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C19" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D19">
-        <v>16</v>
+        <v>266</v>
       </c>
       <c r="E19">
-        <v>6118</v>
+        <v>10173</v>
       </c>
       <c r="F19">
-        <v>9</v>
+        <v>262</v>
       </c>
       <c r="G19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J19">
         <v>2</v>
@@ -1351,7 +1351,7 @@
         <v>85</v>
       </c>
       <c r="L19">
-        <v>0.36</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1359,28 +1359,28 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C20" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D20">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E20">
-        <v>296</v>
+        <v>57353</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G20">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H20">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J20">
         <v>2</v>
@@ -1389,7 +1389,7 @@
         <v>85</v>
       </c>
       <c r="L20">
-        <v>0.02</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1397,28 +1397,28 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C21" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D21">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E21">
-        <v>5647694</v>
+        <v>1754397</v>
       </c>
       <c r="F21">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="G21">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H21">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J21">
         <v>2</v>
@@ -1427,7 +1427,7 @@
         <v>85</v>
       </c>
       <c r="L21">
-        <v>173.9</v>
+        <v>130.3</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1435,28 +1435,28 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C22" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D22">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E22">
-        <v>6912</v>
+        <v>6735507</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G22">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H22">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I22">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J22">
         <v>2</v>
@@ -1465,7 +1465,7 @@
         <v>85</v>
       </c>
       <c r="L22">
-        <v>0.11</v>
+        <v>269.25</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1473,37 +1473,37 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C23" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D23">
-        <v>78</v>
+        <v>17</v>
       </c>
       <c r="E23">
-        <v>139179</v>
+        <v>2762</v>
       </c>
       <c r="F23">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="H23">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I23">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K23" t="s">
         <v>85</v>
       </c>
       <c r="L23">
-        <v>31.18</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1511,37 +1511,37 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C24" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D24">
-        <v>432</v>
+        <v>198</v>
       </c>
       <c r="E24">
-        <v>39000</v>
+        <v>12781</v>
       </c>
       <c r="F24">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="G24">
-        <v>51</v>
+        <v>193</v>
       </c>
       <c r="H24">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="I24">
-        <v>171</v>
+        <v>3</v>
       </c>
       <c r="J24">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K24" t="s">
         <v>85</v>
       </c>
       <c r="L24">
-        <v>3.45</v>
+        <v>6.62</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1549,37 +1549,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C25" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D25">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="E25">
-        <v>154899</v>
+        <v>5751408</v>
       </c>
       <c r="F25">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="G25">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="H25">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="I25">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="J25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K25" t="s">
         <v>85</v>
       </c>
       <c r="L25">
-        <v>9.67</v>
+        <v>293.14</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1587,37 +1587,37 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C26" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D26">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="E26">
-        <v>19297</v>
+        <v>19867</v>
       </c>
       <c r="F26">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H26">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="I26">
-        <v>3</v>
+        <v>65</v>
       </c>
       <c r="J26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K26" t="s">
         <v>85</v>
       </c>
       <c r="L26">
-        <v>0.6899999999999999</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1625,37 +1625,37 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C27" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D27">
-        <v>55</v>
+        <v>202</v>
       </c>
       <c r="E27">
-        <v>1079680</v>
+        <v>4425</v>
       </c>
       <c r="F27">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H27">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="I27">
-        <v>8</v>
+        <v>189</v>
       </c>
       <c r="J27">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K27" t="s">
         <v>85</v>
       </c>
       <c r="L27">
-        <v>85.38</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1663,37 +1663,37 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C28" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D28">
-        <v>202</v>
+        <v>16</v>
       </c>
       <c r="E28">
-        <v>4425</v>
+        <v>21895</v>
       </c>
       <c r="F28">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H28">
-        <v>68</v>
+        <v>5</v>
       </c>
       <c r="I28">
-        <v>134</v>
+        <v>5</v>
       </c>
       <c r="J28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K28" t="s">
         <v>85</v>
       </c>
       <c r="L28">
-        <v>0.1</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1701,28 +1701,28 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C29" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D29">
-        <v>198</v>
+        <v>11</v>
       </c>
       <c r="E29">
-        <v>12781</v>
+        <v>96491</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G29">
-        <v>193</v>
+        <v>1</v>
       </c>
       <c r="H29">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I29">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J29">
         <v>2</v>
@@ -1731,7 +1731,7 @@
         <v>85</v>
       </c>
       <c r="L29">
-        <v>6.62</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1739,37 +1739,37 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C30" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D30">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="E30">
-        <v>1302</v>
+        <v>440</v>
       </c>
       <c r="F30">
+        <v>1</v>
+      </c>
+      <c r="G30">
         <v>0</v>
       </c>
-      <c r="G30">
-        <v>12</v>
-      </c>
       <c r="H30">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I30">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="J30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K30" t="s">
         <v>85</v>
       </c>
       <c r="L30">
-        <v>0.12</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1777,28 +1777,28 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C31" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D31">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E31">
-        <v>712</v>
+        <v>6118</v>
       </c>
       <c r="F31">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G31">
         <v>2</v>
       </c>
       <c r="H31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J31">
         <v>2</v>
@@ -1807,7 +1807,7 @@
         <v>85</v>
       </c>
       <c r="L31">
-        <v>0.02</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1815,28 +1815,28 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C32" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D32">
         <v>19</v>
       </c>
       <c r="E32">
-        <v>668</v>
+        <v>171</v>
       </c>
       <c r="F32">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G32">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H32">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I32">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J32">
         <v>2</v>
@@ -1845,7 +1845,7 @@
         <v>85</v>
       </c>
       <c r="L32">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1853,37 +1853,37 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C33" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D33">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E33">
-        <v>57353</v>
+        <v>3841029</v>
       </c>
       <c r="F33">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G33">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="H33">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I33">
         <v>3</v>
       </c>
       <c r="J33">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K33" t="s">
         <v>85</v>
       </c>
       <c r="L33">
-        <v>1.79</v>
+        <v>148.44</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1891,28 +1891,28 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C34" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D34">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="E34">
-        <v>2700</v>
+        <v>6912</v>
       </c>
       <c r="F34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H34">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="I34">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="J34">
         <v>2</v>
@@ -1921,7 +1921,7 @@
         <v>85</v>
       </c>
       <c r="L34">
-        <v>0.04</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1929,22 +1929,22 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C35" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D35">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="E35">
-        <v>2052</v>
+        <v>1302</v>
       </c>
       <c r="F35">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="G35">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H35">
         <v>2</v>
@@ -1959,7 +1959,7 @@
         <v>85</v>
       </c>
       <c r="L35">
-        <v>0.25</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -1967,37 +1967,37 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C36" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D36">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E36">
-        <v>21895</v>
+        <v>5302</v>
       </c>
       <c r="F36">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G36">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H36">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I36">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K36" t="s">
         <v>85</v>
       </c>
       <c r="L36">
-        <v>0.57</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -2005,37 +2005,37 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C37" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D37">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="E37">
-        <v>29850</v>
+        <v>1352</v>
       </c>
       <c r="F37">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G37">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H37">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="I37">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="J37">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K37" t="s">
         <v>85</v>
       </c>
       <c r="L37">
-        <v>0.95</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2043,37 +2043,37 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C38" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D38">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E38">
-        <v>6735507</v>
+        <v>10324</v>
       </c>
       <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38">
         <v>7</v>
       </c>
-      <c r="G38">
-        <v>2</v>
-      </c>
       <c r="H38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I38">
         <v>3</v>
       </c>
       <c r="J38">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K38" t="s">
         <v>85</v>
       </c>
       <c r="L38">
-        <v>269.25</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2081,22 +2081,22 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D39">
-        <v>170</v>
+        <v>14</v>
       </c>
       <c r="E39">
-        <v>568</v>
+        <v>296</v>
       </c>
       <c r="F39">
         <v>0</v>
       </c>
       <c r="G39">
-        <v>167</v>
+        <v>11</v>
       </c>
       <c r="H39">
         <v>2</v>
@@ -2111,7 +2111,7 @@
         <v>85</v>
       </c>
       <c r="L39">
-        <v>0.64</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2119,28 +2119,28 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C40" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D40">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="E40">
-        <v>440</v>
+        <v>2113275</v>
       </c>
       <c r="F40">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G40">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H40">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="I40">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="J40">
         <v>2</v>
@@ -2149,7 +2149,7 @@
         <v>85</v>
       </c>
       <c r="L40">
-        <v>0.01</v>
+        <v>120</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2157,37 +2157,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C41" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D41">
-        <v>70</v>
+        <v>12</v>
       </c>
       <c r="E41">
-        <v>19867</v>
+        <v>36922</v>
       </c>
       <c r="F41">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G41">
         <v>0</v>
       </c>
       <c r="H41">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="I41">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="J41">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K41" t="s">
         <v>85</v>
       </c>
       <c r="L41">
-        <v>0.32</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2195,37 +2195,37 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C42" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D42">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="E42">
-        <v>81850</v>
+        <v>27443</v>
       </c>
       <c r="F42">
         <v>2</v>
       </c>
       <c r="G42">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H42">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I42">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="J42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K42" t="s">
         <v>85</v>
       </c>
       <c r="L42">
-        <v>1.96</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2233,37 +2233,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C43" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D43">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="E43">
-        <v>2113275</v>
+        <v>19297</v>
       </c>
       <c r="F43">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G43">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H43">
         <v>3</v>
       </c>
       <c r="I43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K43" t="s">
         <v>85</v>
       </c>
       <c r="L43">
-        <v>120</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2271,22 +2271,22 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C44" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D44">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E44">
-        <v>2735</v>
+        <v>668</v>
       </c>
       <c r="F44">
         <v>5</v>
       </c>
       <c r="G44">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H44">
         <v>2</v>
@@ -2301,7 +2301,7 @@
         <v>85</v>
       </c>
       <c r="L44">
-        <v>0.11</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2309,37 +2309,37 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C45" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D45">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="E45">
-        <v>1219</v>
+        <v>668</v>
       </c>
       <c r="F45">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G45">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="H45">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I45">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J45">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K45" t="s">
         <v>85</v>
       </c>
       <c r="L45">
-        <v>0.15</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2347,37 +2347,37 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C46" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D46">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="E46">
-        <v>1249411</v>
+        <v>1079680</v>
       </c>
       <c r="F46">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="G46">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="H46">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I46">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J46">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K46" t="s">
         <v>85</v>
       </c>
       <c r="L46">
-        <v>39.2</v>
+        <v>85.38</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2385,28 +2385,28 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C47" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D47">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E47">
-        <v>1352</v>
+        <v>5288</v>
       </c>
       <c r="F47">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G47">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H47">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I47">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="J47">
         <v>2</v>
@@ -2415,7 +2415,7 @@
         <v>85</v>
       </c>
       <c r="L47">
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2423,28 +2423,28 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C48" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D48">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="E48">
-        <v>5751408</v>
+        <v>12927</v>
       </c>
       <c r="F48">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="G48">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H48">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I48">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J48">
         <v>2</v>
@@ -2453,7 +2453,7 @@
         <v>85</v>
       </c>
       <c r="L48">
-        <v>293.14</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2461,28 +2461,28 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C49" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D49">
-        <v>22</v>
+        <v>78</v>
       </c>
       <c r="E49">
-        <v>11150</v>
+        <v>139179</v>
       </c>
       <c r="F49">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G49">
-        <v>3</v>
+        <v>57</v>
       </c>
       <c r="H49">
         <v>4</v>
       </c>
       <c r="I49">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J49">
         <v>3</v>
@@ -2491,7 +2491,7 @@
         <v>85</v>
       </c>
       <c r="L49">
-        <v>0.6928000000000001</v>
+        <v>31.18</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2499,28 +2499,28 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C50" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D50">
-        <v>15</v>
+        <v>218</v>
       </c>
       <c r="E50">
-        <v>10324</v>
+        <v>11308</v>
       </c>
       <c r="F50">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G50">
-        <v>7</v>
+        <v>204</v>
       </c>
       <c r="H50">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I50">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J50">
         <v>3</v>
@@ -2529,7 +2529,7 @@
         <v>85</v>
       </c>
       <c r="L50">
-        <v>0.37</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2537,37 +2537,37 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C51" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D51">
-        <v>12</v>
+        <v>170</v>
       </c>
       <c r="E51">
-        <v>36922</v>
+        <v>568</v>
       </c>
       <c r="F51">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G51">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="H51">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I51">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J51">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K51" t="s">
         <v>85</v>
       </c>
       <c r="L51">
-        <v>1.03</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2575,37 +2575,37 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C52" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D52">
+        <v>9</v>
+      </c>
+      <c r="E52">
         <v>23</v>
       </c>
-      <c r="E52">
-        <v>27443</v>
-      </c>
       <c r="F52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G52">
         <v>2</v>
       </c>
       <c r="H52">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I52">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="J52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K52" t="s">
         <v>85</v>
       </c>
       <c r="L52">
-        <v>0.9399999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2613,28 +2613,28 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C53" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D53">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E53">
-        <v>668</v>
+        <v>1536</v>
       </c>
       <c r="F53">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G53">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H53">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I53">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J53">
         <v>2</v>
@@ -2643,7 +2643,7 @@
         <v>85</v>
       </c>
       <c r="L53">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2651,37 +2651,37 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C54" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D54">
-        <v>29</v>
+        <v>97</v>
       </c>
       <c r="E54">
-        <v>12927</v>
+        <v>29850</v>
       </c>
       <c r="F54">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="G54">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="H54">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="I54">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="J54">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K54" t="s">
         <v>85</v>
       </c>
       <c r="L54">
-        <v>0.68</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2689,37 +2689,37 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C55" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D55">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E55">
-        <v>1463093</v>
+        <v>2052</v>
       </c>
       <c r="F55">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="G55">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="H55">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I55">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J55">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K55" t="s">
         <v>85</v>
       </c>
       <c r="L55">
-        <v>219.33</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2733,31 +2733,31 @@
         <v>81</v>
       </c>
       <c r="D56">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="E56">
-        <v>299285</v>
+        <v>22318</v>
       </c>
       <c r="F56">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="G56">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="H56">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I56">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J56">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K56" t="s">
         <v>85</v>
       </c>
       <c r="L56">
-        <v>98.17</v>
+        <v>9.93</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2771,31 +2771,31 @@
         <v>82</v>
       </c>
       <c r="D57">
-        <v>25</v>
+        <v>119</v>
       </c>
       <c r="E57">
-        <v>1000</v>
+        <v>11004</v>
       </c>
       <c r="F57">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G57">
-        <v>5</v>
+        <v>112</v>
       </c>
       <c r="H57">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I57">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K57" t="s">
         <v>85</v>
       </c>
       <c r="L57">
-        <v>0.2</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2806,34 +2806,34 @@
         <v>76</v>
       </c>
       <c r="C58" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D58">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="E58">
-        <v>20000</v>
+        <v>81850</v>
       </c>
       <c r="F58">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="G58">
         <v>0</v>
       </c>
       <c r="H58">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I58">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J58">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K58" t="s">
         <v>85</v>
       </c>
       <c r="L58">
-        <v>3.34</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2847,31 +2847,31 @@
         <v>81</v>
       </c>
       <c r="D59">
-        <v>59</v>
+        <v>6</v>
       </c>
       <c r="E59">
-        <v>39644</v>
+        <v>8258</v>
       </c>
       <c r="F59">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G59">
-        <v>59</v>
+        <v>1</v>
       </c>
       <c r="H59">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I59">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J59">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K59" t="s">
         <v>85</v>
       </c>
       <c r="L59">
-        <v>18.71</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2885,31 +2885,31 @@
         <v>81</v>
       </c>
       <c r="D60">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="E60">
-        <v>581012</v>
+        <v>2700</v>
       </c>
       <c r="F60">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G60">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="H60">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="I60">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="J60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K60" t="s">
         <v>85</v>
       </c>
       <c r="L60">
-        <v>255.65</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2920,34 +2920,34 @@
         <v>76</v>
       </c>
       <c r="C61" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D61">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E61">
-        <v>20000</v>
+        <v>4395</v>
       </c>
       <c r="F61">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="G61">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H61">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I61">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J61">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K61" t="s">
         <v>85</v>
       </c>
       <c r="L61">
-        <v>3.2</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -2958,34 +2958,34 @@
         <v>76</v>
       </c>
       <c r="C62" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D62">
-        <v>41</v>
+        <v>192</v>
       </c>
       <c r="E62">
-        <v>494021</v>
+        <v>154899</v>
       </c>
       <c r="F62">
-        <v>4</v>
+        <v>54</v>
       </c>
       <c r="G62">
-        <v>37</v>
+        <v>92</v>
       </c>
       <c r="H62">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="I62">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="J62">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K62" t="s">
         <v>85</v>
       </c>
       <c r="L62">
-        <v>162.04</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -2996,34 +2996,34 @@
         <v>76</v>
       </c>
       <c r="C63" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D63">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="E63">
-        <v>20000</v>
+        <v>1249411</v>
       </c>
       <c r="F63">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="G63">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H63">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I63">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J63">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K63" t="s">
         <v>85</v>
       </c>
       <c r="L63">
-        <v>4.52</v>
+        <v>39.2</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3034,34 +3034,34 @@
         <v>76</v>
       </c>
       <c r="C64" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D64">
-        <v>15</v>
+        <v>112</v>
       </c>
       <c r="E64">
-        <v>32561</v>
+        <v>202305</v>
       </c>
       <c r="F64">
+        <v>14</v>
+      </c>
+      <c r="G64">
+        <v>72</v>
+      </c>
+      <c r="H64">
         <v>9</v>
       </c>
-      <c r="G64">
-        <v>6</v>
-      </c>
-      <c r="H64">
-        <v>1</v>
-      </c>
       <c r="I64">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="J64">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K64" t="s">
         <v>85</v>
       </c>
       <c r="L64">
-        <v>3.91</v>
+        <v>27.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_04_01_2026) - Modality: single_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -52,220 +52,220 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>Same_gen</t>
+  </si>
+  <si>
+    <t>imdb_small</t>
+  </si>
+  <si>
+    <t>trains</t>
+  </si>
+  <si>
+    <t>SAT</t>
+  </si>
+  <si>
+    <t>legalActs</t>
+  </si>
+  <si>
+    <t>Dunur</t>
+  </si>
+  <si>
+    <t>fake_hotels_extended</t>
+  </si>
+  <si>
+    <t>Biodegradability</t>
+  </si>
+  <si>
+    <t>OMOP_CDM_dayz</t>
+  </si>
+  <si>
+    <t>mutagenesis</t>
+  </si>
+  <si>
+    <t>Mesh</t>
+  </si>
+  <si>
+    <t>Pima</t>
+  </si>
+  <si>
+    <t>Countries</t>
+  </si>
+  <si>
+    <t>genes</t>
+  </si>
+  <si>
+    <t>airbnb-simplified</t>
+  </si>
+  <si>
+    <t>Chess</t>
+  </si>
+  <si>
+    <t>Toxicology</t>
+  </si>
+  <si>
+    <t>fake_hotels</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>UTube</t>
+  </si>
+  <si>
+    <t>got_families</t>
+  </si>
+  <si>
+    <t>Hepatitis_std</t>
+  </si>
+  <si>
+    <t>Student_loan</t>
+  </si>
+  <si>
+    <t>multi_table_ID_demo_dataset</t>
+  </si>
+  <si>
+    <t>Pyrimidine</t>
+  </si>
+  <si>
+    <t>CORA</t>
+  </si>
+  <si>
+    <t>imdb_ijs</t>
+  </si>
+  <si>
+    <t>world</t>
+  </si>
+  <si>
+    <t>Elti</t>
+  </si>
+  <si>
+    <t>PTE</t>
+  </si>
+  <si>
+    <t>Carcinogenesis</t>
+  </si>
+  <si>
+    <t>PremierLeague</t>
+  </si>
+  <si>
+    <t>SalesDB</t>
+  </si>
+  <si>
+    <t>Triazine</t>
+  </si>
+  <si>
+    <t>UW_std</t>
+  </si>
+  <si>
+    <t>imdb_MovieLens</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>nations</t>
+  </si>
+  <si>
+    <t>AustralianFootball</t>
+  </si>
+  <si>
+    <t>ftp</t>
+  </si>
+  <si>
+    <t>NCAA</t>
+  </si>
+  <si>
+    <t>restbase</t>
+  </si>
+  <si>
+    <t>TubePricing</t>
+  </si>
+  <si>
+    <t>Accidents</t>
+  </si>
+  <si>
+    <t>financial</t>
+  </si>
+  <si>
+    <t>MuskSmall</t>
+  </si>
+  <si>
+    <t>Atherosclerosis</t>
+  </si>
+  <si>
+    <t>NBA</t>
+  </si>
+  <si>
+    <t>WebKP</t>
+  </si>
+  <si>
+    <t>university</t>
+  </si>
+  <si>
+    <t>FNHK</t>
+  </si>
+  <si>
+    <t>Mooney_Family</t>
+  </si>
+  <si>
+    <t>DCG</t>
+  </si>
+  <si>
+    <t>Bupa</t>
+  </si>
+  <si>
+    <t>expedia_hotel_logs</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
     <t>alarm</t>
   </si>
   <si>
+    <t>news</t>
+  </si>
+  <si>
     <t>intrusion</t>
   </si>
   <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>adult</t>
+  </si>
+  <si>
+    <t>covtype</t>
+  </si>
+  <si>
     <t>insurance</t>
   </si>
   <si>
-    <t>child</t>
-  </si>
-  <si>
-    <t>adult</t>
-  </si>
-  <si>
-    <t>covtype</t>
-  </si>
-  <si>
-    <t>expedia_hotel_logs</t>
-  </si>
-  <si>
-    <t>news</t>
-  </si>
-  <si>
-    <t>census</t>
-  </si>
-  <si>
-    <t>Same_gen</t>
-  </si>
-  <si>
-    <t>imdb_small</t>
-  </si>
-  <si>
-    <t>trains</t>
-  </si>
-  <si>
-    <t>SAT</t>
-  </si>
-  <si>
-    <t>legalActs</t>
-  </si>
-  <si>
-    <t>Dunur</t>
-  </si>
-  <si>
-    <t>fake_hotels_extended</t>
-  </si>
-  <si>
-    <t>Biodegradability</t>
-  </si>
-  <si>
-    <t>OMOP_CDM_dayz</t>
-  </si>
-  <si>
-    <t>mutagenesis</t>
-  </si>
-  <si>
-    <t>Mesh</t>
-  </si>
-  <si>
-    <t>Pima</t>
-  </si>
-  <si>
-    <t>Countries</t>
-  </si>
-  <si>
-    <t>genes</t>
-  </si>
-  <si>
-    <t>airbnb-simplified</t>
-  </si>
-  <si>
-    <t>Chess</t>
-  </si>
-  <si>
-    <t>Toxicology</t>
-  </si>
-  <si>
-    <t>fake_hotels</t>
-  </si>
-  <si>
-    <t>Facebook</t>
-  </si>
-  <si>
-    <t>UTube</t>
-  </si>
-  <si>
-    <t>got_families</t>
-  </si>
-  <si>
-    <t>Hepatitis_std</t>
-  </si>
-  <si>
-    <t>Student_loan</t>
-  </si>
-  <si>
-    <t>multi_table_ID_demo_dataset</t>
-  </si>
-  <si>
-    <t>Pyrimidine</t>
-  </si>
-  <si>
-    <t>CORA</t>
-  </si>
-  <si>
-    <t>imdb_ijs</t>
-  </si>
-  <si>
-    <t>world</t>
-  </si>
-  <si>
-    <t>Elti</t>
-  </si>
-  <si>
-    <t>PTE</t>
-  </si>
-  <si>
-    <t>Carcinogenesis</t>
-  </si>
-  <si>
-    <t>PremierLeague</t>
-  </si>
-  <si>
-    <t>SalesDB</t>
-  </si>
-  <si>
-    <t>Triazine</t>
-  </si>
-  <si>
-    <t>UW_std</t>
-  </si>
-  <si>
-    <t>imdb_MovieLens</t>
-  </si>
-  <si>
-    <t>SAP</t>
-  </si>
-  <si>
-    <t>nations</t>
-  </si>
-  <si>
-    <t>AustralianFootball</t>
-  </si>
-  <si>
-    <t>ftp</t>
-  </si>
-  <si>
-    <t>NCAA</t>
-  </si>
-  <si>
-    <t>restbase</t>
-  </si>
-  <si>
-    <t>TubePricing</t>
-  </si>
-  <si>
-    <t>Accidents</t>
-  </si>
-  <si>
-    <t>financial</t>
-  </si>
-  <si>
-    <t>MuskSmall</t>
-  </si>
-  <si>
-    <t>Atherosclerosis</t>
-  </si>
-  <si>
-    <t>NBA</t>
-  </si>
-  <si>
-    <t>WebKP</t>
-  </si>
-  <si>
-    <t>university</t>
-  </si>
-  <si>
-    <t>FNHK</t>
-  </si>
-  <si>
-    <t>Mooney_Family</t>
-  </si>
-  <si>
-    <t>DCG</t>
-  </si>
-  <si>
-    <t>Bupa</t>
+    <t>multi_table</t>
   </si>
   <si>
     <t>single_table</t>
   </si>
   <si>
-    <t>multi_table</t>
+    <t>HSASynthesizer</t>
+  </si>
+  <si>
+    <t>IndependentSynthesizer</t>
+  </si>
+  <si>
+    <t>HMASynthesizer</t>
+  </si>
+  <si>
+    <t>GaussianCopulaSynthesizer</t>
   </si>
   <si>
     <t>TVAESynthesizer</t>
   </si>
   <si>
-    <t>RealTabFormerSynthesizer</t>
-  </si>
-  <si>
-    <t>SegmentSynthesizer</t>
-  </si>
-  <si>
-    <t>GaussianCopulaSynthesizer</t>
-  </si>
-  <si>
-    <t>HSASynthesizer</t>
-  </si>
-  <si>
-    <t>IndependentSynthesizer</t>
-  </si>
-  <si>
-    <t>HMASynthesizer</t>
+    <t>CopulaGANSynthesizer</t>
+  </si>
+  <si>
+    <t>CTGANSynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -678,31 +678,31 @@
         <v>77</v>
       </c>
       <c r="D2">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="E2">
-        <v>20000</v>
+        <v>1536</v>
       </c>
       <c r="F2">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2" t="s">
         <v>84</v>
       </c>
       <c r="L2">
-        <v>4.52</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -713,34 +713,34 @@
         <v>75</v>
       </c>
       <c r="C3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D3">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="E3">
-        <v>494021</v>
+        <v>4395</v>
       </c>
       <c r="F3">
+        <v>9</v>
+      </c>
+      <c r="G3">
         <v>4</v>
       </c>
-      <c r="G3">
-        <v>37</v>
-      </c>
       <c r="H3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="s">
         <v>84</v>
       </c>
       <c r="L3">
-        <v>162.04</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -751,34 +751,34 @@
         <v>75</v>
       </c>
       <c r="C4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D4">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E4">
-        <v>20000</v>
+        <v>83</v>
       </c>
       <c r="F4">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" t="s">
         <v>84</v>
       </c>
       <c r="L4">
-        <v>3.34</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -792,31 +792,31 @@
         <v>77</v>
       </c>
       <c r="D5">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="E5">
-        <v>20000</v>
+        <v>19867</v>
       </c>
       <c r="F5">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" t="s">
         <v>84</v>
       </c>
       <c r="L5">
-        <v>3.2</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -830,31 +830,31 @@
         <v>78</v>
       </c>
       <c r="D6">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E6">
-        <v>32561</v>
+        <v>1754397</v>
       </c>
       <c r="F6">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="G6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" t="s">
         <v>84</v>
       </c>
       <c r="L6">
-        <v>3.91</v>
+        <v>130.3</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -865,34 +865,34 @@
         <v>75</v>
       </c>
       <c r="C7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D7">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E7">
-        <v>581012</v>
+        <v>440</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K7" t="s">
         <v>84</v>
       </c>
       <c r="L7">
-        <v>255.65</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -903,34 +903,34 @@
         <v>75</v>
       </c>
       <c r="C8" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D8">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E8">
-        <v>1000</v>
+        <v>668</v>
       </c>
       <c r="F8">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="G8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" t="s">
         <v>84</v>
       </c>
       <c r="L8">
-        <v>0.2</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -941,34 +941,34 @@
         <v>75</v>
       </c>
       <c r="C9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D9">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="E9">
-        <v>39644</v>
+        <v>21895</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>59</v>
+        <v>4</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K9" t="s">
         <v>84</v>
       </c>
       <c r="L9">
-        <v>18.71</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -979,34 +979,34 @@
         <v>75</v>
       </c>
       <c r="C10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D10">
-        <v>41</v>
+        <v>432</v>
       </c>
       <c r="E10">
-        <v>299285</v>
+        <v>39000</v>
       </c>
       <c r="F10">
-        <v>29</v>
+        <v>108</v>
       </c>
       <c r="G10">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>171</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="K10" t="s">
         <v>84</v>
       </c>
       <c r="L10">
-        <v>98.17</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1014,37 +1014,37 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D11">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E11">
-        <v>1536</v>
+        <v>10324</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I11">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K11" t="s">
         <v>84</v>
       </c>
       <c r="L11">
-        <v>0.04</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1052,28 +1052,28 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C12" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D12">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="E12">
-        <v>4395</v>
+        <v>2700</v>
       </c>
       <c r="F12">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H12">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="I12">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="J12">
         <v>2</v>
@@ -1082,7 +1082,7 @@
         <v>84</v>
       </c>
       <c r="L12">
-        <v>0.15</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1090,28 +1090,28 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D13">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E13">
-        <v>83</v>
+        <v>6912</v>
       </c>
       <c r="F13">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H13">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J13">
         <v>2</v>
@@ -1120,7 +1120,7 @@
         <v>84</v>
       </c>
       <c r="L13">
-        <v>0.01</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1128,28 +1128,28 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C14" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D14">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E14">
-        <v>19867</v>
+        <v>22318</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="H14">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="I14">
-        <v>65</v>
+        <v>3</v>
       </c>
       <c r="J14">
         <v>2</v>
@@ -1158,7 +1158,7 @@
         <v>84</v>
       </c>
       <c r="L14">
-        <v>0.32</v>
+        <v>9.93</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1166,28 +1166,28 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C15" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D15">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="E15">
-        <v>1754397</v>
+        <v>6118</v>
       </c>
       <c r="F15">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="G15">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J15">
         <v>2</v>
@@ -1196,7 +1196,7 @@
         <v>84</v>
       </c>
       <c r="L15">
-        <v>130.3</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1204,37 +1204,37 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C16" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D16">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="E16">
-        <v>440</v>
+        <v>5751408</v>
       </c>
       <c r="F16">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="I16">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="J16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K16" t="s">
         <v>84</v>
       </c>
       <c r="L16">
-        <v>0.01</v>
+        <v>293.14</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1242,22 +1242,22 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C17" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D17">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="E17">
-        <v>668</v>
+        <v>2052</v>
       </c>
       <c r="F17">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="G17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H17">
         <v>2</v>
@@ -1272,7 +1272,7 @@
         <v>84</v>
       </c>
       <c r="L17">
-        <v>0.07000000000000001</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1280,25 +1280,25 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C18" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="D18">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E18">
-        <v>21895</v>
+        <v>36922</v>
       </c>
       <c r="F18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
         <v>4</v>
-      </c>
-      <c r="H18">
-        <v>5</v>
       </c>
       <c r="I18">
         <v>5</v>
@@ -1310,7 +1310,7 @@
         <v>84</v>
       </c>
       <c r="L18">
-        <v>0.57</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1318,37 +1318,37 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C19" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D19">
-        <v>432</v>
+        <v>15</v>
       </c>
       <c r="E19">
-        <v>39000</v>
+        <v>668</v>
       </c>
       <c r="F19">
-        <v>108</v>
+        <v>5</v>
       </c>
       <c r="G19">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="H19">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="I19">
-        <v>171</v>
+        <v>1</v>
       </c>
       <c r="J19">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K19" t="s">
         <v>84</v>
       </c>
       <c r="L19">
-        <v>3.45</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1356,37 +1356,37 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C20" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D20">
-        <v>15</v>
+        <v>266</v>
       </c>
       <c r="E20">
-        <v>10324</v>
+        <v>10173</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>262</v>
       </c>
       <c r="G20">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K20" t="s">
         <v>84</v>
       </c>
       <c r="L20">
-        <v>0.37</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1394,28 +1394,28 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C21" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D21">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="E21">
-        <v>2700</v>
+        <v>2735</v>
       </c>
       <c r="F21">
+        <v>5</v>
+      </c>
+      <c r="G21">
         <v>0</v>
       </c>
-      <c r="G21">
-        <v>2</v>
-      </c>
       <c r="H21">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="I21">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="J21">
         <v>2</v>
@@ -1424,7 +1424,7 @@
         <v>84</v>
       </c>
       <c r="L21">
-        <v>0.04</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1432,28 +1432,28 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C22" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D22">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="E22">
-        <v>6912</v>
+        <v>23</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G22">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H22">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I22">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J22">
         <v>2</v>
@@ -1462,7 +1462,7 @@
         <v>84</v>
       </c>
       <c r="L22">
-        <v>0.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1470,28 +1470,28 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C23" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D23">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="E23">
-        <v>22318</v>
+        <v>12927</v>
       </c>
       <c r="F23">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G23">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="H23">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I23">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J23">
         <v>2</v>
@@ -1500,7 +1500,7 @@
         <v>84</v>
       </c>
       <c r="L23">
-        <v>9.93</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1508,29 +1508,29 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C24" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D24">
         <v>16</v>
       </c>
       <c r="E24">
-        <v>6118</v>
+        <v>5288</v>
       </c>
       <c r="F24">
+        <v>2</v>
+      </c>
+      <c r="G24">
+        <v>2</v>
+      </c>
+      <c r="H24">
+        <v>10</v>
+      </c>
+      <c r="I24">
         <v>9</v>
       </c>
-      <c r="G24">
-        <v>2</v>
-      </c>
-      <c r="H24">
-        <v>3</v>
-      </c>
-      <c r="I24">
-        <v>3</v>
-      </c>
       <c r="J24">
         <v>2</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>84</v>
       </c>
       <c r="L24">
-        <v>0.36</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1546,37 +1546,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C25" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D25">
         <v>22</v>
       </c>
       <c r="E25">
-        <v>5751408</v>
+        <v>11150</v>
       </c>
       <c r="F25">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="G25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H25">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I25">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K25" t="s">
         <v>84</v>
       </c>
       <c r="L25">
-        <v>293.14</v>
+        <v>0.6928000000000001</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1584,22 +1584,22 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C26" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D26">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="E26">
-        <v>2052</v>
+        <v>296</v>
       </c>
       <c r="F26">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="G26">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="H26">
         <v>2</v>
@@ -1614,7 +1614,7 @@
         <v>84</v>
       </c>
       <c r="L26">
-        <v>0.25</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1622,37 +1622,37 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C27" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D27">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E27">
-        <v>36922</v>
+        <v>57353</v>
       </c>
       <c r="F27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H27">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I27">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K27" t="s">
         <v>84</v>
       </c>
       <c r="L27">
-        <v>1.03</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1660,28 +1660,28 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C28" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D28">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E28">
-        <v>668</v>
+        <v>5647694</v>
       </c>
       <c r="F28">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G28">
         <v>3</v>
       </c>
       <c r="H28">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I28">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J28">
         <v>2</v>
@@ -1690,7 +1690,7 @@
         <v>84</v>
       </c>
       <c r="L28">
-        <v>0.05</v>
+        <v>173.9</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1698,25 +1698,25 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C29" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D29">
-        <v>266</v>
+        <v>25</v>
       </c>
       <c r="E29">
-        <v>10173</v>
+        <v>5302</v>
       </c>
       <c r="F29">
-        <v>262</v>
+        <v>11</v>
       </c>
       <c r="G29">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I29">
         <v>2</v>
@@ -1728,7 +1728,7 @@
         <v>84</v>
       </c>
       <c r="L29">
-        <v>1.38</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1736,28 +1736,28 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C30" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D30">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="E30">
-        <v>2735</v>
+        <v>1352</v>
       </c>
       <c r="F30">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G30">
         <v>0</v>
       </c>
       <c r="H30">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="I30">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="J30">
         <v>2</v>
@@ -1766,7 +1766,7 @@
         <v>84</v>
       </c>
       <c r="L30">
-        <v>0.11</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1774,37 +1774,37 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C31" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D31">
+        <v>97</v>
+      </c>
+      <c r="E31">
+        <v>29850</v>
+      </c>
+      <c r="F31">
+        <v>25</v>
+      </c>
+      <c r="G31">
         <v>9</v>
       </c>
-      <c r="E31">
-        <v>23</v>
-      </c>
-      <c r="F31">
-        <v>3</v>
-      </c>
-      <c r="G31">
-        <v>2</v>
-      </c>
       <c r="H31">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="I31">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="J31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K31" t="s">
         <v>84</v>
       </c>
       <c r="L31">
-        <v>0</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1812,37 +1812,37 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C32" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D32">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="E32">
-        <v>12927</v>
+        <v>27443</v>
       </c>
       <c r="F32">
         <v>2</v>
       </c>
       <c r="G32">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I32">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="J32">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K32" t="s">
         <v>84</v>
       </c>
       <c r="L32">
-        <v>0.68</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1850,37 +1850,37 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C33" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D33">
-        <v>16</v>
+        <v>218</v>
       </c>
       <c r="E33">
-        <v>5288</v>
+        <v>11308</v>
       </c>
       <c r="F33">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G33">
-        <v>2</v>
+        <v>204</v>
       </c>
       <c r="H33">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I33">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J33">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K33" t="s">
         <v>84</v>
       </c>
       <c r="L33">
-        <v>0.09</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1888,22 +1888,22 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C34" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D34">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E34">
-        <v>11150</v>
+        <v>6735507</v>
       </c>
       <c r="F34">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H34">
         <v>4</v>
@@ -1912,13 +1912,13 @@
         <v>3</v>
       </c>
       <c r="J34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K34" t="s">
         <v>84</v>
       </c>
       <c r="L34">
-        <v>0.6928000000000001</v>
+        <v>269.25</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1926,22 +1926,22 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C35" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D35">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E35">
-        <v>296</v>
+        <v>1302</v>
       </c>
       <c r="F35">
         <v>0</v>
       </c>
       <c r="G35">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H35">
         <v>2</v>
@@ -1956,7 +1956,7 @@
         <v>84</v>
       </c>
       <c r="L35">
-        <v>0.02</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -1964,28 +1964,28 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C36" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D36">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E36">
-        <v>57353</v>
+        <v>712</v>
       </c>
       <c r="F36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G36">
         <v>2</v>
       </c>
       <c r="H36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J36">
         <v>2</v>
@@ -1994,7 +1994,7 @@
         <v>84</v>
       </c>
       <c r="L36">
-        <v>1.79</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -2002,22 +2002,22 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C37" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D37">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E37">
-        <v>5647694</v>
+        <v>1249411</v>
       </c>
       <c r="F37">
+        <v>5</v>
+      </c>
+      <c r="G37">
         <v>9</v>
-      </c>
-      <c r="G37">
-        <v>3</v>
       </c>
       <c r="H37">
         <v>7</v>
@@ -2032,7 +2032,7 @@
         <v>84</v>
       </c>
       <c r="L37">
-        <v>173.9</v>
+        <v>39.2</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2040,37 +2040,37 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C38" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="D38">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="E38">
-        <v>5302</v>
+        <v>3841029</v>
       </c>
       <c r="F38">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G38">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="H38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I38">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J38">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K38" t="s">
         <v>84</v>
       </c>
       <c r="L38">
-        <v>0.23</v>
+        <v>148.44</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2078,28 +2078,28 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C39" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D39">
-        <v>32</v>
+        <v>119</v>
       </c>
       <c r="E39">
-        <v>1352</v>
+        <v>11004</v>
       </c>
       <c r="F39">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="H39">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="I39">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="J39">
         <v>2</v>
@@ -2108,7 +2108,7 @@
         <v>84</v>
       </c>
       <c r="L39">
-        <v>0.05</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2116,28 +2116,28 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C40" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D40">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="E40">
-        <v>29850</v>
+        <v>139179</v>
       </c>
       <c r="F40">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="G40">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="H40">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="I40">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="J40">
         <v>3</v>
@@ -2146,7 +2146,7 @@
         <v>84</v>
       </c>
       <c r="L40">
-        <v>0.95</v>
+        <v>31.18</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2154,37 +2154,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C41" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="D41">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="E41">
-        <v>27443</v>
+        <v>96491</v>
       </c>
       <c r="F41">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H41">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I41">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="J41">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K41" t="s">
         <v>84</v>
       </c>
       <c r="L41">
-        <v>0.9399999999999999</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2192,28 +2192,28 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C42" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D42">
-        <v>218</v>
+        <v>112</v>
       </c>
       <c r="E42">
-        <v>11308</v>
+        <v>202305</v>
       </c>
       <c r="F42">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="G42">
-        <v>204</v>
+        <v>72</v>
       </c>
       <c r="H42">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I42">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="J42">
         <v>3</v>
@@ -2222,7 +2222,7 @@
         <v>84</v>
       </c>
       <c r="L42">
-        <v>17.2</v>
+        <v>27.15</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2230,37 +2230,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C43" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D43">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E43">
-        <v>6735507</v>
+        <v>19297</v>
       </c>
       <c r="F43">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G43">
         <v>2</v>
       </c>
       <c r="H43">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I43">
         <v>3</v>
       </c>
       <c r="J43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K43" t="s">
         <v>84</v>
       </c>
       <c r="L43">
-        <v>269.25</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2268,37 +2268,37 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C44" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D44">
-        <v>15</v>
+        <v>192</v>
       </c>
       <c r="E44">
-        <v>1302</v>
+        <v>154899</v>
       </c>
       <c r="F44">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="G44">
-        <v>12</v>
+        <v>92</v>
       </c>
       <c r="H44">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="I44">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="J44">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K44" t="s">
         <v>84</v>
       </c>
       <c r="L44">
-        <v>0.12</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2306,37 +2306,37 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C45" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D45">
+        <v>43</v>
+      </c>
+      <c r="E45">
+        <v>1463093</v>
+      </c>
+      <c r="F45">
+        <v>24</v>
+      </c>
+      <c r="G45">
         <v>14</v>
       </c>
-      <c r="E45">
-        <v>712</v>
-      </c>
-      <c r="F45">
-        <v>4</v>
-      </c>
-      <c r="G45">
-        <v>2</v>
-      </c>
       <c r="H45">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I45">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J45">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K45" t="s">
         <v>84</v>
       </c>
       <c r="L45">
-        <v>0.02</v>
+        <v>219.33</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2344,37 +2344,37 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C46" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D46">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="E46">
-        <v>1249411</v>
+        <v>1079680</v>
       </c>
       <c r="F46">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="G46">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="H46">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I46">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J46">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K46" t="s">
         <v>84</v>
       </c>
       <c r="L46">
-        <v>39.2</v>
+        <v>85.38</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2382,37 +2382,37 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C47" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D47">
-        <v>42</v>
+        <v>170</v>
       </c>
       <c r="E47">
-        <v>3841029</v>
+        <v>568</v>
       </c>
       <c r="F47">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G47">
-        <v>27</v>
+        <v>167</v>
       </c>
       <c r="H47">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I47">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J47">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K47" t="s">
         <v>84</v>
       </c>
       <c r="L47">
-        <v>148.44</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2420,25 +2420,25 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C48" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D48">
-        <v>119</v>
+        <v>198</v>
       </c>
       <c r="E48">
-        <v>11004</v>
+        <v>12781</v>
       </c>
       <c r="F48">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G48">
-        <v>112</v>
+        <v>193</v>
       </c>
       <c r="H48">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I48">
         <v>3</v>
@@ -2450,7 +2450,7 @@
         <v>84</v>
       </c>
       <c r="L48">
-        <v>0.45</v>
+        <v>6.62</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2458,22 +2458,22 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C49" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D49">
-        <v>78</v>
+        <v>33</v>
       </c>
       <c r="E49">
-        <v>139179</v>
+        <v>1219</v>
       </c>
       <c r="F49">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G49">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="H49">
         <v>4</v>
@@ -2488,7 +2488,7 @@
         <v>84</v>
       </c>
       <c r="L49">
-        <v>31.18</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2496,28 +2496,28 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C50" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D50">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E50">
-        <v>96491</v>
+        <v>81850</v>
       </c>
       <c r="F50">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G50">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I50">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J50">
         <v>2</v>
@@ -2526,7 +2526,7 @@
         <v>84</v>
       </c>
       <c r="L50">
-        <v>4.68</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2534,37 +2534,37 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C51" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D51">
-        <v>112</v>
+        <v>19</v>
       </c>
       <c r="E51">
-        <v>202305</v>
+        <v>171</v>
       </c>
       <c r="F51">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G51">
-        <v>72</v>
+        <v>9</v>
       </c>
       <c r="H51">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I51">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="J51">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K51" t="s">
         <v>84</v>
       </c>
       <c r="L51">
-        <v>27.15</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2572,37 +2572,37 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C52" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D52">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="E52">
-        <v>19297</v>
+        <v>2113275</v>
       </c>
       <c r="F52">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G52">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H52">
         <v>3</v>
       </c>
       <c r="I52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K52" t="s">
         <v>84</v>
       </c>
       <c r="L52">
-        <v>0.6899999999999999</v>
+        <v>120</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2610,28 +2610,28 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C53" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D53">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="E53">
-        <v>154899</v>
+        <v>4425</v>
       </c>
       <c r="F53">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="G53">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="H53">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="I53">
-        <v>39</v>
+        <v>189</v>
       </c>
       <c r="J53">
         <v>3</v>
@@ -2640,7 +2640,7 @@
         <v>84</v>
       </c>
       <c r="L53">
-        <v>9.67</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2648,37 +2648,37 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C54" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D54">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="E54">
-        <v>1463093</v>
+        <v>8258</v>
       </c>
       <c r="F54">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="G54">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="H54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I54">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K54" t="s">
         <v>84</v>
       </c>
       <c r="L54">
-        <v>219.33</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2686,37 +2686,37 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C55" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D55">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="E55">
-        <v>1079680</v>
+        <v>2762</v>
       </c>
       <c r="F55">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G55">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="H55">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I55">
         <v>8</v>
       </c>
       <c r="J55">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K55" t="s">
         <v>84</v>
       </c>
       <c r="L55">
-        <v>85.38</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2727,34 +2727,34 @@
         <v>76</v>
       </c>
       <c r="C56" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D56">
-        <v>170</v>
+        <v>25</v>
       </c>
       <c r="E56">
-        <v>568</v>
+        <v>1000</v>
       </c>
       <c r="F56">
+        <v>16</v>
+      </c>
+      <c r="G56">
+        <v>5</v>
+      </c>
+      <c r="H56">
+        <v>1</v>
+      </c>
+      <c r="I56">
         <v>0</v>
       </c>
-      <c r="G56">
-        <v>167</v>
-      </c>
-      <c r="H56">
-        <v>2</v>
-      </c>
-      <c r="I56">
-        <v>1</v>
-      </c>
       <c r="J56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K56" t="s">
         <v>84</v>
       </c>
       <c r="L56">
-        <v>0.64</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2768,31 +2768,31 @@
         <v>81</v>
       </c>
       <c r="D57">
-        <v>198</v>
+        <v>20</v>
       </c>
       <c r="E57">
-        <v>12781</v>
+        <v>20000</v>
       </c>
       <c r="F57">
+        <v>20</v>
+      </c>
+      <c r="G57">
         <v>0</v>
       </c>
-      <c r="G57">
-        <v>193</v>
-      </c>
       <c r="H57">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I57">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K57" t="s">
         <v>84</v>
       </c>
       <c r="L57">
-        <v>6.62</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2806,31 +2806,31 @@
         <v>81</v>
       </c>
       <c r="D58">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E58">
-        <v>1219</v>
+        <v>20000</v>
       </c>
       <c r="F58">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="G58">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H58">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I58">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J58">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K58" t="s">
         <v>84</v>
       </c>
       <c r="L58">
-        <v>0.15</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2844,31 +2844,31 @@
         <v>81</v>
       </c>
       <c r="D59">
-        <v>8</v>
+        <v>59</v>
       </c>
       <c r="E59">
-        <v>81850</v>
+        <v>39644</v>
       </c>
       <c r="F59">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G59">
+        <v>59</v>
+      </c>
+      <c r="H59">
+        <v>1</v>
+      </c>
+      <c r="I59">
         <v>0</v>
       </c>
-      <c r="H59">
-        <v>3</v>
-      </c>
-      <c r="I59">
-        <v>3</v>
-      </c>
       <c r="J59">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K59" t="s">
         <v>84</v>
       </c>
       <c r="L59">
-        <v>1.96</v>
+        <v>18.71</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2879,34 +2879,34 @@
         <v>76</v>
       </c>
       <c r="C60" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D60">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="E60">
-        <v>171</v>
+        <v>494021</v>
       </c>
       <c r="F60">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G60">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="H60">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I60">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K60" t="s">
         <v>84</v>
       </c>
       <c r="L60">
-        <v>0.01</v>
+        <v>162.04</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2917,34 +2917,34 @@
         <v>76</v>
       </c>
       <c r="C61" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D61">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E61">
-        <v>2113275</v>
+        <v>299285</v>
       </c>
       <c r="F61">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="G61">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H61">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I61">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J61">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K61" t="s">
         <v>84</v>
       </c>
       <c r="L61">
-        <v>120</v>
+        <v>98.17</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -2955,34 +2955,34 @@
         <v>76</v>
       </c>
       <c r="C62" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D62">
-        <v>202</v>
+        <v>15</v>
       </c>
       <c r="E62">
-        <v>4425</v>
+        <v>32561</v>
       </c>
       <c r="F62">
+        <v>9</v>
+      </c>
+      <c r="G62">
+        <v>6</v>
+      </c>
+      <c r="H62">
+        <v>1</v>
+      </c>
+      <c r="I62">
         <v>0</v>
       </c>
-      <c r="G62">
-        <v>0</v>
-      </c>
-      <c r="H62">
-        <v>68</v>
-      </c>
-      <c r="I62">
-        <v>189</v>
-      </c>
       <c r="J62">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K62" t="s">
         <v>84</v>
       </c>
       <c r="L62">
-        <v>0.1</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -2993,34 +2993,34 @@
         <v>76</v>
       </c>
       <c r="C63" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D63">
-        <v>6</v>
+        <v>55</v>
       </c>
       <c r="E63">
-        <v>8258</v>
+        <v>581012</v>
       </c>
       <c r="F63">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G63">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="H63">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I63">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J63">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K63" t="s">
         <v>84</v>
       </c>
       <c r="L63">
-        <v>0.25</v>
+        <v>255.65</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3031,34 +3031,34 @@
         <v>76</v>
       </c>
       <c r="C64" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D64">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E64">
-        <v>2762</v>
+        <v>20000</v>
       </c>
       <c r="F64">
+        <v>27</v>
+      </c>
+      <c r="G64">
         <v>0</v>
       </c>
-      <c r="G64">
-        <v>7</v>
-      </c>
       <c r="H64">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I64">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J64">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K64" t="s">
         <v>84</v>
       </c>
       <c r="L64">
-        <v>0.04</v>
+        <v>3.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_05_01_2026) - Modality: single_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="84">
   <si>
     <t>Dataset</t>
   </si>
@@ -214,10 +214,25 @@
     <t>Bupa</t>
   </si>
   <si>
+    <t>insurance</t>
+  </si>
+  <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
     <t>expedia_hotel_logs</t>
   </si>
   <si>
-    <t>child</t>
+    <t>intrusion</t>
+  </si>
+  <si>
+    <t>covtype</t>
+  </si>
+  <si>
+    <t>adult</t>
   </si>
   <si>
     <t>alarm</t>
@@ -226,21 +241,6 @@
     <t>news</t>
   </si>
   <si>
-    <t>intrusion</t>
-  </si>
-  <si>
-    <t>census</t>
-  </si>
-  <si>
-    <t>adult</t>
-  </si>
-  <si>
-    <t>covtype</t>
-  </si>
-  <si>
-    <t>insurance</t>
-  </si>
-  <si>
     <t>multi_table</t>
   </si>
   <si>
@@ -256,16 +256,13 @@
     <t>HMASynthesizer</t>
   </si>
   <si>
+    <t>TVAESynthesizer</t>
+  </si>
+  <si>
+    <t>RealTabFormerSynthesizer</t>
+  </si>
+  <si>
     <t>GaussianCopulaSynthesizer</t>
-  </si>
-  <si>
-    <t>TVAESynthesizer</t>
-  </si>
-  <si>
-    <t>CopulaGANSynthesizer</t>
-  </si>
-  <si>
-    <t>CTGANSynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -699,7 +696,7 @@
         <v>2</v>
       </c>
       <c r="K2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L2">
         <v>0.04</v>
@@ -737,7 +734,7 @@
         <v>2</v>
       </c>
       <c r="K3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L3">
         <v>0.15</v>
@@ -775,7 +772,7 @@
         <v>2</v>
       </c>
       <c r="K4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L4">
         <v>0.01</v>
@@ -813,7 +810,7 @@
         <v>2</v>
       </c>
       <c r="K5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L5">
         <v>0.32</v>
@@ -851,7 +848,7 @@
         <v>2</v>
       </c>
       <c r="K6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L6">
         <v>130.3</v>
@@ -889,7 +886,7 @@
         <v>3</v>
       </c>
       <c r="K7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L7">
         <v>0.01</v>
@@ -927,7 +924,7 @@
         <v>2</v>
       </c>
       <c r="K8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L8">
         <v>0.07000000000000001</v>
@@ -965,7 +962,7 @@
         <v>3</v>
       </c>
       <c r="K9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L9">
         <v>0.57</v>
@@ -1003,7 +1000,7 @@
         <v>9</v>
       </c>
       <c r="K10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L10">
         <v>3.45</v>
@@ -1041,7 +1038,7 @@
         <v>3</v>
       </c>
       <c r="K11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L11">
         <v>0.37</v>
@@ -1079,7 +1076,7 @@
         <v>2</v>
       </c>
       <c r="K12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L12">
         <v>0.04</v>
@@ -1117,7 +1114,7 @@
         <v>2</v>
       </c>
       <c r="K13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L13">
         <v>0.11</v>
@@ -1155,7 +1152,7 @@
         <v>2</v>
       </c>
       <c r="K14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L14">
         <v>9.93</v>
@@ -1193,7 +1190,7 @@
         <v>2</v>
       </c>
       <c r="K15" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L15">
         <v>0.36</v>
@@ -1231,7 +1228,7 @@
         <v>2</v>
       </c>
       <c r="K16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L16">
         <v>293.14</v>
@@ -1269,7 +1266,7 @@
         <v>2</v>
       </c>
       <c r="K17" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L17">
         <v>0.25</v>
@@ -1307,7 +1304,7 @@
         <v>3</v>
       </c>
       <c r="K18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L18">
         <v>1.03</v>
@@ -1345,7 +1342,7 @@
         <v>2</v>
       </c>
       <c r="K19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L19">
         <v>0.05</v>
@@ -1383,7 +1380,7 @@
         <v>2</v>
       </c>
       <c r="K20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L20">
         <v>1.38</v>
@@ -1421,7 +1418,7 @@
         <v>2</v>
       </c>
       <c r="K21" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L21">
         <v>0.11</v>
@@ -1459,7 +1456,7 @@
         <v>2</v>
       </c>
       <c r="K22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L22">
         <v>0</v>
@@ -1497,7 +1494,7 @@
         <v>2</v>
       </c>
       <c r="K23" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L23">
         <v>0.68</v>
@@ -1535,7 +1532,7 @@
         <v>2</v>
       </c>
       <c r="K24" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L24">
         <v>0.09</v>
@@ -1573,7 +1570,7 @@
         <v>3</v>
       </c>
       <c r="K25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L25">
         <v>0.6928000000000001</v>
@@ -1611,7 +1608,7 @@
         <v>2</v>
       </c>
       <c r="K26" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L26">
         <v>0.02</v>
@@ -1649,7 +1646,7 @@
         <v>2</v>
       </c>
       <c r="K27" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L27">
         <v>1.79</v>
@@ -1687,7 +1684,7 @@
         <v>2</v>
       </c>
       <c r="K28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L28">
         <v>173.9</v>
@@ -1725,7 +1722,7 @@
         <v>2</v>
       </c>
       <c r="K29" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L29">
         <v>0.23</v>
@@ -1763,7 +1760,7 @@
         <v>2</v>
       </c>
       <c r="K30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L30">
         <v>0.05</v>
@@ -1801,7 +1798,7 @@
         <v>3</v>
       </c>
       <c r="K31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L31">
         <v>0.95</v>
@@ -1839,7 +1836,7 @@
         <v>3</v>
       </c>
       <c r="K32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L32">
         <v>0.9399999999999999</v>
@@ -1877,7 +1874,7 @@
         <v>3</v>
       </c>
       <c r="K33" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L33">
         <v>17.2</v>
@@ -1915,7 +1912,7 @@
         <v>2</v>
       </c>
       <c r="K34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L34">
         <v>269.25</v>
@@ -1953,7 +1950,7 @@
         <v>2</v>
       </c>
       <c r="K35" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L35">
         <v>0.12</v>
@@ -1991,7 +1988,7 @@
         <v>2</v>
       </c>
       <c r="K36" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L36">
         <v>0.02</v>
@@ -2029,7 +2026,7 @@
         <v>2</v>
       </c>
       <c r="K37" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L37">
         <v>39.2</v>
@@ -2067,7 +2064,7 @@
         <v>3</v>
       </c>
       <c r="K38" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L38">
         <v>148.44</v>
@@ -2105,7 +2102,7 @@
         <v>2</v>
       </c>
       <c r="K39" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L39">
         <v>0.45</v>
@@ -2143,7 +2140,7 @@
         <v>3</v>
       </c>
       <c r="K40" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L40">
         <v>31.18</v>
@@ -2181,7 +2178,7 @@
         <v>2</v>
       </c>
       <c r="K41" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L41">
         <v>4.68</v>
@@ -2219,7 +2216,7 @@
         <v>3</v>
       </c>
       <c r="K42" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L42">
         <v>27.15</v>
@@ -2257,7 +2254,7 @@
         <v>3</v>
       </c>
       <c r="K43" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L43">
         <v>0.6899999999999999</v>
@@ -2295,7 +2292,7 @@
         <v>3</v>
       </c>
       <c r="K44" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L44">
         <v>9.67</v>
@@ -2333,7 +2330,7 @@
         <v>3</v>
       </c>
       <c r="K45" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L45">
         <v>219.33</v>
@@ -2371,7 +2368,7 @@
         <v>4</v>
       </c>
       <c r="K46" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L46">
         <v>85.38</v>
@@ -2409,7 +2406,7 @@
         <v>2</v>
       </c>
       <c r="K47" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L47">
         <v>0.64</v>
@@ -2447,7 +2444,7 @@
         <v>2</v>
       </c>
       <c r="K48" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L48">
         <v>6.62</v>
@@ -2485,7 +2482,7 @@
         <v>3</v>
       </c>
       <c r="K49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L49">
         <v>0.15</v>
@@ -2523,7 +2520,7 @@
         <v>2</v>
       </c>
       <c r="K50" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L50">
         <v>1.96</v>
@@ -2561,7 +2558,7 @@
         <v>2</v>
       </c>
       <c r="K51" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L51">
         <v>0.01</v>
@@ -2599,7 +2596,7 @@
         <v>2</v>
       </c>
       <c r="K52" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L52">
         <v>120</v>
@@ -2637,7 +2634,7 @@
         <v>3</v>
       </c>
       <c r="K53" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L53">
         <v>0.1</v>
@@ -2675,7 +2672,7 @@
         <v>2</v>
       </c>
       <c r="K54" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L54">
         <v>0.25</v>
@@ -2713,7 +2710,7 @@
         <v>2</v>
       </c>
       <c r="K55" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L55">
         <v>0.04</v>
@@ -2730,16 +2727,16 @@
         <v>80</v>
       </c>
       <c r="D56">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E56">
-        <v>1000</v>
+        <v>20000</v>
       </c>
       <c r="F56">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="G56">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H56">
         <v>1</v>
@@ -2751,10 +2748,10 @@
         <v>1</v>
       </c>
       <c r="K56" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L56">
-        <v>0.2</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2768,16 +2765,16 @@
         <v>81</v>
       </c>
       <c r="D57">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="E57">
-        <v>20000</v>
+        <v>299285</v>
       </c>
       <c r="F57">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="G57">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H57">
         <v>1</v>
@@ -2789,10 +2786,10 @@
         <v>1</v>
       </c>
       <c r="K57" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L57">
-        <v>3.2</v>
+        <v>98.17</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2803,16 +2800,16 @@
         <v>76</v>
       </c>
       <c r="C58" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D58">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E58">
         <v>20000</v>
       </c>
       <c r="F58">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="G58">
         <v>0</v>
@@ -2827,10 +2824,10 @@
         <v>1</v>
       </c>
       <c r="K58" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L58">
-        <v>4.52</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2841,19 +2838,19 @@
         <v>76</v>
       </c>
       <c r="C59" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D59">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="E59">
-        <v>39644</v>
+        <v>1000</v>
       </c>
       <c r="F59">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G59">
-        <v>59</v>
+        <v>5</v>
       </c>
       <c r="H59">
         <v>1</v>
@@ -2865,10 +2862,10 @@
         <v>1</v>
       </c>
       <c r="K59" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L59">
-        <v>18.71</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2903,7 +2900,7 @@
         <v>1</v>
       </c>
       <c r="K60" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L60">
         <v>162.04</v>
@@ -2917,19 +2914,19 @@
         <v>76</v>
       </c>
       <c r="C61" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D61">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="E61">
-        <v>299285</v>
+        <v>581012</v>
       </c>
       <c r="F61">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="G61">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="H61">
         <v>1</v>
@@ -2941,10 +2938,10 @@
         <v>1</v>
       </c>
       <c r="K61" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L61">
-        <v>98.17</v>
+        <v>255.65</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -2955,7 +2952,7 @@
         <v>76</v>
       </c>
       <c r="C62" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D62">
         <v>15</v>
@@ -2979,7 +2976,7 @@
         <v>1</v>
       </c>
       <c r="K62" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L62">
         <v>3.91</v>
@@ -2993,19 +2990,19 @@
         <v>76</v>
       </c>
       <c r="C63" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D63">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E63">
-        <v>581012</v>
+        <v>20000</v>
       </c>
       <c r="F63">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="G63">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="H63">
         <v>1</v>
@@ -3017,10 +3014,10 @@
         <v>1</v>
       </c>
       <c r="K63" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L63">
-        <v>255.65</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3031,19 +3028,19 @@
         <v>76</v>
       </c>
       <c r="C64" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D64">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="E64">
-        <v>20000</v>
+        <v>39644</v>
       </c>
       <c r="F64">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="G64">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="H64">
         <v>1</v>
@@ -3055,10 +3052,10 @@
         <v>1</v>
       </c>
       <c r="K64" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L64">
-        <v>3.34</v>
+        <v>18.71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_05_01_2026) - Modality: multi_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="85">
   <si>
     <t>Dataset</t>
   </si>
@@ -52,217 +52,220 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>insurance</t>
+  </si>
+  <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
+    <t>expedia_hotel_logs</t>
+  </si>
+  <si>
+    <t>intrusion</t>
+  </si>
+  <si>
+    <t>covtype</t>
+  </si>
+  <si>
+    <t>adult</t>
+  </si>
+  <si>
+    <t>alarm</t>
+  </si>
+  <si>
+    <t>news</t>
+  </si>
+  <si>
+    <t>Accidents</t>
+  </si>
+  <si>
+    <t>Atherosclerosis</t>
+  </si>
+  <si>
+    <t>AustralianFootball</t>
+  </si>
+  <si>
+    <t>Biodegradability</t>
+  </si>
+  <si>
+    <t>Bupa</t>
+  </si>
+  <si>
+    <t>CORA</t>
+  </si>
+  <si>
+    <t>Carcinogenesis</t>
+  </si>
+  <si>
+    <t>Chess</t>
+  </si>
+  <si>
+    <t>Countries</t>
+  </si>
+  <si>
+    <t>DCG</t>
+  </si>
+  <si>
+    <t>Dunur</t>
+  </si>
+  <si>
+    <t>Elti</t>
+  </si>
+  <si>
+    <t>FNHK</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>Hepatitis_std</t>
+  </si>
+  <si>
+    <t>Mesh</t>
+  </si>
+  <si>
+    <t>Mooney_Family</t>
+  </si>
+  <si>
+    <t>MuskSmall</t>
+  </si>
+  <si>
+    <t>NBA</t>
+  </si>
+  <si>
+    <t>NCAA</t>
+  </si>
+  <si>
+    <t>OMOP_CDM_dayz</t>
+  </si>
+  <si>
+    <t>PTE</t>
+  </si>
+  <si>
+    <t>Pima</t>
+  </si>
+  <si>
+    <t>PremierLeague</t>
+  </si>
+  <si>
+    <t>Pyrimidine</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>SAT</t>
+  </si>
+  <si>
+    <t>SalesDB</t>
+  </si>
+  <si>
     <t>Same_gen</t>
   </si>
   <si>
+    <t>Student_loan</t>
+  </si>
+  <si>
+    <t>Toxicology</t>
+  </si>
+  <si>
+    <t>Triazine</t>
+  </si>
+  <si>
+    <t>TubePricing</t>
+  </si>
+  <si>
+    <t>UTube</t>
+  </si>
+  <si>
+    <t>UW_std</t>
+  </si>
+  <si>
+    <t>WebKP</t>
+  </si>
+  <si>
+    <t>airbnb-simplified</t>
+  </si>
+  <si>
+    <t>fake_hotels</t>
+  </si>
+  <si>
+    <t>fake_hotels_extended</t>
+  </si>
+  <si>
+    <t>financial</t>
+  </si>
+  <si>
+    <t>ftp</t>
+  </si>
+  <si>
+    <t>genes</t>
+  </si>
+  <si>
+    <t>got_families</t>
+  </si>
+  <si>
+    <t>imdb_MovieLens</t>
+  </si>
+  <si>
+    <t>imdb_ijs</t>
+  </si>
+  <si>
     <t>imdb_small</t>
   </si>
   <si>
+    <t>legalActs</t>
+  </si>
+  <si>
+    <t>multi_table_ID_demo_dataset</t>
+  </si>
+  <si>
+    <t>mutagenesis</t>
+  </si>
+  <si>
+    <t>nations</t>
+  </si>
+  <si>
+    <t>restbase</t>
+  </si>
+  <si>
     <t>trains</t>
   </si>
   <si>
-    <t>SAT</t>
-  </si>
-  <si>
-    <t>legalActs</t>
-  </si>
-  <si>
-    <t>Dunur</t>
-  </si>
-  <si>
-    <t>fake_hotels_extended</t>
-  </si>
-  <si>
-    <t>Biodegradability</t>
-  </si>
-  <si>
-    <t>OMOP_CDM_dayz</t>
-  </si>
-  <si>
-    <t>mutagenesis</t>
-  </si>
-  <si>
-    <t>Mesh</t>
-  </si>
-  <si>
-    <t>Pima</t>
-  </si>
-  <si>
-    <t>Countries</t>
-  </si>
-  <si>
-    <t>genes</t>
-  </si>
-  <si>
-    <t>airbnb-simplified</t>
-  </si>
-  <si>
-    <t>Chess</t>
-  </si>
-  <si>
-    <t>Toxicology</t>
-  </si>
-  <si>
-    <t>fake_hotels</t>
-  </si>
-  <si>
-    <t>Facebook</t>
-  </si>
-  <si>
-    <t>UTube</t>
-  </si>
-  <si>
-    <t>got_families</t>
-  </si>
-  <si>
-    <t>Hepatitis_std</t>
-  </si>
-  <si>
-    <t>Student_loan</t>
-  </si>
-  <si>
-    <t>multi_table_ID_demo_dataset</t>
-  </si>
-  <si>
-    <t>Pyrimidine</t>
-  </si>
-  <si>
-    <t>CORA</t>
-  </si>
-  <si>
-    <t>imdb_ijs</t>
+    <t>university</t>
   </si>
   <si>
     <t>world</t>
   </si>
   <si>
-    <t>Elti</t>
-  </si>
-  <si>
-    <t>PTE</t>
-  </si>
-  <si>
-    <t>Carcinogenesis</t>
-  </si>
-  <si>
-    <t>PremierLeague</t>
-  </si>
-  <si>
-    <t>SalesDB</t>
-  </si>
-  <si>
-    <t>Triazine</t>
-  </si>
-  <si>
-    <t>UW_std</t>
-  </si>
-  <si>
-    <t>imdb_MovieLens</t>
-  </si>
-  <si>
-    <t>SAP</t>
-  </si>
-  <si>
-    <t>nations</t>
-  </si>
-  <si>
-    <t>AustralianFootball</t>
-  </si>
-  <si>
-    <t>ftp</t>
-  </si>
-  <si>
-    <t>NCAA</t>
-  </si>
-  <si>
-    <t>restbase</t>
-  </si>
-  <si>
-    <t>TubePricing</t>
-  </si>
-  <si>
-    <t>Accidents</t>
-  </si>
-  <si>
-    <t>financial</t>
-  </si>
-  <si>
-    <t>MuskSmall</t>
-  </si>
-  <si>
-    <t>Atherosclerosis</t>
-  </si>
-  <si>
-    <t>NBA</t>
-  </si>
-  <si>
-    <t>WebKP</t>
-  </si>
-  <si>
-    <t>university</t>
-  </si>
-  <si>
-    <t>FNHK</t>
-  </si>
-  <si>
-    <t>Mooney_Family</t>
-  </si>
-  <si>
-    <t>DCG</t>
-  </si>
-  <si>
-    <t>Bupa</t>
-  </si>
-  <si>
-    <t>insurance</t>
-  </si>
-  <si>
-    <t>census</t>
-  </si>
-  <si>
-    <t>child</t>
-  </si>
-  <si>
-    <t>expedia_hotel_logs</t>
-  </si>
-  <si>
-    <t>intrusion</t>
-  </si>
-  <si>
-    <t>covtype</t>
-  </si>
-  <si>
-    <t>adult</t>
-  </si>
-  <si>
-    <t>alarm</t>
-  </si>
-  <si>
-    <t>news</t>
+    <t>single_table</t>
   </si>
   <si>
     <t>multi_table</t>
   </si>
   <si>
-    <t>single_table</t>
+    <t>TVAESynthesizer</t>
+  </si>
+  <si>
+    <t>RealTabFormerSynthesizer</t>
+  </si>
+  <si>
+    <t>GaussianCopulaSynthesizer</t>
   </si>
   <si>
     <t>HSASynthesizer</t>
   </si>
   <si>
+    <t>HMASynthesizer</t>
+  </si>
+  <si>
     <t>IndependentSynthesizer</t>
   </si>
   <si>
-    <t>HMASynthesizer</t>
-  </si>
-  <si>
-    <t>TVAESynthesizer</t>
-  </si>
-  <si>
-    <t>RealTabFormerSynthesizer</t>
-  </si>
-  <si>
-    <t>GaussianCopulaSynthesizer</t>
+    <t>MultiTableUniformSynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -675,31 +678,31 @@
         <v>77</v>
       </c>
       <c r="D2">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="E2">
-        <v>1536</v>
+        <v>20000</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L2">
-        <v>0.04</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -710,34 +713,34 @@
         <v>75</v>
       </c>
       <c r="C3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D3">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="E3">
-        <v>4395</v>
+        <v>299285</v>
       </c>
       <c r="F3">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="G3">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L3">
-        <v>0.15</v>
+        <v>98.17</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -751,31 +754,31 @@
         <v>77</v>
       </c>
       <c r="D4">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E4">
-        <v>83</v>
+        <v>20000</v>
       </c>
       <c r="F4">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="G4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L4">
-        <v>0.01</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -786,34 +789,34 @@
         <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D5">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="E5">
-        <v>19867</v>
+        <v>1000</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="G5">
+        <v>5</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
         <v>0</v>
       </c>
-      <c r="H5">
-        <v>36</v>
-      </c>
-      <c r="I5">
-        <v>65</v>
-      </c>
       <c r="J5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L5">
-        <v>0.32</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -827,31 +830,31 @@
         <v>78</v>
       </c>
       <c r="D6">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="E6">
-        <v>1754397</v>
+        <v>494021</v>
       </c>
       <c r="F6">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="G6">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="H6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I6">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L6">
-        <v>130.3</v>
+        <v>162.04</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -865,31 +868,31 @@
         <v>77</v>
       </c>
       <c r="D7">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E7">
-        <v>440</v>
+        <v>581012</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7">
+        <v>54</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
         <v>0</v>
       </c>
-      <c r="H7">
-        <v>17</v>
-      </c>
-      <c r="I7">
-        <v>34</v>
-      </c>
       <c r="J7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L7">
-        <v>0.01</v>
+        <v>255.65</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -900,34 +903,34 @@
         <v>75</v>
       </c>
       <c r="C8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D8">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E8">
-        <v>668</v>
+        <v>32561</v>
       </c>
       <c r="F8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G8">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L8">
-        <v>0.07000000000000001</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -938,34 +941,34 @@
         <v>75</v>
       </c>
       <c r="C9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D9">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="E9">
-        <v>21895</v>
+        <v>20000</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L9">
-        <v>0.57</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -976,34 +979,34 @@
         <v>75</v>
       </c>
       <c r="C10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D10">
-        <v>432</v>
+        <v>59</v>
       </c>
       <c r="E10">
-        <v>39000</v>
+        <v>39644</v>
       </c>
       <c r="F10">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="H10">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="I10">
-        <v>171</v>
+        <v>0</v>
       </c>
       <c r="J10">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L10">
-        <v>3.45</v>
+        <v>18.71</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1011,22 +1014,22 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D11">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="E11">
-        <v>10324</v>
+        <v>1463093</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G11">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="H11">
         <v>3</v>
@@ -1038,10 +1041,10 @@
         <v>3</v>
       </c>
       <c r="K11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L11">
-        <v>0.37</v>
+        <v>219.33</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1049,37 +1052,37 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C12" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D12">
-        <v>41</v>
+        <v>198</v>
       </c>
       <c r="E12">
-        <v>2700</v>
+        <v>12781</v>
       </c>
       <c r="F12">
         <v>0</v>
       </c>
       <c r="G12">
-        <v>2</v>
+        <v>193</v>
       </c>
       <c r="H12">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="I12">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="J12">
         <v>2</v>
       </c>
       <c r="K12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L12">
-        <v>0.04</v>
+        <v>6.62</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1087,37 +1090,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D13">
-        <v>18</v>
+        <v>78</v>
       </c>
       <c r="E13">
-        <v>6912</v>
+        <v>139179</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G13">
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="H13">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I13">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L13">
-        <v>0.11</v>
+        <v>31.18</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1125,37 +1128,37 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C14" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D14">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="E14">
-        <v>22318</v>
+        <v>21895</v>
       </c>
       <c r="F14">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G14">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="H14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L14">
-        <v>9.93</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1163,37 +1166,37 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C15" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D15">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E15">
-        <v>6118</v>
+        <v>2762</v>
       </c>
       <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>7</v>
+      </c>
+      <c r="H15">
         <v>9</v>
       </c>
-      <c r="G15">
-        <v>2</v>
-      </c>
-      <c r="H15">
-        <v>3</v>
-      </c>
       <c r="I15">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J15">
         <v>2</v>
       </c>
       <c r="K15" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L15">
-        <v>0.36</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1201,37 +1204,37 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C16" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D16">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E16">
-        <v>5751408</v>
+        <v>57353</v>
       </c>
       <c r="F16">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="G16">
         <v>2</v>
       </c>
       <c r="H16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J16">
         <v>2</v>
       </c>
       <c r="K16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L16">
-        <v>293.14</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1239,37 +1242,37 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C17" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D17">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="E17">
-        <v>2052</v>
+        <v>27443</v>
       </c>
       <c r="F17">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="G17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H17">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="J17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L17">
-        <v>0.25</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1277,37 +1280,37 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C18" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D18">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="E18">
-        <v>36922</v>
+        <v>2052</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H18">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I18">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L18">
-        <v>1.03</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1315,37 +1318,37 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C19" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D19">
-        <v>15</v>
+        <v>68</v>
       </c>
       <c r="E19">
-        <v>668</v>
+        <v>22318</v>
       </c>
       <c r="F19">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G19">
-        <v>3</v>
+        <v>53</v>
       </c>
       <c r="H19">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J19">
         <v>2</v>
       </c>
       <c r="K19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L19">
-        <v>0.05</v>
+        <v>9.93</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1353,37 +1356,37 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C20" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D20">
-        <v>266</v>
+        <v>6</v>
       </c>
       <c r="E20">
-        <v>10173</v>
+        <v>8258</v>
       </c>
       <c r="F20">
-        <v>262</v>
+        <v>2</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H20">
         <v>2</v>
       </c>
       <c r="I20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J20">
         <v>2</v>
       </c>
       <c r="K20" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L20">
-        <v>1.38</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1391,37 +1394,37 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C21" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D21">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="E21">
-        <v>2735</v>
+        <v>440</v>
       </c>
       <c r="F21">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G21">
         <v>0</v>
       </c>
       <c r="H21">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I21">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="J21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L21">
-        <v>0.11</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1429,37 +1432,37 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C22" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D22">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E22">
-        <v>23</v>
+        <v>1352</v>
       </c>
       <c r="F22">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G22">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="I22">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="J22">
         <v>2</v>
       </c>
       <c r="K22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L22">
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1467,37 +1470,37 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C23" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D23">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E23">
-        <v>12927</v>
+        <v>2113275</v>
       </c>
       <c r="F23">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G23">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H23">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I23">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J23">
         <v>2</v>
       </c>
       <c r="K23" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L23">
-        <v>0.68</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1505,37 +1508,37 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C24" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D24">
-        <v>16</v>
+        <v>266</v>
       </c>
       <c r="E24">
-        <v>5288</v>
+        <v>10173</v>
       </c>
       <c r="F24">
-        <v>2</v>
+        <v>262</v>
       </c>
       <c r="G24">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H24">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I24">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="J24">
         <v>2</v>
       </c>
       <c r="K24" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L24">
-        <v>0.09</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1543,37 +1546,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D25">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="E25">
-        <v>11150</v>
+        <v>12927</v>
       </c>
       <c r="F25">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G25">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="H25">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I25">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K25" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L25">
-        <v>0.6928000000000001</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1581,37 +1584,37 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C26" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D26">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="E26">
-        <v>296</v>
+        <v>2700</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="J26">
         <v>2</v>
       </c>
       <c r="K26" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L26">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1619,37 +1622,37 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C27" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D27">
-        <v>10</v>
+        <v>202</v>
       </c>
       <c r="E27">
-        <v>57353</v>
+        <v>4425</v>
       </c>
       <c r="F27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H27">
-        <v>3</v>
+        <v>68</v>
       </c>
       <c r="I27">
-        <v>3</v>
+        <v>189</v>
       </c>
       <c r="J27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K27" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L27">
-        <v>1.79</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1657,37 +1660,37 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D28">
-        <v>25</v>
+        <v>170</v>
       </c>
       <c r="E28">
-        <v>5647694</v>
+        <v>568</v>
       </c>
       <c r="F28">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>3</v>
+        <v>167</v>
       </c>
       <c r="H28">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I28">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J28">
         <v>2</v>
       </c>
       <c r="K28" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L28">
-        <v>173.9</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1695,37 +1698,37 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C29" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D29">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E29">
-        <v>5302</v>
+        <v>1219</v>
       </c>
       <c r="F29">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="G29">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="H29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I29">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K29" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L29">
-        <v>0.23</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1733,37 +1736,37 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C30" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D30">
-        <v>32</v>
+        <v>112</v>
       </c>
       <c r="E30">
-        <v>1352</v>
+        <v>202305</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H30">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I30">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K30" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L30">
-        <v>0.05</v>
+        <v>27.15</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1771,37 +1774,37 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C31" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D31">
-        <v>97</v>
+        <v>432</v>
       </c>
       <c r="E31">
-        <v>29850</v>
+        <v>39000</v>
       </c>
       <c r="F31">
-        <v>25</v>
+        <v>108</v>
       </c>
       <c r="G31">
+        <v>51</v>
+      </c>
+      <c r="H31">
+        <v>39</v>
+      </c>
+      <c r="I31">
+        <v>171</v>
+      </c>
+      <c r="J31">
         <v>9</v>
       </c>
-      <c r="H31">
-        <v>38</v>
-      </c>
-      <c r="I31">
-        <v>39</v>
-      </c>
-      <c r="J31">
-        <v>3</v>
-      </c>
       <c r="K31" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L31">
-        <v>0.95</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1809,37 +1812,37 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C32" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D32">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="E32">
-        <v>27443</v>
+        <v>29850</v>
       </c>
       <c r="F32">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="G32">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H32">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="I32">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="J32">
         <v>3</v>
       </c>
       <c r="K32" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L32">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1847,37 +1850,37 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C33" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D33">
-        <v>218</v>
+        <v>18</v>
       </c>
       <c r="E33">
-        <v>11308</v>
+        <v>6912</v>
       </c>
       <c r="F33">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G33">
-        <v>204</v>
+        <v>8</v>
       </c>
       <c r="H33">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I33">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J33">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K33" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L33">
-        <v>17.2</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1885,37 +1888,37 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C34" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D34">
-        <v>16</v>
+        <v>218</v>
       </c>
       <c r="E34">
-        <v>6735507</v>
+        <v>11308</v>
       </c>
       <c r="F34">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G34">
-        <v>2</v>
+        <v>204</v>
       </c>
       <c r="H34">
         <v>4</v>
       </c>
       <c r="I34">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J34">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K34" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L34">
-        <v>269.25</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1923,22 +1926,22 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C35" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D35">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E35">
-        <v>1302</v>
+        <v>296</v>
       </c>
       <c r="F35">
         <v>0</v>
       </c>
       <c r="G35">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H35">
         <v>2</v>
@@ -1950,10 +1953,10 @@
         <v>2</v>
       </c>
       <c r="K35" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L35">
-        <v>0.12</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -1961,37 +1964,37 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C36" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D36">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="E36">
-        <v>712</v>
+        <v>3841029</v>
       </c>
       <c r="F36">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G36">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="H36">
         <v>4</v>
       </c>
       <c r="I36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K36" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L36">
-        <v>0.02</v>
+        <v>148.44</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -1999,37 +2002,37 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C37" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D37">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="E37">
-        <v>1249411</v>
+        <v>19867</v>
       </c>
       <c r="F37">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G37">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H37">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="I37">
-        <v>6</v>
+        <v>65</v>
       </c>
       <c r="J37">
         <v>2</v>
       </c>
       <c r="K37" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L37">
-        <v>39.2</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2037,22 +2040,22 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C38" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D38">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="E38">
-        <v>3841029</v>
+        <v>6735507</v>
       </c>
       <c r="F38">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G38">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="H38">
         <v>4</v>
@@ -2061,13 +2064,13 @@
         <v>3</v>
       </c>
       <c r="J38">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K38" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L38">
-        <v>148.44</v>
+        <v>269.25</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2075,37 +2078,37 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C39" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D39">
-        <v>119</v>
+        <v>11</v>
       </c>
       <c r="E39">
-        <v>11004</v>
+        <v>1536</v>
       </c>
       <c r="F39">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G39">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="H39">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I39">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J39">
         <v>2</v>
       </c>
       <c r="K39" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L39">
-        <v>0.45</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2113,37 +2116,37 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C40" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D40">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E40">
-        <v>139179</v>
+        <v>5288</v>
       </c>
       <c r="F40">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G40">
-        <v>57</v>
+        <v>2</v>
       </c>
       <c r="H40">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="I40">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K40" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L40">
-        <v>31.18</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2151,37 +2154,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C41" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D41">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E41">
-        <v>96491</v>
+        <v>36922</v>
       </c>
       <c r="F41">
+        <v>3</v>
+      </c>
+      <c r="G41">
+        <v>0</v>
+      </c>
+      <c r="H41">
+        <v>4</v>
+      </c>
+      <c r="I41">
         <v>5</v>
       </c>
-      <c r="G41">
-        <v>1</v>
-      </c>
-      <c r="H41">
-        <v>2</v>
-      </c>
-      <c r="I41">
-        <v>1</v>
-      </c>
       <c r="J41">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K41" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L41">
-        <v>4.68</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2189,37 +2192,37 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C42" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D42">
-        <v>112</v>
+        <v>15</v>
       </c>
       <c r="E42">
-        <v>202305</v>
+        <v>1302</v>
       </c>
       <c r="F42">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G42">
-        <v>72</v>
+        <v>12</v>
       </c>
       <c r="H42">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I42">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="J42">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K42" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L42">
-        <v>27.15</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2227,37 +2230,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C43" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D43">
-        <v>12</v>
+        <v>192</v>
       </c>
       <c r="E43">
-        <v>19297</v>
+        <v>154899</v>
       </c>
       <c r="F43">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="G43">
-        <v>2</v>
+        <v>92</v>
       </c>
       <c r="H43">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="I43">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="J43">
         <v>3</v>
       </c>
       <c r="K43" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L43">
-        <v>0.6899999999999999</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2265,37 +2268,37 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C44" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D44">
-        <v>192</v>
+        <v>8</v>
       </c>
       <c r="E44">
-        <v>154899</v>
+        <v>2735</v>
       </c>
       <c r="F44">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="G44">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="H44">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="I44">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="J44">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K44" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L44">
-        <v>9.67</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2303,37 +2306,37 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C45" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D45">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="E45">
-        <v>1463093</v>
+        <v>712</v>
       </c>
       <c r="F45">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="G45">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H45">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I45">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J45">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K45" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L45">
-        <v>219.33</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2341,37 +2344,37 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C46" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D46">
-        <v>55</v>
+        <v>8</v>
       </c>
       <c r="E46">
-        <v>1079680</v>
+        <v>81850</v>
       </c>
       <c r="F46">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G46">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H46">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I46">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J46">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K46" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L46">
-        <v>85.38</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2379,22 +2382,22 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C47" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D47">
-        <v>170</v>
+        <v>22</v>
       </c>
       <c r="E47">
-        <v>568</v>
+        <v>5751408</v>
       </c>
       <c r="F47">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G47">
-        <v>167</v>
+        <v>2</v>
       </c>
       <c r="H47">
         <v>2</v>
@@ -2406,10 +2409,10 @@
         <v>2</v>
       </c>
       <c r="K47" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L47">
-        <v>0.64</v>
+        <v>293.14</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2417,37 +2420,37 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C48" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D48">
-        <v>198</v>
+        <v>15</v>
       </c>
       <c r="E48">
-        <v>12781</v>
+        <v>668</v>
       </c>
       <c r="F48">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G48">
-        <v>193</v>
+        <v>3</v>
       </c>
       <c r="H48">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I48">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J48">
         <v>2</v>
       </c>
       <c r="K48" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L48">
-        <v>6.62</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2455,37 +2458,37 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C49" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D49">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="E49">
-        <v>1219</v>
+        <v>668</v>
       </c>
       <c r="F49">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G49">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="H49">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I49">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K49" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L49">
-        <v>0.15</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2493,37 +2496,37 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C50" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D50">
+        <v>55</v>
+      </c>
+      <c r="E50">
+        <v>1079680</v>
+      </c>
+      <c r="F50">
+        <v>14</v>
+      </c>
+      <c r="G50">
+        <v>21</v>
+      </c>
+      <c r="H50">
         <v>8</v>
       </c>
-      <c r="E50">
-        <v>81850</v>
-      </c>
-      <c r="F50">
-        <v>2</v>
-      </c>
-      <c r="G50">
-        <v>0</v>
-      </c>
-      <c r="H50">
-        <v>3</v>
-      </c>
       <c r="I50">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J50">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K50" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L50">
-        <v>1.96</v>
+        <v>85.38</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2531,37 +2534,37 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C51" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D51">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E51">
-        <v>171</v>
+        <v>96491</v>
       </c>
       <c r="F51">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G51">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H51">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I51">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J51">
         <v>2</v>
       </c>
       <c r="K51" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L51">
-        <v>0.01</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2569,37 +2572,37 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C52" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D52">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="E52">
-        <v>2113275</v>
+        <v>6118</v>
       </c>
       <c r="F52">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G52">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H52">
         <v>3</v>
       </c>
       <c r="I52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J52">
         <v>2</v>
       </c>
       <c r="K52" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L52">
-        <v>120</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2607,37 +2610,37 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C53" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D53">
-        <v>202</v>
+        <v>9</v>
       </c>
       <c r="E53">
-        <v>4425</v>
+        <v>23</v>
       </c>
       <c r="F53">
+        <v>3</v>
+      </c>
+      <c r="G53">
+        <v>2</v>
+      </c>
+      <c r="H53">
+        <v>3</v>
+      </c>
+      <c r="I53">
+        <v>2</v>
+      </c>
+      <c r="J53">
+        <v>2</v>
+      </c>
+      <c r="K53" t="s">
+        <v>84</v>
+      </c>
+      <c r="L53">
         <v>0</v>
-      </c>
-      <c r="G53">
-        <v>0</v>
-      </c>
-      <c r="H53">
-        <v>68</v>
-      </c>
-      <c r="I53">
-        <v>189</v>
-      </c>
-      <c r="J53">
-        <v>3</v>
-      </c>
-      <c r="K53" t="s">
-        <v>83</v>
-      </c>
-      <c r="L53">
-        <v>0.1</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2645,37 +2648,37 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C54" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D54">
+        <v>27</v>
+      </c>
+      <c r="E54">
+        <v>1249411</v>
+      </c>
+      <c r="F54">
+        <v>5</v>
+      </c>
+      <c r="G54">
+        <v>9</v>
+      </c>
+      <c r="H54">
+        <v>7</v>
+      </c>
+      <c r="I54">
         <v>6</v>
       </c>
-      <c r="E54">
-        <v>8258</v>
-      </c>
-      <c r="F54">
-        <v>2</v>
-      </c>
-      <c r="G54">
-        <v>1</v>
-      </c>
-      <c r="H54">
-        <v>2</v>
-      </c>
-      <c r="I54">
-        <v>1</v>
-      </c>
       <c r="J54">
         <v>2</v>
       </c>
       <c r="K54" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L54">
-        <v>0.25</v>
+        <v>39.2</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2683,37 +2686,37 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C55" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D55">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="E55">
-        <v>2762</v>
+        <v>5647694</v>
       </c>
       <c r="F55">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G55">
+        <v>3</v>
+      </c>
+      <c r="H55">
         <v>7</v>
       </c>
-      <c r="H55">
-        <v>9</v>
-      </c>
       <c r="I55">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J55">
         <v>2</v>
       </c>
       <c r="K55" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L55">
-        <v>0.04</v>
+        <v>173.9</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2727,31 +2730,31 @@
         <v>80</v>
       </c>
       <c r="D56">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E56">
-        <v>20000</v>
+        <v>4395</v>
       </c>
       <c r="F56">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="G56">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H56">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I56">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J56">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K56" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L56">
-        <v>3.34</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2762,34 +2765,34 @@
         <v>76</v>
       </c>
       <c r="C57" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D57">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E57">
-        <v>299285</v>
+        <v>1754397</v>
       </c>
       <c r="F57">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="G57">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H57">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I57">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K57" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L57">
-        <v>98.17</v>
+        <v>130.3</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2803,31 +2806,31 @@
         <v>80</v>
       </c>
       <c r="D58">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E58">
-        <v>20000</v>
+        <v>11150</v>
       </c>
       <c r="F58">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="G58">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H58">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I58">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J58">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K58" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L58">
-        <v>3.2</v>
+        <v>0.6928000000000001</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2838,34 +2841,34 @@
         <v>76</v>
       </c>
       <c r="C59" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D59">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E59">
-        <v>1000</v>
+        <v>10324</v>
       </c>
       <c r="F59">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G59">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H59">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I59">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J59">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K59" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L59">
-        <v>0.2</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2879,31 +2882,31 @@
         <v>81</v>
       </c>
       <c r="D60">
-        <v>41</v>
+        <v>119</v>
       </c>
       <c r="E60">
-        <v>494021</v>
+        <v>11004</v>
       </c>
       <c r="F60">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G60">
-        <v>37</v>
+        <v>112</v>
       </c>
       <c r="H60">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I60">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K60" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L60">
-        <v>162.04</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2917,31 +2920,31 @@
         <v>80</v>
       </c>
       <c r="D61">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="E61">
-        <v>581012</v>
+        <v>19297</v>
       </c>
       <c r="F61">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G61">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="H61">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I61">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J61">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K61" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L61">
-        <v>255.65</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -2952,34 +2955,34 @@
         <v>76</v>
       </c>
       <c r="C62" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D62">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E62">
-        <v>32561</v>
+        <v>83</v>
       </c>
       <c r="F62">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G62">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I62">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K62" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L62">
-        <v>3.91</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -2993,31 +2996,31 @@
         <v>80</v>
       </c>
       <c r="D63">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="E63">
-        <v>20000</v>
+        <v>171</v>
       </c>
       <c r="F63">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="G63">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H63">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I63">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J63">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K63" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L63">
-        <v>4.52</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3031,31 +3034,31 @@
         <v>81</v>
       </c>
       <c r="D64">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="E64">
-        <v>39644</v>
+        <v>5302</v>
       </c>
       <c r="F64">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G64">
-        <v>59</v>
+        <v>9</v>
       </c>
       <c r="H64">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I64">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J64">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K64" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L64">
-        <v>18.71</v>
+        <v>0.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_06_02_2026) - Modality: single_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -52,220 +52,220 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>Accidents</t>
+  </si>
+  <si>
+    <t>Atherosclerosis</t>
+  </si>
+  <si>
+    <t>AustralianFootball</t>
+  </si>
+  <si>
+    <t>Biodegradability</t>
+  </si>
+  <si>
+    <t>Bupa</t>
+  </si>
+  <si>
+    <t>CORA</t>
+  </si>
+  <si>
+    <t>Carcinogenesis</t>
+  </si>
+  <si>
+    <t>Chess</t>
+  </si>
+  <si>
+    <t>Countries</t>
+  </si>
+  <si>
+    <t>DCG</t>
+  </si>
+  <si>
+    <t>Dunur</t>
+  </si>
+  <si>
+    <t>Elti</t>
+  </si>
+  <si>
+    <t>FNHK</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>Hepatitis_std</t>
+  </si>
+  <si>
+    <t>Mesh</t>
+  </si>
+  <si>
+    <t>Mooney_Family</t>
+  </si>
+  <si>
+    <t>MuskSmall</t>
+  </si>
+  <si>
+    <t>NBA</t>
+  </si>
+  <si>
+    <t>NCAA</t>
+  </si>
+  <si>
+    <t>OMOP_CDM_dayz</t>
+  </si>
+  <si>
+    <t>PTE</t>
+  </si>
+  <si>
+    <t>Pima</t>
+  </si>
+  <si>
+    <t>PremierLeague</t>
+  </si>
+  <si>
+    <t>Pyrimidine</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>SAT</t>
+  </si>
+  <si>
+    <t>SalesDB</t>
+  </si>
+  <si>
+    <t>Same_gen</t>
+  </si>
+  <si>
+    <t>Student_loan</t>
+  </si>
+  <si>
+    <t>Toxicology</t>
+  </si>
+  <si>
+    <t>Triazine</t>
+  </si>
+  <si>
+    <t>TubePricing</t>
+  </si>
+  <si>
+    <t>UTube</t>
+  </si>
+  <si>
+    <t>UW_std</t>
+  </si>
+  <si>
+    <t>WebKP</t>
+  </si>
+  <si>
+    <t>airbnb-simplified</t>
+  </si>
+  <si>
+    <t>fake_hotels</t>
+  </si>
+  <si>
+    <t>fake_hotels_extended</t>
+  </si>
+  <si>
+    <t>financial</t>
+  </si>
+  <si>
+    <t>ftp</t>
+  </si>
+  <si>
+    <t>genes</t>
+  </si>
+  <si>
+    <t>got_families</t>
+  </si>
+  <si>
+    <t>imdb_MovieLens</t>
+  </si>
+  <si>
+    <t>imdb_ijs</t>
+  </si>
+  <si>
+    <t>imdb_small</t>
+  </si>
+  <si>
+    <t>legalActs</t>
+  </si>
+  <si>
+    <t>multi_table_ID_demo_dataset</t>
+  </si>
+  <si>
+    <t>mutagenesis</t>
+  </si>
+  <si>
+    <t>nations</t>
+  </si>
+  <si>
+    <t>restbase</t>
+  </si>
+  <si>
+    <t>trains</t>
+  </si>
+  <si>
+    <t>university</t>
+  </si>
+  <si>
+    <t>world</t>
+  </si>
+  <si>
+    <t>adult</t>
+  </si>
+  <si>
+    <t>alarm</t>
+  </si>
+  <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
+    <t>covtype</t>
+  </si>
+  <si>
+    <t>expedia_hotel_logs</t>
+  </si>
+  <si>
     <t>insurance</t>
   </si>
   <si>
-    <t>census</t>
-  </si>
-  <si>
-    <t>child</t>
-  </si>
-  <si>
-    <t>expedia_hotel_logs</t>
-  </si>
-  <si>
     <t>intrusion</t>
   </si>
   <si>
-    <t>covtype</t>
-  </si>
-  <si>
-    <t>adult</t>
-  </si>
-  <si>
-    <t>alarm</t>
-  </si>
-  <si>
     <t>news</t>
   </si>
   <si>
-    <t>Accidents</t>
-  </si>
-  <si>
-    <t>Atherosclerosis</t>
-  </si>
-  <si>
-    <t>AustralianFootball</t>
-  </si>
-  <si>
-    <t>Biodegradability</t>
-  </si>
-  <si>
-    <t>Bupa</t>
-  </si>
-  <si>
-    <t>CORA</t>
-  </si>
-  <si>
-    <t>Carcinogenesis</t>
-  </si>
-  <si>
-    <t>Chess</t>
-  </si>
-  <si>
-    <t>Countries</t>
-  </si>
-  <si>
-    <t>DCG</t>
-  </si>
-  <si>
-    <t>Dunur</t>
-  </si>
-  <si>
-    <t>Elti</t>
-  </si>
-  <si>
-    <t>FNHK</t>
-  </si>
-  <si>
-    <t>Facebook</t>
-  </si>
-  <si>
-    <t>Hepatitis_std</t>
-  </si>
-  <si>
-    <t>Mesh</t>
-  </si>
-  <si>
-    <t>Mooney_Family</t>
-  </si>
-  <si>
-    <t>MuskSmall</t>
-  </si>
-  <si>
-    <t>NBA</t>
-  </si>
-  <si>
-    <t>NCAA</t>
-  </si>
-  <si>
-    <t>OMOP_CDM_dayz</t>
-  </si>
-  <si>
-    <t>PTE</t>
-  </si>
-  <si>
-    <t>Pima</t>
-  </si>
-  <si>
-    <t>PremierLeague</t>
-  </si>
-  <si>
-    <t>Pyrimidine</t>
-  </si>
-  <si>
-    <t>SAP</t>
-  </si>
-  <si>
-    <t>SAT</t>
-  </si>
-  <si>
-    <t>SalesDB</t>
-  </si>
-  <si>
-    <t>Same_gen</t>
-  </si>
-  <si>
-    <t>Student_loan</t>
-  </si>
-  <si>
-    <t>Toxicology</t>
-  </si>
-  <si>
-    <t>Triazine</t>
-  </si>
-  <si>
-    <t>TubePricing</t>
-  </si>
-  <si>
-    <t>UTube</t>
-  </si>
-  <si>
-    <t>UW_std</t>
-  </si>
-  <si>
-    <t>WebKP</t>
-  </si>
-  <si>
-    <t>airbnb-simplified</t>
-  </si>
-  <si>
-    <t>fake_hotels</t>
-  </si>
-  <si>
-    <t>fake_hotels_extended</t>
-  </si>
-  <si>
-    <t>financial</t>
-  </si>
-  <si>
-    <t>ftp</t>
-  </si>
-  <si>
-    <t>genes</t>
-  </si>
-  <si>
-    <t>got_families</t>
-  </si>
-  <si>
-    <t>imdb_MovieLens</t>
-  </si>
-  <si>
-    <t>imdb_ijs</t>
-  </si>
-  <si>
-    <t>imdb_small</t>
-  </si>
-  <si>
-    <t>legalActs</t>
-  </si>
-  <si>
-    <t>multi_table_ID_demo_dataset</t>
-  </si>
-  <si>
-    <t>mutagenesis</t>
-  </si>
-  <si>
-    <t>nations</t>
-  </si>
-  <si>
-    <t>restbase</t>
-  </si>
-  <si>
-    <t>trains</t>
-  </si>
-  <si>
-    <t>university</t>
-  </si>
-  <si>
-    <t>world</t>
+    <t>multi_table</t>
   </si>
   <si>
     <t>single_table</t>
   </si>
   <si>
-    <t>multi_table</t>
+    <t>HSASynthesizer</t>
+  </si>
+  <si>
+    <t>HMASynthesizer</t>
+  </si>
+  <si>
+    <t>IndependentSynthesizer</t>
+  </si>
+  <si>
+    <t>MultiTableUniformSynthesizer</t>
+  </si>
+  <si>
+    <t>RealTabFormerSynthesizer</t>
   </si>
   <si>
     <t>TVAESynthesizer</t>
   </si>
   <si>
-    <t>RealTabFormerSynthesizer</t>
-  </si>
-  <si>
     <t>GaussianCopulaSynthesizer</t>
-  </si>
-  <si>
-    <t>HSASynthesizer</t>
-  </si>
-  <si>
-    <t>HMASynthesizer</t>
-  </si>
-  <si>
-    <t>IndependentSynthesizer</t>
-  </si>
-  <si>
-    <t>MultiTableUniformSynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -678,31 +678,31 @@
         <v>77</v>
       </c>
       <c r="D2">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="E2">
-        <v>20000</v>
+        <v>1463093</v>
       </c>
       <c r="F2">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K2" t="s">
         <v>84</v>
       </c>
       <c r="L2">
-        <v>3.34</v>
+        <v>219.33</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -713,34 +713,34 @@
         <v>75</v>
       </c>
       <c r="C3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D3">
-        <v>41</v>
+        <v>198</v>
       </c>
       <c r="E3">
-        <v>299285</v>
+        <v>12781</v>
       </c>
       <c r="F3">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>12</v>
+        <v>193</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="s">
         <v>84</v>
       </c>
       <c r="L3">
-        <v>98.17</v>
+        <v>6.62</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -754,31 +754,31 @@
         <v>77</v>
       </c>
       <c r="D4">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="E4">
-        <v>20000</v>
+        <v>139179</v>
       </c>
       <c r="F4">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K4" t="s">
         <v>84</v>
       </c>
       <c r="L4">
-        <v>3.2</v>
+        <v>31.18</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -789,34 +789,34 @@
         <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D5">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E5">
-        <v>1000</v>
+        <v>21895</v>
       </c>
       <c r="F5">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
         <v>5</v>
       </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
       <c r="I5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K5" t="s">
         <v>84</v>
       </c>
       <c r="L5">
-        <v>0.2</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -830,31 +830,31 @@
         <v>78</v>
       </c>
       <c r="D6">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="E6">
-        <v>494021</v>
+        <v>2762</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" t="s">
         <v>84</v>
       </c>
       <c r="L6">
-        <v>162.04</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -868,31 +868,31 @@
         <v>77</v>
       </c>
       <c r="D7">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="E7">
-        <v>581012</v>
+        <v>57353</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" t="s">
         <v>84</v>
       </c>
       <c r="L7">
-        <v>255.65</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -906,31 +906,31 @@
         <v>78</v>
       </c>
       <c r="D8">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E8">
-        <v>32561</v>
+        <v>27443</v>
       </c>
       <c r="F8">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G8">
+        <v>2</v>
+      </c>
+      <c r="H8">
         <v>6</v>
       </c>
-      <c r="H8">
-        <v>1</v>
-      </c>
       <c r="I8">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K8" t="s">
         <v>84</v>
       </c>
       <c r="L8">
-        <v>3.91</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -944,31 +944,31 @@
         <v>77</v>
       </c>
       <c r="D9">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="E9">
-        <v>20000</v>
+        <v>2052</v>
       </c>
       <c r="F9">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" t="s">
         <v>84</v>
       </c>
       <c r="L9">
-        <v>4.52</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -979,34 +979,34 @@
         <v>75</v>
       </c>
       <c r="C10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D10">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E10">
-        <v>39644</v>
+        <v>22318</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G10">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" t="s">
         <v>84</v>
       </c>
       <c r="L10">
-        <v>18.71</v>
+        <v>9.93</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1014,37 +1014,37 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D11">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="E11">
-        <v>1463093</v>
+        <v>8258</v>
       </c>
       <c r="F11">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="G11">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="H11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K11" t="s">
         <v>84</v>
       </c>
       <c r="L11">
-        <v>219.33</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1052,37 +1052,37 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C12" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D12">
-        <v>198</v>
+        <v>50</v>
       </c>
       <c r="E12">
-        <v>12781</v>
+        <v>440</v>
       </c>
       <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
         <v>0</v>
       </c>
-      <c r="G12">
-        <v>193</v>
-      </c>
       <c r="H12">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I12">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="J12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K12" t="s">
         <v>84</v>
       </c>
       <c r="L12">
-        <v>6.62</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1090,37 +1090,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D13">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="E13">
-        <v>139179</v>
+        <v>1352</v>
       </c>
       <c r="F13">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I13">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="J13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K13" t="s">
         <v>84</v>
       </c>
       <c r="L13">
-        <v>31.18</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1128,37 +1128,37 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C14" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D14">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="E14">
-        <v>21895</v>
+        <v>2113275</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G14">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I14">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" t="s">
         <v>84</v>
       </c>
       <c r="L14">
-        <v>0.57</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1166,28 +1166,28 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C15" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D15">
-        <v>17</v>
+        <v>266</v>
       </c>
       <c r="E15">
-        <v>2762</v>
+        <v>10173</v>
       </c>
       <c r="F15">
+        <v>262</v>
+      </c>
+      <c r="G15">
         <v>0</v>
       </c>
-      <c r="G15">
-        <v>7</v>
-      </c>
       <c r="H15">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I15">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J15">
         <v>2</v>
@@ -1196,7 +1196,7 @@
         <v>84</v>
       </c>
       <c r="L15">
-        <v>0.04</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1204,28 +1204,28 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C16" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D16">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E16">
-        <v>57353</v>
+        <v>12927</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
       <c r="G16">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H16">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I16">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J16">
         <v>2</v>
@@ -1234,7 +1234,7 @@
         <v>84</v>
       </c>
       <c r="L16">
-        <v>1.79</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1242,37 +1242,37 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C17" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D17">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="E17">
-        <v>27443</v>
+        <v>2700</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G17">
         <v>2</v>
       </c>
       <c r="H17">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="I17">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="J17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K17" t="s">
         <v>84</v>
       </c>
       <c r="L17">
-        <v>0.9399999999999999</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1280,37 +1280,37 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D18">
-        <v>46</v>
+        <v>202</v>
       </c>
       <c r="E18">
-        <v>2052</v>
+        <v>4425</v>
       </c>
       <c r="F18">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>189</v>
       </c>
       <c r="J18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K18" t="s">
         <v>84</v>
       </c>
       <c r="L18">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1318,28 +1318,28 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C19" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D19">
-        <v>68</v>
+        <v>170</v>
       </c>
       <c r="E19">
-        <v>22318</v>
+        <v>568</v>
       </c>
       <c r="F19">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>53</v>
+        <v>167</v>
       </c>
       <c r="H19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J19">
         <v>2</v>
@@ -1348,7 +1348,7 @@
         <v>84</v>
       </c>
       <c r="L19">
-        <v>9.93</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1356,37 +1356,37 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D20">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E20">
-        <v>8258</v>
+        <v>1219</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="H20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J20">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" t="s">
         <v>84</v>
       </c>
       <c r="L20">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1394,28 +1394,28 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C21" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D21">
-        <v>50</v>
+        <v>112</v>
       </c>
       <c r="E21">
-        <v>440</v>
+        <v>202305</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H21">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I21">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="J21">
         <v>3</v>
@@ -1424,7 +1424,7 @@
         <v>84</v>
       </c>
       <c r="L21">
-        <v>0.01</v>
+        <v>27.15</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1432,37 +1432,37 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C22" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D22">
-        <v>32</v>
+        <v>432</v>
       </c>
       <c r="E22">
-        <v>1352</v>
+        <v>39000</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>108</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="H22">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="I22">
-        <v>20</v>
+        <v>171</v>
       </c>
       <c r="J22">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="K22" t="s">
         <v>84</v>
       </c>
       <c r="L22">
-        <v>0.05</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1470,37 +1470,37 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C23" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D23">
-        <v>26</v>
+        <v>97</v>
       </c>
       <c r="E23">
-        <v>2113275</v>
+        <v>29850</v>
       </c>
       <c r="F23">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="G23">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H23">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="I23">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="J23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K23" t="s">
         <v>84</v>
       </c>
       <c r="L23">
-        <v>120</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1508,28 +1508,28 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D24">
-        <v>266</v>
+        <v>18</v>
       </c>
       <c r="E24">
-        <v>10173</v>
+        <v>6912</v>
       </c>
       <c r="F24">
-        <v>262</v>
+        <v>1</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H24">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I24">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J24">
         <v>2</v>
@@ -1538,7 +1538,7 @@
         <v>84</v>
       </c>
       <c r="L24">
-        <v>1.38</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1546,37 +1546,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D25">
-        <v>29</v>
+        <v>218</v>
       </c>
       <c r="E25">
-        <v>12927</v>
+        <v>11308</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G25">
-        <v>14</v>
+        <v>204</v>
       </c>
       <c r="H25">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K25" t="s">
         <v>84</v>
       </c>
       <c r="L25">
-        <v>0.68</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1584,28 +1584,28 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C26" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D26">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E26">
-        <v>2700</v>
+        <v>296</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H26">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="I26">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="J26">
         <v>2</v>
@@ -1614,7 +1614,7 @@
         <v>84</v>
       </c>
       <c r="L26">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1622,28 +1622,28 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C27" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D27">
-        <v>202</v>
+        <v>42</v>
       </c>
       <c r="E27">
-        <v>4425</v>
+        <v>3841029</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="H27">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="I27">
-        <v>189</v>
+        <v>3</v>
       </c>
       <c r="J27">
         <v>3</v>
@@ -1652,7 +1652,7 @@
         <v>84</v>
       </c>
       <c r="L27">
-        <v>0.1</v>
+        <v>148.44</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1660,28 +1660,28 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C28" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D28">
-        <v>170</v>
+        <v>70</v>
       </c>
       <c r="E28">
-        <v>568</v>
+        <v>19867</v>
       </c>
       <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
         <v>0</v>
       </c>
-      <c r="G28">
-        <v>167</v>
-      </c>
       <c r="H28">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="I28">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="J28">
         <v>2</v>
@@ -1690,7 +1690,7 @@
         <v>84</v>
       </c>
       <c r="L28">
-        <v>0.64</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1698,37 +1698,37 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C29" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D29">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E29">
-        <v>1219</v>
+        <v>6735507</v>
       </c>
       <c r="F29">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G29">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="H29">
         <v>4</v>
       </c>
       <c r="I29">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K29" t="s">
         <v>84</v>
       </c>
       <c r="L29">
-        <v>0.15</v>
+        <v>269.25</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1736,37 +1736,37 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C30" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D30">
-        <v>112</v>
+        <v>11</v>
       </c>
       <c r="E30">
-        <v>202305</v>
+        <v>1536</v>
       </c>
       <c r="F30">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G30">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="H30">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I30">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="J30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K30" t="s">
         <v>84</v>
       </c>
       <c r="L30">
-        <v>27.15</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1774,37 +1774,37 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C31" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D31">
-        <v>432</v>
+        <v>16</v>
       </c>
       <c r="E31">
-        <v>39000</v>
+        <v>5288</v>
       </c>
       <c r="F31">
-        <v>108</v>
+        <v>2</v>
       </c>
       <c r="G31">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="H31">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="I31">
-        <v>171</v>
+        <v>9</v>
       </c>
       <c r="J31">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K31" t="s">
         <v>84</v>
       </c>
       <c r="L31">
-        <v>3.45</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1812,28 +1812,28 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C32" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D32">
-        <v>97</v>
+        <v>12</v>
       </c>
       <c r="E32">
-        <v>29850</v>
+        <v>36922</v>
       </c>
       <c r="F32">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="G32">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H32">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="I32">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="J32">
         <v>3</v>
@@ -1842,7 +1842,7 @@
         <v>84</v>
       </c>
       <c r="L32">
-        <v>0.95</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1850,28 +1850,28 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C33" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D33">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E33">
-        <v>6912</v>
+        <v>1302</v>
       </c>
       <c r="F33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H33">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I33">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J33">
         <v>2</v>
@@ -1880,7 +1880,7 @@
         <v>84</v>
       </c>
       <c r="L33">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1888,28 +1888,28 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C34" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D34">
-        <v>218</v>
+        <v>192</v>
       </c>
       <c r="E34">
-        <v>11308</v>
+        <v>154899</v>
       </c>
       <c r="F34">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="G34">
-        <v>204</v>
+        <v>92</v>
       </c>
       <c r="H34">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="I34">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="J34">
         <v>3</v>
@@ -1918,7 +1918,7 @@
         <v>84</v>
       </c>
       <c r="L34">
-        <v>17.2</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1926,23 +1926,23 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C35" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D35">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E35">
-        <v>296</v>
+        <v>2735</v>
       </c>
       <c r="F35">
+        <v>5</v>
+      </c>
+      <c r="G35">
         <v>0</v>
       </c>
-      <c r="G35">
-        <v>11</v>
-      </c>
       <c r="H35">
         <v>2</v>
       </c>
@@ -1956,7 +1956,7 @@
         <v>84</v>
       </c>
       <c r="L35">
-        <v>0.02</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -1964,37 +1964,37 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C36" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D36">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="E36">
-        <v>3841029</v>
+        <v>712</v>
       </c>
       <c r="F36">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G36">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="H36">
         <v>4</v>
       </c>
       <c r="I36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K36" t="s">
         <v>84</v>
       </c>
       <c r="L36">
-        <v>148.44</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -2002,28 +2002,28 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C37" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D37">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="E37">
-        <v>19867</v>
+        <v>81850</v>
       </c>
       <c r="F37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G37">
         <v>0</v>
       </c>
       <c r="H37">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="I37">
-        <v>65</v>
+        <v>3</v>
       </c>
       <c r="J37">
         <v>2</v>
@@ -2032,7 +2032,7 @@
         <v>84</v>
       </c>
       <c r="L37">
-        <v>0.32</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2040,28 +2040,28 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C38" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D38">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E38">
-        <v>6735507</v>
+        <v>5751408</v>
       </c>
       <c r="F38">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="G38">
         <v>2</v>
       </c>
       <c r="H38">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I38">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J38">
         <v>2</v>
@@ -2070,7 +2070,7 @@
         <v>84</v>
       </c>
       <c r="L38">
-        <v>269.25</v>
+        <v>293.14</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2078,28 +2078,28 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C39" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D39">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E39">
-        <v>1536</v>
+        <v>668</v>
       </c>
       <c r="F39">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H39">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I39">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J39">
         <v>2</v>
@@ -2108,7 +2108,7 @@
         <v>84</v>
       </c>
       <c r="L39">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2116,28 +2116,28 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C40" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D40">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E40">
-        <v>5288</v>
+        <v>668</v>
       </c>
       <c r="F40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H40">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I40">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J40">
         <v>2</v>
@@ -2146,7 +2146,7 @@
         <v>84</v>
       </c>
       <c r="L40">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2154,37 +2154,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C41" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D41">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="E41">
-        <v>36922</v>
+        <v>1079680</v>
       </c>
       <c r="F41">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H41">
+        <v>8</v>
+      </c>
+      <c r="I41">
+        <v>8</v>
+      </c>
+      <c r="J41">
         <v>4</v>
       </c>
-      <c r="I41">
-        <v>5</v>
-      </c>
-      <c r="J41">
-        <v>3</v>
-      </c>
       <c r="K41" t="s">
         <v>84</v>
       </c>
       <c r="L41">
-        <v>1.03</v>
+        <v>85.38</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2192,22 +2192,22 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C42" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D42">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E42">
-        <v>1302</v>
+        <v>96491</v>
       </c>
       <c r="F42">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G42">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -2222,7 +2222,7 @@
         <v>84</v>
       </c>
       <c r="L42">
-        <v>0.12</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2230,37 +2230,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C43" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D43">
-        <v>192</v>
+        <v>16</v>
       </c>
       <c r="E43">
-        <v>154899</v>
+        <v>6118</v>
       </c>
       <c r="F43">
-        <v>54</v>
+        <v>9</v>
       </c>
       <c r="G43">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="H43">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="I43">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="J43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K43" t="s">
         <v>84</v>
       </c>
       <c r="L43">
-        <v>9.67</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2268,37 +2268,37 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C44" t="s">
         <v>80</v>
       </c>
       <c r="D44">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E44">
-        <v>2735</v>
+        <v>23</v>
       </c>
       <c r="F44">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G44">
+        <v>2</v>
+      </c>
+      <c r="H44">
+        <v>3</v>
+      </c>
+      <c r="I44">
+        <v>2</v>
+      </c>
+      <c r="J44">
+        <v>2</v>
+      </c>
+      <c r="K44" t="s">
+        <v>84</v>
+      </c>
+      <c r="L44">
         <v>0</v>
-      </c>
-      <c r="H44">
-        <v>2</v>
-      </c>
-      <c r="I44">
-        <v>1</v>
-      </c>
-      <c r="J44">
-        <v>2</v>
-      </c>
-      <c r="K44" t="s">
-        <v>84</v>
-      </c>
-      <c r="L44">
-        <v>0.11</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2306,28 +2306,28 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C45" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D45">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="E45">
-        <v>712</v>
+        <v>1249411</v>
       </c>
       <c r="F45">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G45">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H45">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I45">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J45">
         <v>2</v>
@@ -2336,7 +2336,7 @@
         <v>84</v>
       </c>
       <c r="L45">
-        <v>0.02</v>
+        <v>39.2</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2344,28 +2344,28 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C46" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D46">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E46">
-        <v>81850</v>
+        <v>5647694</v>
       </c>
       <c r="F46">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H46">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I46">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J46">
         <v>2</v>
@@ -2374,7 +2374,7 @@
         <v>84</v>
       </c>
       <c r="L46">
-        <v>1.96</v>
+        <v>173.9</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2382,28 +2382,28 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C47" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D47">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E47">
-        <v>5751408</v>
+        <v>4395</v>
       </c>
       <c r="F47">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G47">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H47">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I47">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J47">
         <v>2</v>
@@ -2412,7 +2412,7 @@
         <v>84</v>
       </c>
       <c r="L47">
-        <v>293.14</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2420,28 +2420,28 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C48" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D48">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E48">
-        <v>668</v>
+        <v>1754397</v>
       </c>
       <c r="F48">
+        <v>18</v>
+      </c>
+      <c r="G48">
+        <v>8</v>
+      </c>
+      <c r="H48">
         <v>5</v>
       </c>
-      <c r="G48">
-        <v>3</v>
-      </c>
-      <c r="H48">
-        <v>2</v>
-      </c>
       <c r="I48">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J48">
         <v>2</v>
@@ -2450,7 +2450,7 @@
         <v>84</v>
       </c>
       <c r="L48">
-        <v>0.05</v>
+        <v>130.3</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2458,37 +2458,37 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C49" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D49">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E49">
-        <v>668</v>
+        <v>11150</v>
       </c>
       <c r="F49">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G49">
         <v>3</v>
       </c>
       <c r="H49">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I49">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J49">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K49" t="s">
         <v>84</v>
       </c>
       <c r="L49">
-        <v>0.07000000000000001</v>
+        <v>0.6928000000000001</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2496,37 +2496,37 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C50" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D50">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="E50">
-        <v>1079680</v>
+        <v>10324</v>
       </c>
       <c r="F50">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G50">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="H50">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I50">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J50">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K50" t="s">
         <v>84</v>
       </c>
       <c r="L50">
-        <v>85.38</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2534,28 +2534,28 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C51" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D51">
-        <v>11</v>
+        <v>119</v>
       </c>
       <c r="E51">
-        <v>96491</v>
+        <v>11004</v>
       </c>
       <c r="F51">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G51">
-        <v>1</v>
+        <v>112</v>
       </c>
       <c r="H51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I51">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J51">
         <v>2</v>
@@ -2564,7 +2564,7 @@
         <v>84</v>
       </c>
       <c r="L51">
-        <v>4.68</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2572,19 +2572,19 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C52" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D52">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E52">
-        <v>6118</v>
+        <v>19297</v>
       </c>
       <c r="F52">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G52">
         <v>2</v>
@@ -2596,13 +2596,13 @@
         <v>3</v>
       </c>
       <c r="J52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K52" t="s">
         <v>84</v>
       </c>
       <c r="L52">
-        <v>0.36</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2610,28 +2610,28 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C53" t="s">
+        <v>77</v>
+      </c>
+      <c r="D53">
+        <v>13</v>
+      </c>
+      <c r="E53">
         <v>83</v>
       </c>
-      <c r="D53">
-        <v>9</v>
-      </c>
-      <c r="E53">
-        <v>23</v>
-      </c>
       <c r="F53">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G53">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H53">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J53">
         <v>2</v>
@@ -2640,7 +2640,7 @@
         <v>84</v>
       </c>
       <c r="L53">
-        <v>0</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2648,28 +2648,28 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C54" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D54">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E54">
-        <v>1249411</v>
+        <v>171</v>
       </c>
       <c r="F54">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G54">
         <v>9</v>
       </c>
       <c r="H54">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I54">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J54">
         <v>2</v>
@@ -2678,7 +2678,7 @@
         <v>84</v>
       </c>
       <c r="L54">
-        <v>39.2</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2686,28 +2686,28 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C55" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D55">
         <v>25</v>
       </c>
       <c r="E55">
-        <v>5647694</v>
+        <v>5302</v>
       </c>
       <c r="F55">
+        <v>11</v>
+      </c>
+      <c r="G55">
         <v>9</v>
       </c>
-      <c r="G55">
-        <v>3</v>
-      </c>
       <c r="H55">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I55">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J55">
         <v>2</v>
@@ -2716,7 +2716,7 @@
         <v>84</v>
       </c>
       <c r="L55">
-        <v>173.9</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2727,34 +2727,34 @@
         <v>76</v>
       </c>
       <c r="C56" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D56">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E56">
-        <v>4395</v>
+        <v>32561</v>
       </c>
       <c r="F56">
         <v>9</v>
       </c>
       <c r="G56">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H56">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I56">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K56" t="s">
         <v>84</v>
       </c>
       <c r="L56">
-        <v>0.15</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2768,31 +2768,31 @@
         <v>82</v>
       </c>
       <c r="D57">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E57">
-        <v>1754397</v>
+        <v>20000</v>
       </c>
       <c r="F57">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="G57">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H57">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I57">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K57" t="s">
         <v>84</v>
       </c>
       <c r="L57">
-        <v>130.3</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2803,34 +2803,34 @@
         <v>76</v>
       </c>
       <c r="C58" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D58">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="E58">
-        <v>11150</v>
+        <v>299285</v>
       </c>
       <c r="F58">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="G58">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H58">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I58">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J58">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K58" t="s">
         <v>84</v>
       </c>
       <c r="L58">
-        <v>0.6928000000000001</v>
+        <v>98.17</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2841,34 +2841,34 @@
         <v>76</v>
       </c>
       <c r="C59" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D59">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E59">
-        <v>10324</v>
+        <v>20000</v>
       </c>
       <c r="F59">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="G59">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H59">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I59">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J59">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K59" t="s">
         <v>84</v>
       </c>
       <c r="L59">
-        <v>0.37</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2879,34 +2879,34 @@
         <v>76</v>
       </c>
       <c r="C60" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D60">
-        <v>119</v>
+        <v>55</v>
       </c>
       <c r="E60">
-        <v>11004</v>
+        <v>581012</v>
       </c>
       <c r="F60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G60">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="H60">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I60">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K60" t="s">
         <v>84</v>
       </c>
       <c r="L60">
-        <v>0.45</v>
+        <v>255.65</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2917,34 +2917,34 @@
         <v>76</v>
       </c>
       <c r="C61" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D61">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E61">
-        <v>19297</v>
+        <v>1000</v>
       </c>
       <c r="F61">
+        <v>16</v>
+      </c>
+      <c r="G61">
         <v>5</v>
       </c>
-      <c r="G61">
-        <v>2</v>
-      </c>
       <c r="H61">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I61">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J61">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K61" t="s">
         <v>84</v>
       </c>
       <c r="L61">
-        <v>0.6899999999999999</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -2955,34 +2955,34 @@
         <v>76</v>
       </c>
       <c r="C62" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D62">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E62">
-        <v>83</v>
+        <v>20000</v>
       </c>
       <c r="F62">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="G62">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H62">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I62">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J62">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K62" t="s">
         <v>84</v>
       </c>
       <c r="L62">
-        <v>0.01</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -2993,34 +2993,34 @@
         <v>76</v>
       </c>
       <c r="C63" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D63">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="E63">
-        <v>171</v>
+        <v>494021</v>
       </c>
       <c r="F63">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G63">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="H63">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I63">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J63">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K63" t="s">
         <v>84</v>
       </c>
       <c r="L63">
-        <v>0.01</v>
+        <v>162.04</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3034,31 +3034,31 @@
         <v>81</v>
       </c>
       <c r="D64">
-        <v>25</v>
+        <v>59</v>
       </c>
       <c r="E64">
-        <v>5302</v>
+        <v>39644</v>
       </c>
       <c r="F64">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="G64">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="H64">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I64">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J64">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K64" t="s">
         <v>84</v>
       </c>
       <c r="L64">
-        <v>0.23</v>
+        <v>18.71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_06_02_2026) - Modality: multi_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="101">
   <si>
     <t>Dataset</t>
   </si>
@@ -52,6 +52,33 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>adult</t>
+  </si>
+  <si>
+    <t>alarm</t>
+  </si>
+  <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
+    <t>covtype</t>
+  </si>
+  <si>
+    <t>expedia_hotel_logs</t>
+  </si>
+  <si>
+    <t>insurance</t>
+  </si>
+  <si>
+    <t>intrusion</t>
+  </si>
+  <si>
+    <t>news</t>
+  </si>
+  <si>
     <t>Accidents</t>
   </si>
   <si>
@@ -214,61 +241,82 @@
     <t>world</t>
   </si>
   <si>
-    <t>adult</t>
-  </si>
-  <si>
-    <t>alarm</t>
-  </si>
-  <si>
-    <t>census</t>
-  </si>
-  <si>
-    <t>child</t>
-  </si>
-  <si>
-    <t>covtype</t>
-  </si>
-  <si>
-    <t>expedia_hotel_logs</t>
-  </si>
-  <si>
-    <t>insurance</t>
-  </si>
-  <si>
-    <t>intrusion</t>
-  </si>
-  <si>
-    <t>news</t>
+    <t>MovieLens</t>
+  </si>
+  <si>
+    <t>Telstra</t>
+  </si>
+  <si>
+    <t>instacart_marketbasket_ml</t>
+  </si>
+  <si>
+    <t>rel-amazon</t>
+  </si>
+  <si>
+    <t>rel-arxiv</t>
+  </si>
+  <si>
+    <t>rel-avito</t>
+  </si>
+  <si>
+    <t>rel-event</t>
+  </si>
+  <si>
+    <t>rel-f1</t>
+  </si>
+  <si>
+    <t>rel-hm</t>
+  </si>
+  <si>
+    <t>rel-ratebeer</t>
+  </si>
+  <si>
+    <t>rel-salt</t>
+  </si>
+  <si>
+    <t>rel-stack</t>
+  </si>
+  <si>
+    <t>rel-trial</t>
+  </si>
+  <si>
+    <t>rossmann</t>
+  </si>
+  <si>
+    <t>walmart</t>
+  </si>
+  <si>
+    <t>single_table</t>
   </si>
   <si>
     <t>multi_table</t>
   </si>
   <si>
-    <t>single_table</t>
+    <t>RealTabFormerSynthesizer</t>
+  </si>
+  <si>
+    <t>TVAESynthesizer</t>
+  </si>
+  <si>
+    <t>GaussianCopulaSynthesizer</t>
   </si>
   <si>
     <t>HSASynthesizer</t>
   </si>
   <si>
+    <t>IndependentSynthesizer</t>
+  </si>
+  <si>
     <t>HMASynthesizer</t>
   </si>
   <si>
-    <t>IndependentSynthesizer</t>
-  </si>
-  <si>
     <t>MultiTableUniformSynthesizer</t>
   </si>
   <si>
-    <t>RealTabFormerSynthesizer</t>
-  </si>
-  <si>
-    <t>TVAESynthesizer</t>
-  </si>
-  <si>
-    <t>GaussianCopulaSynthesizer</t>
-  </si>
-  <si>
     <t>Public</t>
+  </si>
+  <si>
+    <t>Private</t>
   </si>
 </sst>
 </file>
@@ -626,7 +674,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -672,37 +720,37 @@
         <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="C2" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="D2">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="E2">
-        <v>1463093</v>
+        <v>32561</v>
       </c>
       <c r="F2">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L2">
-        <v>219.33</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -710,37 +758,37 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="D3">
-        <v>198</v>
+        <v>37</v>
       </c>
       <c r="E3">
-        <v>12781</v>
+        <v>20000</v>
       </c>
       <c r="F3">
+        <v>37</v>
+      </c>
+      <c r="G3">
         <v>0</v>
       </c>
-      <c r="G3">
-        <v>193</v>
-      </c>
       <c r="H3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L3">
-        <v>6.62</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -748,37 +796,37 @@
         <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="C4" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="D4">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="E4">
-        <v>139179</v>
+        <v>299285</v>
       </c>
       <c r="F4">
+        <v>29</v>
+      </c>
+      <c r="G4">
         <v>12</v>
       </c>
-      <c r="G4">
-        <v>57</v>
-      </c>
       <c r="H4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L4">
-        <v>31.18</v>
+        <v>98.17</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -786,37 +834,37 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="C5" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="D5">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E5">
-        <v>21895</v>
+        <v>20000</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K5" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L5">
-        <v>0.57</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -824,37 +872,37 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="D6">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="E6">
-        <v>2762</v>
+        <v>581012</v>
       </c>
       <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>54</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
         <v>0</v>
       </c>
-      <c r="G6">
-        <v>7</v>
-      </c>
-      <c r="H6">
-        <v>9</v>
-      </c>
-      <c r="I6">
-        <v>8</v>
-      </c>
       <c r="J6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L6">
-        <v>0.04</v>
+        <v>255.65</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -862,37 +910,37 @@
         <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="D7">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E7">
-        <v>57353</v>
+        <v>1000</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L7">
-        <v>1.79</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -900,37 +948,37 @@
         <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="D8">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E8">
-        <v>27443</v>
+        <v>20000</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="G8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K8" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L8">
-        <v>0.9399999999999999</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -938,37 +986,37 @@
         <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="C9" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="D9">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E9">
-        <v>2052</v>
+        <v>494021</v>
       </c>
       <c r="F9">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L9">
-        <v>0.25</v>
+        <v>162.04</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -976,37 +1024,37 @@
         <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="C10" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="D10">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E10">
-        <v>22318</v>
+        <v>39644</v>
       </c>
       <c r="F10">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="H10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L10">
-        <v>9.93</v>
+        <v>18.71</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1014,37 +1062,37 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C11" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D11">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="E11">
-        <v>8258</v>
+        <v>1463093</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K11" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L11">
-        <v>0.25</v>
+        <v>219.33</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1052,37 +1100,37 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C12" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="D12">
-        <v>50</v>
+        <v>198</v>
       </c>
       <c r="E12">
-        <v>440</v>
+        <v>12781</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="H12">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I12">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="J12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K12" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L12">
-        <v>0.01</v>
+        <v>6.62</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1090,37 +1138,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D13">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="E13">
-        <v>1352</v>
+        <v>139179</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="H13">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="I13">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="J13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L13">
-        <v>0.05</v>
+        <v>31.18</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1128,37 +1176,37 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C14" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="D14">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="E14">
-        <v>2113275</v>
+        <v>21895</v>
       </c>
       <c r="F14">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G14">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L14">
-        <v>120</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1166,37 +1214,37 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C15" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="D15">
-        <v>266</v>
+        <v>17</v>
       </c>
       <c r="E15">
-        <v>10173</v>
+        <v>2762</v>
       </c>
       <c r="F15">
-        <v>262</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J15">
         <v>2</v>
       </c>
       <c r="K15" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L15">
-        <v>1.38</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1204,37 +1252,37 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D16">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E16">
-        <v>12927</v>
+        <v>57353</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
       <c r="G16">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I16">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J16">
         <v>2</v>
       </c>
       <c r="K16" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L16">
-        <v>0.68</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1242,37 +1290,37 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C17" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="D17">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="E17">
-        <v>2700</v>
+        <v>27443</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G17">
         <v>2</v>
       </c>
       <c r="H17">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="I17">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="J17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L17">
-        <v>0.04</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1280,37 +1328,37 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D18">
-        <v>202</v>
+        <v>46</v>
       </c>
       <c r="E18">
-        <v>4425</v>
+        <v>2052</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H18">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="I18">
-        <v>189</v>
+        <v>1</v>
       </c>
       <c r="J18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K18" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L18">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1318,37 +1366,37 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C19" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D19">
-        <v>170</v>
+        <v>68</v>
       </c>
       <c r="E19">
-        <v>568</v>
+        <v>22318</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G19">
-        <v>167</v>
+        <v>53</v>
       </c>
       <c r="H19">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J19">
         <v>2</v>
       </c>
       <c r="K19" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L19">
-        <v>0.64</v>
+        <v>9.93</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1356,37 +1404,37 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C20" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="D20">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E20">
-        <v>1219</v>
+        <v>8258</v>
       </c>
       <c r="F20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G20">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="H20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I20">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K20" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L20">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1394,37 +1442,37 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C21" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D21">
-        <v>112</v>
+        <v>50</v>
       </c>
       <c r="E21">
-        <v>202305</v>
+        <v>440</v>
       </c>
       <c r="F21">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G21">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="H21">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="I21">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="J21">
         <v>3</v>
       </c>
       <c r="K21" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L21">
-        <v>27.15</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1432,37 +1480,37 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C22" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D22">
-        <v>432</v>
+        <v>32</v>
       </c>
       <c r="E22">
-        <v>39000</v>
+        <v>1352</v>
       </c>
       <c r="F22">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="G22">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="I22">
-        <v>171</v>
+        <v>20</v>
       </c>
       <c r="J22">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K22" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L22">
-        <v>3.45</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1470,37 +1518,37 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C23" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="D23">
-        <v>97</v>
+        <v>26</v>
       </c>
       <c r="E23">
-        <v>29850</v>
+        <v>2113275</v>
       </c>
       <c r="F23">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G23">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H23">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="I23">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="J23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K23" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L23">
-        <v>0.95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1508,37 +1556,37 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C24" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D24">
-        <v>18</v>
+        <v>266</v>
       </c>
       <c r="E24">
-        <v>6912</v>
+        <v>10173</v>
       </c>
       <c r="F24">
-        <v>1</v>
+        <v>262</v>
       </c>
       <c r="G24">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H24">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I24">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J24">
         <v>2</v>
       </c>
       <c r="K24" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L24">
-        <v>0.11</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1546,37 +1594,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C25" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="D25">
-        <v>218</v>
+        <v>29</v>
       </c>
       <c r="E25">
-        <v>11308</v>
+        <v>12927</v>
       </c>
       <c r="F25">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G25">
-        <v>204</v>
+        <v>14</v>
       </c>
       <c r="H25">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K25" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L25">
-        <v>17.2</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1584,37 +1632,37 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C26" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="D26">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="E26">
-        <v>296</v>
+        <v>2700</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="J26">
         <v>2</v>
       </c>
       <c r="K26" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L26">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1622,37 +1670,37 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C27" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D27">
-        <v>42</v>
+        <v>202</v>
       </c>
       <c r="E27">
-        <v>3841029</v>
+        <v>4425</v>
       </c>
       <c r="F27">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="H27">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="I27">
-        <v>3</v>
+        <v>189</v>
       </c>
       <c r="J27">
         <v>3</v>
       </c>
       <c r="K27" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L27">
-        <v>148.44</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1660,37 +1708,37 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C28" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="D28">
-        <v>70</v>
+        <v>170</v>
       </c>
       <c r="E28">
-        <v>19867</v>
+        <v>568</v>
       </c>
       <c r="F28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="H28">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="I28">
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="J28">
         <v>2</v>
       </c>
       <c r="K28" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L28">
-        <v>0.32</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1698,37 +1746,37 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C29" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="D29">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E29">
-        <v>6735507</v>
+        <v>1219</v>
       </c>
       <c r="F29">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G29">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="H29">
         <v>4</v>
       </c>
       <c r="I29">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K29" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L29">
-        <v>269.25</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1736,37 +1784,37 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C30" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="D30">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="E30">
-        <v>1536</v>
+        <v>202305</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H30">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I30">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="J30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K30" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L30">
-        <v>0.04</v>
+        <v>27.15</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1774,37 +1822,37 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C31" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="D31">
-        <v>16</v>
+        <v>432</v>
       </c>
       <c r="E31">
-        <v>5288</v>
+        <v>39000</v>
       </c>
       <c r="F31">
-        <v>2</v>
+        <v>108</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="H31">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="I31">
+        <v>171</v>
+      </c>
+      <c r="J31">
         <v>9</v>
       </c>
-      <c r="J31">
-        <v>2</v>
-      </c>
       <c r="K31" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L31">
-        <v>0.09</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1812,37 +1860,37 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C32" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D32">
-        <v>12</v>
+        <v>97</v>
       </c>
       <c r="E32">
-        <v>36922</v>
+        <v>29850</v>
       </c>
       <c r="F32">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H32">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="I32">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="J32">
         <v>3</v>
       </c>
       <c r="K32" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L32">
-        <v>1.03</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1850,37 +1898,37 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C33" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="D33">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E33">
-        <v>1302</v>
+        <v>6912</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I33">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J33">
         <v>2</v>
       </c>
       <c r="K33" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L33">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1888,37 +1936,37 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C34" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="D34">
-        <v>192</v>
+        <v>218</v>
       </c>
       <c r="E34">
-        <v>154899</v>
+        <v>11308</v>
       </c>
       <c r="F34">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="G34">
-        <v>92</v>
+        <v>204</v>
       </c>
       <c r="H34">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="I34">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="J34">
         <v>3</v>
       </c>
       <c r="K34" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L34">
-        <v>9.67</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1926,22 +1974,22 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C35" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="D35">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E35">
-        <v>2735</v>
+        <v>296</v>
       </c>
       <c r="F35">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G35">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H35">
         <v>2</v>
@@ -1953,10 +2001,10 @@
         <v>2</v>
       </c>
       <c r="K35" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L35">
-        <v>0.11</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -1964,37 +2012,37 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C36" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="D36">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="E36">
-        <v>712</v>
+        <v>3841029</v>
       </c>
       <c r="F36">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G36">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="H36">
         <v>4</v>
       </c>
       <c r="I36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K36" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L36">
-        <v>0.02</v>
+        <v>148.44</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -2002,37 +2050,37 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C37" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D37">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="E37">
-        <v>81850</v>
+        <v>19867</v>
       </c>
       <c r="F37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G37">
         <v>0</v>
       </c>
       <c r="H37">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="I37">
-        <v>3</v>
+        <v>65</v>
       </c>
       <c r="J37">
         <v>2</v>
       </c>
       <c r="K37" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L37">
-        <v>1.96</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2040,37 +2088,37 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C38" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="D38">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E38">
-        <v>5751408</v>
+        <v>6735507</v>
       </c>
       <c r="F38">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G38">
         <v>2</v>
       </c>
       <c r="H38">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I38">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J38">
         <v>2</v>
       </c>
       <c r="K38" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L38">
-        <v>293.14</v>
+        <v>269.25</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2078,37 +2126,37 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C39" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D39">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E39">
-        <v>668</v>
+        <v>1536</v>
       </c>
       <c r="F39">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G39">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H39">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I39">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J39">
         <v>2</v>
       </c>
       <c r="K39" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L39">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2116,37 +2164,37 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C40" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="D40">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E40">
-        <v>668</v>
+        <v>5288</v>
       </c>
       <c r="F40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H40">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I40">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J40">
         <v>2</v>
       </c>
       <c r="K40" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L40">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2154,37 +2202,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C41" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="D41">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="E41">
-        <v>1079680</v>
+        <v>36922</v>
       </c>
       <c r="F41">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G41">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H41">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I41">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J41">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K41" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L41">
-        <v>85.38</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2192,22 +2240,22 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C42" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="D42">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E42">
-        <v>96491</v>
+        <v>1302</v>
       </c>
       <c r="F42">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -2219,10 +2267,10 @@
         <v>2</v>
       </c>
       <c r="K42" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L42">
-        <v>4.68</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2230,37 +2278,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C43" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="D43">
-        <v>16</v>
+        <v>192</v>
       </c>
       <c r="E43">
-        <v>6118</v>
+        <v>154899</v>
       </c>
       <c r="F43">
-        <v>9</v>
+        <v>54</v>
       </c>
       <c r="G43">
-        <v>2</v>
+        <v>92</v>
       </c>
       <c r="H43">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="I43">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="J43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K43" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L43">
-        <v>0.36</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2268,37 +2316,37 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C44" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="D44">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E44">
-        <v>23</v>
+        <v>2735</v>
       </c>
       <c r="F44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G44">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H44">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I44">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J44">
         <v>2</v>
       </c>
       <c r="K44" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L44">
-        <v>0</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2306,37 +2354,37 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C45" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D45">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="E45">
-        <v>1249411</v>
+        <v>712</v>
       </c>
       <c r="F45">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G45">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H45">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I45">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J45">
         <v>2</v>
       </c>
       <c r="K45" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L45">
-        <v>39.2</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2344,37 +2392,37 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C46" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="D46">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="E46">
-        <v>5647694</v>
+        <v>81850</v>
       </c>
       <c r="F46">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G46">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H46">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I46">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J46">
         <v>2</v>
       </c>
       <c r="K46" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L46">
-        <v>173.9</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2382,37 +2430,37 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C47" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="D47">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E47">
-        <v>4395</v>
+        <v>5751408</v>
       </c>
       <c r="F47">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G47">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H47">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I47">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J47">
         <v>2</v>
       </c>
       <c r="K47" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L47">
-        <v>0.15</v>
+        <v>293.14</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2420,37 +2468,37 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C48" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="D48">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E48">
-        <v>1754397</v>
+        <v>668</v>
       </c>
       <c r="F48">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="G48">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H48">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I48">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J48">
         <v>2</v>
       </c>
       <c r="K48" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L48">
-        <v>130.3</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2458,37 +2506,37 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C49" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="D49">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E49">
-        <v>11150</v>
+        <v>668</v>
       </c>
       <c r="F49">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G49">
         <v>3</v>
       </c>
       <c r="H49">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I49">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K49" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L49">
-        <v>0.6928000000000001</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2496,37 +2544,37 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C50" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D50">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="E50">
-        <v>10324</v>
+        <v>1079680</v>
       </c>
       <c r="F50">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="G50">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="H50">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I50">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J50">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K50" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L50">
-        <v>0.37</v>
+        <v>85.38</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2534,37 +2582,37 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C51" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="D51">
-        <v>119</v>
+        <v>11</v>
       </c>
       <c r="E51">
-        <v>11004</v>
+        <v>96491</v>
       </c>
       <c r="F51">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G51">
-        <v>112</v>
+        <v>1</v>
       </c>
       <c r="H51">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I51">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J51">
         <v>2</v>
       </c>
       <c r="K51" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L51">
-        <v>0.45</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2572,19 +2620,19 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C52" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D52">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E52">
-        <v>19297</v>
+        <v>6118</v>
       </c>
       <c r="F52">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G52">
         <v>2</v>
@@ -2596,13 +2644,13 @@
         <v>3</v>
       </c>
       <c r="J52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K52" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L52">
-        <v>0.6899999999999999</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2610,37 +2658,37 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C53" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D53">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E53">
-        <v>83</v>
+        <v>23</v>
       </c>
       <c r="F53">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G53">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I53">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J53">
         <v>2</v>
       </c>
       <c r="K53" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L53">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2648,37 +2696,37 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C54" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="D54">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E54">
-        <v>171</v>
+        <v>1249411</v>
       </c>
       <c r="F54">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G54">
         <v>9</v>
       </c>
       <c r="H54">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I54">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J54">
         <v>2</v>
       </c>
       <c r="K54" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L54">
-        <v>0.01</v>
+        <v>39.2</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2686,37 +2734,37 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C55" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="D55">
         <v>25</v>
       </c>
       <c r="E55">
-        <v>5302</v>
+        <v>5647694</v>
       </c>
       <c r="F55">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G55">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H55">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I55">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J55">
         <v>2</v>
       </c>
       <c r="K55" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L55">
-        <v>0.23</v>
+        <v>173.9</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2724,37 +2772,37 @@
         <v>66</v>
       </c>
       <c r="B56" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="C56" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="D56">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E56">
-        <v>32561</v>
+        <v>4395</v>
       </c>
       <c r="F56">
         <v>9</v>
       </c>
       <c r="G56">
+        <v>4</v>
+      </c>
+      <c r="H56">
+        <v>7</v>
+      </c>
+      <c r="I56">
         <v>6</v>
       </c>
-      <c r="H56">
-        <v>1</v>
-      </c>
-      <c r="I56">
-        <v>0</v>
-      </c>
       <c r="J56">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K56" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L56">
-        <v>3.91</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2762,37 +2810,37 @@
         <v>67</v>
       </c>
       <c r="B57" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="C57" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="D57">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E57">
-        <v>20000</v>
+        <v>1754397</v>
       </c>
       <c r="F57">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="G57">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H57">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I57">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K57" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L57">
-        <v>4.52</v>
+        <v>130.3</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2800,37 +2848,37 @@
         <v>68</v>
       </c>
       <c r="B58" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="C58" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="D58">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="E58">
-        <v>299285</v>
+        <v>11150</v>
       </c>
       <c r="F58">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="G58">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H58">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I58">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J58">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K58" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L58">
-        <v>98.17</v>
+        <v>0.6928000000000001</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2838,37 +2886,37 @@
         <v>69</v>
       </c>
       <c r="B59" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="C59" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="D59">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E59">
-        <v>20000</v>
+        <v>10324</v>
       </c>
       <c r="F59">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="G59">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H59">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I59">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J59">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K59" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L59">
-        <v>3.2</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2876,37 +2924,37 @@
         <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="C60" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="D60">
-        <v>55</v>
+        <v>119</v>
       </c>
       <c r="E60">
-        <v>581012</v>
+        <v>11004</v>
       </c>
       <c r="F60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G60">
-        <v>54</v>
+        <v>112</v>
       </c>
       <c r="H60">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I60">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K60" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L60">
-        <v>255.65</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2914,37 +2962,37 @@
         <v>71</v>
       </c>
       <c r="B61" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="C61" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="D61">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E61">
-        <v>1000</v>
+        <v>19297</v>
       </c>
       <c r="F61">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="G61">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H61">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I61">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J61">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K61" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L61">
-        <v>0.2</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -2952,37 +3000,37 @@
         <v>72</v>
       </c>
       <c r="B62" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="C62" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="D62">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E62">
-        <v>20000</v>
+        <v>83</v>
       </c>
       <c r="F62">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="G62">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I62">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K62" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L62">
-        <v>3.34</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -2990,37 +3038,37 @@
         <v>73</v>
       </c>
       <c r="B63" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="C63" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="D63">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="E63">
-        <v>494021</v>
+        <v>171</v>
       </c>
       <c r="F63">
+        <v>1</v>
+      </c>
+      <c r="G63">
+        <v>9</v>
+      </c>
+      <c r="H63">
+        <v>5</v>
+      </c>
+      <c r="I63">
         <v>4</v>
       </c>
-      <c r="G63">
-        <v>37</v>
-      </c>
-      <c r="H63">
-        <v>1</v>
-      </c>
-      <c r="I63">
-        <v>0</v>
-      </c>
       <c r="J63">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K63" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="L63">
-        <v>162.04</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3028,37 +3076,607 @@
         <v>74</v>
       </c>
       <c r="B64" t="s">
+        <v>91</v>
+      </c>
+      <c r="C64" t="s">
+        <v>97</v>
+      </c>
+      <c r="D64">
+        <v>25</v>
+      </c>
+      <c r="E64">
+        <v>5302</v>
+      </c>
+      <c r="F64">
+        <v>11</v>
+      </c>
+      <c r="G64">
+        <v>9</v>
+      </c>
+      <c r="H64">
+        <v>3</v>
+      </c>
+      <c r="I64">
+        <v>2</v>
+      </c>
+      <c r="J64">
+        <v>2</v>
+      </c>
+      <c r="K64" t="s">
+        <v>99</v>
+      </c>
+      <c r="L64">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12">
+      <c r="A65" t="s">
+        <v>75</v>
+      </c>
+      <c r="B65" t="s">
+        <v>91</v>
+      </c>
+      <c r="C65" t="s">
+        <v>98</v>
+      </c>
+      <c r="D65">
+        <v>19</v>
+      </c>
+      <c r="E65">
+        <v>32231279</v>
+      </c>
+      <c r="F65">
+        <v>4</v>
+      </c>
+      <c r="G65">
+        <v>2</v>
+      </c>
+      <c r="H65">
+        <v>6</v>
+      </c>
+      <c r="I65">
+        <v>5</v>
+      </c>
+      <c r="J65">
+        <v>2</v>
+      </c>
+      <c r="K65" t="s">
+        <v>100</v>
+      </c>
+      <c r="L65">
+        <v>937.268</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12">
+      <c r="A66" t="s">
         <v>76</v>
       </c>
-      <c r="C64" t="s">
+      <c r="B66" t="s">
+        <v>91</v>
+      </c>
+      <c r="C66" t="s">
+        <v>95</v>
+      </c>
+      <c r="D66">
+        <v>15</v>
+      </c>
+      <c r="E66">
+        <v>148021</v>
+      </c>
+      <c r="F66">
+        <v>5</v>
+      </c>
+      <c r="G66">
+        <v>2</v>
+      </c>
+      <c r="H66">
+        <v>5</v>
+      </c>
+      <c r="I66">
+        <v>4</v>
+      </c>
+      <c r="J66">
+        <v>2</v>
+      </c>
+      <c r="K66" t="s">
+        <v>100</v>
+      </c>
+      <c r="L66">
+        <v>3.87</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12">
+      <c r="A67" t="s">
+        <v>77</v>
+      </c>
+      <c r="B67" t="s">
+        <v>91</v>
+      </c>
+      <c r="C67" t="s">
+        <v>95</v>
+      </c>
+      <c r="D67">
+        <v>12</v>
+      </c>
+      <c r="E67">
+        <v>173933</v>
+      </c>
+      <c r="F67">
+        <v>4</v>
+      </c>
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67">
+        <v>3</v>
+      </c>
+      <c r="I67">
+        <v>2</v>
+      </c>
+      <c r="J67">
+        <v>3</v>
+      </c>
+      <c r="K67" t="s">
+        <v>100</v>
+      </c>
+      <c r="L67">
+        <v>8.081517</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12">
+      <c r="A68" t="s">
+        <v>78</v>
+      </c>
+      <c r="B68" t="s">
+        <v>91</v>
+      </c>
+      <c r="C68" t="s">
+        <v>97</v>
+      </c>
+      <c r="D68">
+        <v>15</v>
+      </c>
+      <c r="E68">
+        <v>15000713</v>
+      </c>
+      <c r="F68">
+        <v>4</v>
+      </c>
+      <c r="G68">
+        <v>1</v>
+      </c>
+      <c r="H68">
+        <v>3</v>
+      </c>
+      <c r="I68">
+        <v>2</v>
+      </c>
+      <c r="J68">
+        <v>2</v>
+      </c>
+      <c r="K68" t="s">
+        <v>100</v>
+      </c>
+      <c r="L68">
+        <v>650.54</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12">
+      <c r="A69" t="s">
+        <v>79</v>
+      </c>
+      <c r="B69" t="s">
+        <v>91</v>
+      </c>
+      <c r="C69" t="s">
+        <v>97</v>
+      </c>
+      <c r="D69">
+        <v>21</v>
+      </c>
+      <c r="E69">
+        <v>2146112</v>
+      </c>
+      <c r="F69">
+        <v>1</v>
+      </c>
+      <c r="G69">
+        <v>0</v>
+      </c>
+      <c r="H69">
+        <v>6</v>
+      </c>
+      <c r="I69">
+        <v>6</v>
+      </c>
+      <c r="J69">
+        <v>2</v>
+      </c>
+      <c r="K69" t="s">
+        <v>100</v>
+      </c>
+      <c r="L69">
+        <v>61.659</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12">
+      <c r="A70" t="s">
+        <v>80</v>
+      </c>
+      <c r="B70" t="s">
+        <v>91</v>
+      </c>
+      <c r="C70" t="s">
+        <v>97</v>
+      </c>
+      <c r="D70">
+        <v>42</v>
+      </c>
+      <c r="E70">
+        <v>20679117</v>
+      </c>
+      <c r="F70">
+        <v>7</v>
+      </c>
+      <c r="G70">
+        <v>2</v>
+      </c>
+      <c r="H70">
+        <v>8</v>
+      </c>
+      <c r="I70">
+        <v>11</v>
+      </c>
+      <c r="J70">
+        <v>3</v>
+      </c>
+      <c r="K70" t="s">
+        <v>100</v>
+      </c>
+      <c r="L70">
+        <v>1043.242</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12">
+      <c r="A71" t="s">
         <v>81</v>
       </c>
-      <c r="D64">
-        <v>59</v>
-      </c>
-      <c r="E64">
-        <v>39644</v>
-      </c>
-      <c r="F64">
+      <c r="B71" t="s">
+        <v>91</v>
+      </c>
+      <c r="C71" t="s">
+        <v>97</v>
+      </c>
+      <c r="D71">
+        <v>129</v>
+      </c>
+      <c r="E71">
+        <v>41328337</v>
+      </c>
+      <c r="F71">
+        <v>10</v>
+      </c>
+      <c r="G71">
+        <v>102</v>
+      </c>
+      <c r="H71">
+        <v>5</v>
+      </c>
+      <c r="I71">
+        <v>7</v>
+      </c>
+      <c r="J71">
+        <v>3</v>
+      </c>
+      <c r="K71" t="s">
+        <v>100</v>
+      </c>
+      <c r="L71">
+        <v>3005.995</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12">
+      <c r="A72" t="s">
+        <v>82</v>
+      </c>
+      <c r="B72" t="s">
+        <v>91</v>
+      </c>
+      <c r="C72" t="s">
+        <v>95</v>
+      </c>
+      <c r="D72">
+        <v>67</v>
+      </c>
+      <c r="E72">
+        <v>74063</v>
+      </c>
+      <c r="F72">
+        <v>4</v>
+      </c>
+      <c r="G72">
+        <v>21</v>
+      </c>
+      <c r="H72">
+        <v>9</v>
+      </c>
+      <c r="I72">
+        <v>13</v>
+      </c>
+      <c r="J72">
+        <v>3</v>
+      </c>
+      <c r="K72" t="s">
+        <v>100</v>
+      </c>
+      <c r="L72">
+        <v>5.537</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12">
+      <c r="A73" t="s">
+        <v>83</v>
+      </c>
+      <c r="B73" t="s">
+        <v>91</v>
+      </c>
+      <c r="C73" t="s">
+        <v>96</v>
+      </c>
+      <c r="D73">
+        <v>37</v>
+      </c>
+      <c r="E73">
+        <v>16664809</v>
+      </c>
+      <c r="F73">
+        <v>30</v>
+      </c>
+      <c r="G73">
+        <v>2</v>
+      </c>
+      <c r="H73">
+        <v>3</v>
+      </c>
+      <c r="I73">
+        <v>2</v>
+      </c>
+      <c r="J73">
+        <v>2</v>
+      </c>
+      <c r="K73" t="s">
+        <v>100</v>
+      </c>
+      <c r="L73">
+        <v>737.283</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12">
+      <c r="A74" t="s">
+        <v>84</v>
+      </c>
+      <c r="B74" t="s">
+        <v>91</v>
+      </c>
+      <c r="C74" t="s">
+        <v>97</v>
+      </c>
+      <c r="D74">
+        <v>221</v>
+      </c>
+      <c r="E74">
+        <v>13787005</v>
+      </c>
+      <c r="F74">
+        <v>69</v>
+      </c>
+      <c r="G74">
+        <v>40</v>
+      </c>
+      <c r="H74">
+        <v>13</v>
+      </c>
+      <c r="I74">
+        <v>21</v>
+      </c>
+      <c r="J74">
+        <v>6</v>
+      </c>
+      <c r="K74" t="s">
+        <v>100</v>
+      </c>
+      <c r="L74">
+        <v>1736.28</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12">
+      <c r="A75" t="s">
+        <v>85</v>
+      </c>
+      <c r="B75" t="s">
+        <v>91</v>
+      </c>
+      <c r="C75" t="s">
+        <v>96</v>
+      </c>
+      <c r="D75">
+        <v>31</v>
+      </c>
+      <c r="E75">
+        <v>4257145</v>
+      </c>
+      <c r="F75">
+        <v>17</v>
+      </c>
+      <c r="G75">
         <v>0</v>
       </c>
-      <c r="G64">
-        <v>59</v>
-      </c>
-      <c r="H64">
-        <v>1</v>
-      </c>
-      <c r="I64">
+      <c r="H75">
+        <v>4</v>
+      </c>
+      <c r="I75">
+        <v>6</v>
+      </c>
+      <c r="J75">
+        <v>3</v>
+      </c>
+      <c r="K75" t="s">
+        <v>100</v>
+      </c>
+      <c r="L75">
+        <v>287.3467</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12">
+      <c r="A76" t="s">
+        <v>86</v>
+      </c>
+      <c r="B76" t="s">
+        <v>91</v>
+      </c>
+      <c r="C76" t="s">
+        <v>97</v>
+      </c>
+      <c r="D76">
+        <v>51</v>
+      </c>
+      <c r="E76">
+        <v>4247264</v>
+      </c>
+      <c r="F76">
+        <v>10</v>
+      </c>
+      <c r="G76">
         <v>0</v>
       </c>
-      <c r="J64">
-        <v>1</v>
-      </c>
-      <c r="K64" t="s">
-        <v>84</v>
-      </c>
-      <c r="L64">
-        <v>18.71</v>
+      <c r="H76">
+        <v>7</v>
+      </c>
+      <c r="I76">
+        <v>10</v>
+      </c>
+      <c r="J76">
+        <v>3</v>
+      </c>
+      <c r="K76" t="s">
+        <v>100</v>
+      </c>
+      <c r="L76">
+        <v>246.836575</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12">
+      <c r="A77" t="s">
+        <v>87</v>
+      </c>
+      <c r="B77" t="s">
+        <v>91</v>
+      </c>
+      <c r="C77" t="s">
+        <v>95</v>
+      </c>
+      <c r="D77">
+        <v>140</v>
+      </c>
+      <c r="E77">
+        <v>5434924</v>
+      </c>
+      <c r="F77">
+        <v>51</v>
+      </c>
+      <c r="G77">
+        <v>15</v>
+      </c>
+      <c r="H77">
+        <v>15</v>
+      </c>
+      <c r="I77">
+        <v>15</v>
+      </c>
+      <c r="J77">
+        <v>3</v>
+      </c>
+      <c r="K77" t="s">
+        <v>100</v>
+      </c>
+      <c r="L77">
+        <v>372.106</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12">
+      <c r="A78" t="s">
+        <v>88</v>
+      </c>
+      <c r="B78" t="s">
+        <v>91</v>
+      </c>
+      <c r="C78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D78">
+        <v>19</v>
+      </c>
+      <c r="E78">
+        <v>1018324</v>
+      </c>
+      <c r="F78">
+        <v>5</v>
+      </c>
+      <c r="G78">
+        <v>10</v>
+      </c>
+      <c r="H78">
+        <v>2</v>
+      </c>
+      <c r="I78">
+        <v>1</v>
+      </c>
+      <c r="J78">
+        <v>2</v>
+      </c>
+      <c r="K78" t="s">
+        <v>100</v>
+      </c>
+      <c r="L78">
+        <v>73.33</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12">
+      <c r="A79" t="s">
+        <v>89</v>
+      </c>
+      <c r="B79" t="s">
+        <v>91</v>
+      </c>
+      <c r="C79" t="s">
+        <v>97</v>
+      </c>
+      <c r="D79">
+        <v>20</v>
+      </c>
+      <c r="E79">
+        <v>429805</v>
+      </c>
+      <c r="F79">
+        <v>3</v>
+      </c>
+      <c r="G79">
+        <v>12</v>
+      </c>
+      <c r="H79">
+        <v>3</v>
+      </c>
+      <c r="I79">
+        <v>2</v>
+      </c>
+      <c r="J79">
+        <v>2</v>
+      </c>
+      <c r="K79" t="s">
+        <v>100</v>
+      </c>
+      <c r="L79">
+        <v>14.64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_07_02_2026) - Modality: single_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="102">
   <si>
     <t>Dataset</t>
   </si>
@@ -52,6 +52,213 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>Accidents</t>
+  </si>
+  <si>
+    <t>Atherosclerosis</t>
+  </si>
+  <si>
+    <t>AustralianFootball</t>
+  </si>
+  <si>
+    <t>Biodegradability</t>
+  </si>
+  <si>
+    <t>Bupa</t>
+  </si>
+  <si>
+    <t>CORA</t>
+  </si>
+  <si>
+    <t>Carcinogenesis</t>
+  </si>
+  <si>
+    <t>Chess</t>
+  </si>
+  <si>
+    <t>Countries</t>
+  </si>
+  <si>
+    <t>DCG</t>
+  </si>
+  <si>
+    <t>Dunur</t>
+  </si>
+  <si>
+    <t>Elti</t>
+  </si>
+  <si>
+    <t>FNHK</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>Hepatitis_std</t>
+  </si>
+  <si>
+    <t>Mesh</t>
+  </si>
+  <si>
+    <t>Mooney_Family</t>
+  </si>
+  <si>
+    <t>MuskSmall</t>
+  </si>
+  <si>
+    <t>NBA</t>
+  </si>
+  <si>
+    <t>NCAA</t>
+  </si>
+  <si>
+    <t>OMOP_CDM_dayz</t>
+  </si>
+  <si>
+    <t>PTE</t>
+  </si>
+  <si>
+    <t>Pima</t>
+  </si>
+  <si>
+    <t>PremierLeague</t>
+  </si>
+  <si>
+    <t>Pyrimidine</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>SAT</t>
+  </si>
+  <si>
+    <t>SalesDB</t>
+  </si>
+  <si>
+    <t>Same_gen</t>
+  </si>
+  <si>
+    <t>Student_loan</t>
+  </si>
+  <si>
+    <t>Toxicology</t>
+  </si>
+  <si>
+    <t>Triazine</t>
+  </si>
+  <si>
+    <t>TubePricing</t>
+  </si>
+  <si>
+    <t>UTube</t>
+  </si>
+  <si>
+    <t>UW_std</t>
+  </si>
+  <si>
+    <t>WebKP</t>
+  </si>
+  <si>
+    <t>airbnb-simplified</t>
+  </si>
+  <si>
+    <t>fake_hotels</t>
+  </si>
+  <si>
+    <t>fake_hotels_extended</t>
+  </si>
+  <si>
+    <t>financial</t>
+  </si>
+  <si>
+    <t>ftp</t>
+  </si>
+  <si>
+    <t>genes</t>
+  </si>
+  <si>
+    <t>got_families</t>
+  </si>
+  <si>
+    <t>imdb_MovieLens</t>
+  </si>
+  <si>
+    <t>imdb_ijs</t>
+  </si>
+  <si>
+    <t>imdb_small</t>
+  </si>
+  <si>
+    <t>legalActs</t>
+  </si>
+  <si>
+    <t>multi_table_ID_demo_dataset</t>
+  </si>
+  <si>
+    <t>mutagenesis</t>
+  </si>
+  <si>
+    <t>nations</t>
+  </si>
+  <si>
+    <t>restbase</t>
+  </si>
+  <si>
+    <t>trains</t>
+  </si>
+  <si>
+    <t>university</t>
+  </si>
+  <si>
+    <t>world</t>
+  </si>
+  <si>
+    <t>MovieLens</t>
+  </si>
+  <si>
+    <t>Telstra</t>
+  </si>
+  <si>
+    <t>instacart_marketbasket_ml</t>
+  </si>
+  <si>
+    <t>rel-amazon</t>
+  </si>
+  <si>
+    <t>rel-arxiv</t>
+  </si>
+  <si>
+    <t>rel-avito</t>
+  </si>
+  <si>
+    <t>rel-event</t>
+  </si>
+  <si>
+    <t>rel-f1</t>
+  </si>
+  <si>
+    <t>rel-hm</t>
+  </si>
+  <si>
+    <t>rel-ratebeer</t>
+  </si>
+  <si>
+    <t>rel-salt</t>
+  </si>
+  <si>
+    <t>rel-stack</t>
+  </si>
+  <si>
+    <t>rel-trial</t>
+  </si>
+  <si>
+    <t>rossmann</t>
+  </si>
+  <si>
+    <t>walmart</t>
+  </si>
+  <si>
     <t>adult</t>
   </si>
   <si>
@@ -79,217 +286,22 @@
     <t>news</t>
   </si>
   <si>
-    <t>Accidents</t>
-  </si>
-  <si>
-    <t>Atherosclerosis</t>
-  </si>
-  <si>
-    <t>AustralianFootball</t>
-  </si>
-  <si>
-    <t>Biodegradability</t>
-  </si>
-  <si>
-    <t>Bupa</t>
-  </si>
-  <si>
-    <t>CORA</t>
-  </si>
-  <si>
-    <t>Carcinogenesis</t>
-  </si>
-  <si>
-    <t>Chess</t>
-  </si>
-  <si>
-    <t>Countries</t>
-  </si>
-  <si>
-    <t>DCG</t>
-  </si>
-  <si>
-    <t>Dunur</t>
-  </si>
-  <si>
-    <t>Elti</t>
-  </si>
-  <si>
-    <t>FNHK</t>
-  </si>
-  <si>
-    <t>Facebook</t>
-  </si>
-  <si>
-    <t>Hepatitis_std</t>
-  </si>
-  <si>
-    <t>Mesh</t>
-  </si>
-  <si>
-    <t>Mooney_Family</t>
-  </si>
-  <si>
-    <t>MuskSmall</t>
-  </si>
-  <si>
-    <t>NBA</t>
-  </si>
-  <si>
-    <t>NCAA</t>
-  </si>
-  <si>
-    <t>OMOP_CDM_dayz</t>
-  </si>
-  <si>
-    <t>PTE</t>
-  </si>
-  <si>
-    <t>Pima</t>
-  </si>
-  <si>
-    <t>PremierLeague</t>
-  </si>
-  <si>
-    <t>Pyrimidine</t>
-  </si>
-  <si>
-    <t>SAP</t>
-  </si>
-  <si>
-    <t>SAT</t>
-  </si>
-  <si>
-    <t>SalesDB</t>
-  </si>
-  <si>
-    <t>Same_gen</t>
-  </si>
-  <si>
-    <t>Student_loan</t>
-  </si>
-  <si>
-    <t>Toxicology</t>
-  </si>
-  <si>
-    <t>Triazine</t>
-  </si>
-  <si>
-    <t>TubePricing</t>
-  </si>
-  <si>
-    <t>UTube</t>
-  </si>
-  <si>
-    <t>UW_std</t>
-  </si>
-  <si>
-    <t>WebKP</t>
-  </si>
-  <si>
-    <t>airbnb-simplified</t>
-  </si>
-  <si>
-    <t>fake_hotels</t>
-  </si>
-  <si>
-    <t>fake_hotels_extended</t>
-  </si>
-  <si>
-    <t>financial</t>
-  </si>
-  <si>
-    <t>ftp</t>
-  </si>
-  <si>
-    <t>genes</t>
-  </si>
-  <si>
-    <t>got_families</t>
-  </si>
-  <si>
-    <t>imdb_MovieLens</t>
-  </si>
-  <si>
-    <t>imdb_ijs</t>
-  </si>
-  <si>
-    <t>imdb_small</t>
-  </si>
-  <si>
-    <t>legalActs</t>
-  </si>
-  <si>
-    <t>multi_table_ID_demo_dataset</t>
-  </si>
-  <si>
-    <t>mutagenesis</t>
-  </si>
-  <si>
-    <t>nations</t>
-  </si>
-  <si>
-    <t>restbase</t>
-  </si>
-  <si>
-    <t>trains</t>
-  </si>
-  <si>
-    <t>university</t>
-  </si>
-  <si>
-    <t>world</t>
-  </si>
-  <si>
-    <t>MovieLens</t>
-  </si>
-  <si>
-    <t>Telstra</t>
-  </si>
-  <si>
-    <t>instacart_marketbasket_ml</t>
-  </si>
-  <si>
-    <t>rel-amazon</t>
-  </si>
-  <si>
-    <t>rel-arxiv</t>
-  </si>
-  <si>
-    <t>rel-avito</t>
-  </si>
-  <si>
-    <t>rel-event</t>
-  </si>
-  <si>
-    <t>rel-f1</t>
-  </si>
-  <si>
-    <t>rel-hm</t>
-  </si>
-  <si>
-    <t>rel-ratebeer</t>
-  </si>
-  <si>
-    <t>rel-salt</t>
-  </si>
-  <si>
-    <t>rel-stack</t>
-  </si>
-  <si>
-    <t>rel-trial</t>
-  </si>
-  <si>
-    <t>rossmann</t>
-  </si>
-  <si>
-    <t>walmart</t>
+    <t>multi_table</t>
   </si>
   <si>
     <t>single_table</t>
   </si>
   <si>
-    <t>multi_table</t>
+    <t>HSASynthesizer</t>
+  </si>
+  <si>
+    <t>IndependentSynthesizer</t>
+  </si>
+  <si>
+    <t>HMASynthesizer</t>
+  </si>
+  <si>
+    <t>MultiTableUniformSynthesizer</t>
   </si>
   <si>
     <t>RealTabFormerSynthesizer</t>
@@ -301,16 +313,7 @@
     <t>GaussianCopulaSynthesizer</t>
   </si>
   <si>
-    <t>HSASynthesizer</t>
-  </si>
-  <si>
-    <t>IndependentSynthesizer</t>
-  </si>
-  <si>
-    <t>HMASynthesizer</t>
-  </si>
-  <si>
-    <t>MultiTableUniformSynthesizer</t>
+    <t>SegmentSynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -726,31 +729,31 @@
         <v>92</v>
       </c>
       <c r="D2">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="E2">
-        <v>32561</v>
+        <v>1463093</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="G2">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L2">
-        <v>3.91</v>
+        <v>219.33</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -764,31 +767,31 @@
         <v>93</v>
       </c>
       <c r="D3">
-        <v>37</v>
+        <v>198</v>
       </c>
       <c r="E3">
-        <v>20000</v>
+        <v>12781</v>
       </c>
       <c r="F3">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L3">
-        <v>4.52</v>
+        <v>6.62</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -802,31 +805,31 @@
         <v>92</v>
       </c>
       <c r="D4">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="E4">
-        <v>299285</v>
+        <v>139179</v>
       </c>
       <c r="F4">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="G4">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L4">
-        <v>98.17</v>
+        <v>31.18</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -837,34 +840,34 @@
         <v>90</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D5">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E5">
-        <v>20000</v>
+        <v>21895</v>
       </c>
       <c r="F5">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L5">
-        <v>3.2</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -878,31 +881,31 @@
         <v>93</v>
       </c>
       <c r="D6">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="E6">
-        <v>581012</v>
+        <v>2762</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>54</v>
+        <v>7</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L6">
-        <v>255.65</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -913,34 +916,34 @@
         <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D7">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E7">
-        <v>1000</v>
+        <v>57353</v>
       </c>
       <c r="F7">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L7">
-        <v>0.2</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -951,34 +954,34 @@
         <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D8">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E8">
-        <v>20000</v>
+        <v>27443</v>
       </c>
       <c r="F8">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L8">
-        <v>3.34</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -992,31 +995,31 @@
         <v>92</v>
       </c>
       <c r="D9">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="E9">
-        <v>494021</v>
+        <v>2052</v>
       </c>
       <c r="F9">
+        <v>39</v>
+      </c>
+      <c r="G9">
         <v>4</v>
       </c>
-      <c r="G9">
-        <v>37</v>
-      </c>
       <c r="H9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L9">
-        <v>162.04</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -1030,31 +1033,31 @@
         <v>92</v>
       </c>
       <c r="D10">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E10">
-        <v>39644</v>
+        <v>22318</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G10">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L10">
-        <v>18.71</v>
+        <v>9.93</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1062,37 +1065,37 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C11" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D11">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="E11">
-        <v>1463093</v>
+        <v>8258</v>
       </c>
       <c r="F11">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="G11">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="H11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L11">
-        <v>219.33</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1100,37 +1103,37 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C12" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D12">
-        <v>198</v>
+        <v>50</v>
       </c>
       <c r="E12">
-        <v>12781</v>
+        <v>440</v>
       </c>
       <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
         <v>0</v>
       </c>
-      <c r="G12">
-        <v>193</v>
-      </c>
       <c r="H12">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I12">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="J12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L12">
-        <v>6.62</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1138,37 +1141,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C13" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D13">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="E13">
-        <v>139179</v>
+        <v>1352</v>
       </c>
       <c r="F13">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I13">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="J13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L13">
-        <v>31.18</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1176,37 +1179,37 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C14" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D14">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="E14">
-        <v>21895</v>
+        <v>2113275</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G14">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I14">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L14">
-        <v>0.57</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1214,37 +1217,37 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C15" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D15">
-        <v>17</v>
+        <v>266</v>
       </c>
       <c r="E15">
-        <v>2762</v>
+        <v>10173</v>
       </c>
       <c r="F15">
+        <v>262</v>
+      </c>
+      <c r="G15">
         <v>0</v>
       </c>
-      <c r="G15">
-        <v>7</v>
-      </c>
       <c r="H15">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I15">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J15">
         <v>2</v>
       </c>
       <c r="K15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L15">
-        <v>0.04</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1252,37 +1255,37 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C16" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D16">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E16">
-        <v>57353</v>
+        <v>12927</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
       <c r="G16">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H16">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I16">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J16">
         <v>2</v>
       </c>
       <c r="K16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L16">
-        <v>1.79</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1290,37 +1293,37 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C17" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D17">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="E17">
-        <v>27443</v>
+        <v>2700</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G17">
         <v>2</v>
       </c>
       <c r="H17">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="I17">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="J17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L17">
-        <v>0.9399999999999999</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1328,37 +1331,37 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C18" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D18">
-        <v>46</v>
+        <v>202</v>
       </c>
       <c r="E18">
-        <v>2052</v>
+        <v>4425</v>
       </c>
       <c r="F18">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>189</v>
       </c>
       <c r="J18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L18">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1366,37 +1369,37 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D19">
-        <v>68</v>
+        <v>170</v>
       </c>
       <c r="E19">
-        <v>22318</v>
+        <v>568</v>
       </c>
       <c r="F19">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>53</v>
+        <v>167</v>
       </c>
       <c r="H19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J19">
         <v>2</v>
       </c>
       <c r="K19" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L19">
-        <v>9.93</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1404,37 +1407,37 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C20" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D20">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E20">
-        <v>8258</v>
+        <v>1219</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="H20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J20">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L20">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1442,37 +1445,37 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D21">
-        <v>50</v>
+        <v>112</v>
       </c>
       <c r="E21">
-        <v>440</v>
+        <v>202305</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H21">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I21">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="J21">
         <v>3</v>
       </c>
       <c r="K21" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L21">
-        <v>0.01</v>
+        <v>27.15</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1480,37 +1483,37 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C22" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D22">
-        <v>32</v>
+        <v>432</v>
       </c>
       <c r="E22">
-        <v>1352</v>
+        <v>39000</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>108</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="H22">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="I22">
-        <v>20</v>
+        <v>171</v>
       </c>
       <c r="J22">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="K22" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L22">
-        <v>0.05</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1518,37 +1521,37 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C23" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23">
         <v>97</v>
       </c>
-      <c r="D23">
-        <v>26</v>
-      </c>
       <c r="E23">
-        <v>2113275</v>
+        <v>29850</v>
       </c>
       <c r="F23">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="G23">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H23">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="I23">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="J23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K23" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L23">
-        <v>120</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1556,37 +1559,37 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D24">
-        <v>266</v>
+        <v>18</v>
       </c>
       <c r="E24">
-        <v>10173</v>
+        <v>6912</v>
       </c>
       <c r="F24">
-        <v>262</v>
+        <v>1</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H24">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I24">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J24">
         <v>2</v>
       </c>
       <c r="K24" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L24">
-        <v>1.38</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1594,37 +1597,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C25" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D25">
-        <v>29</v>
+        <v>218</v>
       </c>
       <c r="E25">
-        <v>12927</v>
+        <v>11308</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G25">
-        <v>14</v>
+        <v>204</v>
       </c>
       <c r="H25">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K25" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L25">
-        <v>0.68</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1632,37 +1635,37 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C26" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D26">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E26">
-        <v>2700</v>
+        <v>296</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H26">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="I26">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="J26">
         <v>2</v>
       </c>
       <c r="K26" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L26">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1670,37 +1673,37 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C27" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D27">
-        <v>202</v>
+        <v>42</v>
       </c>
       <c r="E27">
-        <v>4425</v>
+        <v>3841029</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="H27">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="I27">
-        <v>189</v>
+        <v>3</v>
       </c>
       <c r="J27">
         <v>3</v>
       </c>
       <c r="K27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L27">
-        <v>0.1</v>
+        <v>148.44</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1708,37 +1711,37 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C28" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D28">
-        <v>170</v>
+        <v>70</v>
       </c>
       <c r="E28">
-        <v>568</v>
+        <v>19867</v>
       </c>
       <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
         <v>0</v>
       </c>
-      <c r="G28">
-        <v>167</v>
-      </c>
       <c r="H28">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="I28">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="J28">
         <v>2</v>
       </c>
       <c r="K28" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L28">
-        <v>0.64</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1746,37 +1749,37 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C29" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D29">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E29">
-        <v>1219</v>
+        <v>6735507</v>
       </c>
       <c r="F29">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G29">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="H29">
         <v>4</v>
       </c>
       <c r="I29">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K29" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L29">
-        <v>0.15</v>
+        <v>269.25</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1784,37 +1787,37 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C30" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D30">
-        <v>112</v>
+        <v>11</v>
       </c>
       <c r="E30">
-        <v>202305</v>
+        <v>1536</v>
       </c>
       <c r="F30">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G30">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="H30">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I30">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="J30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L30">
-        <v>27.15</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1822,37 +1825,37 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C31" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D31">
-        <v>432</v>
+        <v>16</v>
       </c>
       <c r="E31">
-        <v>39000</v>
+        <v>5288</v>
       </c>
       <c r="F31">
-        <v>108</v>
+        <v>2</v>
       </c>
       <c r="G31">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="H31">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="I31">
-        <v>171</v>
+        <v>9</v>
       </c>
       <c r="J31">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K31" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L31">
-        <v>3.45</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1860,37 +1863,37 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C32" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D32">
-        <v>97</v>
+        <v>12</v>
       </c>
       <c r="E32">
-        <v>29850</v>
+        <v>36922</v>
       </c>
       <c r="F32">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="G32">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H32">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="I32">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="J32">
         <v>3</v>
       </c>
       <c r="K32" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L32">
-        <v>0.95</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1898,37 +1901,37 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C33" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D33">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E33">
-        <v>6912</v>
+        <v>1302</v>
       </c>
       <c r="F33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H33">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I33">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J33">
         <v>2</v>
       </c>
       <c r="K33" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L33">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1936,37 +1939,37 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C34" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D34">
-        <v>218</v>
+        <v>192</v>
       </c>
       <c r="E34">
-        <v>11308</v>
+        <v>154899</v>
       </c>
       <c r="F34">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="G34">
-        <v>204</v>
+        <v>92</v>
       </c>
       <c r="H34">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="I34">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="J34">
         <v>3</v>
       </c>
       <c r="K34" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L34">
-        <v>17.2</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1974,23 +1977,23 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C35" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D35">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E35">
-        <v>296</v>
+        <v>2735</v>
       </c>
       <c r="F35">
+        <v>5</v>
+      </c>
+      <c r="G35">
         <v>0</v>
       </c>
-      <c r="G35">
-        <v>11</v>
-      </c>
       <c r="H35">
         <v>2</v>
       </c>
@@ -2001,10 +2004,10 @@
         <v>2</v>
       </c>
       <c r="K35" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L35">
-        <v>0.02</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -2012,37 +2015,37 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C36" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D36">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="E36">
-        <v>3841029</v>
+        <v>712</v>
       </c>
       <c r="F36">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G36">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="H36">
         <v>4</v>
       </c>
       <c r="I36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K36" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L36">
-        <v>148.44</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -2050,37 +2053,37 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C37" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D37">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="E37">
-        <v>19867</v>
+        <v>81850</v>
       </c>
       <c r="F37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G37">
         <v>0</v>
       </c>
       <c r="H37">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="I37">
-        <v>65</v>
+        <v>3</v>
       </c>
       <c r="J37">
         <v>2</v>
       </c>
       <c r="K37" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L37">
-        <v>0.32</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2088,37 +2091,37 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C38" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D38">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E38">
-        <v>6735507</v>
+        <v>5751408</v>
       </c>
       <c r="F38">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="G38">
         <v>2</v>
       </c>
       <c r="H38">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I38">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J38">
         <v>2</v>
       </c>
       <c r="K38" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L38">
-        <v>269.25</v>
+        <v>293.14</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2126,37 +2129,37 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C39" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D39">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E39">
-        <v>1536</v>
+        <v>668</v>
       </c>
       <c r="F39">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H39">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I39">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J39">
         <v>2</v>
       </c>
       <c r="K39" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L39">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2164,37 +2167,37 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C40" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D40">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E40">
-        <v>5288</v>
+        <v>668</v>
       </c>
       <c r="F40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H40">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I40">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J40">
         <v>2</v>
       </c>
       <c r="K40" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L40">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2202,37 +2205,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C41" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D41">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="E41">
-        <v>36922</v>
+        <v>1079680</v>
       </c>
       <c r="F41">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H41">
+        <v>8</v>
+      </c>
+      <c r="I41">
+        <v>8</v>
+      </c>
+      <c r="J41">
         <v>4</v>
       </c>
-      <c r="I41">
-        <v>5</v>
-      </c>
-      <c r="J41">
-        <v>3</v>
-      </c>
       <c r="K41" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L41">
-        <v>1.03</v>
+        <v>85.38</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2240,22 +2243,22 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C42" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D42">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E42">
-        <v>1302</v>
+        <v>96491</v>
       </c>
       <c r="F42">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G42">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -2267,10 +2270,10 @@
         <v>2</v>
       </c>
       <c r="K42" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L42">
-        <v>0.12</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2278,37 +2281,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C43" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D43">
-        <v>192</v>
+        <v>16</v>
       </c>
       <c r="E43">
-        <v>154899</v>
+        <v>6118</v>
       </c>
       <c r="F43">
-        <v>54</v>
+        <v>9</v>
       </c>
       <c r="G43">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="H43">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="I43">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="J43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K43" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L43">
-        <v>9.67</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2316,37 +2319,37 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C44" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D44">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E44">
-        <v>2735</v>
+        <v>23</v>
       </c>
       <c r="F44">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G44">
+        <v>2</v>
+      </c>
+      <c r="H44">
+        <v>3</v>
+      </c>
+      <c r="I44">
+        <v>2</v>
+      </c>
+      <c r="J44">
+        <v>2</v>
+      </c>
+      <c r="K44" t="s">
+        <v>100</v>
+      </c>
+      <c r="L44">
         <v>0</v>
-      </c>
-      <c r="H44">
-        <v>2</v>
-      </c>
-      <c r="I44">
-        <v>1</v>
-      </c>
-      <c r="J44">
-        <v>2</v>
-      </c>
-      <c r="K44" t="s">
-        <v>99</v>
-      </c>
-      <c r="L44">
-        <v>0.11</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2354,37 +2357,37 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C45" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D45">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="E45">
-        <v>712</v>
+        <v>1249411</v>
       </c>
       <c r="F45">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G45">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H45">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I45">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J45">
         <v>2</v>
       </c>
       <c r="K45" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L45">
-        <v>0.02</v>
+        <v>39.2</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2392,37 +2395,37 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C46" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D46">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E46">
-        <v>81850</v>
+        <v>5647694</v>
       </c>
       <c r="F46">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H46">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I46">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J46">
         <v>2</v>
       </c>
       <c r="K46" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L46">
-        <v>1.96</v>
+        <v>173.9</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2430,37 +2433,37 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C47" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D47">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E47">
-        <v>5751408</v>
+        <v>4395</v>
       </c>
       <c r="F47">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G47">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H47">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I47">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J47">
         <v>2</v>
       </c>
       <c r="K47" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L47">
-        <v>293.14</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2468,37 +2471,37 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C48" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D48">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E48">
-        <v>668</v>
+        <v>1754397</v>
       </c>
       <c r="F48">
+        <v>18</v>
+      </c>
+      <c r="G48">
+        <v>8</v>
+      </c>
+      <c r="H48">
         <v>5</v>
       </c>
-      <c r="G48">
-        <v>3</v>
-      </c>
-      <c r="H48">
-        <v>2</v>
-      </c>
       <c r="I48">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J48">
         <v>2</v>
       </c>
       <c r="K48" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L48">
-        <v>0.05</v>
+        <v>130.3</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2506,37 +2509,37 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C49" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D49">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E49">
-        <v>668</v>
+        <v>11150</v>
       </c>
       <c r="F49">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G49">
         <v>3</v>
       </c>
       <c r="H49">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I49">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J49">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K49" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L49">
-        <v>0.07000000000000001</v>
+        <v>0.6928000000000001</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2544,37 +2547,37 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C50" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D50">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="E50">
-        <v>1079680</v>
+        <v>10324</v>
       </c>
       <c r="F50">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G50">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="H50">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I50">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J50">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K50" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L50">
-        <v>85.38</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2582,37 +2585,37 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C51" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D51">
-        <v>11</v>
+        <v>119</v>
       </c>
       <c r="E51">
-        <v>96491</v>
+        <v>11004</v>
       </c>
       <c r="F51">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G51">
-        <v>1</v>
+        <v>112</v>
       </c>
       <c r="H51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I51">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J51">
         <v>2</v>
       </c>
       <c r="K51" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L51">
-        <v>4.68</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2620,19 +2623,19 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C52" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D52">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E52">
-        <v>6118</v>
+        <v>19297</v>
       </c>
       <c r="F52">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G52">
         <v>2</v>
@@ -2644,13 +2647,13 @@
         <v>3</v>
       </c>
       <c r="J52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K52" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L52">
-        <v>0.36</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2658,37 +2661,37 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C53" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D53">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E53">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="F53">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G53">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H53">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J53">
         <v>2</v>
       </c>
       <c r="K53" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L53">
-        <v>0</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2696,37 +2699,37 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C54" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D54">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E54">
-        <v>1249411</v>
+        <v>171</v>
       </c>
       <c r="F54">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G54">
         <v>9</v>
       </c>
       <c r="H54">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I54">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J54">
         <v>2</v>
       </c>
       <c r="K54" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L54">
-        <v>39.2</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2734,37 +2737,37 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C55" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D55">
         <v>25</v>
       </c>
       <c r="E55">
-        <v>5647694</v>
+        <v>5302</v>
       </c>
       <c r="F55">
+        <v>11</v>
+      </c>
+      <c r="G55">
         <v>9</v>
       </c>
-      <c r="G55">
-        <v>3</v>
-      </c>
       <c r="H55">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I55">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J55">
         <v>2</v>
       </c>
       <c r="K55" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L55">
-        <v>173.9</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2772,37 +2775,37 @@
         <v>66</v>
       </c>
       <c r="B56" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C56" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D56">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E56">
-        <v>4395</v>
+        <v>32231279</v>
       </c>
       <c r="F56">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G56">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H56">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I56">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J56">
         <v>2</v>
       </c>
       <c r="K56" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L56">
-        <v>0.15</v>
+        <v>937.268</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2810,37 +2813,37 @@
         <v>67</v>
       </c>
       <c r="B57" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C57" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D57">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E57">
-        <v>1754397</v>
+        <v>148021</v>
       </c>
       <c r="F57">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="G57">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H57">
         <v>5</v>
       </c>
       <c r="I57">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J57">
         <v>2</v>
       </c>
       <c r="K57" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L57">
-        <v>130.3</v>
+        <v>3.87</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2848,37 +2851,37 @@
         <v>68</v>
       </c>
       <c r="B58" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C58" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D58">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="E58">
-        <v>11150</v>
+        <v>173933</v>
       </c>
       <c r="F58">
         <v>4</v>
       </c>
       <c r="G58">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I58">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J58">
         <v>3</v>
       </c>
       <c r="K58" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L58">
-        <v>0.6928000000000001</v>
+        <v>8.081517</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2886,37 +2889,37 @@
         <v>69</v>
       </c>
       <c r="B59" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C59" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D59">
         <v>15</v>
       </c>
       <c r="E59">
-        <v>10324</v>
+        <v>15000713</v>
       </c>
       <c r="F59">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G59">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H59">
         <v>3</v>
       </c>
       <c r="I59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K59" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L59">
-        <v>0.37</v>
+        <v>650.54</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2924,37 +2927,37 @@
         <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C60" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D60">
-        <v>119</v>
+        <v>21</v>
       </c>
       <c r="E60">
-        <v>11004</v>
+        <v>2146112</v>
       </c>
       <c r="F60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G60">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="H60">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I60">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J60">
         <v>2</v>
       </c>
       <c r="K60" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L60">
-        <v>0.45</v>
+        <v>61.659</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2962,37 +2965,37 @@
         <v>71</v>
       </c>
       <c r="B61" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C61" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D61">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="E61">
-        <v>19297</v>
+        <v>20679117</v>
       </c>
       <c r="F61">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G61">
         <v>2</v>
       </c>
       <c r="H61">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I61">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J61">
         <v>3</v>
       </c>
       <c r="K61" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L61">
-        <v>0.6899999999999999</v>
+        <v>1043.242</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -3000,37 +3003,37 @@
         <v>72</v>
       </c>
       <c r="B62" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C62" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D62">
-        <v>13</v>
+        <v>129</v>
       </c>
       <c r="E62">
-        <v>83</v>
+        <v>41328337</v>
       </c>
       <c r="F62">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G62">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="H62">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I62">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K62" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L62">
-        <v>0.01</v>
+        <v>3005.995</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -3038,37 +3041,37 @@
         <v>73</v>
       </c>
       <c r="B63" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C63" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D63">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="E63">
-        <v>171</v>
+        <v>74063</v>
       </c>
       <c r="F63">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G63">
+        <v>21</v>
+      </c>
+      <c r="H63">
         <v>9</v>
       </c>
-      <c r="H63">
-        <v>5</v>
-      </c>
       <c r="I63">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="J63">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K63" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L63">
-        <v>0.01</v>
+        <v>5.537</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3076,22 +3079,22 @@
         <v>74</v>
       </c>
       <c r="B64" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C64" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D64">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="E64">
-        <v>5302</v>
+        <v>16664809</v>
       </c>
       <c r="F64">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="G64">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H64">
         <v>3</v>
@@ -3103,10 +3106,10 @@
         <v>2</v>
       </c>
       <c r="K64" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L64">
-        <v>0.23</v>
+        <v>737.283</v>
       </c>
     </row>
     <row r="65" spans="1:12">
@@ -3114,37 +3117,37 @@
         <v>75</v>
       </c>
       <c r="B65" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C65" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D65">
-        <v>19</v>
+        <v>221</v>
       </c>
       <c r="E65">
-        <v>32231279</v>
+        <v>13787005</v>
       </c>
       <c r="F65">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="G65">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="H65">
+        <v>13</v>
+      </c>
+      <c r="I65">
+        <v>21</v>
+      </c>
+      <c r="J65">
         <v>6</v>
       </c>
-      <c r="I65">
-        <v>5</v>
-      </c>
-      <c r="J65">
-        <v>2</v>
-      </c>
       <c r="K65" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L65">
-        <v>937.268</v>
+        <v>1736.28</v>
       </c>
     </row>
     <row r="66" spans="1:12">
@@ -3152,37 +3155,37 @@
         <v>76</v>
       </c>
       <c r="B66" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C66" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D66">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="E66">
-        <v>148021</v>
+        <v>4257145</v>
       </c>
       <c r="F66">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="G66">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I66">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J66">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K66" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L66">
-        <v>3.87</v>
+        <v>287.3467</v>
       </c>
     </row>
     <row r="67" spans="1:12">
@@ -3190,37 +3193,37 @@
         <v>77</v>
       </c>
       <c r="B67" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C67" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D67">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="E67">
-        <v>173933</v>
+        <v>4247264</v>
       </c>
       <c r="F67">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G67">
         <v>0</v>
       </c>
       <c r="H67">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I67">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J67">
         <v>3</v>
       </c>
       <c r="K67" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L67">
-        <v>8.081517</v>
+        <v>246.836575</v>
       </c>
     </row>
     <row r="68" spans="1:12">
@@ -3228,37 +3231,37 @@
         <v>78</v>
       </c>
       <c r="B68" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C68" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D68">
+        <v>140</v>
+      </c>
+      <c r="E68">
+        <v>5434924</v>
+      </c>
+      <c r="F68">
+        <v>51</v>
+      </c>
+      <c r="G68">
         <v>15</v>
       </c>
-      <c r="E68">
-        <v>15000713</v>
-      </c>
-      <c r="F68">
-        <v>4</v>
-      </c>
-      <c r="G68">
-        <v>1</v>
-      </c>
       <c r="H68">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="I68">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="J68">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K68" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L68">
-        <v>650.54</v>
+        <v>372.106</v>
       </c>
     </row>
     <row r="69" spans="1:12">
@@ -3266,37 +3269,37 @@
         <v>79</v>
       </c>
       <c r="B69" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C69" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D69">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E69">
-        <v>2146112</v>
+        <v>1018324</v>
       </c>
       <c r="F69">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G69">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H69">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I69">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J69">
         <v>2</v>
       </c>
       <c r="K69" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L69">
-        <v>61.659</v>
+        <v>73.33</v>
       </c>
     </row>
     <row r="70" spans="1:12">
@@ -3304,37 +3307,37 @@
         <v>80</v>
       </c>
       <c r="B70" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C70" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D70">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="E70">
-        <v>20679117</v>
+        <v>429805</v>
       </c>
       <c r="F70">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G70">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H70">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I70">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J70">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K70" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L70">
-        <v>1043.242</v>
+        <v>14.64</v>
       </c>
     </row>
     <row r="71" spans="1:12">
@@ -3345,34 +3348,34 @@
         <v>91</v>
       </c>
       <c r="C71" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D71">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="E71">
-        <v>41328337</v>
+        <v>32561</v>
       </c>
       <c r="F71">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G71">
-        <v>102</v>
+        <v>6</v>
       </c>
       <c r="H71">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I71">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J71">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K71" t="s">
         <v>100</v>
       </c>
       <c r="L71">
-        <v>3005.995</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="72" spans="1:12">
@@ -3383,34 +3386,34 @@
         <v>91</v>
       </c>
       <c r="C72" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D72">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="E72">
-        <v>74063</v>
+        <v>20000</v>
       </c>
       <c r="F72">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="G72">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H72">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I72">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J72">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K72" t="s">
         <v>100</v>
       </c>
       <c r="L72">
-        <v>5.537</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="73" spans="1:12">
@@ -3424,31 +3427,31 @@
         <v>96</v>
       </c>
       <c r="D73">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E73">
-        <v>16664809</v>
+        <v>299285</v>
       </c>
       <c r="F73">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G73">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H73">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I73">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K73" t="s">
         <v>100</v>
       </c>
       <c r="L73">
-        <v>737.283</v>
+        <v>98.17</v>
       </c>
     </row>
     <row r="74" spans="1:12">
@@ -3462,31 +3465,31 @@
         <v>97</v>
       </c>
       <c r="D74">
-        <v>221</v>
+        <v>20</v>
       </c>
       <c r="E74">
-        <v>13787005</v>
+        <v>20000</v>
       </c>
       <c r="F74">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="G74">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="H74">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="I74">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="J74">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K74" t="s">
         <v>100</v>
       </c>
       <c r="L74">
-        <v>1736.28</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="75" spans="1:12">
@@ -3497,34 +3500,34 @@
         <v>91</v>
       </c>
       <c r="C75" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D75">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="E75">
-        <v>4257145</v>
+        <v>581012</v>
       </c>
       <c r="F75">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="G75">
+        <v>54</v>
+      </c>
+      <c r="H75">
+        <v>1</v>
+      </c>
+      <c r="I75">
         <v>0</v>
       </c>
-      <c r="H75">
-        <v>4</v>
-      </c>
-      <c r="I75">
-        <v>6</v>
-      </c>
       <c r="J75">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K75" t="s">
         <v>100</v>
       </c>
       <c r="L75">
-        <v>287.3467</v>
+        <v>255.65</v>
       </c>
     </row>
     <row r="76" spans="1:12">
@@ -3535,34 +3538,34 @@
         <v>91</v>
       </c>
       <c r="C76" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D76">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="E76">
-        <v>4247264</v>
+        <v>1000</v>
       </c>
       <c r="F76">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G76">
+        <v>5</v>
+      </c>
+      <c r="H76">
+        <v>1</v>
+      </c>
+      <c r="I76">
         <v>0</v>
       </c>
-      <c r="H76">
-        <v>7</v>
-      </c>
-      <c r="I76">
-        <v>10</v>
-      </c>
       <c r="J76">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K76" t="s">
         <v>100</v>
       </c>
       <c r="L76">
-        <v>246.836575</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="77" spans="1:12">
@@ -3573,34 +3576,34 @@
         <v>91</v>
       </c>
       <c r="C77" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D77">
-        <v>140</v>
+        <v>27</v>
       </c>
       <c r="E77">
-        <v>5434924</v>
+        <v>20000</v>
       </c>
       <c r="F77">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="G77">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H77">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="I77">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J77">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K77" t="s">
         <v>100</v>
       </c>
       <c r="L77">
-        <v>372.106</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="78" spans="1:12">
@@ -3611,34 +3614,34 @@
         <v>91</v>
       </c>
       <c r="C78" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D78">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="E78">
-        <v>1018324</v>
+        <v>494021</v>
       </c>
       <c r="F78">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G78">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="H78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K78" t="s">
         <v>100</v>
       </c>
       <c r="L78">
-        <v>73.33</v>
+        <v>162.04</v>
       </c>
     </row>
     <row r="79" spans="1:12">
@@ -3649,34 +3652,34 @@
         <v>91</v>
       </c>
       <c r="C79" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D79">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="E79">
-        <v>429805</v>
+        <v>39644</v>
       </c>
       <c r="F79">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G79">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="H79">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I79">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J79">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K79" t="s">
         <v>100</v>
       </c>
       <c r="L79">
-        <v>14.64</v>
+        <v>18.71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_07_02_2026) - Modality: multi_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -52,6 +52,33 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>adult</t>
+  </si>
+  <si>
+    <t>alarm</t>
+  </si>
+  <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
+    <t>covtype</t>
+  </si>
+  <si>
+    <t>expedia_hotel_logs</t>
+  </si>
+  <si>
+    <t>insurance</t>
+  </si>
+  <si>
+    <t>intrusion</t>
+  </si>
+  <si>
+    <t>news</t>
+  </si>
+  <si>
     <t>Accidents</t>
   </si>
   <si>
@@ -259,61 +286,34 @@
     <t>walmart</t>
   </si>
   <si>
-    <t>adult</t>
-  </si>
-  <si>
-    <t>alarm</t>
-  </si>
-  <si>
-    <t>census</t>
-  </si>
-  <si>
-    <t>child</t>
-  </si>
-  <si>
-    <t>covtype</t>
-  </si>
-  <si>
-    <t>expedia_hotel_logs</t>
-  </si>
-  <si>
-    <t>insurance</t>
-  </si>
-  <si>
-    <t>intrusion</t>
-  </si>
-  <si>
-    <t>news</t>
+    <t>single_table</t>
   </si>
   <si>
     <t>multi_table</t>
   </si>
   <si>
-    <t>single_table</t>
+    <t>RealTabFormerSynthesizer</t>
+  </si>
+  <si>
+    <t>TVAESynthesizer</t>
+  </si>
+  <si>
+    <t>GaussianCopulaSynthesizer</t>
+  </si>
+  <si>
+    <t>SegmentSynthesizer</t>
   </si>
   <si>
     <t>HSASynthesizer</t>
   </si>
   <si>
+    <t>HMASynthesizer</t>
+  </si>
+  <si>
     <t>IndependentSynthesizer</t>
   </si>
   <si>
-    <t>HMASynthesizer</t>
-  </si>
-  <si>
     <t>MultiTableUniformSynthesizer</t>
-  </si>
-  <si>
-    <t>RealTabFormerSynthesizer</t>
-  </si>
-  <si>
-    <t>TVAESynthesizer</t>
-  </si>
-  <si>
-    <t>GaussianCopulaSynthesizer</t>
-  </si>
-  <si>
-    <t>SegmentSynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -729,31 +729,31 @@
         <v>92</v>
       </c>
       <c r="D2">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="E2">
-        <v>1463093</v>
+        <v>32561</v>
       </c>
       <c r="F2">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2" t="s">
         <v>100</v>
       </c>
       <c r="L2">
-        <v>219.33</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -767,31 +767,31 @@
         <v>93</v>
       </c>
       <c r="D3">
-        <v>198</v>
+        <v>37</v>
       </c>
       <c r="E3">
-        <v>12781</v>
+        <v>20000</v>
       </c>
       <c r="F3">
+        <v>37</v>
+      </c>
+      <c r="G3">
         <v>0</v>
       </c>
-      <c r="G3">
-        <v>193</v>
-      </c>
       <c r="H3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" t="s">
         <v>100</v>
       </c>
       <c r="L3">
-        <v>6.62</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -805,31 +805,31 @@
         <v>92</v>
       </c>
       <c r="D4">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="E4">
-        <v>139179</v>
+        <v>299285</v>
       </c>
       <c r="F4">
+        <v>29</v>
+      </c>
+      <c r="G4">
         <v>12</v>
       </c>
-      <c r="G4">
-        <v>57</v>
-      </c>
       <c r="H4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4" t="s">
         <v>100</v>
       </c>
       <c r="L4">
-        <v>31.18</v>
+        <v>98.17</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -840,34 +840,34 @@
         <v>90</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D5">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E5">
-        <v>21895</v>
+        <v>20000</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K5" t="s">
         <v>100</v>
       </c>
       <c r="L5">
-        <v>0.57</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -881,31 +881,31 @@
         <v>93</v>
       </c>
       <c r="D6">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="E6">
-        <v>2762</v>
+        <v>581012</v>
       </c>
       <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>54</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
         <v>0</v>
       </c>
-      <c r="G6">
-        <v>7</v>
-      </c>
-      <c r="H6">
-        <v>9</v>
-      </c>
-      <c r="I6">
-        <v>8</v>
-      </c>
       <c r="J6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" t="s">
         <v>100</v>
       </c>
       <c r="L6">
-        <v>0.04</v>
+        <v>255.65</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -916,34 +916,34 @@
         <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D7">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E7">
-        <v>57353</v>
+        <v>1000</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" t="s">
         <v>100</v>
       </c>
       <c r="L7">
-        <v>1.79</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -954,34 +954,34 @@
         <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D8">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E8">
-        <v>27443</v>
+        <v>20000</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="G8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K8" t="s">
         <v>100</v>
       </c>
       <c r="L8">
-        <v>0.9399999999999999</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -995,31 +995,31 @@
         <v>92</v>
       </c>
       <c r="D9">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E9">
-        <v>2052</v>
+        <v>494021</v>
       </c>
       <c r="F9">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" t="s">
         <v>100</v>
       </c>
       <c r="L9">
-        <v>0.25</v>
+        <v>162.04</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -1033,31 +1033,31 @@
         <v>92</v>
       </c>
       <c r="D10">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E10">
-        <v>22318</v>
+        <v>39644</v>
       </c>
       <c r="F10">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="H10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" t="s">
         <v>100</v>
       </c>
       <c r="L10">
-        <v>9.93</v>
+        <v>18.71</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1065,37 +1065,37 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C11" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D11">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="E11">
-        <v>8258</v>
+        <v>1463093</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K11" t="s">
         <v>100</v>
       </c>
       <c r="L11">
-        <v>0.25</v>
+        <v>219.33</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1103,37 +1103,37 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C12" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D12">
-        <v>50</v>
+        <v>198</v>
       </c>
       <c r="E12">
-        <v>440</v>
+        <v>12781</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="H12">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I12">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="J12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K12" t="s">
         <v>100</v>
       </c>
       <c r="L12">
-        <v>0.01</v>
+        <v>6.62</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1141,37 +1141,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C13" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D13">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="E13">
-        <v>1352</v>
+        <v>139179</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="H13">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="I13">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="J13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13" t="s">
         <v>100</v>
       </c>
       <c r="L13">
-        <v>0.05</v>
+        <v>31.18</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1179,37 +1179,37 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C14" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D14">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="E14">
-        <v>2113275</v>
+        <v>21895</v>
       </c>
       <c r="F14">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G14">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" t="s">
         <v>100</v>
       </c>
       <c r="L14">
-        <v>120</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1217,28 +1217,28 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D15">
-        <v>266</v>
+        <v>17</v>
       </c>
       <c r="E15">
-        <v>10173</v>
+        <v>2762</v>
       </c>
       <c r="F15">
-        <v>262</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J15">
         <v>2</v>
@@ -1247,7 +1247,7 @@
         <v>100</v>
       </c>
       <c r="L15">
-        <v>1.38</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1255,28 +1255,28 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D16">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E16">
-        <v>12927</v>
+        <v>57353</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
       <c r="G16">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I16">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J16">
         <v>2</v>
@@ -1285,7 +1285,7 @@
         <v>100</v>
       </c>
       <c r="L16">
-        <v>0.68</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1293,37 +1293,37 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C17" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D17">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="E17">
-        <v>2700</v>
+        <v>27443</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G17">
         <v>2</v>
       </c>
       <c r="H17">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="I17">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="J17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17" t="s">
         <v>100</v>
       </c>
       <c r="L17">
-        <v>0.04</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1331,37 +1331,37 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D18">
-        <v>202</v>
+        <v>46</v>
       </c>
       <c r="E18">
-        <v>4425</v>
+        <v>2052</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H18">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="I18">
-        <v>189</v>
+        <v>1</v>
       </c>
       <c r="J18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K18" t="s">
         <v>100</v>
       </c>
       <c r="L18">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1369,28 +1369,28 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C19" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D19">
-        <v>170</v>
+        <v>68</v>
       </c>
       <c r="E19">
-        <v>568</v>
+        <v>22318</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G19">
-        <v>167</v>
+        <v>53</v>
       </c>
       <c r="H19">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J19">
         <v>2</v>
@@ -1399,7 +1399,7 @@
         <v>100</v>
       </c>
       <c r="L19">
-        <v>0.64</v>
+        <v>9.93</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1407,37 +1407,37 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C20" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D20">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E20">
-        <v>1219</v>
+        <v>8258</v>
       </c>
       <c r="F20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G20">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="H20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I20">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K20" t="s">
         <v>100</v>
       </c>
       <c r="L20">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1445,28 +1445,28 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C21" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D21">
-        <v>112</v>
+        <v>50</v>
       </c>
       <c r="E21">
-        <v>202305</v>
+        <v>440</v>
       </c>
       <c r="F21">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G21">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="H21">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="I21">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="J21">
         <v>3</v>
@@ -1475,7 +1475,7 @@
         <v>100</v>
       </c>
       <c r="L21">
-        <v>27.15</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1483,37 +1483,37 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C22" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D22">
-        <v>432</v>
+        <v>32</v>
       </c>
       <c r="E22">
-        <v>39000</v>
+        <v>1352</v>
       </c>
       <c r="F22">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="G22">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="I22">
-        <v>171</v>
+        <v>20</v>
       </c>
       <c r="J22">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K22" t="s">
         <v>100</v>
       </c>
       <c r="L22">
-        <v>3.45</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1521,37 +1521,37 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C23" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D23">
-        <v>97</v>
+        <v>26</v>
       </c>
       <c r="E23">
-        <v>29850</v>
+        <v>2113275</v>
       </c>
       <c r="F23">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G23">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H23">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="I23">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="J23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K23" t="s">
         <v>100</v>
       </c>
       <c r="L23">
-        <v>0.95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1559,28 +1559,28 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C24" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D24">
-        <v>18</v>
+        <v>266</v>
       </c>
       <c r="E24">
-        <v>6912</v>
+        <v>10173</v>
       </c>
       <c r="F24">
-        <v>1</v>
+        <v>262</v>
       </c>
       <c r="G24">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H24">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I24">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J24">
         <v>2</v>
@@ -1589,7 +1589,7 @@
         <v>100</v>
       </c>
       <c r="L24">
-        <v>0.11</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1597,37 +1597,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C25" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D25">
-        <v>218</v>
+        <v>29</v>
       </c>
       <c r="E25">
-        <v>11308</v>
+        <v>12927</v>
       </c>
       <c r="F25">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G25">
-        <v>204</v>
+        <v>14</v>
       </c>
       <c r="H25">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K25" t="s">
         <v>100</v>
       </c>
       <c r="L25">
-        <v>17.2</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1635,28 +1635,28 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C26" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D26">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="E26">
-        <v>296</v>
+        <v>2700</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="J26">
         <v>2</v>
@@ -1665,7 +1665,7 @@
         <v>100</v>
       </c>
       <c r="L26">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1673,28 +1673,28 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C27" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D27">
-        <v>42</v>
+        <v>202</v>
       </c>
       <c r="E27">
-        <v>3841029</v>
+        <v>4425</v>
       </c>
       <c r="F27">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="H27">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="I27">
-        <v>3</v>
+        <v>189</v>
       </c>
       <c r="J27">
         <v>3</v>
@@ -1703,7 +1703,7 @@
         <v>100</v>
       </c>
       <c r="L27">
-        <v>148.44</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1711,28 +1711,28 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C28" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D28">
-        <v>70</v>
+        <v>170</v>
       </c>
       <c r="E28">
-        <v>19867</v>
+        <v>568</v>
       </c>
       <c r="F28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="H28">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="I28">
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="J28">
         <v>2</v>
@@ -1741,7 +1741,7 @@
         <v>100</v>
       </c>
       <c r="L28">
-        <v>0.32</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1749,37 +1749,37 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C29" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D29">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E29">
-        <v>6735507</v>
+        <v>1219</v>
       </c>
       <c r="F29">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G29">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="H29">
         <v>4</v>
       </c>
       <c r="I29">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K29" t="s">
         <v>100</v>
       </c>
       <c r="L29">
-        <v>269.25</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1787,37 +1787,37 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C30" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D30">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="E30">
-        <v>1536</v>
+        <v>202305</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H30">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I30">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="J30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K30" t="s">
         <v>100</v>
       </c>
       <c r="L30">
-        <v>0.04</v>
+        <v>27.15</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1825,37 +1825,37 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C31" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D31">
-        <v>16</v>
+        <v>432</v>
       </c>
       <c r="E31">
-        <v>5288</v>
+        <v>39000</v>
       </c>
       <c r="F31">
-        <v>2</v>
+        <v>108</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="H31">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="I31">
+        <v>171</v>
+      </c>
+      <c r="J31">
         <v>9</v>
       </c>
-      <c r="J31">
-        <v>2</v>
-      </c>
       <c r="K31" t="s">
         <v>100</v>
       </c>
       <c r="L31">
-        <v>0.09</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1863,28 +1863,28 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C32" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D32">
-        <v>12</v>
+        <v>97</v>
       </c>
       <c r="E32">
-        <v>36922</v>
+        <v>29850</v>
       </c>
       <c r="F32">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H32">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="I32">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="J32">
         <v>3</v>
@@ -1893,7 +1893,7 @@
         <v>100</v>
       </c>
       <c r="L32">
-        <v>1.03</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1901,28 +1901,28 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C33" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D33">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E33">
-        <v>1302</v>
+        <v>6912</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I33">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J33">
         <v>2</v>
@@ -1931,7 +1931,7 @@
         <v>100</v>
       </c>
       <c r="L33">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1939,28 +1939,28 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C34" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D34">
-        <v>192</v>
+        <v>218</v>
       </c>
       <c r="E34">
-        <v>154899</v>
+        <v>11308</v>
       </c>
       <c r="F34">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="G34">
-        <v>92</v>
+        <v>204</v>
       </c>
       <c r="H34">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="I34">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="J34">
         <v>3</v>
@@ -1969,7 +1969,7 @@
         <v>100</v>
       </c>
       <c r="L34">
-        <v>9.67</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1977,22 +1977,22 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C35" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D35">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E35">
-        <v>2735</v>
+        <v>296</v>
       </c>
       <c r="F35">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G35">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H35">
         <v>2</v>
@@ -2007,7 +2007,7 @@
         <v>100</v>
       </c>
       <c r="L35">
-        <v>0.11</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -2015,37 +2015,37 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C36" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D36">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="E36">
-        <v>712</v>
+        <v>3841029</v>
       </c>
       <c r="F36">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G36">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="H36">
         <v>4</v>
       </c>
       <c r="I36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K36" t="s">
         <v>100</v>
       </c>
       <c r="L36">
-        <v>0.02</v>
+        <v>148.44</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -2053,28 +2053,28 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C37" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D37">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="E37">
-        <v>81850</v>
+        <v>19867</v>
       </c>
       <c r="F37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G37">
         <v>0</v>
       </c>
       <c r="H37">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="I37">
-        <v>3</v>
+        <v>65</v>
       </c>
       <c r="J37">
         <v>2</v>
@@ -2083,7 +2083,7 @@
         <v>100</v>
       </c>
       <c r="L37">
-        <v>1.96</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2091,28 +2091,28 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C38" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D38">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E38">
-        <v>5751408</v>
+        <v>6735507</v>
       </c>
       <c r="F38">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G38">
         <v>2</v>
       </c>
       <c r="H38">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I38">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J38">
         <v>2</v>
@@ -2121,7 +2121,7 @@
         <v>100</v>
       </c>
       <c r="L38">
-        <v>293.14</v>
+        <v>269.25</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2129,28 +2129,28 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C39" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D39">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E39">
-        <v>668</v>
+        <v>1536</v>
       </c>
       <c r="F39">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G39">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H39">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I39">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J39">
         <v>2</v>
@@ -2159,7 +2159,7 @@
         <v>100</v>
       </c>
       <c r="L39">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2167,28 +2167,28 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C40" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D40">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E40">
-        <v>668</v>
+        <v>5288</v>
       </c>
       <c r="F40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H40">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I40">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J40">
         <v>2</v>
@@ -2197,7 +2197,7 @@
         <v>100</v>
       </c>
       <c r="L40">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2205,37 +2205,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C41" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D41">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="E41">
-        <v>1079680</v>
+        <v>36922</v>
       </c>
       <c r="F41">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G41">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H41">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I41">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J41">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K41" t="s">
         <v>100</v>
       </c>
       <c r="L41">
-        <v>85.38</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2243,22 +2243,22 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C42" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D42">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E42">
-        <v>96491</v>
+        <v>1302</v>
       </c>
       <c r="F42">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -2273,7 +2273,7 @@
         <v>100</v>
       </c>
       <c r="L42">
-        <v>4.68</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2281,37 +2281,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C43" t="s">
+        <v>98</v>
+      </c>
+      <c r="D43">
+        <v>192</v>
+      </c>
+      <c r="E43">
+        <v>154899</v>
+      </c>
+      <c r="F43">
+        <v>54</v>
+      </c>
+      <c r="G43">
         <v>92</v>
       </c>
-      <c r="D43">
-        <v>16</v>
-      </c>
-      <c r="E43">
-        <v>6118</v>
-      </c>
-      <c r="F43">
-        <v>9</v>
-      </c>
-      <c r="G43">
-        <v>2</v>
-      </c>
       <c r="H43">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="I43">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="J43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K43" t="s">
         <v>100</v>
       </c>
       <c r="L43">
-        <v>0.36</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2319,28 +2319,28 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C44" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D44">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E44">
-        <v>23</v>
+        <v>2735</v>
       </c>
       <c r="F44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G44">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H44">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I44">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J44">
         <v>2</v>
@@ -2349,7 +2349,7 @@
         <v>100</v>
       </c>
       <c r="L44">
-        <v>0</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2357,28 +2357,28 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C45" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D45">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="E45">
-        <v>1249411</v>
+        <v>712</v>
       </c>
       <c r="F45">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G45">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H45">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I45">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J45">
         <v>2</v>
@@ -2387,7 +2387,7 @@
         <v>100</v>
       </c>
       <c r="L45">
-        <v>39.2</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2395,28 +2395,28 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C46" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D46">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="E46">
-        <v>5647694</v>
+        <v>81850</v>
       </c>
       <c r="F46">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G46">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H46">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I46">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J46">
         <v>2</v>
@@ -2425,7 +2425,7 @@
         <v>100</v>
       </c>
       <c r="L46">
-        <v>173.9</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2433,28 +2433,28 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C47" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D47">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E47">
-        <v>4395</v>
+        <v>5751408</v>
       </c>
       <c r="F47">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G47">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H47">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I47">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J47">
         <v>2</v>
@@ -2463,7 +2463,7 @@
         <v>100</v>
       </c>
       <c r="L47">
-        <v>0.15</v>
+        <v>293.14</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2471,28 +2471,28 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C48" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D48">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E48">
-        <v>1754397</v>
+        <v>668</v>
       </c>
       <c r="F48">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="G48">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H48">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I48">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J48">
         <v>2</v>
@@ -2501,7 +2501,7 @@
         <v>100</v>
       </c>
       <c r="L48">
-        <v>130.3</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2509,37 +2509,37 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C49" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D49">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E49">
-        <v>11150</v>
+        <v>668</v>
       </c>
       <c r="F49">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G49">
         <v>3</v>
       </c>
       <c r="H49">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I49">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K49" t="s">
         <v>100</v>
       </c>
       <c r="L49">
-        <v>0.6928000000000001</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2547,37 +2547,37 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C50" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D50">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="E50">
-        <v>10324</v>
+        <v>1079680</v>
       </c>
       <c r="F50">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="G50">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="H50">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I50">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J50">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K50" t="s">
         <v>100</v>
       </c>
       <c r="L50">
-        <v>0.37</v>
+        <v>85.38</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2585,28 +2585,28 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C51" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D51">
-        <v>119</v>
+        <v>11</v>
       </c>
       <c r="E51">
-        <v>11004</v>
+        <v>96491</v>
       </c>
       <c r="F51">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G51">
-        <v>112</v>
+        <v>1</v>
       </c>
       <c r="H51">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I51">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J51">
         <v>2</v>
@@ -2615,7 +2615,7 @@
         <v>100</v>
       </c>
       <c r="L51">
-        <v>0.45</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2623,19 +2623,19 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C52" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D52">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E52">
-        <v>19297</v>
+        <v>6118</v>
       </c>
       <c r="F52">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G52">
         <v>2</v>
@@ -2647,13 +2647,13 @@
         <v>3</v>
       </c>
       <c r="J52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K52" t="s">
         <v>100</v>
       </c>
       <c r="L52">
-        <v>0.6899999999999999</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2661,28 +2661,28 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C53" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D53">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E53">
-        <v>83</v>
+        <v>23</v>
       </c>
       <c r="F53">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G53">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I53">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J53">
         <v>2</v>
@@ -2691,7 +2691,7 @@
         <v>100</v>
       </c>
       <c r="L53">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2699,28 +2699,28 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C54" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D54">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E54">
-        <v>171</v>
+        <v>1249411</v>
       </c>
       <c r="F54">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G54">
         <v>9</v>
       </c>
       <c r="H54">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I54">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J54">
         <v>2</v>
@@ -2729,7 +2729,7 @@
         <v>100</v>
       </c>
       <c r="L54">
-        <v>0.01</v>
+        <v>39.2</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2737,28 +2737,28 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C55" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D55">
         <v>25</v>
       </c>
       <c r="E55">
-        <v>5302</v>
+        <v>5647694</v>
       </c>
       <c r="F55">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G55">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H55">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I55">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J55">
         <v>2</v>
@@ -2767,7 +2767,7 @@
         <v>100</v>
       </c>
       <c r="L55">
-        <v>0.23</v>
+        <v>173.9</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2775,37 +2775,37 @@
         <v>66</v>
       </c>
       <c r="B56" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C56" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D56">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="E56">
-        <v>32231279</v>
+        <v>4395</v>
       </c>
       <c r="F56">
+        <v>9</v>
+      </c>
+      <c r="G56">
         <v>4</v>
       </c>
-      <c r="G56">
-        <v>2</v>
-      </c>
       <c r="H56">
+        <v>7</v>
+      </c>
+      <c r="I56">
         <v>6</v>
       </c>
-      <c r="I56">
-        <v>5</v>
-      </c>
       <c r="J56">
         <v>2</v>
       </c>
       <c r="K56" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L56">
-        <v>937.268</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2813,37 +2813,37 @@
         <v>67</v>
       </c>
       <c r="B57" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C57" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D57">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E57">
-        <v>148021</v>
+        <v>1754397</v>
       </c>
       <c r="F57">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="G57">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H57">
         <v>5</v>
       </c>
       <c r="I57">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J57">
         <v>2</v>
       </c>
       <c r="K57" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L57">
-        <v>3.87</v>
+        <v>130.3</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2851,37 +2851,37 @@
         <v>68</v>
       </c>
       <c r="B58" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C58" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D58">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E58">
-        <v>173933</v>
+        <v>11150</v>
       </c>
       <c r="F58">
         <v>4</v>
       </c>
       <c r="G58">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H58">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J58">
         <v>3</v>
       </c>
       <c r="K58" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L58">
-        <v>8.081517</v>
+        <v>0.6928000000000001</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2889,37 +2889,37 @@
         <v>69</v>
       </c>
       <c r="B59" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C59" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D59">
         <v>15</v>
       </c>
       <c r="E59">
-        <v>15000713</v>
+        <v>10324</v>
       </c>
       <c r="F59">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G59">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H59">
         <v>3</v>
       </c>
       <c r="I59">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J59">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K59" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L59">
-        <v>650.54</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2927,37 +2927,37 @@
         <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C60" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D60">
-        <v>21</v>
+        <v>119</v>
       </c>
       <c r="E60">
-        <v>2146112</v>
+        <v>11004</v>
       </c>
       <c r="F60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G60">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="H60">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I60">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J60">
         <v>2</v>
       </c>
       <c r="K60" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L60">
-        <v>61.659</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2965,37 +2965,37 @@
         <v>71</v>
       </c>
       <c r="B61" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C61" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D61">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E61">
-        <v>20679117</v>
+        <v>19297</v>
       </c>
       <c r="F61">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G61">
         <v>2</v>
       </c>
       <c r="H61">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I61">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="J61">
         <v>3</v>
       </c>
       <c r="K61" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L61">
-        <v>1043.242</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -3003,37 +3003,37 @@
         <v>72</v>
       </c>
       <c r="B62" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C62" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D62">
-        <v>129</v>
+        <v>13</v>
       </c>
       <c r="E62">
-        <v>41328337</v>
+        <v>83</v>
       </c>
       <c r="F62">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G62">
-        <v>102</v>
+        <v>4</v>
       </c>
       <c r="H62">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I62">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K62" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L62">
-        <v>3005.995</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -3041,37 +3041,37 @@
         <v>73</v>
       </c>
       <c r="B63" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C63" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D63">
-        <v>67</v>
+        <v>19</v>
       </c>
       <c r="E63">
-        <v>74063</v>
+        <v>171</v>
       </c>
       <c r="F63">
+        <v>1</v>
+      </c>
+      <c r="G63">
+        <v>9</v>
+      </c>
+      <c r="H63">
+        <v>5</v>
+      </c>
+      <c r="I63">
         <v>4</v>
       </c>
-      <c r="G63">
-        <v>21</v>
-      </c>
-      <c r="H63">
-        <v>9</v>
-      </c>
-      <c r="I63">
-        <v>13</v>
-      </c>
       <c r="J63">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K63" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L63">
-        <v>5.537</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3079,22 +3079,22 @@
         <v>74</v>
       </c>
       <c r="B64" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C64" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D64">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="E64">
-        <v>16664809</v>
+        <v>5302</v>
       </c>
       <c r="F64">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H64">
         <v>3</v>
@@ -3106,10 +3106,10 @@
         <v>2</v>
       </c>
       <c r="K64" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L64">
-        <v>737.283</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="65" spans="1:12">
@@ -3117,37 +3117,37 @@
         <v>75</v>
       </c>
       <c r="B65" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C65" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D65">
-        <v>221</v>
+        <v>19</v>
       </c>
       <c r="E65">
-        <v>13787005</v>
+        <v>32231279</v>
       </c>
       <c r="F65">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="G65">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="H65">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="I65">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="J65">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K65" t="s">
         <v>101</v>
       </c>
       <c r="L65">
-        <v>1736.28</v>
+        <v>937.268</v>
       </c>
     </row>
     <row r="66" spans="1:12">
@@ -3155,37 +3155,37 @@
         <v>76</v>
       </c>
       <c r="B66" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C66" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D66">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="E66">
-        <v>4257145</v>
+        <v>148021</v>
       </c>
       <c r="F66">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="G66">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H66">
+        <v>5</v>
+      </c>
+      <c r="I66">
         <v>4</v>
       </c>
-      <c r="I66">
-        <v>6</v>
-      </c>
       <c r="J66">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K66" t="s">
         <v>101</v>
       </c>
       <c r="L66">
-        <v>287.3467</v>
+        <v>3.87</v>
       </c>
     </row>
     <row r="67" spans="1:12">
@@ -3193,28 +3193,28 @@
         <v>77</v>
       </c>
       <c r="B67" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C67" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D67">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="E67">
-        <v>4247264</v>
+        <v>173933</v>
       </c>
       <c r="F67">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G67">
         <v>0</v>
       </c>
       <c r="H67">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I67">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J67">
         <v>3</v>
@@ -3223,7 +3223,7 @@
         <v>101</v>
       </c>
       <c r="L67">
-        <v>246.836575</v>
+        <v>8.081517</v>
       </c>
     </row>
     <row r="68" spans="1:12">
@@ -3231,37 +3231,37 @@
         <v>78</v>
       </c>
       <c r="B68" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C68" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D68">
-        <v>140</v>
+        <v>15</v>
       </c>
       <c r="E68">
-        <v>5434924</v>
+        <v>15000713</v>
       </c>
       <c r="F68">
-        <v>51</v>
+        <v>4</v>
       </c>
       <c r="G68">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="H68">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="I68">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="J68">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K68" t="s">
         <v>101</v>
       </c>
       <c r="L68">
-        <v>372.106</v>
+        <v>650.54</v>
       </c>
     </row>
     <row r="69" spans="1:12">
@@ -3269,28 +3269,28 @@
         <v>79</v>
       </c>
       <c r="B69" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C69" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D69">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E69">
-        <v>1018324</v>
+        <v>2146112</v>
       </c>
       <c r="F69">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G69">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H69">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I69">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J69">
         <v>2</v>
@@ -3299,7 +3299,7 @@
         <v>101</v>
       </c>
       <c r="L69">
-        <v>73.33</v>
+        <v>61.659</v>
       </c>
     </row>
     <row r="70" spans="1:12">
@@ -3307,37 +3307,37 @@
         <v>80</v>
       </c>
       <c r="B70" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C70" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D70">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="E70">
-        <v>429805</v>
+        <v>20679117</v>
       </c>
       <c r="F70">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G70">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H70">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I70">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="J70">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K70" t="s">
         <v>101</v>
       </c>
       <c r="L70">
-        <v>14.64</v>
+        <v>1043.242</v>
       </c>
     </row>
     <row r="71" spans="1:12">
@@ -3348,34 +3348,34 @@
         <v>91</v>
       </c>
       <c r="C71" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D71">
-        <v>15</v>
+        <v>129</v>
       </c>
       <c r="E71">
-        <v>32561</v>
+        <v>41328337</v>
       </c>
       <c r="F71">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G71">
-        <v>6</v>
+        <v>102</v>
       </c>
       <c r="H71">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I71">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J71">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K71" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L71">
-        <v>3.91</v>
+        <v>3005.995</v>
       </c>
     </row>
     <row r="72" spans="1:12">
@@ -3386,34 +3386,34 @@
         <v>91</v>
       </c>
       <c r="C72" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D72">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="E72">
-        <v>20000</v>
+        <v>74063</v>
       </c>
       <c r="F72">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="G72">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H72">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I72">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J72">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K72" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L72">
-        <v>4.52</v>
+        <v>5.537</v>
       </c>
     </row>
     <row r="73" spans="1:12">
@@ -3424,34 +3424,34 @@
         <v>91</v>
       </c>
       <c r="C73" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D73">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E73">
-        <v>299285</v>
+        <v>16664809</v>
       </c>
       <c r="F73">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G73">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H73">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I73">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K73" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L73">
-        <v>98.17</v>
+        <v>737.283</v>
       </c>
     </row>
     <row r="74" spans="1:12">
@@ -3465,31 +3465,31 @@
         <v>97</v>
       </c>
       <c r="D74">
-        <v>20</v>
+        <v>221</v>
       </c>
       <c r="E74">
-        <v>20000</v>
+        <v>13787005</v>
       </c>
       <c r="F74">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="G74">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="H74">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="I74">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="J74">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K74" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L74">
-        <v>3.2</v>
+        <v>1736.28</v>
       </c>
     </row>
     <row r="75" spans="1:12">
@@ -3500,34 +3500,34 @@
         <v>91</v>
       </c>
       <c r="C75" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D75">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="E75">
-        <v>581012</v>
+        <v>4257145</v>
       </c>
       <c r="F75">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="G75">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="H75">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I75">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J75">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K75" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L75">
-        <v>255.65</v>
+        <v>287.3467</v>
       </c>
     </row>
     <row r="76" spans="1:12">
@@ -3538,34 +3538,34 @@
         <v>91</v>
       </c>
       <c r="C76" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D76">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="E76">
-        <v>1000</v>
+        <v>4247264</v>
       </c>
       <c r="F76">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G76">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H76">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I76">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J76">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K76" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L76">
-        <v>0.2</v>
+        <v>246.836575</v>
       </c>
     </row>
     <row r="77" spans="1:12">
@@ -3576,34 +3576,34 @@
         <v>91</v>
       </c>
       <c r="C77" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D77">
-        <v>27</v>
+        <v>140</v>
       </c>
       <c r="E77">
-        <v>20000</v>
+        <v>5434924</v>
       </c>
       <c r="F77">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="G77">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H77">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="I77">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J77">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K77" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L77">
-        <v>3.34</v>
+        <v>372.106</v>
       </c>
     </row>
     <row r="78" spans="1:12">
@@ -3614,34 +3614,34 @@
         <v>91</v>
       </c>
       <c r="C78" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D78">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="E78">
-        <v>494021</v>
+        <v>1018324</v>
       </c>
       <c r="F78">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G78">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="H78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K78" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L78">
-        <v>162.04</v>
+        <v>73.33</v>
       </c>
     </row>
     <row r="79" spans="1:12">
@@ -3652,34 +3652,34 @@
         <v>91</v>
       </c>
       <c r="C79" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D79">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="E79">
-        <v>39644</v>
+        <v>429805</v>
       </c>
       <c r="F79">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G79">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="H79">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I79">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K79" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L79">
-        <v>18.71</v>
+        <v>14.64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_08_01_2026) - Modality: single_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="101">
   <si>
     <t>Dataset</t>
   </si>
@@ -52,6 +52,213 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>Accidents</t>
+  </si>
+  <si>
+    <t>Atherosclerosis</t>
+  </si>
+  <si>
+    <t>AustralianFootball</t>
+  </si>
+  <si>
+    <t>Biodegradability</t>
+  </si>
+  <si>
+    <t>Bupa</t>
+  </si>
+  <si>
+    <t>CORA</t>
+  </si>
+  <si>
+    <t>Carcinogenesis</t>
+  </si>
+  <si>
+    <t>Chess</t>
+  </si>
+  <si>
+    <t>Countries</t>
+  </si>
+  <si>
+    <t>DCG</t>
+  </si>
+  <si>
+    <t>Dunur</t>
+  </si>
+  <si>
+    <t>Elti</t>
+  </si>
+  <si>
+    <t>FNHK</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>Hepatitis_std</t>
+  </si>
+  <si>
+    <t>Mesh</t>
+  </si>
+  <si>
+    <t>Mooney_Family</t>
+  </si>
+  <si>
+    <t>MuskSmall</t>
+  </si>
+  <si>
+    <t>NBA</t>
+  </si>
+  <si>
+    <t>NCAA</t>
+  </si>
+  <si>
+    <t>OMOP_CDM_dayz</t>
+  </si>
+  <si>
+    <t>PTE</t>
+  </si>
+  <si>
+    <t>Pima</t>
+  </si>
+  <si>
+    <t>PremierLeague</t>
+  </si>
+  <si>
+    <t>Pyrimidine</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>SAT</t>
+  </si>
+  <si>
+    <t>SalesDB</t>
+  </si>
+  <si>
+    <t>Same_gen</t>
+  </si>
+  <si>
+    <t>Student_loan</t>
+  </si>
+  <si>
+    <t>Toxicology</t>
+  </si>
+  <si>
+    <t>Triazine</t>
+  </si>
+  <si>
+    <t>TubePricing</t>
+  </si>
+  <si>
+    <t>UTube</t>
+  </si>
+  <si>
+    <t>UW_std</t>
+  </si>
+  <si>
+    <t>WebKP</t>
+  </si>
+  <si>
+    <t>airbnb-simplified</t>
+  </si>
+  <si>
+    <t>fake_hotels</t>
+  </si>
+  <si>
+    <t>fake_hotels_extended</t>
+  </si>
+  <si>
+    <t>financial</t>
+  </si>
+  <si>
+    <t>ftp</t>
+  </si>
+  <si>
+    <t>genes</t>
+  </si>
+  <si>
+    <t>got_families</t>
+  </si>
+  <si>
+    <t>imdb_MovieLens</t>
+  </si>
+  <si>
+    <t>imdb_ijs</t>
+  </si>
+  <si>
+    <t>imdb_small</t>
+  </si>
+  <si>
+    <t>legalActs</t>
+  </si>
+  <si>
+    <t>multi_table_ID_demo_dataset</t>
+  </si>
+  <si>
+    <t>mutagenesis</t>
+  </si>
+  <si>
+    <t>nations</t>
+  </si>
+  <si>
+    <t>restbase</t>
+  </si>
+  <si>
+    <t>trains</t>
+  </si>
+  <si>
+    <t>university</t>
+  </si>
+  <si>
+    <t>world</t>
+  </si>
+  <si>
+    <t>MovieLens</t>
+  </si>
+  <si>
+    <t>Telstra</t>
+  </si>
+  <si>
+    <t>instacart_marketbasket_ml</t>
+  </si>
+  <si>
+    <t>rel-amazon</t>
+  </si>
+  <si>
+    <t>rel-arxiv</t>
+  </si>
+  <si>
+    <t>rel-avito</t>
+  </si>
+  <si>
+    <t>rel-event</t>
+  </si>
+  <si>
+    <t>rel-f1</t>
+  </si>
+  <si>
+    <t>rel-hm</t>
+  </si>
+  <si>
+    <t>rel-ratebeer</t>
+  </si>
+  <si>
+    <t>rel-salt</t>
+  </si>
+  <si>
+    <t>rel-stack</t>
+  </si>
+  <si>
+    <t>rel-trial</t>
+  </si>
+  <si>
+    <t>rossmann</t>
+  </si>
+  <si>
+    <t>walmart</t>
+  </si>
+  <si>
     <t>adult</t>
   </si>
   <si>
@@ -79,217 +286,22 @@
     <t>news</t>
   </si>
   <si>
-    <t>Accidents</t>
-  </si>
-  <si>
-    <t>Atherosclerosis</t>
-  </si>
-  <si>
-    <t>AustralianFootball</t>
-  </si>
-  <si>
-    <t>Biodegradability</t>
-  </si>
-  <si>
-    <t>Bupa</t>
-  </si>
-  <si>
-    <t>CORA</t>
-  </si>
-  <si>
-    <t>Carcinogenesis</t>
-  </si>
-  <si>
-    <t>Chess</t>
-  </si>
-  <si>
-    <t>Countries</t>
-  </si>
-  <si>
-    <t>DCG</t>
-  </si>
-  <si>
-    <t>Dunur</t>
-  </si>
-  <si>
-    <t>Elti</t>
-  </si>
-  <si>
-    <t>FNHK</t>
-  </si>
-  <si>
-    <t>Facebook</t>
-  </si>
-  <si>
-    <t>Hepatitis_std</t>
-  </si>
-  <si>
-    <t>Mesh</t>
-  </si>
-  <si>
-    <t>Mooney_Family</t>
-  </si>
-  <si>
-    <t>MuskSmall</t>
-  </si>
-  <si>
-    <t>NBA</t>
-  </si>
-  <si>
-    <t>NCAA</t>
-  </si>
-  <si>
-    <t>OMOP_CDM_dayz</t>
-  </si>
-  <si>
-    <t>PTE</t>
-  </si>
-  <si>
-    <t>Pima</t>
-  </si>
-  <si>
-    <t>PremierLeague</t>
-  </si>
-  <si>
-    <t>Pyrimidine</t>
-  </si>
-  <si>
-    <t>SAP</t>
-  </si>
-  <si>
-    <t>SAT</t>
-  </si>
-  <si>
-    <t>SalesDB</t>
-  </si>
-  <si>
-    <t>Same_gen</t>
-  </si>
-  <si>
-    <t>Student_loan</t>
-  </si>
-  <si>
-    <t>Toxicology</t>
-  </si>
-  <si>
-    <t>Triazine</t>
-  </si>
-  <si>
-    <t>TubePricing</t>
-  </si>
-  <si>
-    <t>UTube</t>
-  </si>
-  <si>
-    <t>UW_std</t>
-  </si>
-  <si>
-    <t>WebKP</t>
-  </si>
-  <si>
-    <t>airbnb-simplified</t>
-  </si>
-  <si>
-    <t>fake_hotels</t>
-  </si>
-  <si>
-    <t>fake_hotels_extended</t>
-  </si>
-  <si>
-    <t>financial</t>
-  </si>
-  <si>
-    <t>ftp</t>
-  </si>
-  <si>
-    <t>genes</t>
-  </si>
-  <si>
-    <t>got_families</t>
-  </si>
-  <si>
-    <t>imdb_MovieLens</t>
-  </si>
-  <si>
-    <t>imdb_ijs</t>
-  </si>
-  <si>
-    <t>imdb_small</t>
-  </si>
-  <si>
-    <t>legalActs</t>
-  </si>
-  <si>
-    <t>multi_table_ID_demo_dataset</t>
-  </si>
-  <si>
-    <t>mutagenesis</t>
-  </si>
-  <si>
-    <t>nations</t>
-  </si>
-  <si>
-    <t>restbase</t>
-  </si>
-  <si>
-    <t>trains</t>
-  </si>
-  <si>
-    <t>university</t>
-  </si>
-  <si>
-    <t>world</t>
-  </si>
-  <si>
-    <t>MovieLens</t>
-  </si>
-  <si>
-    <t>Telstra</t>
-  </si>
-  <si>
-    <t>instacart_marketbasket_ml</t>
-  </si>
-  <si>
-    <t>rel-amazon</t>
-  </si>
-  <si>
-    <t>rel-arxiv</t>
-  </si>
-  <si>
-    <t>rel-avito</t>
-  </si>
-  <si>
-    <t>rel-event</t>
-  </si>
-  <si>
-    <t>rel-f1</t>
-  </si>
-  <si>
-    <t>rel-hm</t>
-  </si>
-  <si>
-    <t>rel-ratebeer</t>
-  </si>
-  <si>
-    <t>rel-salt</t>
-  </si>
-  <si>
-    <t>rel-stack</t>
-  </si>
-  <si>
-    <t>rel-trial</t>
-  </si>
-  <si>
-    <t>rossmann</t>
-  </si>
-  <si>
-    <t>walmart</t>
+    <t>multi_table</t>
   </si>
   <si>
     <t>single_table</t>
   </si>
   <si>
-    <t>multi_table</t>
+    <t>HSASynthesizer</t>
+  </si>
+  <si>
+    <t>HMASynthesizer</t>
+  </si>
+  <si>
+    <t>IndependentSynthesizer</t>
+  </si>
+  <si>
+    <t>MultiTableUniformSynthesizer</t>
   </si>
   <si>
     <t>RealTabFormerSynthesizer</t>
@@ -299,21 +311,6 @@
   </si>
   <si>
     <t>GaussianCopulaSynthesizer</t>
-  </si>
-  <si>
-    <t>SegmentSynthesizer</t>
-  </si>
-  <si>
-    <t>HSASynthesizer</t>
-  </si>
-  <si>
-    <t>HMASynthesizer</t>
-  </si>
-  <si>
-    <t>IndependentSynthesizer</t>
-  </si>
-  <si>
-    <t>MultiTableUniformSynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -729,31 +726,31 @@
         <v>92</v>
       </c>
       <c r="D2">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="E2">
-        <v>32561</v>
+        <v>1463093</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="G2">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L2">
-        <v>3.91</v>
+        <v>219.33</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -764,34 +761,34 @@
         <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D3">
-        <v>37</v>
+        <v>198</v>
       </c>
       <c r="E3">
-        <v>20000</v>
+        <v>12781</v>
       </c>
       <c r="F3">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L3">
-        <v>4.52</v>
+        <v>6.62</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -805,31 +802,31 @@
         <v>92</v>
       </c>
       <c r="D4">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="E4">
-        <v>299285</v>
+        <v>139179</v>
       </c>
       <c r="F4">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="G4">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L4">
-        <v>98.17</v>
+        <v>31.18</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -843,31 +840,31 @@
         <v>93</v>
       </c>
       <c r="D5">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E5">
-        <v>20000</v>
+        <v>21895</v>
       </c>
       <c r="F5">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L5">
-        <v>3.2</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -878,34 +875,34 @@
         <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D6">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="E6">
-        <v>581012</v>
+        <v>2762</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>54</v>
+        <v>7</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L6">
-        <v>255.65</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -916,34 +913,34 @@
         <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D7">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E7">
-        <v>1000</v>
+        <v>57353</v>
       </c>
       <c r="F7">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L7">
-        <v>0.2</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -954,34 +951,34 @@
         <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D8">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E8">
-        <v>20000</v>
+        <v>27443</v>
       </c>
       <c r="F8">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L8">
-        <v>3.34</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -995,31 +992,31 @@
         <v>92</v>
       </c>
       <c r="D9">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="E9">
-        <v>494021</v>
+        <v>2052</v>
       </c>
       <c r="F9">
+        <v>39</v>
+      </c>
+      <c r="G9">
         <v>4</v>
       </c>
-      <c r="G9">
-        <v>37</v>
-      </c>
       <c r="H9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L9">
-        <v>162.04</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -1033,31 +1030,31 @@
         <v>92</v>
       </c>
       <c r="D10">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E10">
-        <v>39644</v>
+        <v>22318</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G10">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L10">
-        <v>18.71</v>
+        <v>9.93</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1065,37 +1062,37 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C11" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D11">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="E11">
-        <v>1463093</v>
+        <v>8258</v>
       </c>
       <c r="F11">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="G11">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="H11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L11">
-        <v>219.33</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1103,37 +1100,37 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C12" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D12">
-        <v>198</v>
+        <v>50</v>
       </c>
       <c r="E12">
-        <v>12781</v>
+        <v>440</v>
       </c>
       <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
         <v>0</v>
       </c>
-      <c r="G12">
-        <v>193</v>
-      </c>
       <c r="H12">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I12">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="J12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L12">
-        <v>6.62</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1141,37 +1138,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C13" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D13">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="E13">
-        <v>139179</v>
+        <v>1352</v>
       </c>
       <c r="F13">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I13">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="J13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L13">
-        <v>31.18</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1179,37 +1176,37 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C14" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D14">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="E14">
-        <v>21895</v>
+        <v>2113275</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G14">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I14">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L14">
-        <v>0.57</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1217,37 +1214,37 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C15" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D15">
-        <v>17</v>
+        <v>266</v>
       </c>
       <c r="E15">
-        <v>2762</v>
+        <v>10173</v>
       </c>
       <c r="F15">
+        <v>262</v>
+      </c>
+      <c r="G15">
         <v>0</v>
       </c>
-      <c r="G15">
-        <v>7</v>
-      </c>
       <c r="H15">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I15">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J15">
         <v>2</v>
       </c>
       <c r="K15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L15">
-        <v>0.04</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1255,37 +1252,37 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C16" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D16">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E16">
-        <v>57353</v>
+        <v>12927</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
       <c r="G16">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H16">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I16">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J16">
         <v>2</v>
       </c>
       <c r="K16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L16">
-        <v>1.79</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1293,37 +1290,37 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C17" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D17">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="E17">
-        <v>27443</v>
+        <v>2700</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G17">
         <v>2</v>
       </c>
       <c r="H17">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="I17">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="J17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L17">
-        <v>0.9399999999999999</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1331,37 +1328,37 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C18" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D18">
-        <v>46</v>
+        <v>202</v>
       </c>
       <c r="E18">
-        <v>2052</v>
+        <v>4425</v>
       </c>
       <c r="F18">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>189</v>
       </c>
       <c r="J18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L18">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1369,37 +1366,37 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C19" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D19">
-        <v>68</v>
+        <v>170</v>
       </c>
       <c r="E19">
-        <v>22318</v>
+        <v>568</v>
       </c>
       <c r="F19">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>53</v>
+        <v>167</v>
       </c>
       <c r="H19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J19">
         <v>2</v>
       </c>
       <c r="K19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L19">
-        <v>9.93</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1407,37 +1404,37 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C20" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D20">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E20">
-        <v>8258</v>
+        <v>1219</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="H20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J20">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L20">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1445,37 +1442,37 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D21">
-        <v>50</v>
+        <v>112</v>
       </c>
       <c r="E21">
-        <v>440</v>
+        <v>202305</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H21">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I21">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="J21">
         <v>3</v>
       </c>
       <c r="K21" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L21">
-        <v>0.01</v>
+        <v>27.15</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1483,37 +1480,37 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C22" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D22">
-        <v>32</v>
+        <v>432</v>
       </c>
       <c r="E22">
-        <v>1352</v>
+        <v>39000</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>108</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="H22">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="I22">
-        <v>20</v>
+        <v>171</v>
       </c>
       <c r="J22">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="K22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L22">
-        <v>0.05</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1521,37 +1518,37 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C23" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23">
         <v>97</v>
       </c>
-      <c r="D23">
-        <v>26</v>
-      </c>
       <c r="E23">
-        <v>2113275</v>
+        <v>29850</v>
       </c>
       <c r="F23">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="G23">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H23">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="I23">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="J23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K23" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L23">
-        <v>120</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1559,37 +1556,37 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D24">
-        <v>266</v>
+        <v>18</v>
       </c>
       <c r="E24">
-        <v>10173</v>
+        <v>6912</v>
       </c>
       <c r="F24">
-        <v>262</v>
+        <v>1</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H24">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I24">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J24">
         <v>2</v>
       </c>
       <c r="K24" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L24">
-        <v>1.38</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1597,37 +1594,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C25" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D25">
-        <v>29</v>
+        <v>218</v>
       </c>
       <c r="E25">
-        <v>12927</v>
+        <v>11308</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G25">
-        <v>14</v>
+        <v>204</v>
       </c>
       <c r="H25">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K25" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L25">
-        <v>0.68</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1635,37 +1632,37 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C26" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D26">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E26">
-        <v>2700</v>
+        <v>296</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H26">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="I26">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="J26">
         <v>2</v>
       </c>
       <c r="K26" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L26">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1673,37 +1670,37 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C27" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D27">
-        <v>202</v>
+        <v>42</v>
       </c>
       <c r="E27">
-        <v>4425</v>
+        <v>3841029</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="H27">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="I27">
-        <v>189</v>
+        <v>3</v>
       </c>
       <c r="J27">
         <v>3</v>
       </c>
       <c r="K27" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L27">
-        <v>0.1</v>
+        <v>148.44</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1711,37 +1708,37 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C28" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D28">
-        <v>170</v>
+        <v>70</v>
       </c>
       <c r="E28">
-        <v>568</v>
+        <v>19867</v>
       </c>
       <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
         <v>0</v>
       </c>
-      <c r="G28">
-        <v>167</v>
-      </c>
       <c r="H28">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="I28">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="J28">
         <v>2</v>
       </c>
       <c r="K28" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L28">
-        <v>0.64</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1749,37 +1746,37 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C29" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D29">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E29">
-        <v>1219</v>
+        <v>6735507</v>
       </c>
       <c r="F29">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G29">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="H29">
         <v>4</v>
       </c>
       <c r="I29">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K29" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L29">
-        <v>0.15</v>
+        <v>269.25</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1787,37 +1784,37 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C30" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D30">
-        <v>112</v>
+        <v>11</v>
       </c>
       <c r="E30">
-        <v>202305</v>
+        <v>1536</v>
       </c>
       <c r="F30">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G30">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="H30">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I30">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="J30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L30">
-        <v>27.15</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1825,37 +1822,37 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C31" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D31">
-        <v>432</v>
+        <v>16</v>
       </c>
       <c r="E31">
-        <v>39000</v>
+        <v>5288</v>
       </c>
       <c r="F31">
-        <v>108</v>
+        <v>2</v>
       </c>
       <c r="G31">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="H31">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="I31">
-        <v>171</v>
+        <v>9</v>
       </c>
       <c r="J31">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K31" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L31">
-        <v>3.45</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1863,37 +1860,37 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C32" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D32">
-        <v>97</v>
+        <v>12</v>
       </c>
       <c r="E32">
-        <v>29850</v>
+        <v>36922</v>
       </c>
       <c r="F32">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="G32">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H32">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="I32">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="J32">
         <v>3</v>
       </c>
       <c r="K32" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L32">
-        <v>0.95</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1901,37 +1898,37 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C33" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D33">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E33">
-        <v>6912</v>
+        <v>1302</v>
       </c>
       <c r="F33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H33">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I33">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J33">
         <v>2</v>
       </c>
       <c r="K33" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L33">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1939,37 +1936,37 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C34" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D34">
-        <v>218</v>
+        <v>192</v>
       </c>
       <c r="E34">
-        <v>11308</v>
+        <v>154899</v>
       </c>
       <c r="F34">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="G34">
-        <v>204</v>
+        <v>92</v>
       </c>
       <c r="H34">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="I34">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="J34">
         <v>3</v>
       </c>
       <c r="K34" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L34">
-        <v>17.2</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1977,23 +1974,23 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C35" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D35">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E35">
-        <v>296</v>
+        <v>2735</v>
       </c>
       <c r="F35">
+        <v>5</v>
+      </c>
+      <c r="G35">
         <v>0</v>
       </c>
-      <c r="G35">
-        <v>11</v>
-      </c>
       <c r="H35">
         <v>2</v>
       </c>
@@ -2004,10 +2001,10 @@
         <v>2</v>
       </c>
       <c r="K35" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L35">
-        <v>0.02</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -2015,37 +2012,37 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C36" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D36">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="E36">
-        <v>3841029</v>
+        <v>712</v>
       </c>
       <c r="F36">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G36">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="H36">
         <v>4</v>
       </c>
       <c r="I36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K36" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L36">
-        <v>148.44</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -2053,37 +2050,37 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C37" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D37">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="E37">
-        <v>19867</v>
+        <v>81850</v>
       </c>
       <c r="F37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G37">
         <v>0</v>
       </c>
       <c r="H37">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="I37">
-        <v>65</v>
+        <v>3</v>
       </c>
       <c r="J37">
         <v>2</v>
       </c>
       <c r="K37" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L37">
-        <v>0.32</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2091,37 +2088,37 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C38" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D38">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E38">
-        <v>6735507</v>
+        <v>5751408</v>
       </c>
       <c r="F38">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="G38">
         <v>2</v>
       </c>
       <c r="H38">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I38">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J38">
         <v>2</v>
       </c>
       <c r="K38" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L38">
-        <v>269.25</v>
+        <v>293.14</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2129,37 +2126,37 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C39" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D39">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E39">
-        <v>1536</v>
+        <v>668</v>
       </c>
       <c r="F39">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H39">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I39">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J39">
         <v>2</v>
       </c>
       <c r="K39" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L39">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2167,37 +2164,37 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C40" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D40">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E40">
-        <v>5288</v>
+        <v>668</v>
       </c>
       <c r="F40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H40">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I40">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J40">
         <v>2</v>
       </c>
       <c r="K40" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L40">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2205,37 +2202,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C41" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D41">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="E41">
-        <v>36922</v>
+        <v>1079680</v>
       </c>
       <c r="F41">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H41">
+        <v>8</v>
+      </c>
+      <c r="I41">
+        <v>8</v>
+      </c>
+      <c r="J41">
         <v>4</v>
       </c>
-      <c r="I41">
-        <v>5</v>
-      </c>
-      <c r="J41">
-        <v>3</v>
-      </c>
       <c r="K41" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L41">
-        <v>1.03</v>
+        <v>85.38</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2243,22 +2240,22 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C42" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D42">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E42">
-        <v>1302</v>
+        <v>96491</v>
       </c>
       <c r="F42">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G42">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -2270,10 +2267,10 @@
         <v>2</v>
       </c>
       <c r="K42" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L42">
-        <v>0.12</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2281,37 +2278,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C43" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D43">
-        <v>192</v>
+        <v>16</v>
       </c>
       <c r="E43">
-        <v>154899</v>
+        <v>6118</v>
       </c>
       <c r="F43">
-        <v>54</v>
+        <v>9</v>
       </c>
       <c r="G43">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="H43">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="I43">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="J43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K43" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L43">
-        <v>9.67</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2319,37 +2316,37 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C44" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D44">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E44">
-        <v>2735</v>
+        <v>23</v>
       </c>
       <c r="F44">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G44">
+        <v>2</v>
+      </c>
+      <c r="H44">
+        <v>3</v>
+      </c>
+      <c r="I44">
+        <v>2</v>
+      </c>
+      <c r="J44">
+        <v>2</v>
+      </c>
+      <c r="K44" t="s">
+        <v>99</v>
+      </c>
+      <c r="L44">
         <v>0</v>
-      </c>
-      <c r="H44">
-        <v>2</v>
-      </c>
-      <c r="I44">
-        <v>1</v>
-      </c>
-      <c r="J44">
-        <v>2</v>
-      </c>
-      <c r="K44" t="s">
-        <v>100</v>
-      </c>
-      <c r="L44">
-        <v>0.11</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2357,37 +2354,37 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C45" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D45">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="E45">
-        <v>712</v>
+        <v>1249411</v>
       </c>
       <c r="F45">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G45">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H45">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I45">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J45">
         <v>2</v>
       </c>
       <c r="K45" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L45">
-        <v>0.02</v>
+        <v>39.2</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2395,37 +2392,37 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C46" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D46">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E46">
-        <v>81850</v>
+        <v>5647694</v>
       </c>
       <c r="F46">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H46">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I46">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J46">
         <v>2</v>
       </c>
       <c r="K46" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L46">
-        <v>1.96</v>
+        <v>173.9</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2433,37 +2430,37 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C47" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D47">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E47">
-        <v>5751408</v>
+        <v>4395</v>
       </c>
       <c r="F47">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G47">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H47">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I47">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J47">
         <v>2</v>
       </c>
       <c r="K47" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L47">
-        <v>293.14</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2471,37 +2468,37 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C48" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D48">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E48">
-        <v>668</v>
+        <v>1754397</v>
       </c>
       <c r="F48">
+        <v>18</v>
+      </c>
+      <c r="G48">
+        <v>8</v>
+      </c>
+      <c r="H48">
         <v>5</v>
       </c>
-      <c r="G48">
-        <v>3</v>
-      </c>
-      <c r="H48">
-        <v>2</v>
-      </c>
       <c r="I48">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J48">
         <v>2</v>
       </c>
       <c r="K48" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L48">
-        <v>0.05</v>
+        <v>130.3</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2509,37 +2506,37 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C49" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D49">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E49">
-        <v>668</v>
+        <v>11150</v>
       </c>
       <c r="F49">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G49">
         <v>3</v>
       </c>
       <c r="H49">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I49">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J49">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K49" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L49">
-        <v>0.07000000000000001</v>
+        <v>0.6928000000000001</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2547,37 +2544,37 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C50" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D50">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="E50">
-        <v>1079680</v>
+        <v>10324</v>
       </c>
       <c r="F50">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G50">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="H50">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I50">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J50">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K50" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L50">
-        <v>85.38</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2585,37 +2582,37 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C51" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D51">
-        <v>11</v>
+        <v>119</v>
       </c>
       <c r="E51">
-        <v>96491</v>
+        <v>11004</v>
       </c>
       <c r="F51">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G51">
-        <v>1</v>
+        <v>112</v>
       </c>
       <c r="H51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I51">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J51">
         <v>2</v>
       </c>
       <c r="K51" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L51">
-        <v>4.68</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2623,19 +2620,19 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C52" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D52">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E52">
-        <v>6118</v>
+        <v>19297</v>
       </c>
       <c r="F52">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G52">
         <v>2</v>
@@ -2647,13 +2644,13 @@
         <v>3</v>
       </c>
       <c r="J52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K52" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L52">
-        <v>0.36</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2661,37 +2658,37 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C53" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D53">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E53">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="F53">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G53">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H53">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J53">
         <v>2</v>
       </c>
       <c r="K53" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L53">
-        <v>0</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2699,37 +2696,37 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C54" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D54">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E54">
-        <v>1249411</v>
+        <v>171</v>
       </c>
       <c r="F54">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G54">
         <v>9</v>
       </c>
       <c r="H54">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I54">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J54">
         <v>2</v>
       </c>
       <c r="K54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L54">
-        <v>39.2</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2737,37 +2734,37 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C55" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="D55">
         <v>25</v>
       </c>
       <c r="E55">
-        <v>5647694</v>
+        <v>5302</v>
       </c>
       <c r="F55">
+        <v>11</v>
+      </c>
+      <c r="G55">
         <v>9</v>
       </c>
-      <c r="G55">
-        <v>3</v>
-      </c>
       <c r="H55">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I55">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J55">
         <v>2</v>
       </c>
       <c r="K55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L55">
-        <v>173.9</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2775,28 +2772,28 @@
         <v>66</v>
       </c>
       <c r="B56" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C56" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D56">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E56">
-        <v>4395</v>
+        <v>32231279</v>
       </c>
       <c r="F56">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G56">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H56">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I56">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J56">
         <v>2</v>
@@ -2805,7 +2802,7 @@
         <v>100</v>
       </c>
       <c r="L56">
-        <v>0.15</v>
+        <v>937.268</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2813,28 +2810,28 @@
         <v>67</v>
       </c>
       <c r="B57" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C57" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D57">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E57">
-        <v>1754397</v>
+        <v>148021</v>
       </c>
       <c r="F57">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="G57">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H57">
         <v>5</v>
       </c>
       <c r="I57">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J57">
         <v>2</v>
@@ -2843,7 +2840,7 @@
         <v>100</v>
       </c>
       <c r="L57">
-        <v>130.3</v>
+        <v>3.87</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2851,28 +2848,28 @@
         <v>68</v>
       </c>
       <c r="B58" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C58" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D58">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="E58">
-        <v>11150</v>
+        <v>173933</v>
       </c>
       <c r="F58">
         <v>4</v>
       </c>
       <c r="G58">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I58">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J58">
         <v>3</v>
@@ -2881,7 +2878,7 @@
         <v>100</v>
       </c>
       <c r="L58">
-        <v>0.6928000000000001</v>
+        <v>8.081517</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2889,37 +2886,37 @@
         <v>69</v>
       </c>
       <c r="B59" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C59" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D59">
         <v>15</v>
       </c>
       <c r="E59">
-        <v>10324</v>
+        <v>15000713</v>
       </c>
       <c r="F59">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G59">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H59">
         <v>3</v>
       </c>
       <c r="I59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K59" t="s">
         <v>100</v>
       </c>
       <c r="L59">
-        <v>0.37</v>
+        <v>650.54</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2927,28 +2924,28 @@
         <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C60" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D60">
-        <v>119</v>
+        <v>21</v>
       </c>
       <c r="E60">
-        <v>11004</v>
+        <v>2146112</v>
       </c>
       <c r="F60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G60">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="H60">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I60">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J60">
         <v>2</v>
@@ -2957,7 +2954,7 @@
         <v>100</v>
       </c>
       <c r="L60">
-        <v>0.45</v>
+        <v>61.659</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2965,28 +2962,28 @@
         <v>71</v>
       </c>
       <c r="B61" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C61" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D61">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="E61">
-        <v>19297</v>
+        <v>20679117</v>
       </c>
       <c r="F61">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G61">
         <v>2</v>
       </c>
       <c r="H61">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I61">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J61">
         <v>3</v>
@@ -2995,7 +2992,7 @@
         <v>100</v>
       </c>
       <c r="L61">
-        <v>0.6899999999999999</v>
+        <v>1043.242</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -3003,37 +3000,37 @@
         <v>72</v>
       </c>
       <c r="B62" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C62" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D62">
-        <v>13</v>
+        <v>129</v>
       </c>
       <c r="E62">
-        <v>83</v>
+        <v>41328337</v>
       </c>
       <c r="F62">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G62">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="H62">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I62">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K62" t="s">
         <v>100</v>
       </c>
       <c r="L62">
-        <v>0.01</v>
+        <v>3005.995</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -3041,37 +3038,37 @@
         <v>73</v>
       </c>
       <c r="B63" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C63" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D63">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="E63">
-        <v>171</v>
+        <v>74063</v>
       </c>
       <c r="F63">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G63">
+        <v>21</v>
+      </c>
+      <c r="H63">
         <v>9</v>
       </c>
-      <c r="H63">
-        <v>5</v>
-      </c>
       <c r="I63">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="J63">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K63" t="s">
         <v>100</v>
       </c>
       <c r="L63">
-        <v>0.01</v>
+        <v>5.537</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3079,22 +3076,22 @@
         <v>74</v>
       </c>
       <c r="B64" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C64" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D64">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="E64">
-        <v>5302</v>
+        <v>16664809</v>
       </c>
       <c r="F64">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="G64">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H64">
         <v>3</v>
@@ -3109,7 +3106,7 @@
         <v>100</v>
       </c>
       <c r="L64">
-        <v>0.23</v>
+        <v>737.283</v>
       </c>
     </row>
     <row r="65" spans="1:12">
@@ -3117,37 +3114,37 @@
         <v>75</v>
       </c>
       <c r="B65" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C65" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="D65">
-        <v>19</v>
+        <v>221</v>
       </c>
       <c r="E65">
-        <v>32231279</v>
+        <v>13787005</v>
       </c>
       <c r="F65">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="G65">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="H65">
+        <v>13</v>
+      </c>
+      <c r="I65">
+        <v>21</v>
+      </c>
+      <c r="J65">
         <v>6</v>
       </c>
-      <c r="I65">
-        <v>5</v>
-      </c>
-      <c r="J65">
-        <v>2</v>
-      </c>
       <c r="K65" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L65">
-        <v>937.268</v>
+        <v>1736.28</v>
       </c>
     </row>
     <row r="66" spans="1:12">
@@ -3155,37 +3152,37 @@
         <v>76</v>
       </c>
       <c r="B66" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C66" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D66">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="E66">
-        <v>148021</v>
+        <v>4257145</v>
       </c>
       <c r="F66">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="G66">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I66">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J66">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K66" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L66">
-        <v>3.87</v>
+        <v>287.3467</v>
       </c>
     </row>
     <row r="67" spans="1:12">
@@ -3193,37 +3190,37 @@
         <v>77</v>
       </c>
       <c r="B67" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C67" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D67">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="E67">
-        <v>173933</v>
+        <v>4247264</v>
       </c>
       <c r="F67">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G67">
         <v>0</v>
       </c>
       <c r="H67">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I67">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J67">
         <v>3</v>
       </c>
       <c r="K67" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L67">
-        <v>8.081517</v>
+        <v>246.836575</v>
       </c>
     </row>
     <row r="68" spans="1:12">
@@ -3231,37 +3228,37 @@
         <v>78</v>
       </c>
       <c r="B68" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C68" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D68">
+        <v>140</v>
+      </c>
+      <c r="E68">
+        <v>5434924</v>
+      </c>
+      <c r="F68">
+        <v>51</v>
+      </c>
+      <c r="G68">
         <v>15</v>
       </c>
-      <c r="E68">
-        <v>15000713</v>
-      </c>
-      <c r="F68">
-        <v>4</v>
-      </c>
-      <c r="G68">
-        <v>1</v>
-      </c>
       <c r="H68">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="I68">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="J68">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K68" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L68">
-        <v>650.54</v>
+        <v>372.106</v>
       </c>
     </row>
     <row r="69" spans="1:12">
@@ -3269,37 +3266,37 @@
         <v>79</v>
       </c>
       <c r="B69" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C69" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D69">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E69">
-        <v>2146112</v>
+        <v>1018324</v>
       </c>
       <c r="F69">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G69">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H69">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I69">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J69">
         <v>2</v>
       </c>
       <c r="K69" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L69">
-        <v>61.659</v>
+        <v>73.33</v>
       </c>
     </row>
     <row r="70" spans="1:12">
@@ -3307,37 +3304,37 @@
         <v>80</v>
       </c>
       <c r="B70" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C70" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D70">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="E70">
-        <v>20679117</v>
+        <v>429805</v>
       </c>
       <c r="F70">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G70">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H70">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I70">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J70">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K70" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L70">
-        <v>1043.242</v>
+        <v>14.64</v>
       </c>
     </row>
     <row r="71" spans="1:12">
@@ -3348,34 +3345,34 @@
         <v>91</v>
       </c>
       <c r="C71" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D71">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="E71">
-        <v>41328337</v>
+        <v>32561</v>
       </c>
       <c r="F71">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G71">
-        <v>102</v>
+        <v>6</v>
       </c>
       <c r="H71">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I71">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J71">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K71" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L71">
-        <v>3005.995</v>
+        <v>20.848</v>
       </c>
     </row>
     <row r="72" spans="1:12">
@@ -3386,34 +3383,34 @@
         <v>91</v>
       </c>
       <c r="C72" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D72">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="E72">
-        <v>74063</v>
+        <v>20000</v>
       </c>
       <c r="F72">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="G72">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H72">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I72">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J72">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K72" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L72">
-        <v>5.537</v>
+        <v>33.428</v>
       </c>
     </row>
     <row r="73" spans="1:12">
@@ -3424,34 +3421,34 @@
         <v>91</v>
       </c>
       <c r="C73" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D73">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E73">
-        <v>16664809</v>
+        <v>299285</v>
       </c>
       <c r="F73">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G73">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H73">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I73">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K73" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L73">
-        <v>737.283</v>
+        <v>647.349</v>
       </c>
     </row>
     <row r="74" spans="1:12">
@@ -3462,34 +3459,34 @@
         <v>91</v>
       </c>
       <c r="C74" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D74">
-        <v>221</v>
+        <v>20</v>
       </c>
       <c r="E74">
-        <v>13787005</v>
+        <v>20000</v>
       </c>
       <c r="F74">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="G74">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="H74">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="I74">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="J74">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K74" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L74">
-        <v>1736.28</v>
+        <v>24.462</v>
       </c>
     </row>
     <row r="75" spans="1:12">
@@ -3500,34 +3497,34 @@
         <v>91</v>
       </c>
       <c r="C75" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D75">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="E75">
-        <v>4257145</v>
+        <v>581012</v>
       </c>
       <c r="F75">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="G75">
+        <v>54</v>
+      </c>
+      <c r="H75">
+        <v>1</v>
+      </c>
+      <c r="I75">
         <v>0</v>
       </c>
-      <c r="H75">
-        <v>4</v>
-      </c>
-      <c r="I75">
-        <v>6</v>
-      </c>
       <c r="J75">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K75" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L75">
-        <v>287.3467</v>
+        <v>255.645</v>
       </c>
     </row>
     <row r="76" spans="1:12">
@@ -3538,34 +3535,34 @@
         <v>91</v>
       </c>
       <c r="C76" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D76">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="E76">
-        <v>4247264</v>
+        <v>1000</v>
       </c>
       <c r="F76">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G76">
+        <v>5</v>
+      </c>
+      <c r="H76">
+        <v>1</v>
+      </c>
+      <c r="I76">
         <v>0</v>
       </c>
-      <c r="H76">
-        <v>7</v>
-      </c>
-      <c r="I76">
-        <v>10</v>
-      </c>
       <c r="J76">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K76" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L76">
-        <v>246.836575</v>
+        <v>0.444</v>
       </c>
     </row>
     <row r="77" spans="1:12">
@@ -3576,34 +3573,34 @@
         <v>91</v>
       </c>
       <c r="C77" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D77">
-        <v>140</v>
+        <v>27</v>
       </c>
       <c r="E77">
-        <v>5434924</v>
+        <v>20000</v>
       </c>
       <c r="F77">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="G77">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H77">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="I77">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J77">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K77" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L77">
-        <v>372.106</v>
+        <v>24.82</v>
       </c>
     </row>
     <row r="78" spans="1:12">
@@ -3614,34 +3611,34 @@
         <v>91</v>
       </c>
       <c r="C78" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D78">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="E78">
-        <v>1018324</v>
+        <v>494021</v>
       </c>
       <c r="F78">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G78">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="H78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K78" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L78">
-        <v>73.33</v>
+        <v>266.086</v>
       </c>
     </row>
     <row r="79" spans="1:12">
@@ -3652,34 +3649,34 @@
         <v>91</v>
       </c>
       <c r="C79" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D79">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="E79">
-        <v>429805</v>
+        <v>39644</v>
       </c>
       <c r="F79">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G79">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="H79">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I79">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J79">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K79" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L79">
-        <v>14.64</v>
+        <v>18.712</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_08_01_2026) - Modality: multi_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -52,6 +52,33 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>adult</t>
+  </si>
+  <si>
+    <t>alarm</t>
+  </si>
+  <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
+    <t>covtype</t>
+  </si>
+  <si>
+    <t>expedia_hotel_logs</t>
+  </si>
+  <si>
+    <t>insurance</t>
+  </si>
+  <si>
+    <t>intrusion</t>
+  </si>
+  <si>
+    <t>news</t>
+  </si>
+  <si>
     <t>Accidents</t>
   </si>
   <si>
@@ -259,37 +286,19 @@
     <t>walmart</t>
   </si>
   <si>
-    <t>adult</t>
-  </si>
-  <si>
-    <t>alarm</t>
-  </si>
-  <si>
-    <t>census</t>
-  </si>
-  <si>
-    <t>child</t>
-  </si>
-  <si>
-    <t>covtype</t>
-  </si>
-  <si>
-    <t>expedia_hotel_logs</t>
-  </si>
-  <si>
-    <t>insurance</t>
-  </si>
-  <si>
-    <t>intrusion</t>
-  </si>
-  <si>
-    <t>news</t>
+    <t>single_table</t>
   </si>
   <si>
     <t>multi_table</t>
   </si>
   <si>
-    <t>single_table</t>
+    <t>RealTabFormerSynthesizer</t>
+  </si>
+  <si>
+    <t>TVAESynthesizer</t>
+  </si>
+  <si>
+    <t>GaussianCopulaSynthesizer</t>
   </si>
   <si>
     <t>HSASynthesizer</t>
@@ -302,15 +311,6 @@
   </si>
   <si>
     <t>MultiTableUniformSynthesizer</t>
-  </si>
-  <si>
-    <t>RealTabFormerSynthesizer</t>
-  </si>
-  <si>
-    <t>TVAESynthesizer</t>
-  </si>
-  <si>
-    <t>GaussianCopulaSynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -726,31 +726,31 @@
         <v>92</v>
       </c>
       <c r="D2">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="E2">
-        <v>1463093</v>
+        <v>32561</v>
       </c>
       <c r="F2">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2" t="s">
         <v>99</v>
       </c>
       <c r="L2">
-        <v>219.33</v>
+        <v>20.848</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -761,34 +761,34 @@
         <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D3">
-        <v>198</v>
+        <v>37</v>
       </c>
       <c r="E3">
-        <v>12781</v>
+        <v>20000</v>
       </c>
       <c r="F3">
+        <v>37</v>
+      </c>
+      <c r="G3">
         <v>0</v>
       </c>
-      <c r="G3">
-        <v>193</v>
-      </c>
       <c r="H3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" t="s">
         <v>99</v>
       </c>
       <c r="L3">
-        <v>6.62</v>
+        <v>33.428</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -802,31 +802,31 @@
         <v>92</v>
       </c>
       <c r="D4">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="E4">
-        <v>139179</v>
+        <v>299285</v>
       </c>
       <c r="F4">
+        <v>29</v>
+      </c>
+      <c r="G4">
         <v>12</v>
       </c>
-      <c r="G4">
-        <v>57</v>
-      </c>
       <c r="H4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4" t="s">
         <v>99</v>
       </c>
       <c r="L4">
-        <v>31.18</v>
+        <v>647.349</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -837,34 +837,34 @@
         <v>90</v>
       </c>
       <c r="C5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D5">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E5">
-        <v>21895</v>
+        <v>20000</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K5" t="s">
         <v>99</v>
       </c>
       <c r="L5">
-        <v>0.57</v>
+        <v>24.462</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -875,34 +875,34 @@
         <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D6">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="E6">
-        <v>2762</v>
+        <v>581012</v>
       </c>
       <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>54</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
         <v>0</v>
       </c>
-      <c r="G6">
-        <v>7</v>
-      </c>
-      <c r="H6">
-        <v>9</v>
-      </c>
-      <c r="I6">
-        <v>8</v>
-      </c>
       <c r="J6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" t="s">
         <v>99</v>
       </c>
       <c r="L6">
-        <v>0.04</v>
+        <v>255.645</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -913,34 +913,34 @@
         <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D7">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E7">
-        <v>57353</v>
+        <v>1000</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" t="s">
         <v>99</v>
       </c>
       <c r="L7">
-        <v>1.79</v>
+        <v>0.444</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -954,31 +954,31 @@
         <v>93</v>
       </c>
       <c r="D8">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E8">
-        <v>27443</v>
+        <v>20000</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="G8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K8" t="s">
         <v>99</v>
       </c>
       <c r="L8">
-        <v>0.9399999999999999</v>
+        <v>24.82</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -992,31 +992,31 @@
         <v>92</v>
       </c>
       <c r="D9">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E9">
-        <v>2052</v>
+        <v>494021</v>
       </c>
       <c r="F9">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" t="s">
         <v>99</v>
       </c>
       <c r="L9">
-        <v>0.25</v>
+        <v>266.086</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -1030,31 +1030,31 @@
         <v>92</v>
       </c>
       <c r="D10">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E10">
-        <v>22318</v>
+        <v>39644</v>
       </c>
       <c r="F10">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="H10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" t="s">
         <v>99</v>
       </c>
       <c r="L10">
-        <v>9.93</v>
+        <v>18.712</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1062,37 +1062,37 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C11" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D11">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="E11">
-        <v>8258</v>
+        <v>1463093</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K11" t="s">
         <v>99</v>
       </c>
       <c r="L11">
-        <v>0.25</v>
+        <v>1029.07</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1100,37 +1100,37 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C12" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D12">
-        <v>50</v>
+        <v>198</v>
       </c>
       <c r="E12">
-        <v>440</v>
+        <v>12781</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="H12">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I12">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="J12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K12" t="s">
         <v>99</v>
       </c>
       <c r="L12">
-        <v>0.01</v>
+        <v>7.22</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1138,37 +1138,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C13" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D13">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="E13">
-        <v>1352</v>
+        <v>139179</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="H13">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="I13">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="J13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13" t="s">
         <v>99</v>
       </c>
       <c r="L13">
-        <v>0.05</v>
+        <v>57.799</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1176,37 +1176,37 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C14" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D14">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="E14">
-        <v>2113275</v>
+        <v>21895</v>
       </c>
       <c r="F14">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G14">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" t="s">
         <v>99</v>
       </c>
       <c r="L14">
-        <v>120</v>
+        <v>4.414</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1214,28 +1214,28 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D15">
-        <v>266</v>
+        <v>17</v>
       </c>
       <c r="E15">
-        <v>10173</v>
+        <v>2762</v>
       </c>
       <c r="F15">
-        <v>262</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J15">
         <v>2</v>
@@ -1244,7 +1244,7 @@
         <v>99</v>
       </c>
       <c r="L15">
-        <v>1.38</v>
+        <v>0.204</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1252,28 +1252,28 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D16">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E16">
-        <v>12927</v>
+        <v>57353</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
       <c r="G16">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I16">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J16">
         <v>2</v>
@@ -1282,7 +1282,7 @@
         <v>99</v>
       </c>
       <c r="L16">
-        <v>0.68</v>
+        <v>8.178000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1290,37 +1290,37 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C17" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D17">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="E17">
-        <v>2700</v>
+        <v>27443</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G17">
         <v>2</v>
       </c>
       <c r="H17">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="I17">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="J17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17" t="s">
         <v>99</v>
       </c>
       <c r="L17">
-        <v>0.04</v>
+        <v>5.962</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1328,37 +1328,37 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D18">
-        <v>202</v>
+        <v>46</v>
       </c>
       <c r="E18">
-        <v>4425</v>
+        <v>2052</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H18">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="I18">
-        <v>189</v>
+        <v>1</v>
       </c>
       <c r="J18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K18" t="s">
         <v>99</v>
       </c>
       <c r="L18">
-        <v>0.1</v>
+        <v>1.762</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1366,28 +1366,28 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C19" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D19">
-        <v>170</v>
+        <v>68</v>
       </c>
       <c r="E19">
-        <v>568</v>
+        <v>22318</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G19">
-        <v>167</v>
+        <v>53</v>
       </c>
       <c r="H19">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J19">
         <v>2</v>
@@ -1396,7 +1396,7 @@
         <v>99</v>
       </c>
       <c r="L19">
-        <v>0.64</v>
+        <v>17.769</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1404,37 +1404,37 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C20" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D20">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E20">
-        <v>1219</v>
+        <v>8258</v>
       </c>
       <c r="F20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G20">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="H20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I20">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K20" t="s">
         <v>99</v>
       </c>
       <c r="L20">
-        <v>0.15</v>
+        <v>1.072</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1442,28 +1442,28 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C21" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D21">
-        <v>112</v>
+        <v>50</v>
       </c>
       <c r="E21">
-        <v>202305</v>
+        <v>440</v>
       </c>
       <c r="F21">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G21">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="H21">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="I21">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="J21">
         <v>3</v>
@@ -1472,7 +1472,7 @@
         <v>99</v>
       </c>
       <c r="L21">
-        <v>27.15</v>
+        <v>0.08599999999999999</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1480,37 +1480,37 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C22" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D22">
-        <v>432</v>
+        <v>32</v>
       </c>
       <c r="E22">
-        <v>39000</v>
+        <v>1352</v>
       </c>
       <c r="F22">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="G22">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="I22">
-        <v>171</v>
+        <v>20</v>
       </c>
       <c r="J22">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K22" t="s">
         <v>99</v>
       </c>
       <c r="L22">
-        <v>3.45</v>
+        <v>0.266</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1518,37 +1518,37 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C23" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D23">
-        <v>97</v>
+        <v>26</v>
       </c>
       <c r="E23">
-        <v>29850</v>
+        <v>2113275</v>
       </c>
       <c r="F23">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G23">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H23">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="I23">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="J23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K23" t="s">
         <v>99</v>
       </c>
       <c r="L23">
-        <v>0.95</v>
+        <v>409.557</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1556,28 +1556,28 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C24" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D24">
-        <v>18</v>
+        <v>266</v>
       </c>
       <c r="E24">
-        <v>6912</v>
+        <v>10173</v>
       </c>
       <c r="F24">
-        <v>1</v>
+        <v>262</v>
       </c>
       <c r="G24">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H24">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I24">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J24">
         <v>2</v>
@@ -1586,7 +1586,7 @@
         <v>99</v>
       </c>
       <c r="L24">
-        <v>0.11</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1594,37 +1594,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C25" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D25">
-        <v>218</v>
+        <v>29</v>
       </c>
       <c r="E25">
-        <v>11308</v>
+        <v>12927</v>
       </c>
       <c r="F25">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G25">
-        <v>204</v>
+        <v>14</v>
       </c>
       <c r="H25">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K25" t="s">
         <v>99</v>
       </c>
       <c r="L25">
-        <v>17.2</v>
+        <v>1.043</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1632,28 +1632,28 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C26" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D26">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="E26">
-        <v>296</v>
+        <v>2700</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="J26">
         <v>2</v>
@@ -1662,7 +1662,7 @@
         <v>99</v>
       </c>
       <c r="L26">
-        <v>0.02</v>
+        <v>0.237</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1670,28 +1670,28 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C27" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D27">
-        <v>42</v>
+        <v>202</v>
       </c>
       <c r="E27">
-        <v>3841029</v>
+        <v>4425</v>
       </c>
       <c r="F27">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="H27">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="I27">
-        <v>3</v>
+        <v>189</v>
       </c>
       <c r="J27">
         <v>3</v>
@@ -1700,7 +1700,7 @@
         <v>99</v>
       </c>
       <c r="L27">
-        <v>148.44</v>
+        <v>0.829</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1708,28 +1708,28 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C28" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D28">
-        <v>70</v>
+        <v>170</v>
       </c>
       <c r="E28">
-        <v>19867</v>
+        <v>568</v>
       </c>
       <c r="F28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="H28">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="I28">
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="J28">
         <v>2</v>
@@ -1738,7 +1738,7 @@
         <v>99</v>
       </c>
       <c r="L28">
-        <v>0.32</v>
+        <v>0.702</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1746,37 +1746,37 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C29" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D29">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E29">
-        <v>6735507</v>
+        <v>1219</v>
       </c>
       <c r="F29">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G29">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="H29">
         <v>4</v>
       </c>
       <c r="I29">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K29" t="s">
         <v>99</v>
       </c>
       <c r="L29">
-        <v>269.25</v>
+        <v>0.222</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1784,37 +1784,37 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C30" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D30">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="E30">
-        <v>1536</v>
+        <v>202305</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H30">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I30">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="J30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K30" t="s">
         <v>99</v>
       </c>
       <c r="L30">
-        <v>0.04</v>
+        <v>50.824</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1822,37 +1822,37 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C31" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D31">
-        <v>16</v>
+        <v>432</v>
       </c>
       <c r="E31">
-        <v>5288</v>
+        <v>39000</v>
       </c>
       <c r="F31">
-        <v>2</v>
+        <v>108</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="H31">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="I31">
+        <v>171</v>
+      </c>
+      <c r="J31">
         <v>9</v>
       </c>
-      <c r="J31">
-        <v>2</v>
-      </c>
       <c r="K31" t="s">
         <v>99</v>
       </c>
       <c r="L31">
-        <v>0.09</v>
+        <v>26.461</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1860,28 +1860,28 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C32" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D32">
-        <v>12</v>
+        <v>97</v>
       </c>
       <c r="E32">
-        <v>36922</v>
+        <v>29850</v>
       </c>
       <c r="F32">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H32">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="I32">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="J32">
         <v>3</v>
@@ -1890,7 +1890,7 @@
         <v>99</v>
       </c>
       <c r="L32">
-        <v>1.03</v>
+        <v>5.806</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1898,28 +1898,28 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C33" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D33">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E33">
-        <v>1302</v>
+        <v>6912</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I33">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J33">
         <v>2</v>
@@ -1928,7 +1928,7 @@
         <v>99</v>
       </c>
       <c r="L33">
-        <v>0.12</v>
+        <v>0.514</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1936,28 +1936,28 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C34" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D34">
-        <v>192</v>
+        <v>218</v>
       </c>
       <c r="E34">
-        <v>154899</v>
+        <v>11308</v>
       </c>
       <c r="F34">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="G34">
-        <v>92</v>
+        <v>204</v>
       </c>
       <c r="H34">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="I34">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="J34">
         <v>3</v>
@@ -1966,7 +1966,7 @@
         <v>99</v>
       </c>
       <c r="L34">
-        <v>9.67</v>
+        <v>19.145</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1974,22 +1974,22 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C35" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D35">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E35">
-        <v>2735</v>
+        <v>296</v>
       </c>
       <c r="F35">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G35">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H35">
         <v>2</v>
@@ -2004,7 +2004,7 @@
         <v>99</v>
       </c>
       <c r="L35">
-        <v>0.11</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -2012,37 +2012,37 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C36" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D36">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="E36">
-        <v>712</v>
+        <v>3841029</v>
       </c>
       <c r="F36">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G36">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="H36">
         <v>4</v>
       </c>
       <c r="I36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K36" t="s">
         <v>99</v>
       </c>
       <c r="L36">
-        <v>0.02</v>
+        <v>504.868</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -2050,28 +2050,28 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C37" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D37">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="E37">
-        <v>81850</v>
+        <v>19867</v>
       </c>
       <c r="F37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G37">
         <v>0</v>
       </c>
       <c r="H37">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="I37">
-        <v>3</v>
+        <v>65</v>
       </c>
       <c r="J37">
         <v>2</v>
@@ -2080,7 +2080,7 @@
         <v>99</v>
       </c>
       <c r="L37">
-        <v>1.96</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2088,28 +2088,28 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C38" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D38">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E38">
-        <v>5751408</v>
+        <v>6735507</v>
       </c>
       <c r="F38">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G38">
         <v>2</v>
       </c>
       <c r="H38">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I38">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J38">
         <v>2</v>
@@ -2118,7 +2118,7 @@
         <v>99</v>
       </c>
       <c r="L38">
-        <v>293.14</v>
+        <v>272.229</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2126,28 +2126,28 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C39" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D39">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E39">
-        <v>668</v>
+        <v>1536</v>
       </c>
       <c r="F39">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G39">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H39">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I39">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J39">
         <v>2</v>
@@ -2156,7 +2156,7 @@
         <v>99</v>
       </c>
       <c r="L39">
-        <v>0.05</v>
+        <v>0.302</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2164,28 +2164,28 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C40" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D40">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E40">
-        <v>668</v>
+        <v>5288</v>
       </c>
       <c r="F40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H40">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I40">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J40">
         <v>2</v>
@@ -2194,7 +2194,7 @@
         <v>99</v>
       </c>
       <c r="L40">
-        <v>0.07000000000000001</v>
+        <v>0.609</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2202,37 +2202,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C41" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D41">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="E41">
-        <v>1079680</v>
+        <v>36922</v>
       </c>
       <c r="F41">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G41">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H41">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I41">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J41">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K41" t="s">
         <v>99</v>
       </c>
       <c r="L41">
-        <v>85.38</v>
+        <v>8.368</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2240,22 +2240,22 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C42" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D42">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E42">
-        <v>96491</v>
+        <v>1302</v>
       </c>
       <c r="F42">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -2270,7 +2270,7 @@
         <v>99</v>
       </c>
       <c r="L42">
-        <v>4.68</v>
+        <v>0.179</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2278,37 +2278,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C43" t="s">
+        <v>95</v>
+      </c>
+      <c r="D43">
+        <v>192</v>
+      </c>
+      <c r="E43">
+        <v>154899</v>
+      </c>
+      <c r="F43">
+        <v>54</v>
+      </c>
+      <c r="G43">
         <v>92</v>
       </c>
-      <c r="D43">
-        <v>16</v>
-      </c>
-      <c r="E43">
-        <v>6118</v>
-      </c>
-      <c r="F43">
-        <v>9</v>
-      </c>
-      <c r="G43">
-        <v>2</v>
-      </c>
       <c r="H43">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="I43">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="J43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K43" t="s">
         <v>99</v>
       </c>
       <c r="L43">
-        <v>0.36</v>
+        <v>40.634</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2316,28 +2316,28 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C44" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D44">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E44">
-        <v>23</v>
+        <v>2735</v>
       </c>
       <c r="F44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G44">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H44">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I44">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J44">
         <v>2</v>
@@ -2346,7 +2346,7 @@
         <v>99</v>
       </c>
       <c r="L44">
-        <v>0</v>
+        <v>0.6830000000000001</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2354,28 +2354,28 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C45" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D45">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="E45">
-        <v>1249411</v>
+        <v>712</v>
       </c>
       <c r="F45">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G45">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H45">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I45">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J45">
         <v>2</v>
@@ -2384,7 +2384,7 @@
         <v>99</v>
       </c>
       <c r="L45">
-        <v>39.2</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2392,28 +2392,28 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C46" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D46">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="E46">
-        <v>5647694</v>
+        <v>81850</v>
       </c>
       <c r="F46">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G46">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H46">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I46">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J46">
         <v>2</v>
@@ -2422,7 +2422,7 @@
         <v>99</v>
       </c>
       <c r="L46">
-        <v>173.9</v>
+        <v>22.794</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2430,28 +2430,28 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C47" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D47">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E47">
-        <v>4395</v>
+        <v>5751408</v>
       </c>
       <c r="F47">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G47">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H47">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I47">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J47">
         <v>2</v>
@@ -2460,7 +2460,7 @@
         <v>99</v>
       </c>
       <c r="L47">
-        <v>0.15</v>
+        <v>2058.564</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2468,28 +2468,28 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C48" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D48">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E48">
-        <v>1754397</v>
+        <v>668</v>
       </c>
       <c r="F48">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="G48">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H48">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I48">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J48">
         <v>2</v>
@@ -2498,7 +2498,7 @@
         <v>99</v>
       </c>
       <c r="L48">
-        <v>130.3</v>
+        <v>0.308</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2506,37 +2506,37 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C49" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D49">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E49">
-        <v>11150</v>
+        <v>668</v>
       </c>
       <c r="F49">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G49">
         <v>3</v>
       </c>
       <c r="H49">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I49">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K49" t="s">
         <v>99</v>
       </c>
       <c r="L49">
-        <v>0.6928000000000001</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2544,37 +2544,37 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C50" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D50">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="E50">
-        <v>10324</v>
+        <v>1079680</v>
       </c>
       <c r="F50">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="G50">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="H50">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I50">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J50">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K50" t="s">
         <v>99</v>
       </c>
       <c r="L50">
-        <v>0.37</v>
+        <v>336.452</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2582,28 +2582,28 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C51" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D51">
-        <v>119</v>
+        <v>11</v>
       </c>
       <c r="E51">
-        <v>11004</v>
+        <v>96491</v>
       </c>
       <c r="F51">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G51">
-        <v>112</v>
+        <v>1</v>
       </c>
       <c r="H51">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I51">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J51">
         <v>2</v>
@@ -2612,7 +2612,7 @@
         <v>99</v>
       </c>
       <c r="L51">
-        <v>0.45</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2620,19 +2620,19 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C52" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D52">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E52">
-        <v>19297</v>
+        <v>6118</v>
       </c>
       <c r="F52">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G52">
         <v>2</v>
@@ -2644,13 +2644,13 @@
         <v>3</v>
       </c>
       <c r="J52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K52" t="s">
         <v>99</v>
       </c>
       <c r="L52">
-        <v>0.6899999999999999</v>
+        <v>2.908</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2658,28 +2658,28 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C53" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D53">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E53">
-        <v>83</v>
+        <v>23</v>
       </c>
       <c r="F53">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G53">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I53">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J53">
         <v>2</v>
@@ -2688,7 +2688,7 @@
         <v>99</v>
       </c>
       <c r="L53">
-        <v>0.01</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2696,28 +2696,28 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C54" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D54">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E54">
-        <v>171</v>
+        <v>1249411</v>
       </c>
       <c r="F54">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G54">
         <v>9</v>
       </c>
       <c r="H54">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I54">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J54">
         <v>2</v>
@@ -2726,7 +2726,7 @@
         <v>99</v>
       </c>
       <c r="L54">
-        <v>0.01</v>
+        <v>114.714</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2734,28 +2734,28 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C55" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D55">
         <v>25</v>
       </c>
       <c r="E55">
-        <v>5302</v>
+        <v>5647694</v>
       </c>
       <c r="F55">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G55">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H55">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I55">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J55">
         <v>2</v>
@@ -2764,7 +2764,7 @@
         <v>99</v>
       </c>
       <c r="L55">
-        <v>0.23</v>
+        <v>857.134</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2772,37 +2772,37 @@
         <v>66</v>
       </c>
       <c r="B56" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C56" t="s">
         <v>95</v>
       </c>
       <c r="D56">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="E56">
-        <v>32231279</v>
+        <v>4395</v>
       </c>
       <c r="F56">
+        <v>9</v>
+      </c>
+      <c r="G56">
         <v>4</v>
       </c>
-      <c r="G56">
-        <v>2</v>
-      </c>
       <c r="H56">
+        <v>7</v>
+      </c>
+      <c r="I56">
         <v>6</v>
       </c>
-      <c r="I56">
-        <v>5</v>
-      </c>
       <c r="J56">
         <v>2</v>
       </c>
       <c r="K56" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L56">
-        <v>937.268</v>
+        <v>0.772</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2810,37 +2810,37 @@
         <v>67</v>
       </c>
       <c r="B57" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C57" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D57">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E57">
-        <v>148021</v>
+        <v>1754397</v>
       </c>
       <c r="F57">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="G57">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H57">
         <v>5</v>
       </c>
       <c r="I57">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J57">
         <v>2</v>
       </c>
       <c r="K57" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L57">
-        <v>3.87</v>
+        <v>773.989</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2848,37 +2848,37 @@
         <v>68</v>
       </c>
       <c r="B58" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C58" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D58">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E58">
-        <v>173933</v>
+        <v>11150</v>
       </c>
       <c r="F58">
         <v>4</v>
       </c>
       <c r="G58">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H58">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J58">
         <v>3</v>
       </c>
       <c r="K58" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L58">
-        <v>8.081517</v>
+        <v>2.596</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2886,37 +2886,37 @@
         <v>69</v>
       </c>
       <c r="B59" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C59" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D59">
         <v>15</v>
       </c>
       <c r="E59">
-        <v>15000713</v>
+        <v>10324</v>
       </c>
       <c r="F59">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G59">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H59">
         <v>3</v>
       </c>
       <c r="I59">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J59">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K59" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L59">
-        <v>650.54</v>
+        <v>2.065</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2924,37 +2924,37 @@
         <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C60" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D60">
-        <v>21</v>
+        <v>119</v>
       </c>
       <c r="E60">
-        <v>2146112</v>
+        <v>11004</v>
       </c>
       <c r="F60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G60">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="H60">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I60">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J60">
         <v>2</v>
       </c>
       <c r="K60" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L60">
-        <v>61.659</v>
+        <v>1.833</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2962,37 +2962,37 @@
         <v>71</v>
       </c>
       <c r="B61" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C61" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D61">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E61">
-        <v>20679117</v>
+        <v>19297</v>
       </c>
       <c r="F61">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G61">
         <v>2</v>
       </c>
       <c r="H61">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I61">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="J61">
         <v>3</v>
       </c>
       <c r="K61" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L61">
-        <v>1043.242</v>
+        <v>3.573</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -3000,37 +3000,37 @@
         <v>72</v>
       </c>
       <c r="B62" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C62" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D62">
-        <v>129</v>
+        <v>13</v>
       </c>
       <c r="E62">
-        <v>41328337</v>
+        <v>83</v>
       </c>
       <c r="F62">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G62">
-        <v>102</v>
+        <v>4</v>
       </c>
       <c r="H62">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I62">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K62" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L62">
-        <v>3005.995</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -3038,37 +3038,37 @@
         <v>73</v>
       </c>
       <c r="B63" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C63" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D63">
-        <v>67</v>
+        <v>19</v>
       </c>
       <c r="E63">
-        <v>74063</v>
+        <v>171</v>
       </c>
       <c r="F63">
+        <v>1</v>
+      </c>
+      <c r="G63">
+        <v>9</v>
+      </c>
+      <c r="H63">
+        <v>5</v>
+      </c>
+      <c r="I63">
         <v>4</v>
       </c>
-      <c r="G63">
-        <v>21</v>
-      </c>
-      <c r="H63">
-        <v>9</v>
-      </c>
-      <c r="I63">
-        <v>13</v>
-      </c>
       <c r="J63">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K63" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L63">
-        <v>5.537</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3076,22 +3076,22 @@
         <v>74</v>
       </c>
       <c r="B64" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C64" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D64">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="E64">
-        <v>16664809</v>
+        <v>5302</v>
       </c>
       <c r="F64">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H64">
         <v>3</v>
@@ -3103,10 +3103,10 @@
         <v>2</v>
       </c>
       <c r="K64" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L64">
-        <v>737.283</v>
+        <v>1.266</v>
       </c>
     </row>
     <row r="65" spans="1:12">
@@ -3114,37 +3114,37 @@
         <v>75</v>
       </c>
       <c r="B65" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C65" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D65">
-        <v>221</v>
+        <v>19</v>
       </c>
       <c r="E65">
-        <v>13787005</v>
+        <v>32231279</v>
       </c>
       <c r="F65">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="G65">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="H65">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="I65">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="J65">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K65" t="s">
         <v>100</v>
       </c>
       <c r="L65">
-        <v>1736.28</v>
+        <v>969.1849999999999</v>
       </c>
     </row>
     <row r="66" spans="1:12">
@@ -3152,37 +3152,37 @@
         <v>76</v>
       </c>
       <c r="B66" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C66" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D66">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="E66">
-        <v>4257145</v>
+        <v>148021</v>
       </c>
       <c r="F66">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="G66">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H66">
+        <v>5</v>
+      </c>
+      <c r="I66">
         <v>4</v>
       </c>
-      <c r="I66">
-        <v>6</v>
-      </c>
       <c r="J66">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K66" t="s">
         <v>100</v>
       </c>
       <c r="L66">
-        <v>287.3467</v>
+        <v>20.369</v>
       </c>
     </row>
     <row r="67" spans="1:12">
@@ -3190,28 +3190,28 @@
         <v>77</v>
       </c>
       <c r="B67" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C67" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D67">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="E67">
-        <v>4247264</v>
+        <v>173933</v>
       </c>
       <c r="F67">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G67">
         <v>0</v>
       </c>
       <c r="H67">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I67">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J67">
         <v>3</v>
@@ -3220,7 +3220,7 @@
         <v>100</v>
       </c>
       <c r="L67">
-        <v>246.836575</v>
+        <v>40.435</v>
       </c>
     </row>
     <row r="68" spans="1:12">
@@ -3228,37 +3228,37 @@
         <v>78</v>
       </c>
       <c r="B68" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C68" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D68">
-        <v>140</v>
+        <v>15</v>
       </c>
       <c r="E68">
-        <v>5434924</v>
+        <v>15000713</v>
       </c>
       <c r="F68">
-        <v>51</v>
+        <v>4</v>
       </c>
       <c r="G68">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="H68">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="I68">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="J68">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K68" t="s">
         <v>100</v>
       </c>
       <c r="L68">
-        <v>372.106</v>
+        <v>10786.244</v>
       </c>
     </row>
     <row r="69" spans="1:12">
@@ -3266,28 +3266,28 @@
         <v>79</v>
       </c>
       <c r="B69" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C69" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D69">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E69">
-        <v>1018324</v>
+        <v>2146112</v>
       </c>
       <c r="F69">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G69">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H69">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I69">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J69">
         <v>2</v>
@@ -3296,7 +3296,7 @@
         <v>100</v>
       </c>
       <c r="L69">
-        <v>73.33</v>
+        <v>523.1</v>
       </c>
     </row>
     <row r="70" spans="1:12">
@@ -3304,37 +3304,37 @@
         <v>80</v>
       </c>
       <c r="B70" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C70" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D70">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="E70">
-        <v>429805</v>
+        <v>20679117</v>
       </c>
       <c r="F70">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G70">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H70">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I70">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="J70">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K70" t="s">
         <v>100</v>
       </c>
       <c r="L70">
-        <v>14.64</v>
+        <v>2754.622</v>
       </c>
     </row>
     <row r="71" spans="1:12">
@@ -3348,31 +3348,31 @@
         <v>96</v>
       </c>
       <c r="D71">
-        <v>15</v>
+        <v>129</v>
       </c>
       <c r="E71">
-        <v>32561</v>
+        <v>41328337</v>
       </c>
       <c r="F71">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G71">
-        <v>6</v>
+        <v>102</v>
       </c>
       <c r="H71">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I71">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J71">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K71" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L71">
-        <v>20.848</v>
+        <v>4578.511</v>
       </c>
     </row>
     <row r="72" spans="1:12">
@@ -3383,34 +3383,34 @@
         <v>91</v>
       </c>
       <c r="C72" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D72">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="E72">
-        <v>20000</v>
+        <v>74063</v>
       </c>
       <c r="F72">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="G72">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H72">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I72">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J72">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K72" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L72">
-        <v>33.428</v>
+        <v>10.695</v>
       </c>
     </row>
     <row r="73" spans="1:12">
@@ -3421,34 +3421,34 @@
         <v>91</v>
       </c>
       <c r="C73" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D73">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E73">
-        <v>299285</v>
+        <v>16664809</v>
       </c>
       <c r="F73">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G73">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H73">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I73">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K73" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L73">
-        <v>647.349</v>
+        <v>2008.983</v>
       </c>
     </row>
     <row r="74" spans="1:12">
@@ -3462,31 +3462,31 @@
         <v>96</v>
       </c>
       <c r="D74">
-        <v>20</v>
+        <v>221</v>
       </c>
       <c r="E74">
-        <v>20000</v>
+        <v>13787005</v>
       </c>
       <c r="F74">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="G74">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="H74">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="I74">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="J74">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K74" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L74">
-        <v>24.462</v>
+        <v>9343.481</v>
       </c>
     </row>
     <row r="75" spans="1:12">
@@ -3497,34 +3497,34 @@
         <v>91</v>
       </c>
       <c r="C75" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D75">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="E75">
-        <v>581012</v>
+        <v>4257145</v>
       </c>
       <c r="F75">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="G75">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="H75">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I75">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J75">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K75" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L75">
-        <v>255.645</v>
+        <v>748.396</v>
       </c>
     </row>
     <row r="76" spans="1:12">
@@ -3535,34 +3535,34 @@
         <v>91</v>
       </c>
       <c r="C76" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D76">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="E76">
-        <v>1000</v>
+        <v>4247264</v>
       </c>
       <c r="F76">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G76">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H76">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I76">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J76">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K76" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L76">
-        <v>0.444</v>
+        <v>2679.668</v>
       </c>
     </row>
     <row r="77" spans="1:12">
@@ -3573,34 +3573,34 @@
         <v>91</v>
       </c>
       <c r="C77" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D77">
-        <v>27</v>
+        <v>140</v>
       </c>
       <c r="E77">
-        <v>20000</v>
+        <v>5434924</v>
       </c>
       <c r="F77">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="G77">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H77">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="I77">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J77">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K77" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L77">
-        <v>24.82</v>
+        <v>3006.228</v>
       </c>
     </row>
     <row r="78" spans="1:12">
@@ -3614,31 +3614,31 @@
         <v>96</v>
       </c>
       <c r="D78">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="E78">
-        <v>494021</v>
+        <v>1018324</v>
       </c>
       <c r="F78">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G78">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="H78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K78" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L78">
-        <v>266.086</v>
+        <v>184.365</v>
       </c>
     </row>
     <row r="79" spans="1:12">
@@ -3652,31 +3652,31 @@
         <v>96</v>
       </c>
       <c r="D79">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="E79">
-        <v>39644</v>
+        <v>429805</v>
       </c>
       <c r="F79">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G79">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="H79">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I79">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K79" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L79">
-        <v>18.712</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_09_01_2026) - Modality: single_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="102">
   <si>
     <t>Dataset</t>
   </si>
@@ -52,6 +52,213 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>Accidents</t>
+  </si>
+  <si>
+    <t>Atherosclerosis</t>
+  </si>
+  <si>
+    <t>AustralianFootball</t>
+  </si>
+  <si>
+    <t>Biodegradability</t>
+  </si>
+  <si>
+    <t>Bupa</t>
+  </si>
+  <si>
+    <t>CORA</t>
+  </si>
+  <si>
+    <t>Carcinogenesis</t>
+  </si>
+  <si>
+    <t>Chess</t>
+  </si>
+  <si>
+    <t>Countries</t>
+  </si>
+  <si>
+    <t>DCG</t>
+  </si>
+  <si>
+    <t>Dunur</t>
+  </si>
+  <si>
+    <t>Elti</t>
+  </si>
+  <si>
+    <t>FNHK</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>Hepatitis_std</t>
+  </si>
+  <si>
+    <t>Mesh</t>
+  </si>
+  <si>
+    <t>Mooney_Family</t>
+  </si>
+  <si>
+    <t>MuskSmall</t>
+  </si>
+  <si>
+    <t>NBA</t>
+  </si>
+  <si>
+    <t>NCAA</t>
+  </si>
+  <si>
+    <t>OMOP_CDM_dayz</t>
+  </si>
+  <si>
+    <t>PTE</t>
+  </si>
+  <si>
+    <t>Pima</t>
+  </si>
+  <si>
+    <t>PremierLeague</t>
+  </si>
+  <si>
+    <t>Pyrimidine</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>SAT</t>
+  </si>
+  <si>
+    <t>SalesDB</t>
+  </si>
+  <si>
+    <t>Same_gen</t>
+  </si>
+  <si>
+    <t>Student_loan</t>
+  </si>
+  <si>
+    <t>Toxicology</t>
+  </si>
+  <si>
+    <t>Triazine</t>
+  </si>
+  <si>
+    <t>TubePricing</t>
+  </si>
+  <si>
+    <t>UTube</t>
+  </si>
+  <si>
+    <t>UW_std</t>
+  </si>
+  <si>
+    <t>WebKP</t>
+  </si>
+  <si>
+    <t>airbnb-simplified</t>
+  </si>
+  <si>
+    <t>fake_hotels</t>
+  </si>
+  <si>
+    <t>fake_hotels_extended</t>
+  </si>
+  <si>
+    <t>financial</t>
+  </si>
+  <si>
+    <t>ftp</t>
+  </si>
+  <si>
+    <t>genes</t>
+  </si>
+  <si>
+    <t>got_families</t>
+  </si>
+  <si>
+    <t>imdb_MovieLens</t>
+  </si>
+  <si>
+    <t>imdb_ijs</t>
+  </si>
+  <si>
+    <t>imdb_small</t>
+  </si>
+  <si>
+    <t>legalActs</t>
+  </si>
+  <si>
+    <t>multi_table_ID_demo_dataset</t>
+  </si>
+  <si>
+    <t>mutagenesis</t>
+  </si>
+  <si>
+    <t>nations</t>
+  </si>
+  <si>
+    <t>restbase</t>
+  </si>
+  <si>
+    <t>trains</t>
+  </si>
+  <si>
+    <t>university</t>
+  </si>
+  <si>
+    <t>world</t>
+  </si>
+  <si>
+    <t>MovieLens</t>
+  </si>
+  <si>
+    <t>Telstra</t>
+  </si>
+  <si>
+    <t>instacart_marketbasket_ml</t>
+  </si>
+  <si>
+    <t>rel-amazon</t>
+  </si>
+  <si>
+    <t>rel-arxiv</t>
+  </si>
+  <si>
+    <t>rel-avito</t>
+  </si>
+  <si>
+    <t>rel-event</t>
+  </si>
+  <si>
+    <t>rel-f1</t>
+  </si>
+  <si>
+    <t>rel-hm</t>
+  </si>
+  <si>
+    <t>rel-ratebeer</t>
+  </si>
+  <si>
+    <t>rel-salt</t>
+  </si>
+  <si>
+    <t>rel-stack</t>
+  </si>
+  <si>
+    <t>rel-trial</t>
+  </si>
+  <si>
+    <t>rossmann</t>
+  </si>
+  <si>
+    <t>walmart</t>
+  </si>
+  <si>
     <t>adult</t>
   </si>
   <si>
@@ -79,238 +286,34 @@
     <t>news</t>
   </si>
   <si>
-    <t>Accidents</t>
-  </si>
-  <si>
-    <t>Atherosclerosis</t>
-  </si>
-  <si>
-    <t>AustralianFootball</t>
-  </si>
-  <si>
-    <t>Biodegradability</t>
-  </si>
-  <si>
-    <t>Bupa</t>
-  </si>
-  <si>
-    <t>CORA</t>
-  </si>
-  <si>
-    <t>Carcinogenesis</t>
-  </si>
-  <si>
-    <t>Chess</t>
-  </si>
-  <si>
-    <t>Countries</t>
-  </si>
-  <si>
-    <t>DCG</t>
-  </si>
-  <si>
-    <t>Dunur</t>
-  </si>
-  <si>
-    <t>Elti</t>
-  </si>
-  <si>
-    <t>FNHK</t>
-  </si>
-  <si>
-    <t>Facebook</t>
-  </si>
-  <si>
-    <t>Hepatitis_std</t>
-  </si>
-  <si>
-    <t>Mesh</t>
-  </si>
-  <si>
-    <t>Mooney_Family</t>
-  </si>
-  <si>
-    <t>MuskSmall</t>
-  </si>
-  <si>
-    <t>NBA</t>
-  </si>
-  <si>
-    <t>NCAA</t>
-  </si>
-  <si>
-    <t>OMOP_CDM_dayz</t>
-  </si>
-  <si>
-    <t>PTE</t>
-  </si>
-  <si>
-    <t>Pima</t>
-  </si>
-  <si>
-    <t>PremierLeague</t>
-  </si>
-  <si>
-    <t>Pyrimidine</t>
-  </si>
-  <si>
-    <t>SAP</t>
-  </si>
-  <si>
-    <t>SAT</t>
-  </si>
-  <si>
-    <t>SalesDB</t>
-  </si>
-  <si>
-    <t>Same_gen</t>
-  </si>
-  <si>
-    <t>Student_loan</t>
-  </si>
-  <si>
-    <t>Toxicology</t>
-  </si>
-  <si>
-    <t>Triazine</t>
-  </si>
-  <si>
-    <t>TubePricing</t>
-  </si>
-  <si>
-    <t>UTube</t>
-  </si>
-  <si>
-    <t>UW_std</t>
-  </si>
-  <si>
-    <t>WebKP</t>
-  </si>
-  <si>
-    <t>airbnb-simplified</t>
-  </si>
-  <si>
-    <t>fake_hotels</t>
-  </si>
-  <si>
-    <t>fake_hotels_extended</t>
-  </si>
-  <si>
-    <t>financial</t>
-  </si>
-  <si>
-    <t>ftp</t>
-  </si>
-  <si>
-    <t>genes</t>
-  </si>
-  <si>
-    <t>got_families</t>
-  </si>
-  <si>
-    <t>imdb_MovieLens</t>
-  </si>
-  <si>
-    <t>imdb_ijs</t>
-  </si>
-  <si>
-    <t>imdb_small</t>
-  </si>
-  <si>
-    <t>legalActs</t>
-  </si>
-  <si>
-    <t>multi_table_ID_demo_dataset</t>
-  </si>
-  <si>
-    <t>mutagenesis</t>
-  </si>
-  <si>
-    <t>nations</t>
-  </si>
-  <si>
-    <t>restbase</t>
-  </si>
-  <si>
-    <t>trains</t>
-  </si>
-  <si>
-    <t>university</t>
-  </si>
-  <si>
-    <t>world</t>
-  </si>
-  <si>
-    <t>MovieLens</t>
-  </si>
-  <si>
-    <t>Telstra</t>
-  </si>
-  <si>
-    <t>instacart_marketbasket_ml</t>
-  </si>
-  <si>
-    <t>rel-amazon</t>
-  </si>
-  <si>
-    <t>rel-arxiv</t>
-  </si>
-  <si>
-    <t>rel-avito</t>
-  </si>
-  <si>
-    <t>rel-event</t>
-  </si>
-  <si>
-    <t>rel-f1</t>
-  </si>
-  <si>
-    <t>rel-hm</t>
-  </si>
-  <si>
-    <t>rel-ratebeer</t>
-  </si>
-  <si>
-    <t>rel-salt</t>
-  </si>
-  <si>
-    <t>rel-stack</t>
-  </si>
-  <si>
-    <t>rel-trial</t>
-  </si>
-  <si>
-    <t>rossmann</t>
-  </si>
-  <si>
-    <t>walmart</t>
+    <t>multi_table</t>
   </si>
   <si>
     <t>single_table</t>
   </si>
   <si>
-    <t>multi_table</t>
+    <t>HSASynthesizer</t>
+  </si>
+  <si>
+    <t>HMASynthesizer</t>
+  </si>
+  <si>
+    <t>IndependentSynthesizer</t>
+  </si>
+  <si>
+    <t>MultiTableUniformSynthesizer</t>
   </si>
   <si>
     <t>RealTabFormerSynthesizer</t>
   </si>
   <si>
+    <t>TabDDPMSynthesizer</t>
+  </si>
+  <si>
     <t>TVAESynthesizer</t>
   </si>
   <si>
     <t>GaussianCopulaSynthesizer</t>
-  </si>
-  <si>
-    <t>HSASynthesizer</t>
-  </si>
-  <si>
-    <t>HMASynthesizer</t>
-  </si>
-  <si>
-    <t>IndependentSynthesizer</t>
-  </si>
-  <si>
-    <t>MultiTableUniformSynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -726,31 +729,31 @@
         <v>92</v>
       </c>
       <c r="D2">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="E2">
-        <v>32561</v>
+        <v>1463093</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="G2">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L2">
-        <v>20.848</v>
+        <v>1029.07</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -761,34 +764,34 @@
         <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D3">
-        <v>37</v>
+        <v>198</v>
       </c>
       <c r="E3">
-        <v>20000</v>
+        <v>12781</v>
       </c>
       <c r="F3">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L3">
-        <v>33.428</v>
+        <v>7.22</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -802,31 +805,31 @@
         <v>92</v>
       </c>
       <c r="D4">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="E4">
-        <v>299285</v>
+        <v>139179</v>
       </c>
       <c r="F4">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="G4">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L4">
-        <v>647.349</v>
+        <v>57.799</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -837,34 +840,34 @@
         <v>90</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D5">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E5">
-        <v>20000</v>
+        <v>21895</v>
       </c>
       <c r="F5">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L5">
-        <v>24.462</v>
+        <v>4.414</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -875,34 +878,34 @@
         <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D6">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="E6">
-        <v>581012</v>
+        <v>2762</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>54</v>
+        <v>7</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L6">
-        <v>255.645</v>
+        <v>0.204</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -913,34 +916,34 @@
         <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D7">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E7">
-        <v>1000</v>
+        <v>57353</v>
       </c>
       <c r="F7">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L7">
-        <v>0.444</v>
+        <v>8.178000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -954,31 +957,31 @@
         <v>93</v>
       </c>
       <c r="D8">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E8">
-        <v>20000</v>
+        <v>27443</v>
       </c>
       <c r="F8">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L8">
-        <v>24.82</v>
+        <v>5.962</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -992,31 +995,31 @@
         <v>92</v>
       </c>
       <c r="D9">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="E9">
-        <v>494021</v>
+        <v>2052</v>
       </c>
       <c r="F9">
+        <v>39</v>
+      </c>
+      <c r="G9">
         <v>4</v>
       </c>
-      <c r="G9">
-        <v>37</v>
-      </c>
       <c r="H9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L9">
-        <v>266.086</v>
+        <v>1.762</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -1030,31 +1033,31 @@
         <v>92</v>
       </c>
       <c r="D10">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E10">
-        <v>39644</v>
+        <v>22318</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G10">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L10">
-        <v>18.712</v>
+        <v>17.769</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1062,37 +1065,37 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C11" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D11">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="E11">
-        <v>1463093</v>
+        <v>8258</v>
       </c>
       <c r="F11">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="G11">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="H11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L11">
-        <v>1029.07</v>
+        <v>1.072</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1100,37 +1103,37 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C12" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D12">
-        <v>198</v>
+        <v>50</v>
       </c>
       <c r="E12">
-        <v>12781</v>
+        <v>440</v>
       </c>
       <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
         <v>0</v>
       </c>
-      <c r="G12">
-        <v>193</v>
-      </c>
       <c r="H12">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I12">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="J12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L12">
-        <v>7.22</v>
+        <v>0.08599999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1138,37 +1141,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C13" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D13">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="E13">
-        <v>139179</v>
+        <v>1352</v>
       </c>
       <c r="F13">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I13">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="J13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L13">
-        <v>57.799</v>
+        <v>0.266</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1176,37 +1179,37 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C14" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D14">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="E14">
-        <v>21895</v>
+        <v>2113275</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G14">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I14">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L14">
-        <v>4.414</v>
+        <v>409.557</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1214,37 +1217,37 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C15" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D15">
-        <v>17</v>
+        <v>266</v>
       </c>
       <c r="E15">
-        <v>2762</v>
+        <v>10173</v>
       </c>
       <c r="F15">
+        <v>262</v>
+      </c>
+      <c r="G15">
         <v>0</v>
       </c>
-      <c r="G15">
-        <v>7</v>
-      </c>
       <c r="H15">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I15">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J15">
         <v>2</v>
       </c>
       <c r="K15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L15">
-        <v>0.204</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1252,37 +1255,37 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C16" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D16">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E16">
-        <v>57353</v>
+        <v>12927</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
       <c r="G16">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H16">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I16">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J16">
         <v>2</v>
       </c>
       <c r="K16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L16">
-        <v>8.178000000000001</v>
+        <v>1.043</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1290,37 +1293,37 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C17" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D17">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="E17">
-        <v>27443</v>
+        <v>2700</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G17">
         <v>2</v>
       </c>
       <c r="H17">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="I17">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="J17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L17">
-        <v>5.962</v>
+        <v>0.237</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1328,37 +1331,37 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C18" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D18">
-        <v>46</v>
+        <v>202</v>
       </c>
       <c r="E18">
-        <v>2052</v>
+        <v>4425</v>
       </c>
       <c r="F18">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>189</v>
       </c>
       <c r="J18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L18">
-        <v>1.762</v>
+        <v>0.829</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1366,37 +1369,37 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D19">
-        <v>68</v>
+        <v>170</v>
       </c>
       <c r="E19">
-        <v>22318</v>
+        <v>568</v>
       </c>
       <c r="F19">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>53</v>
+        <v>167</v>
       </c>
       <c r="H19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J19">
         <v>2</v>
       </c>
       <c r="K19" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L19">
-        <v>17.769</v>
+        <v>0.702</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1404,37 +1407,37 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C20" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D20">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E20">
-        <v>8258</v>
+        <v>1219</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="H20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J20">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L20">
-        <v>1.072</v>
+        <v>0.222</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1442,37 +1445,37 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D21">
-        <v>50</v>
+        <v>112</v>
       </c>
       <c r="E21">
-        <v>440</v>
+        <v>202305</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H21">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I21">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="J21">
         <v>3</v>
       </c>
       <c r="K21" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L21">
-        <v>0.08599999999999999</v>
+        <v>50.824</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1480,37 +1483,37 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C22" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D22">
-        <v>32</v>
+        <v>432</v>
       </c>
       <c r="E22">
-        <v>1352</v>
+        <v>39000</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>108</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="H22">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="I22">
-        <v>20</v>
+        <v>171</v>
       </c>
       <c r="J22">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="K22" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L22">
-        <v>0.266</v>
+        <v>26.461</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1518,37 +1521,37 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C23" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D23">
-        <v>26</v>
+        <v>97</v>
       </c>
       <c r="E23">
-        <v>2113275</v>
+        <v>29850</v>
       </c>
       <c r="F23">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="G23">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H23">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="I23">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="J23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K23" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L23">
-        <v>409.557</v>
+        <v>5.806</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1556,37 +1559,37 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D24">
-        <v>266</v>
+        <v>18</v>
       </c>
       <c r="E24">
-        <v>10173</v>
+        <v>6912</v>
       </c>
       <c r="F24">
-        <v>262</v>
+        <v>1</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H24">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I24">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J24">
         <v>2</v>
       </c>
       <c r="K24" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L24">
-        <v>1.94</v>
+        <v>0.514</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1594,37 +1597,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C25" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D25">
-        <v>29</v>
+        <v>218</v>
       </c>
       <c r="E25">
-        <v>12927</v>
+        <v>11308</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G25">
-        <v>14</v>
+        <v>204</v>
       </c>
       <c r="H25">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K25" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L25">
-        <v>1.043</v>
+        <v>19.145</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1632,37 +1635,37 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C26" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D26">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E26">
-        <v>2700</v>
+        <v>296</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H26">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="I26">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="J26">
         <v>2</v>
       </c>
       <c r="K26" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L26">
-        <v>0.237</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1670,37 +1673,37 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C27" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D27">
-        <v>202</v>
+        <v>42</v>
       </c>
       <c r="E27">
-        <v>4425</v>
+        <v>3841029</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="H27">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="I27">
-        <v>189</v>
+        <v>3</v>
       </c>
       <c r="J27">
         <v>3</v>
       </c>
       <c r="K27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L27">
-        <v>0.829</v>
+        <v>504.868</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1708,37 +1711,37 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C28" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D28">
-        <v>170</v>
+        <v>70</v>
       </c>
       <c r="E28">
-        <v>568</v>
+        <v>19867</v>
       </c>
       <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
         <v>0</v>
       </c>
-      <c r="G28">
-        <v>167</v>
-      </c>
       <c r="H28">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="I28">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="J28">
         <v>2</v>
       </c>
       <c r="K28" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L28">
-        <v>0.702</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1746,37 +1749,37 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C29" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D29">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E29">
-        <v>1219</v>
+        <v>6735507</v>
       </c>
       <c r="F29">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G29">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="H29">
         <v>4</v>
       </c>
       <c r="I29">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K29" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L29">
-        <v>0.222</v>
+        <v>272.229</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1784,37 +1787,37 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C30" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D30">
-        <v>112</v>
+        <v>11</v>
       </c>
       <c r="E30">
-        <v>202305</v>
+        <v>1536</v>
       </c>
       <c r="F30">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G30">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="H30">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I30">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="J30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L30">
-        <v>50.824</v>
+        <v>0.302</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1822,37 +1825,37 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C31" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D31">
-        <v>432</v>
+        <v>16</v>
       </c>
       <c r="E31">
-        <v>39000</v>
+        <v>5288</v>
       </c>
       <c r="F31">
-        <v>108</v>
+        <v>2</v>
       </c>
       <c r="G31">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="H31">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="I31">
-        <v>171</v>
+        <v>9</v>
       </c>
       <c r="J31">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K31" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L31">
-        <v>26.461</v>
+        <v>0.609</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1860,37 +1863,37 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C32" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D32">
-        <v>97</v>
+        <v>12</v>
       </c>
       <c r="E32">
-        <v>29850</v>
+        <v>36922</v>
       </c>
       <c r="F32">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="G32">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H32">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="I32">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="J32">
         <v>3</v>
       </c>
       <c r="K32" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L32">
-        <v>5.806</v>
+        <v>8.368</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1898,37 +1901,37 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C33" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D33">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E33">
-        <v>6912</v>
+        <v>1302</v>
       </c>
       <c r="F33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H33">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I33">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J33">
         <v>2</v>
       </c>
       <c r="K33" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L33">
-        <v>0.514</v>
+        <v>0.179</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1936,37 +1939,37 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C34" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D34">
-        <v>218</v>
+        <v>192</v>
       </c>
       <c r="E34">
-        <v>11308</v>
+        <v>154899</v>
       </c>
       <c r="F34">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="G34">
-        <v>204</v>
+        <v>92</v>
       </c>
       <c r="H34">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="I34">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="J34">
         <v>3</v>
       </c>
       <c r="K34" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L34">
-        <v>19.145</v>
+        <v>40.634</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1974,23 +1977,23 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C35" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D35">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E35">
-        <v>296</v>
+        <v>2735</v>
       </c>
       <c r="F35">
+        <v>5</v>
+      </c>
+      <c r="G35">
         <v>0</v>
       </c>
-      <c r="G35">
-        <v>11</v>
-      </c>
       <c r="H35">
         <v>2</v>
       </c>
@@ -2001,10 +2004,10 @@
         <v>2</v>
       </c>
       <c r="K35" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L35">
-        <v>0.034</v>
+        <v>0.6830000000000001</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -2012,37 +2015,37 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C36" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D36">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="E36">
-        <v>3841029</v>
+        <v>712</v>
       </c>
       <c r="F36">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G36">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="H36">
         <v>4</v>
       </c>
       <c r="I36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K36" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L36">
-        <v>504.868</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -2050,37 +2053,37 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C37" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D37">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="E37">
-        <v>19867</v>
+        <v>81850</v>
       </c>
       <c r="F37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G37">
         <v>0</v>
       </c>
       <c r="H37">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="I37">
-        <v>65</v>
+        <v>3</v>
       </c>
       <c r="J37">
         <v>2</v>
       </c>
       <c r="K37" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L37">
-        <v>1.38</v>
+        <v>22.794</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2088,37 +2091,37 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C38" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D38">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E38">
-        <v>6735507</v>
+        <v>5751408</v>
       </c>
       <c r="F38">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="G38">
         <v>2</v>
       </c>
       <c r="H38">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I38">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J38">
         <v>2</v>
       </c>
       <c r="K38" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L38">
-        <v>272.229</v>
+        <v>2058.564</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2126,37 +2129,37 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C39" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D39">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E39">
-        <v>1536</v>
+        <v>668</v>
       </c>
       <c r="F39">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H39">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I39">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J39">
         <v>2</v>
       </c>
       <c r="K39" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L39">
-        <v>0.302</v>
+        <v>0.308</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2164,37 +2167,37 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C40" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D40">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E40">
-        <v>5288</v>
+        <v>668</v>
       </c>
       <c r="F40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H40">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I40">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J40">
         <v>2</v>
       </c>
       <c r="K40" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L40">
-        <v>0.609</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2202,37 +2205,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C41" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D41">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="E41">
-        <v>36922</v>
+        <v>1079680</v>
       </c>
       <c r="F41">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H41">
+        <v>8</v>
+      </c>
+      <c r="I41">
+        <v>8</v>
+      </c>
+      <c r="J41">
         <v>4</v>
       </c>
-      <c r="I41">
-        <v>5</v>
-      </c>
-      <c r="J41">
-        <v>3</v>
-      </c>
       <c r="K41" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L41">
-        <v>8.368</v>
+        <v>336.452</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2240,22 +2243,22 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C42" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D42">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E42">
-        <v>1302</v>
+        <v>96491</v>
       </c>
       <c r="F42">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G42">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -2267,10 +2270,10 @@
         <v>2</v>
       </c>
       <c r="K42" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L42">
-        <v>0.179</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2278,37 +2281,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C43" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D43">
-        <v>192</v>
+        <v>16</v>
       </c>
       <c r="E43">
-        <v>154899</v>
+        <v>6118</v>
       </c>
       <c r="F43">
-        <v>54</v>
+        <v>9</v>
       </c>
       <c r="G43">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="H43">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="I43">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="J43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K43" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L43">
-        <v>40.634</v>
+        <v>2.908</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2316,37 +2319,37 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C44" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D44">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E44">
-        <v>2735</v>
+        <v>23</v>
       </c>
       <c r="F44">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G44">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H44">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I44">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J44">
         <v>2</v>
       </c>
       <c r="K44" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L44">
-        <v>0.6830000000000001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2354,37 +2357,37 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C45" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D45">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="E45">
-        <v>712</v>
+        <v>1249411</v>
       </c>
       <c r="F45">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G45">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H45">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I45">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J45">
         <v>2</v>
       </c>
       <c r="K45" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L45">
-        <v>0.091</v>
+        <v>114.714</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2392,37 +2395,37 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C46" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D46">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E46">
-        <v>81850</v>
+        <v>5647694</v>
       </c>
       <c r="F46">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H46">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I46">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J46">
         <v>2</v>
       </c>
       <c r="K46" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L46">
-        <v>22.794</v>
+        <v>857.134</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2430,37 +2433,37 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C47" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D47">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E47">
-        <v>5751408</v>
+        <v>4395</v>
       </c>
       <c r="F47">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G47">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H47">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I47">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J47">
         <v>2</v>
       </c>
       <c r="K47" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L47">
-        <v>2058.564</v>
+        <v>0.772</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2468,37 +2471,37 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C48" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D48">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E48">
-        <v>668</v>
+        <v>1754397</v>
       </c>
       <c r="F48">
+        <v>18</v>
+      </c>
+      <c r="G48">
+        <v>8</v>
+      </c>
+      <c r="H48">
         <v>5</v>
       </c>
-      <c r="G48">
-        <v>3</v>
-      </c>
-      <c r="H48">
-        <v>2</v>
-      </c>
       <c r="I48">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J48">
         <v>2</v>
       </c>
       <c r="K48" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L48">
-        <v>0.308</v>
+        <v>773.989</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2506,37 +2509,37 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C49" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D49">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E49">
-        <v>668</v>
+        <v>11150</v>
       </c>
       <c r="F49">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G49">
         <v>3</v>
       </c>
       <c r="H49">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I49">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J49">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K49" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L49">
-        <v>0.42</v>
+        <v>2.596</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2544,37 +2547,37 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C50" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D50">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="E50">
-        <v>1079680</v>
+        <v>10324</v>
       </c>
       <c r="F50">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G50">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="H50">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I50">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J50">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K50" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L50">
-        <v>336.452</v>
+        <v>2.065</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2582,37 +2585,37 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C51" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D51">
-        <v>11</v>
+        <v>119</v>
       </c>
       <c r="E51">
-        <v>96491</v>
+        <v>11004</v>
       </c>
       <c r="F51">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G51">
-        <v>1</v>
+        <v>112</v>
       </c>
       <c r="H51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I51">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J51">
         <v>2</v>
       </c>
       <c r="K51" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L51">
-        <v>33.67</v>
+        <v>1.833</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2620,19 +2623,19 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C52" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D52">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E52">
-        <v>6118</v>
+        <v>19297</v>
       </c>
       <c r="F52">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G52">
         <v>2</v>
@@ -2644,13 +2647,13 @@
         <v>3</v>
       </c>
       <c r="J52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K52" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L52">
-        <v>2.908</v>
+        <v>3.573</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2658,37 +2661,37 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C53" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D53">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E53">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="F53">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G53">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H53">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J53">
         <v>2</v>
       </c>
       <c r="K53" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L53">
-        <v>0.002</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2696,37 +2699,37 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C54" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D54">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E54">
-        <v>1249411</v>
+        <v>171</v>
       </c>
       <c r="F54">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G54">
         <v>9</v>
       </c>
       <c r="H54">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I54">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J54">
         <v>2</v>
       </c>
       <c r="K54" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L54">
-        <v>114.714</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2734,37 +2737,37 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C55" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D55">
         <v>25</v>
       </c>
       <c r="E55">
-        <v>5647694</v>
+        <v>5302</v>
       </c>
       <c r="F55">
+        <v>11</v>
+      </c>
+      <c r="G55">
         <v>9</v>
       </c>
-      <c r="G55">
-        <v>3</v>
-      </c>
       <c r="H55">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I55">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J55">
         <v>2</v>
       </c>
       <c r="K55" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L55">
-        <v>857.134</v>
+        <v>1.266</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2772,37 +2775,37 @@
         <v>66</v>
       </c>
       <c r="B56" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C56" t="s">
         <v>95</v>
       </c>
       <c r="D56">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E56">
-        <v>4395</v>
+        <v>32231279</v>
       </c>
       <c r="F56">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G56">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H56">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I56">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J56">
         <v>2</v>
       </c>
       <c r="K56" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L56">
-        <v>0.772</v>
+        <v>969.1849999999999</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2810,37 +2813,37 @@
         <v>67</v>
       </c>
       <c r="B57" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C57" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D57">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E57">
-        <v>1754397</v>
+        <v>148021</v>
       </c>
       <c r="F57">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="G57">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H57">
         <v>5</v>
       </c>
       <c r="I57">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J57">
         <v>2</v>
       </c>
       <c r="K57" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L57">
-        <v>773.989</v>
+        <v>20.369</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2848,37 +2851,37 @@
         <v>68</v>
       </c>
       <c r="B58" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C58" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D58">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="E58">
-        <v>11150</v>
+        <v>173933</v>
       </c>
       <c r="F58">
         <v>4</v>
       </c>
       <c r="G58">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I58">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J58">
         <v>3</v>
       </c>
       <c r="K58" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L58">
-        <v>2.596</v>
+        <v>40.435</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2886,37 +2889,37 @@
         <v>69</v>
       </c>
       <c r="B59" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C59" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D59">
         <v>15</v>
       </c>
       <c r="E59">
-        <v>10324</v>
+        <v>15000713</v>
       </c>
       <c r="F59">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G59">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H59">
         <v>3</v>
       </c>
       <c r="I59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K59" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L59">
-        <v>2.065</v>
+        <v>10786.244</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2924,37 +2927,37 @@
         <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C60" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D60">
-        <v>119</v>
+        <v>21</v>
       </c>
       <c r="E60">
-        <v>11004</v>
+        <v>2146112</v>
       </c>
       <c r="F60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G60">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="H60">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I60">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J60">
         <v>2</v>
       </c>
       <c r="K60" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L60">
-        <v>1.833</v>
+        <v>523.1</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2962,37 +2965,37 @@
         <v>71</v>
       </c>
       <c r="B61" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C61" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D61">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="E61">
-        <v>19297</v>
+        <v>20679117</v>
       </c>
       <c r="F61">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G61">
         <v>2</v>
       </c>
       <c r="H61">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I61">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J61">
         <v>3</v>
       </c>
       <c r="K61" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L61">
-        <v>3.573</v>
+        <v>2754.622</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -3000,37 +3003,37 @@
         <v>72</v>
       </c>
       <c r="B62" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C62" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D62">
-        <v>13</v>
+        <v>129</v>
       </c>
       <c r="E62">
-        <v>83</v>
+        <v>41328337</v>
       </c>
       <c r="F62">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G62">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="H62">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I62">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K62" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L62">
-        <v>0.024</v>
+        <v>4578.511</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -3038,37 +3041,37 @@
         <v>73</v>
       </c>
       <c r="B63" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C63" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D63">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="E63">
-        <v>171</v>
+        <v>74063</v>
       </c>
       <c r="F63">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G63">
+        <v>21</v>
+      </c>
+      <c r="H63">
         <v>9</v>
       </c>
-      <c r="H63">
-        <v>5</v>
-      </c>
       <c r="I63">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="J63">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K63" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L63">
-        <v>0.013</v>
+        <v>10.695</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3076,22 +3079,22 @@
         <v>74</v>
       </c>
       <c r="B64" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C64" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D64">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="E64">
-        <v>5302</v>
+        <v>16664809</v>
       </c>
       <c r="F64">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="G64">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H64">
         <v>3</v>
@@ -3103,10 +3106,10 @@
         <v>2</v>
       </c>
       <c r="K64" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L64">
-        <v>1.266</v>
+        <v>2008.983</v>
       </c>
     </row>
     <row r="65" spans="1:12">
@@ -3114,37 +3117,37 @@
         <v>75</v>
       </c>
       <c r="B65" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C65" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="D65">
-        <v>19</v>
+        <v>221</v>
       </c>
       <c r="E65">
-        <v>32231279</v>
+        <v>13787005</v>
       </c>
       <c r="F65">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="G65">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="H65">
+        <v>13</v>
+      </c>
+      <c r="I65">
+        <v>21</v>
+      </c>
+      <c r="J65">
         <v>6</v>
       </c>
-      <c r="I65">
-        <v>5</v>
-      </c>
-      <c r="J65">
-        <v>2</v>
-      </c>
       <c r="K65" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L65">
-        <v>969.1849999999999</v>
+        <v>9343.481</v>
       </c>
     </row>
     <row r="66" spans="1:12">
@@ -3152,37 +3155,37 @@
         <v>76</v>
       </c>
       <c r="B66" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C66" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D66">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="E66">
-        <v>148021</v>
+        <v>4257145</v>
       </c>
       <c r="F66">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="G66">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I66">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J66">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K66" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L66">
-        <v>20.369</v>
+        <v>748.396</v>
       </c>
     </row>
     <row r="67" spans="1:12">
@@ -3190,37 +3193,37 @@
         <v>77</v>
       </c>
       <c r="B67" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C67" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D67">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="E67">
-        <v>173933</v>
+        <v>4247264</v>
       </c>
       <c r="F67">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G67">
         <v>0</v>
       </c>
       <c r="H67">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I67">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J67">
         <v>3</v>
       </c>
       <c r="K67" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L67">
-        <v>40.435</v>
+        <v>2679.668</v>
       </c>
     </row>
     <row r="68" spans="1:12">
@@ -3228,37 +3231,37 @@
         <v>78</v>
       </c>
       <c r="B68" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C68" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D68">
+        <v>140</v>
+      </c>
+      <c r="E68">
+        <v>5434924</v>
+      </c>
+      <c r="F68">
+        <v>51</v>
+      </c>
+      <c r="G68">
         <v>15</v>
       </c>
-      <c r="E68">
-        <v>15000713</v>
-      </c>
-      <c r="F68">
-        <v>4</v>
-      </c>
-      <c r="G68">
-        <v>1</v>
-      </c>
       <c r="H68">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="I68">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="J68">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K68" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L68">
-        <v>10786.244</v>
+        <v>3006.228</v>
       </c>
     </row>
     <row r="69" spans="1:12">
@@ -3266,37 +3269,37 @@
         <v>79</v>
       </c>
       <c r="B69" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C69" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D69">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E69">
-        <v>2146112</v>
+        <v>1018324</v>
       </c>
       <c r="F69">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G69">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H69">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I69">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J69">
         <v>2</v>
       </c>
       <c r="K69" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L69">
-        <v>523.1</v>
+        <v>184.365</v>
       </c>
     </row>
     <row r="70" spans="1:12">
@@ -3304,37 +3307,37 @@
         <v>80</v>
       </c>
       <c r="B70" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C70" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D70">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="E70">
-        <v>20679117</v>
+        <v>429805</v>
       </c>
       <c r="F70">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G70">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H70">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I70">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J70">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K70" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L70">
-        <v>2754.622</v>
+        <v>40</v>
       </c>
     </row>
     <row r="71" spans="1:12">
@@ -3348,31 +3351,31 @@
         <v>96</v>
       </c>
       <c r="D71">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="E71">
-        <v>41328337</v>
+        <v>32561</v>
       </c>
       <c r="F71">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G71">
-        <v>102</v>
+        <v>6</v>
       </c>
       <c r="H71">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I71">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J71">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K71" t="s">
         <v>100</v>
       </c>
       <c r="L71">
-        <v>4578.511</v>
+        <v>20.848</v>
       </c>
     </row>
     <row r="72" spans="1:12">
@@ -3383,34 +3386,34 @@
         <v>91</v>
       </c>
       <c r="C72" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D72">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="E72">
-        <v>74063</v>
+        <v>20000</v>
       </c>
       <c r="F72">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="G72">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H72">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I72">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J72">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K72" t="s">
         <v>100</v>
       </c>
       <c r="L72">
-        <v>10.695</v>
+        <v>33.428</v>
       </c>
     </row>
     <row r="73" spans="1:12">
@@ -3421,34 +3424,34 @@
         <v>91</v>
       </c>
       <c r="C73" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D73">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E73">
-        <v>16664809</v>
+        <v>299285</v>
       </c>
       <c r="F73">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G73">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H73">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I73">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K73" t="s">
         <v>100</v>
       </c>
       <c r="L73">
-        <v>2008.983</v>
+        <v>647.349</v>
       </c>
     </row>
     <row r="74" spans="1:12">
@@ -3459,34 +3462,34 @@
         <v>91</v>
       </c>
       <c r="C74" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D74">
-        <v>221</v>
+        <v>20</v>
       </c>
       <c r="E74">
-        <v>13787005</v>
+        <v>20000</v>
       </c>
       <c r="F74">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="G74">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="H74">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="I74">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="J74">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K74" t="s">
         <v>100</v>
       </c>
       <c r="L74">
-        <v>9343.481</v>
+        <v>24.462</v>
       </c>
     </row>
     <row r="75" spans="1:12">
@@ -3497,34 +3500,34 @@
         <v>91</v>
       </c>
       <c r="C75" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D75">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="E75">
-        <v>4257145</v>
+        <v>581012</v>
       </c>
       <c r="F75">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="G75">
+        <v>54</v>
+      </c>
+      <c r="H75">
+        <v>1</v>
+      </c>
+      <c r="I75">
         <v>0</v>
       </c>
-      <c r="H75">
-        <v>4</v>
-      </c>
-      <c r="I75">
-        <v>6</v>
-      </c>
       <c r="J75">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K75" t="s">
         <v>100</v>
       </c>
       <c r="L75">
-        <v>748.396</v>
+        <v>255.645</v>
       </c>
     </row>
     <row r="76" spans="1:12">
@@ -3535,34 +3538,34 @@
         <v>91</v>
       </c>
       <c r="C76" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D76">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="E76">
-        <v>4247264</v>
+        <v>1000</v>
       </c>
       <c r="F76">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G76">
+        <v>5</v>
+      </c>
+      <c r="H76">
+        <v>1</v>
+      </c>
+      <c r="I76">
         <v>0</v>
       </c>
-      <c r="H76">
-        <v>7</v>
-      </c>
-      <c r="I76">
-        <v>10</v>
-      </c>
       <c r="J76">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K76" t="s">
         <v>100</v>
       </c>
       <c r="L76">
-        <v>2679.668</v>
+        <v>0.444</v>
       </c>
     </row>
     <row r="77" spans="1:12">
@@ -3573,34 +3576,34 @@
         <v>91</v>
       </c>
       <c r="C77" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D77">
-        <v>140</v>
+        <v>27</v>
       </c>
       <c r="E77">
-        <v>5434924</v>
+        <v>20000</v>
       </c>
       <c r="F77">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="G77">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H77">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="I77">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J77">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K77" t="s">
         <v>100</v>
       </c>
       <c r="L77">
-        <v>3006.228</v>
+        <v>24.82</v>
       </c>
     </row>
     <row r="78" spans="1:12">
@@ -3614,31 +3617,31 @@
         <v>96</v>
       </c>
       <c r="D78">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="E78">
-        <v>1018324</v>
+        <v>494021</v>
       </c>
       <c r="F78">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G78">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="H78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K78" t="s">
         <v>100</v>
       </c>
       <c r="L78">
-        <v>184.365</v>
+        <v>266.086</v>
       </c>
     </row>
     <row r="79" spans="1:12">
@@ -3652,31 +3655,31 @@
         <v>96</v>
       </c>
       <c r="D79">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="E79">
-        <v>429805</v>
+        <v>39644</v>
       </c>
       <c r="F79">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G79">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="H79">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I79">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J79">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K79" t="s">
         <v>100</v>
       </c>
       <c r="L79">
-        <v>40</v>
+        <v>18.712</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload SDGym Benchmark Results (SDGym_results_09_02_2026) - Modality: multi_table
</commit_message>
<xml_diff>
--- a/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
+++ b/assets/sdgym-leaderboard-files/Dataset_Details.xlsx
@@ -52,6 +52,33 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>adult</t>
+  </si>
+  <si>
+    <t>alarm</t>
+  </si>
+  <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
+    <t>covtype</t>
+  </si>
+  <si>
+    <t>expedia_hotel_logs</t>
+  </si>
+  <si>
+    <t>insurance</t>
+  </si>
+  <si>
+    <t>intrusion</t>
+  </si>
+  <si>
+    <t>news</t>
+  </si>
+  <si>
     <t>Accidents</t>
   </si>
   <si>
@@ -259,61 +286,34 @@
     <t>walmart</t>
   </si>
   <si>
-    <t>adult</t>
-  </si>
-  <si>
-    <t>alarm</t>
-  </si>
-  <si>
-    <t>census</t>
-  </si>
-  <si>
-    <t>child</t>
-  </si>
-  <si>
-    <t>covtype</t>
-  </si>
-  <si>
-    <t>expedia_hotel_logs</t>
-  </si>
-  <si>
-    <t>insurance</t>
-  </si>
-  <si>
-    <t>intrusion</t>
-  </si>
-  <si>
-    <t>news</t>
+    <t>single_table</t>
   </si>
   <si>
     <t>multi_table</t>
   </si>
   <si>
-    <t>single_table</t>
+    <t>RealTabFormerSynthesizer</t>
+  </si>
+  <si>
+    <t>TabDDPMSynthesizer</t>
+  </si>
+  <si>
+    <t>TVAESynthesizer</t>
+  </si>
+  <si>
+    <t>GaussianCopulaSynthesizer</t>
   </si>
   <si>
     <t>HSASynthesizer</t>
   </si>
   <si>
+    <t>ClavaDDPMSynthesizer</t>
+  </si>
+  <si>
+    <t>IndependentSynthesizer</t>
+  </si>
+  <si>
     <t>HMASynthesizer</t>
-  </si>
-  <si>
-    <t>IndependentSynthesizer</t>
-  </si>
-  <si>
-    <t>MultiTableUniformSynthesizer</t>
-  </si>
-  <si>
-    <t>RealTabFormerSynthesizer</t>
-  </si>
-  <si>
-    <t>TabDDPMSynthesizer</t>
-  </si>
-  <si>
-    <t>TVAESynthesizer</t>
-  </si>
-  <si>
-    <t>GaussianCopulaSynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -729,31 +729,31 @@
         <v>92</v>
       </c>
       <c r="D2">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="E2">
-        <v>1463093</v>
+        <v>32561</v>
       </c>
       <c r="F2">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2" t="s">
         <v>100</v>
       </c>
       <c r="L2">
-        <v>1029.07</v>
+        <v>20.848</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -764,34 +764,34 @@
         <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D3">
-        <v>198</v>
+        <v>37</v>
       </c>
       <c r="E3">
-        <v>12781</v>
+        <v>20000</v>
       </c>
       <c r="F3">
+        <v>37</v>
+      </c>
+      <c r="G3">
         <v>0</v>
       </c>
-      <c r="G3">
-        <v>193</v>
-      </c>
       <c r="H3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" t="s">
         <v>100</v>
       </c>
       <c r="L3">
-        <v>7.22</v>
+        <v>33.428</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -802,34 +802,34 @@
         <v>90</v>
       </c>
       <c r="C4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D4">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="E4">
-        <v>139179</v>
+        <v>299285</v>
       </c>
       <c r="F4">
+        <v>29</v>
+      </c>
+      <c r="G4">
         <v>12</v>
       </c>
-      <c r="G4">
-        <v>57</v>
-      </c>
       <c r="H4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4" t="s">
         <v>100</v>
       </c>
       <c r="L4">
-        <v>57.799</v>
+        <v>647.349</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -843,31 +843,31 @@
         <v>93</v>
       </c>
       <c r="D5">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E5">
-        <v>21895</v>
+        <v>20000</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K5" t="s">
         <v>100</v>
       </c>
       <c r="L5">
-        <v>4.414</v>
+        <v>24.462</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -878,34 +878,34 @@
         <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D6">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="E6">
-        <v>2762</v>
+        <v>581012</v>
       </c>
       <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>54</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
         <v>0</v>
       </c>
-      <c r="G6">
-        <v>7</v>
-      </c>
-      <c r="H6">
-        <v>9</v>
-      </c>
-      <c r="I6">
-        <v>8</v>
-      </c>
       <c r="J6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" t="s">
         <v>100</v>
       </c>
       <c r="L6">
-        <v>0.204</v>
+        <v>255.645</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -916,34 +916,34 @@
         <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D7">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E7">
-        <v>57353</v>
+        <v>1000</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" t="s">
         <v>100</v>
       </c>
       <c r="L7">
-        <v>8.178000000000001</v>
+        <v>0.444</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -957,31 +957,31 @@
         <v>93</v>
       </c>
       <c r="D8">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E8">
-        <v>27443</v>
+        <v>20000</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="G8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K8" t="s">
         <v>100</v>
       </c>
       <c r="L8">
-        <v>5.962</v>
+        <v>24.82</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -995,31 +995,31 @@
         <v>92</v>
       </c>
       <c r="D9">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E9">
-        <v>2052</v>
+        <v>494021</v>
       </c>
       <c r="F9">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" t="s">
         <v>100</v>
       </c>
       <c r="L9">
-        <v>1.762</v>
+        <v>266.086</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -1033,31 +1033,31 @@
         <v>92</v>
       </c>
       <c r="D10">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E10">
-        <v>22318</v>
+        <v>39644</v>
       </c>
       <c r="F10">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="H10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" t="s">
         <v>100</v>
       </c>
       <c r="L10">
-        <v>17.769</v>
+        <v>18.712</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1065,37 +1065,37 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C11" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D11">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="E11">
-        <v>8258</v>
+        <v>1463093</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K11" t="s">
         <v>100</v>
       </c>
       <c r="L11">
-        <v>1.072</v>
+        <v>1029.07</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1103,37 +1103,37 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C12" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D12">
-        <v>50</v>
+        <v>198</v>
       </c>
       <c r="E12">
-        <v>440</v>
+        <v>12781</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="H12">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I12">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="J12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K12" t="s">
         <v>100</v>
       </c>
       <c r="L12">
-        <v>0.08599999999999999</v>
+        <v>7.22</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1141,37 +1141,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C13" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D13">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="E13">
-        <v>1352</v>
+        <v>139179</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="H13">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="I13">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="J13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13" t="s">
         <v>100</v>
       </c>
       <c r="L13">
-        <v>0.266</v>
+        <v>57.799</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1179,37 +1179,37 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C14" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D14">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="E14">
-        <v>2113275</v>
+        <v>21895</v>
       </c>
       <c r="F14">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G14">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" t="s">
         <v>100</v>
       </c>
       <c r="L14">
-        <v>409.557</v>
+        <v>4.414</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1217,28 +1217,28 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D15">
-        <v>266</v>
+        <v>17</v>
       </c>
       <c r="E15">
-        <v>10173</v>
+        <v>2762</v>
       </c>
       <c r="F15">
-        <v>262</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J15">
         <v>2</v>
@@ -1247,7 +1247,7 @@
         <v>100</v>
       </c>
       <c r="L15">
-        <v>1.94</v>
+        <v>0.204</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1255,28 +1255,28 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D16">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E16">
-        <v>12927</v>
+        <v>57353</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
       <c r="G16">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I16">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J16">
         <v>2</v>
@@ -1285,7 +1285,7 @@
         <v>100</v>
       </c>
       <c r="L16">
-        <v>1.043</v>
+        <v>8.178000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1293,37 +1293,37 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C17" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D17">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="E17">
-        <v>2700</v>
+        <v>27443</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G17">
         <v>2</v>
       </c>
       <c r="H17">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="I17">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="J17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17" t="s">
         <v>100</v>
       </c>
       <c r="L17">
-        <v>0.237</v>
+        <v>5.962</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1331,37 +1331,37 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D18">
-        <v>202</v>
+        <v>46</v>
       </c>
       <c r="E18">
-        <v>4425</v>
+        <v>2052</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H18">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="I18">
-        <v>189</v>
+        <v>1</v>
       </c>
       <c r="J18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K18" t="s">
         <v>100</v>
       </c>
       <c r="L18">
-        <v>0.829</v>
+        <v>1.762</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1369,28 +1369,28 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C19" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D19">
-        <v>170</v>
+        <v>68</v>
       </c>
       <c r="E19">
-        <v>568</v>
+        <v>22318</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G19">
-        <v>167</v>
+        <v>53</v>
       </c>
       <c r="H19">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J19">
         <v>2</v>
@@ -1399,7 +1399,7 @@
         <v>100</v>
       </c>
       <c r="L19">
-        <v>0.702</v>
+        <v>17.769</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1407,37 +1407,37 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D20">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E20">
-        <v>1219</v>
+        <v>8258</v>
       </c>
       <c r="F20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G20">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="H20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I20">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K20" t="s">
         <v>100</v>
       </c>
       <c r="L20">
-        <v>0.222</v>
+        <v>1.072</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1445,28 +1445,28 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C21" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D21">
-        <v>112</v>
+        <v>50</v>
       </c>
       <c r="E21">
-        <v>202305</v>
+        <v>440</v>
       </c>
       <c r="F21">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G21">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="H21">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="I21">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="J21">
         <v>3</v>
@@ -1475,7 +1475,7 @@
         <v>100</v>
       </c>
       <c r="L21">
-        <v>50.824</v>
+        <v>0.08599999999999999</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1483,37 +1483,37 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C22" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D22">
-        <v>432</v>
+        <v>32</v>
       </c>
       <c r="E22">
-        <v>39000</v>
+        <v>1352</v>
       </c>
       <c r="F22">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="G22">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="I22">
-        <v>171</v>
+        <v>20</v>
       </c>
       <c r="J22">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K22" t="s">
         <v>100</v>
       </c>
       <c r="L22">
-        <v>26.461</v>
+        <v>0.266</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1521,37 +1521,37 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C23" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="D23">
-        <v>97</v>
+        <v>26</v>
       </c>
       <c r="E23">
-        <v>29850</v>
+        <v>2113275</v>
       </c>
       <c r="F23">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G23">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H23">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="I23">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="J23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K23" t="s">
         <v>100</v>
       </c>
       <c r="L23">
-        <v>5.806</v>
+        <v>409.557</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1559,28 +1559,28 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C24" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D24">
-        <v>18</v>
+        <v>266</v>
       </c>
       <c r="E24">
-        <v>6912</v>
+        <v>10173</v>
       </c>
       <c r="F24">
-        <v>1</v>
+        <v>262</v>
       </c>
       <c r="G24">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H24">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I24">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J24">
         <v>2</v>
@@ -1589,7 +1589,7 @@
         <v>100</v>
       </c>
       <c r="L24">
-        <v>0.514</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1597,37 +1597,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C25" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D25">
-        <v>218</v>
+        <v>29</v>
       </c>
       <c r="E25">
-        <v>11308</v>
+        <v>12927</v>
       </c>
       <c r="F25">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G25">
-        <v>204</v>
+        <v>14</v>
       </c>
       <c r="H25">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K25" t="s">
         <v>100</v>
       </c>
       <c r="L25">
-        <v>19.145</v>
+        <v>1.043</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1635,28 +1635,28 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C26" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D26">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="E26">
-        <v>296</v>
+        <v>2700</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="J26">
         <v>2</v>
@@ -1665,7 +1665,7 @@
         <v>100</v>
       </c>
       <c r="L26">
-        <v>0.034</v>
+        <v>0.237</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1673,28 +1673,28 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C27" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D27">
-        <v>42</v>
+        <v>202</v>
       </c>
       <c r="E27">
-        <v>3841029</v>
+        <v>4425</v>
       </c>
       <c r="F27">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="H27">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="I27">
-        <v>3</v>
+        <v>189</v>
       </c>
       <c r="J27">
         <v>3</v>
@@ -1703,7 +1703,7 @@
         <v>100</v>
       </c>
       <c r="L27">
-        <v>504.868</v>
+        <v>0.829</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1711,28 +1711,28 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C28" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D28">
-        <v>70</v>
+        <v>170</v>
       </c>
       <c r="E28">
-        <v>19867</v>
+        <v>568</v>
       </c>
       <c r="F28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="H28">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="I28">
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="J28">
         <v>2</v>
@@ -1741,7 +1741,7 @@
         <v>100</v>
       </c>
       <c r="L28">
-        <v>1.38</v>
+        <v>0.702</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1749,37 +1749,37 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C29" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D29">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E29">
-        <v>6735507</v>
+        <v>1219</v>
       </c>
       <c r="F29">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G29">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="H29">
         <v>4</v>
       </c>
       <c r="I29">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K29" t="s">
         <v>100</v>
       </c>
       <c r="L29">
-        <v>272.229</v>
+        <v>0.222</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1787,37 +1787,37 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C30" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D30">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="E30">
-        <v>1536</v>
+        <v>202305</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H30">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I30">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="J30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K30" t="s">
         <v>100</v>
       </c>
       <c r="L30">
-        <v>0.302</v>
+        <v>50.824</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1825,37 +1825,37 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C31" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D31">
-        <v>16</v>
+        <v>432</v>
       </c>
       <c r="E31">
-        <v>5288</v>
+        <v>39000</v>
       </c>
       <c r="F31">
-        <v>2</v>
+        <v>108</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="H31">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="I31">
+        <v>171</v>
+      </c>
+      <c r="J31">
         <v>9</v>
       </c>
-      <c r="J31">
-        <v>2</v>
-      </c>
       <c r="K31" t="s">
         <v>100</v>
       </c>
       <c r="L31">
-        <v>0.609</v>
+        <v>26.461</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1863,28 +1863,28 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C32" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D32">
-        <v>12</v>
+        <v>97</v>
       </c>
       <c r="E32">
-        <v>36922</v>
+        <v>29850</v>
       </c>
       <c r="F32">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H32">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="I32">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="J32">
         <v>3</v>
@@ -1893,7 +1893,7 @@
         <v>100</v>
       </c>
       <c r="L32">
-        <v>8.368</v>
+        <v>5.806</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1901,28 +1901,28 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C33" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D33">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E33">
-        <v>1302</v>
+        <v>6912</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I33">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J33">
         <v>2</v>
@@ -1931,7 +1931,7 @@
         <v>100</v>
       </c>
       <c r="L33">
-        <v>0.179</v>
+        <v>0.514</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1939,28 +1939,28 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C34" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D34">
-        <v>192</v>
+        <v>218</v>
       </c>
       <c r="E34">
-        <v>154899</v>
+        <v>11308</v>
       </c>
       <c r="F34">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="G34">
-        <v>92</v>
+        <v>204</v>
       </c>
       <c r="H34">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="I34">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="J34">
         <v>3</v>
@@ -1969,7 +1969,7 @@
         <v>100</v>
       </c>
       <c r="L34">
-        <v>40.634</v>
+        <v>19.145</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1977,22 +1977,22 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C35" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D35">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E35">
-        <v>2735</v>
+        <v>296</v>
       </c>
       <c r="F35">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G35">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H35">
         <v>2</v>
@@ -2007,7 +2007,7 @@
         <v>100</v>
       </c>
       <c r="L35">
-        <v>0.6830000000000001</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -2015,37 +2015,37 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C36" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D36">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="E36">
-        <v>712</v>
+        <v>3841029</v>
       </c>
       <c r="F36">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G36">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="H36">
         <v>4</v>
       </c>
       <c r="I36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K36" t="s">
         <v>100</v>
       </c>
       <c r="L36">
-        <v>0.091</v>
+        <v>504.868</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -2053,28 +2053,28 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C37" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D37">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="E37">
-        <v>81850</v>
+        <v>19867</v>
       </c>
       <c r="F37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G37">
         <v>0</v>
       </c>
       <c r="H37">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="I37">
-        <v>3</v>
+        <v>65</v>
       </c>
       <c r="J37">
         <v>2</v>
@@ -2083,7 +2083,7 @@
         <v>100</v>
       </c>
       <c r="L37">
-        <v>22.794</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2091,28 +2091,28 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C38" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D38">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E38">
-        <v>5751408</v>
+        <v>6735507</v>
       </c>
       <c r="F38">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G38">
         <v>2</v>
       </c>
       <c r="H38">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I38">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J38">
         <v>2</v>
@@ -2121,7 +2121,7 @@
         <v>100</v>
       </c>
       <c r="L38">
-        <v>2058.564</v>
+        <v>272.229</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2129,28 +2129,28 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C39" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D39">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E39">
-        <v>668</v>
+        <v>1536</v>
       </c>
       <c r="F39">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G39">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H39">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I39">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J39">
         <v>2</v>
@@ -2159,7 +2159,7 @@
         <v>100</v>
       </c>
       <c r="L39">
-        <v>0.308</v>
+        <v>0.302</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2167,28 +2167,28 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C40" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D40">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E40">
-        <v>668</v>
+        <v>5288</v>
       </c>
       <c r="F40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H40">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I40">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J40">
         <v>2</v>
@@ -2197,7 +2197,7 @@
         <v>100</v>
       </c>
       <c r="L40">
-        <v>0.42</v>
+        <v>0.609</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2205,37 +2205,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C41" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D41">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="E41">
-        <v>1079680</v>
+        <v>36922</v>
       </c>
       <c r="F41">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G41">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H41">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I41">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J41">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K41" t="s">
         <v>100</v>
       </c>
       <c r="L41">
-        <v>336.452</v>
+        <v>8.368</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2243,22 +2243,22 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C42" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="D42">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E42">
-        <v>96491</v>
+        <v>1302</v>
       </c>
       <c r="F42">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -2273,7 +2273,7 @@
         <v>100</v>
       </c>
       <c r="L42">
-        <v>33.67</v>
+        <v>0.179</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2281,37 +2281,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C43" t="s">
+        <v>98</v>
+      </c>
+      <c r="D43">
+        <v>192</v>
+      </c>
+      <c r="E43">
+        <v>154899</v>
+      </c>
+      <c r="F43">
+        <v>54</v>
+      </c>
+      <c r="G43">
         <v>92</v>
       </c>
-      <c r="D43">
-        <v>16</v>
-      </c>
-      <c r="E43">
-        <v>6118</v>
-      </c>
-      <c r="F43">
-        <v>9</v>
-      </c>
-      <c r="G43">
-        <v>2</v>
-      </c>
       <c r="H43">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="I43">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="J43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K43" t="s">
         <v>100</v>
       </c>
       <c r="L43">
-        <v>2.908</v>
+        <v>40.634</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2319,28 +2319,28 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C44" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D44">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E44">
-        <v>23</v>
+        <v>2735</v>
       </c>
       <c r="F44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G44">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H44">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I44">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J44">
         <v>2</v>
@@ -2349,7 +2349,7 @@
         <v>100</v>
       </c>
       <c r="L44">
-        <v>0.002</v>
+        <v>0.6830000000000001</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2357,28 +2357,28 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C45" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D45">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="E45">
-        <v>1249411</v>
+        <v>712</v>
       </c>
       <c r="F45">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G45">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H45">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I45">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J45">
         <v>2</v>
@@ -2387,7 +2387,7 @@
         <v>100</v>
       </c>
       <c r="L45">
-        <v>114.714</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2395,28 +2395,28 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C46" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D46">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="E46">
-        <v>5647694</v>
+        <v>81850</v>
       </c>
       <c r="F46">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G46">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H46">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I46">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J46">
         <v>2</v>
@@ -2425,7 +2425,7 @@
         <v>100</v>
       </c>
       <c r="L46">
-        <v>857.134</v>
+        <v>22.794</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2433,28 +2433,28 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C47" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D47">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E47">
-        <v>4395</v>
+        <v>5751408</v>
       </c>
       <c r="F47">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G47">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H47">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I47">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J47">
         <v>2</v>
@@ -2463,7 +2463,7 @@
         <v>100</v>
       </c>
       <c r="L47">
-        <v>0.772</v>
+        <v>2058.564</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2471,28 +2471,28 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C48" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D48">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E48">
-        <v>1754397</v>
+        <v>668</v>
       </c>
       <c r="F48">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="G48">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H48">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I48">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J48">
         <v>2</v>
@@ -2501,7 +2501,7 @@
         <v>100</v>
       </c>
       <c r="L48">
-        <v>773.989</v>
+        <v>0.308</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2509,37 +2509,37 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C49" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D49">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E49">
-        <v>11150</v>
+        <v>668</v>
       </c>
       <c r="F49">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G49">
         <v>3</v>
       </c>
       <c r="H49">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I49">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K49" t="s">
         <v>100</v>
       </c>
       <c r="L49">
-        <v>2.596</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2547,37 +2547,37 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C50" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D50">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="E50">
-        <v>10324</v>
+        <v>1079680</v>
       </c>
       <c r="F50">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="G50">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="H50">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I50">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J50">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K50" t="s">
         <v>100</v>
       </c>
       <c r="L50">
-        <v>2.065</v>
+        <v>336.452</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2585,28 +2585,28 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C51" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D51">
-        <v>119</v>
+        <v>11</v>
       </c>
       <c r="E51">
-        <v>11004</v>
+        <v>96491</v>
       </c>
       <c r="F51">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G51">
-        <v>112</v>
+        <v>1</v>
       </c>
       <c r="H51">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I51">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J51">
         <v>2</v>
@@ -2615,7 +2615,7 @@
         <v>100</v>
       </c>
       <c r="L51">
-        <v>1.833</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2623,19 +2623,19 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C52" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D52">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E52">
-        <v>19297</v>
+        <v>6118</v>
       </c>
       <c r="F52">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G52">
         <v>2</v>
@@ -2647,13 +2647,13 @@
         <v>3</v>
       </c>
       <c r="J52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K52" t="s">
         <v>100</v>
       </c>
       <c r="L52">
-        <v>3.573</v>
+        <v>2.908</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2661,28 +2661,28 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C53" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D53">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E53">
-        <v>83</v>
+        <v>23</v>
       </c>
       <c r="F53">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G53">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I53">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J53">
         <v>2</v>
@@ -2691,7 +2691,7 @@
         <v>100</v>
       </c>
       <c r="L53">
-        <v>0.024</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2699,28 +2699,28 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C54" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D54">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E54">
-        <v>171</v>
+        <v>1249411</v>
       </c>
       <c r="F54">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G54">
         <v>9</v>
       </c>
       <c r="H54">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I54">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J54">
         <v>2</v>
@@ -2729,7 +2729,7 @@
         <v>100</v>
       </c>
       <c r="L54">
-        <v>0.013</v>
+        <v>114.714</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2737,28 +2737,28 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C55" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D55">
         <v>25</v>
       </c>
       <c r="E55">
-        <v>5302</v>
+        <v>5647694</v>
       </c>
       <c r="F55">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G55">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H55">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I55">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J55">
         <v>2</v>
@@ -2767,7 +2767,7 @@
         <v>100</v>
       </c>
       <c r="L55">
-        <v>1.266</v>
+        <v>857.134</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2775,37 +2775,37 @@
         <v>66</v>
       </c>
       <c r="B56" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C56" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D56">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="E56">
-        <v>32231279</v>
+        <v>4395</v>
       </c>
       <c r="F56">
+        <v>9</v>
+      </c>
+      <c r="G56">
         <v>4</v>
       </c>
-      <c r="G56">
-        <v>2</v>
-      </c>
       <c r="H56">
+        <v>7</v>
+      </c>
+      <c r="I56">
         <v>6</v>
       </c>
-      <c r="I56">
-        <v>5</v>
-      </c>
       <c r="J56">
         <v>2</v>
       </c>
       <c r="K56" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L56">
-        <v>969.1849999999999</v>
+        <v>0.772</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2813,37 +2813,37 @@
         <v>67</v>
       </c>
       <c r="B57" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C57" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D57">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E57">
-        <v>148021</v>
+        <v>1754397</v>
       </c>
       <c r="F57">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="G57">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H57">
         <v>5</v>
       </c>
       <c r="I57">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J57">
         <v>2</v>
       </c>
       <c r="K57" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L57">
-        <v>20.369</v>
+        <v>773.989</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2851,37 +2851,37 @@
         <v>68</v>
       </c>
       <c r="B58" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C58" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D58">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E58">
-        <v>173933</v>
+        <v>11150</v>
       </c>
       <c r="F58">
         <v>4</v>
       </c>
       <c r="G58">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H58">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J58">
         <v>3</v>
       </c>
       <c r="K58" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L58">
-        <v>40.435</v>
+        <v>2.596</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2889,37 +2889,37 @@
         <v>69</v>
       </c>
       <c r="B59" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C59" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D59">
         <v>15</v>
       </c>
       <c r="E59">
-        <v>15000713</v>
+        <v>10324</v>
       </c>
       <c r="F59">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G59">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H59">
         <v>3</v>
       </c>
       <c r="I59">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J59">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K59" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L59">
-        <v>10786.244</v>
+        <v>2.065</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2927,37 +2927,37 @@
         <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C60" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D60">
-        <v>21</v>
+        <v>119</v>
       </c>
       <c r="E60">
-        <v>2146112</v>
+        <v>11004</v>
       </c>
       <c r="F60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G60">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="H60">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I60">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J60">
         <v>2</v>
       </c>
       <c r="K60" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L60">
-        <v>523.1</v>
+        <v>1.833</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2965,37 +2965,37 @@
         <v>71</v>
       </c>
       <c r="B61" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C61" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D61">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E61">
-        <v>20679117</v>
+        <v>19297</v>
       </c>
       <c r="F61">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G61">
         <v>2</v>
       </c>
       <c r="H61">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I61">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="J61">
         <v>3</v>
       </c>
       <c r="K61" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L61">
-        <v>2754.622</v>
+        <v>3.573</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -3003,37 +3003,37 @@
         <v>72</v>
       </c>
       <c r="B62" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C62" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D62">
-        <v>129</v>
+        <v>13</v>
       </c>
       <c r="E62">
-        <v>41328337</v>
+        <v>83</v>
       </c>
       <c r="F62">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G62">
-        <v>102</v>
+        <v>4</v>
       </c>
       <c r="H62">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I62">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K62" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L62">
-        <v>4578.511</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -3041,37 +3041,37 @@
         <v>73</v>
       </c>
       <c r="B63" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C63" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D63">
-        <v>67</v>
+        <v>19</v>
       </c>
       <c r="E63">
-        <v>74063</v>
+        <v>171</v>
       </c>
       <c r="F63">
+        <v>1</v>
+      </c>
+      <c r="G63">
+        <v>9</v>
+      </c>
+      <c r="H63">
+        <v>5</v>
+      </c>
+      <c r="I63">
         <v>4</v>
       </c>
-      <c r="G63">
-        <v>21</v>
-      </c>
-      <c r="H63">
-        <v>9</v>
-      </c>
-      <c r="I63">
-        <v>13</v>
-      </c>
       <c r="J63">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K63" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L63">
-        <v>10.695</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3079,22 +3079,22 @@
         <v>74</v>
       </c>
       <c r="B64" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C64" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D64">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="E64">
-        <v>16664809</v>
+        <v>5302</v>
       </c>
       <c r="F64">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H64">
         <v>3</v>
@@ -3106,10 +3106,10 @@
         <v>2</v>
       </c>
       <c r="K64" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L64">
-        <v>2008.983</v>
+        <v>1.266</v>
       </c>
     </row>
     <row r="65" spans="1:12">
@@ -3117,37 +3117,37 @@
         <v>75</v>
       </c>
       <c r="B65" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C65" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D65">
-        <v>221</v>
+        <v>19</v>
       </c>
       <c r="E65">
-        <v>13787005</v>
+        <v>32231279</v>
       </c>
       <c r="F65">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="G65">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="H65">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="I65">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="J65">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K65" t="s">
         <v>101</v>
       </c>
       <c r="L65">
-        <v>9343.481</v>
+        <v>969.1849999999999</v>
       </c>
     </row>
     <row r="66" spans="1:12">
@@ -3155,37 +3155,37 @@
         <v>76</v>
       </c>
       <c r="B66" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C66" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D66">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="E66">
-        <v>4257145</v>
+        <v>148021</v>
       </c>
       <c r="F66">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="G66">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H66">
+        <v>5</v>
+      </c>
+      <c r="I66">
         <v>4</v>
       </c>
-      <c r="I66">
-        <v>6</v>
-      </c>
       <c r="J66">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K66" t="s">
         <v>101</v>
       </c>
       <c r="L66">
-        <v>748.396</v>
+        <v>20.369</v>
       </c>
     </row>
     <row r="67" spans="1:12">
@@ -3193,28 +3193,28 @@
         <v>77</v>
       </c>
       <c r="B67" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C67" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D67">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="E67">
-        <v>4247264</v>
+        <v>173933</v>
       </c>
       <c r="F67">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G67">
         <v>0</v>
       </c>
       <c r="H67">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I67">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J67">
         <v>3</v>
@@ -3223,7 +3223,7 @@
         <v>101</v>
       </c>
       <c r="L67">
-        <v>2679.668</v>
+        <v>40.435</v>
       </c>
     </row>
     <row r="68" spans="1:12">
@@ -3231,37 +3231,37 @@
         <v>78</v>
       </c>
       <c r="B68" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C68" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D68">
-        <v>140</v>
+        <v>15</v>
       </c>
       <c r="E68">
-        <v>5434924</v>
+        <v>15000713</v>
       </c>
       <c r="F68">
-        <v>51</v>
+        <v>4</v>
       </c>
       <c r="G68">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="H68">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="I68">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="J68">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K68" t="s">
         <v>101</v>
       </c>
       <c r="L68">
-        <v>3006.228</v>
+        <v>10786.244</v>
       </c>
     </row>
     <row r="69" spans="1:12">
@@ -3269,28 +3269,28 @@
         <v>79</v>
       </c>
       <c r="B69" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C69" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D69">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E69">
-        <v>1018324</v>
+        <v>2146112</v>
       </c>
       <c r="F69">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G69">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H69">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I69">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J69">
         <v>2</v>
@@ -3299,7 +3299,7 @@
         <v>101</v>
       </c>
       <c r="L69">
-        <v>184.365</v>
+        <v>523.1</v>
       </c>
     </row>
     <row r="70" spans="1:12">
@@ -3307,37 +3307,37 @@
         <v>80</v>
       </c>
       <c r="B70" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C70" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D70">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="E70">
-        <v>429805</v>
+        <v>20679117</v>
       </c>
       <c r="F70">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G70">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H70">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I70">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="J70">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K70" t="s">
         <v>101</v>
       </c>
       <c r="L70">
-        <v>40</v>
+        <v>2754.622</v>
       </c>
     </row>
     <row r="71" spans="1:12">
@@ -3348,34 +3348,34 @@
         <v>91</v>
       </c>
       <c r="C71" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D71">
-        <v>15</v>
+        <v>129</v>
       </c>
       <c r="E71">
-        <v>32561</v>
+        <v>41328337</v>
       </c>
       <c r="F71">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G71">
-        <v>6</v>
+        <v>102</v>
       </c>
       <c r="H71">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I71">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J71">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K71" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L71">
-        <v>20.848</v>
+        <v>4578.511</v>
       </c>
     </row>
     <row r="72" spans="1:12">
@@ -3386,34 +3386,34 @@
         <v>91</v>
       </c>
       <c r="C72" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D72">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="E72">
-        <v>20000</v>
+        <v>74063</v>
       </c>
       <c r="F72">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="G72">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H72">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I72">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J72">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K72" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L72">
-        <v>33.428</v>
+        <v>10.695</v>
       </c>
     </row>
     <row r="73" spans="1:12">
@@ -3427,31 +3427,31 @@
         <v>98</v>
       </c>
       <c r="D73">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E73">
-        <v>299285</v>
+        <v>16664809</v>
       </c>
       <c r="F73">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G73">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H73">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I73">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K73" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L73">
-        <v>647.349</v>
+        <v>2008.983</v>
       </c>
     </row>
     <row r="74" spans="1:12">
@@ -3465,31 +3465,31 @@
         <v>97</v>
       </c>
       <c r="D74">
-        <v>20</v>
+        <v>221</v>
       </c>
       <c r="E74">
-        <v>20000</v>
+        <v>13787005</v>
       </c>
       <c r="F74">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="G74">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="H74">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="I74">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="J74">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K74" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L74">
-        <v>24.462</v>
+        <v>9343.481</v>
       </c>
     </row>
     <row r="75" spans="1:12">
@@ -3500,34 +3500,34 @@
         <v>91</v>
       </c>
       <c r="C75" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D75">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="E75">
-        <v>581012</v>
+        <v>4257145</v>
       </c>
       <c r="F75">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="G75">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="H75">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I75">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J75">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K75" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L75">
-        <v>255.645</v>
+        <v>748.396</v>
       </c>
     </row>
     <row r="76" spans="1:12">
@@ -3538,34 +3538,34 @@
         <v>91</v>
       </c>
       <c r="C76" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D76">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="E76">
-        <v>1000</v>
+        <v>4247264</v>
       </c>
       <c r="F76">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G76">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H76">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I76">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J76">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K76" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L76">
-        <v>0.444</v>
+        <v>2679.668</v>
       </c>
     </row>
     <row r="77" spans="1:12">
@@ -3576,34 +3576,34 @@
         <v>91</v>
       </c>
       <c r="C77" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D77">
-        <v>27</v>
+        <v>140</v>
       </c>
       <c r="E77">
-        <v>20000</v>
+        <v>5434924</v>
       </c>
       <c r="F77">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="G77">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H77">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="I77">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J77">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K77" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L77">
-        <v>24.82</v>
+        <v>3006.228</v>
       </c>
     </row>
     <row r="78" spans="1:12">
@@ -3614,34 +3614,34 @@
         <v>91</v>
       </c>
       <c r="C78" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D78">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="E78">
-        <v>494021</v>
+        <v>1018324</v>
       </c>
       <c r="F78">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G78">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="H78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K78" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L78">
-        <v>266.086</v>
+        <v>184.365</v>
       </c>
     </row>
     <row r="79" spans="1:12">
@@ -3652,34 +3652,34 @@
         <v>91</v>
       </c>
       <c r="C79" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D79">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="E79">
-        <v>39644</v>
+        <v>429805</v>
       </c>
       <c r="F79">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G79">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="H79">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I79">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K79" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L79">
-        <v>18.712</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>